<commit_message>
Mise à jour automatique 2026-07-22
</commit_message>
<xml_diff>
--- a/maxit_store_history.xlsx
+++ b/maxit_store_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U449"/>
+  <dimension ref="A1:U481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35833,7 +35833,6 @@
       <c r="O418" t="n">
         <v>20</v>
       </c>
-      <c r="P418" t="inlineStr"/>
       <c r="Q418" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -35854,7 +35853,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U418" t="inlineStr"/>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
@@ -35917,7 +35915,6 @@
       <c r="N419" t="n">
         <v>319</v>
       </c>
-      <c r="P419" t="inlineStr"/>
       <c r="R419" t="inlineStr">
         <is>
           <t>6.4.8</t>
@@ -35933,7 +35930,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U419" t="inlineStr"/>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
@@ -36003,7 +35999,6 @@
       <c r="O420" t="n">
         <v>38</v>
       </c>
-      <c r="P420" t="inlineStr"/>
       <c r="Q420" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -36024,7 +36019,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U420" t="inlineStr"/>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
@@ -36090,7 +36084,6 @@
       <c r="O421" t="n">
         <v>38</v>
       </c>
-      <c r="P421" t="inlineStr"/>
       <c r="R421" t="inlineStr">
         <is>
           <t>10.0.6</t>
@@ -36108,7 +36101,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U421" t="inlineStr"/>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
@@ -36178,7 +36170,6 @@
       <c r="O422" t="n">
         <v>11</v>
       </c>
-      <c r="P422" t="inlineStr"/>
       <c r="Q422" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -36199,7 +36190,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U422" t="inlineStr"/>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
@@ -36288,7 +36278,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U423" t="inlineStr"/>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
@@ -36358,7 +36347,6 @@
       <c r="O424" t="n">
         <v>12</v>
       </c>
-      <c r="P424" t="inlineStr"/>
       <c r="Q424" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -36379,7 +36367,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U424" t="inlineStr"/>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
@@ -36445,7 +36432,6 @@
       <c r="O425" t="n">
         <v>8</v>
       </c>
-      <c r="P425" t="inlineStr"/>
       <c r="R425" t="inlineStr">
         <is>
           <t>21.1.0</t>
@@ -36463,7 +36449,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U425" t="inlineStr"/>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
@@ -36533,7 +36518,6 @@
       <c r="O426" t="n">
         <v>139</v>
       </c>
-      <c r="P426" t="inlineStr"/>
       <c r="Q426" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -36554,7 +36538,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U426" t="inlineStr"/>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
@@ -36639,7 +36622,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U427" t="inlineStr"/>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
@@ -36706,7 +36688,6 @@
       <c r="N428" t="n">
         <v>38259</v>
       </c>
-      <c r="P428" t="inlineStr"/>
       <c r="Q428" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -36727,7 +36708,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U428" t="inlineStr"/>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -36793,7 +36773,6 @@
       <c r="O429" t="n">
         <v>3</v>
       </c>
-      <c r="P429" t="inlineStr"/>
       <c r="R429" t="inlineStr">
         <is>
           <t>6.5.2</t>
@@ -36812,7 +36791,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U429" t="inlineStr"/>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
@@ -36882,7 +36860,6 @@
       <c r="O430" t="n">
         <v>26</v>
       </c>
-      <c r="P430" t="inlineStr"/>
       <c r="Q430" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -36903,7 +36880,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U430" t="inlineStr"/>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
@@ -36969,7 +36945,6 @@
       <c r="O431" t="n">
         <v>6</v>
       </c>
-      <c r="P431" t="inlineStr"/>
       <c r="R431" t="inlineStr">
         <is>
           <t>5.0.2</t>
@@ -36987,7 +36962,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U431" t="inlineStr"/>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
@@ -37057,7 +37031,6 @@
       <c r="O432" t="n">
         <v>109</v>
       </c>
-      <c r="P432" t="inlineStr"/>
       <c r="Q432" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -37078,7 +37051,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U432" t="inlineStr"/>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
@@ -37166,7 +37138,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U433" t="inlineStr"/>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
@@ -37236,7 +37207,6 @@
       <c r="O434" t="n">
         <v>62</v>
       </c>
-      <c r="P434" t="inlineStr"/>
       <c r="Q434" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -37257,7 +37227,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U434" t="inlineStr"/>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
@@ -37323,7 +37292,6 @@
       <c r="O435" t="n">
         <v>39</v>
       </c>
-      <c r="P435" t="inlineStr"/>
       <c r="R435" t="inlineStr">
         <is>
           <t>10.0.21</t>
@@ -37342,7 +37310,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U435" t="inlineStr"/>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
@@ -37412,7 +37379,6 @@
       <c r="O436" t="n">
         <v>11</v>
       </c>
-      <c r="P436" t="inlineStr"/>
       <c r="Q436" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -37433,7 +37399,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U436" t="inlineStr"/>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
@@ -37519,7 +37484,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U437" t="inlineStr"/>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -37589,7 +37553,6 @@
       <c r="O438" t="n">
         <v>16</v>
       </c>
-      <c r="P438" t="inlineStr"/>
       <c r="Q438" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -37610,7 +37573,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U438" t="inlineStr"/>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
@@ -37696,7 +37658,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U439" t="inlineStr"/>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
@@ -37766,7 +37727,6 @@
       <c r="O440" t="n">
         <v>89</v>
       </c>
-      <c r="P440" t="inlineStr"/>
       <c r="Q440" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -37787,7 +37747,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U440" t="inlineStr"/>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
@@ -37870,7 +37829,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U441" t="inlineStr"/>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
@@ -37940,7 +37898,6 @@
       <c r="O442" t="n">
         <v>12</v>
       </c>
-      <c r="P442" t="inlineStr"/>
       <c r="Q442" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -37961,7 +37918,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U442" t="inlineStr"/>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
@@ -38050,7 +38006,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U443" t="inlineStr"/>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
@@ -38120,7 +38075,6 @@
       <c r="O444" t="n">
         <v>13</v>
       </c>
-      <c r="P444" t="inlineStr"/>
       <c r="Q444" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -38141,7 +38095,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U444" t="inlineStr"/>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
@@ -38228,7 +38181,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U445" t="inlineStr"/>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
@@ -38298,7 +38250,6 @@
       <c r="O446" t="n">
         <v>47</v>
       </c>
-      <c r="P446" t="inlineStr"/>
       <c r="Q446" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -38319,7 +38270,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U446" t="inlineStr"/>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
@@ -38385,7 +38335,6 @@
       <c r="O447" t="n">
         <v>44</v>
       </c>
-      <c r="P447" t="inlineStr"/>
       <c r="R447" t="inlineStr">
         <is>
           <t>7.3.1</t>
@@ -38406,7 +38355,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U447" t="inlineStr"/>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
@@ -38476,7 +38424,6 @@
       <c r="O448" t="n">
         <v>22</v>
       </c>
-      <c r="P448" t="inlineStr"/>
       <c r="Q448" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -38497,7 +38444,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U448" t="inlineStr"/>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
@@ -38563,7 +38509,6 @@
       <c r="O449" t="n">
         <v>60</v>
       </c>
-      <c r="P449" t="inlineStr"/>
       <c r="R449" t="inlineStr">
         <is>
           <t>10.1.0</t>
@@ -38582,7 +38527,2825 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U449" t="inlineStr"/>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogn</t>
+        </is>
+      </c>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J450" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K450" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L450" t="b">
+        <v>0</v>
+      </c>
+      <c r="M450" t="n">
+        <v>4.443459</v>
+      </c>
+      <c r="N450" t="n">
+        <v>9210</v>
+      </c>
+      <c r="O450" t="n">
+        <v>15</v>
+      </c>
+      <c r="P450" t="inlineStr"/>
+      <c r="Q450" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R450" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S450" t="inlineStr">
+        <is>
+          <t>Bien plus qu&amp;#39;une application, un véritable assistant personnel pour une vie connectée et simplifiée.&lt;br&gt;Suivi de consommation: Votre tableau de bord tout-en-un pour une gestion simplifiée !&lt;br&gt;- Gestion de votre offre: Accédez à une vue détaillée de votre offre actuelle et de vos forfaits Orange</t>
+        </is>
+      </c>
+      <c r="T450" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U450" t="inlineStr"/>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G451" t="n">
+        <v>1177999485</v>
+      </c>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K451" t="n">
+        <v>0</v>
+      </c>
+      <c r="L451" t="b">
+        <v>1</v>
+      </c>
+      <c r="M451" t="n">
+        <v>3.89969</v>
+      </c>
+      <c r="N451" t="n">
+        <v>319</v>
+      </c>
+      <c r="P451" t="inlineStr"/>
+      <c r="R451" t="inlineStr">
+        <is>
+          <t>6.4.8</t>
+        </is>
+      </c>
+      <c r="S451" t="inlineStr">
+        <is>
+          <t>La fusion d’Orange et Moi et Orange Money donne naissance à Max it, la nouvelle Super Application Tout-en-Un. Profitez du suivi de consommation, de paiements mobiles, de toutes les fonctionnalités Orange et Moi et Money avec un large éventail de divertissements, le tout regroupé en un seul endroit !</t>
+        </is>
+      </c>
+      <c r="T451" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U451" t="inlineStr"/>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.otn</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J452" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K452" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L452" t="b">
+        <v>0</v>
+      </c>
+      <c r="M452" t="n">
+        <v>3.970176</v>
+      </c>
+      <c r="N452" t="n">
+        <v>35355</v>
+      </c>
+      <c r="O452" t="n">
+        <v>36</v>
+      </c>
+      <c r="P452" t="inlineStr"/>
+      <c r="Q452" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R452" t="inlineStr">
+        <is>
+          <t>10.0.6</t>
+        </is>
+      </c>
+      <c r="S452" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Max it par Orange Tunisie facilite votre vie au quotidien !&lt;/h2&gt;&lt;br&gt;&lt;br&gt;Welcome sur Max it !&lt;br&gt;Accédez rapidement à vos fonctionnalités Max it préférées et profitez également de contenus exclusifs, d’activités divertissantes, et de jeux interactifs pour une expérience enrichissante avec la roue</t>
+        </is>
+      </c>
+      <c r="T452" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U452" t="inlineStr"/>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G453" t="n">
+        <v>1146892088</v>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J453" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K453" t="n">
+        <v>0</v>
+      </c>
+      <c r="L453" t="b">
+        <v>1</v>
+      </c>
+      <c r="M453" t="n">
+        <v>3.02812</v>
+      </c>
+      <c r="N453" t="n">
+        <v>1636</v>
+      </c>
+      <c r="O453" t="n">
+        <v>35</v>
+      </c>
+      <c r="P453" t="inlineStr"/>
+      <c r="R453" t="inlineStr">
+        <is>
+          <t>10.0.6</t>
+        </is>
+      </c>
+      <c r="S453" t="inlineStr">
+        <is>
+          <t>Max it by Orange Tunisie : Votre appli incontournable pour une vie connectée
+Welcome sur Max it : Découvrez fonctionnalités, jeux &amp; contenus de divertissement by Orange Tunisie !
+Trouvez vite vos fonctionnalités Max it favorites et explorez des contenus exclusifs et des jeux pour une expérience im</t>
+        </is>
+      </c>
+      <c r="T453" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U453" t="inlineStr"/>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osl</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J454" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K454" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L454" t="b">
+        <v>0</v>
+      </c>
+      <c r="M454" t="n">
+        <v>4.420561</v>
+      </c>
+      <c r="N454" t="n">
+        <v>2109</v>
+      </c>
+      <c r="O454" t="n">
+        <v>11</v>
+      </c>
+      <c r="P454" t="inlineStr"/>
+      <c r="Q454" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R454" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S454" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it is a free application, which allows Orange Sierra Leone prepaid and postpaid customers to:&lt;br&gt;&lt;br&gt;- Consult your account in real time: minutes, sms, internet&lt;br&gt;- Top up your account or a friend account &lt;br&gt;- Buy Internet Bundles&lt;br&gt;- Discover the latest offers and promotions &lt;br&gt;- Access to </t>
+        </is>
+      </c>
+      <c r="T454" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U454" t="inlineStr"/>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G455" t="n">
+        <v>6443607903</v>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J455" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K455" t="n">
+        <v>0</v>
+      </c>
+      <c r="L455" t="b">
+        <v>1</v>
+      </c>
+      <c r="M455" t="n">
+        <v>3.69948</v>
+      </c>
+      <c r="N455" t="n">
+        <v>193</v>
+      </c>
+      <c r="O455" t="n">
+        <v>2</v>
+      </c>
+      <c r="P455" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R455" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The merger of My Orange &amp; Orange Money has given birth to Max it the all-in-one super app, a free application which allows all Orange Sierra Leone customers to 
+Track calls, SMS, and Data usage and monitor balance. 
+Make a secure mobile/Orange Money payment.
+Easily transfer credit to other users </t>
+        </is>
+      </c>
+      <c r="T455" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U455" t="inlineStr"/>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osn</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>Orange Sénégal</t>
+        </is>
+      </c>
+      <c r="J456" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K456" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L456" t="b">
+        <v>0</v>
+      </c>
+      <c r="M456" t="n">
+        <v>4.3126817</v>
+      </c>
+      <c r="N456" t="n">
+        <v>51104</v>
+      </c>
+      <c r="O456" t="n">
+        <v>11</v>
+      </c>
+      <c r="P456" t="inlineStr"/>
+      <c r="Q456" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R456" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S456" t="inlineStr">
+        <is>
+          <t>Lu bees ak Max it ! &lt;br&gt;Une application repensée pour être plus simple, plus rapide et adaptée à vos besoins. Une expérience optimisée pour faciliter vos usages au quotidien, avec des parcours simplifiés et un accès plus fluide à vos services. Que vous soyez client Orange ou non, Max it vous accompa</t>
+        </is>
+      </c>
+      <c r="T456" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U456" t="inlineStr"/>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G457" t="n">
+        <v>1039327980</v>
+      </c>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>Orange Senegal</t>
+        </is>
+      </c>
+      <c r="J457" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K457" t="n">
+        <v>0</v>
+      </c>
+      <c r="L457" t="b">
+        <v>1</v>
+      </c>
+      <c r="M457" t="n">
+        <v>4.16972</v>
+      </c>
+      <c r="N457" t="n">
+        <v>30202</v>
+      </c>
+      <c r="O457" t="n">
+        <v>8</v>
+      </c>
+      <c r="P457" t="inlineStr"/>
+      <c r="R457" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S457" t="inlineStr">
+        <is>
+          <t>Here is the English translation:
+Welcome to Max it!
+A redesigned app to be simpler, faster, and tailored to your needs. An optimized experience to make your daily life easier, with streamlined journeys and smoother access to your services. Whether you are an Orange customer or not, Max it is your e</t>
+        </is>
+      </c>
+      <c r="T457" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U457" t="inlineStr"/>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>com.orange.meditel.mediteletmoi</t>
+        </is>
+      </c>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>Orange Maroc</t>
+        </is>
+      </c>
+      <c r="J458" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K458" t="inlineStr">
+        <is>
+          <t>MAD 0.00</t>
+        </is>
+      </c>
+      <c r="L458" t="b">
+        <v>0</v>
+      </c>
+      <c r="M458" t="n">
+        <v>3.7242568</v>
+      </c>
+      <c r="N458" t="n">
+        <v>110880</v>
+      </c>
+      <c r="O458" t="n">
+        <v>150</v>
+      </c>
+      <c r="P458" t="inlineStr"/>
+      <c r="Q458" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R458" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S458" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l&amp;#39;expérience mobile réinventé&lt;br&gt;&lt;br&gt;Max it, c&amp;#39;est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d&amp;#39;une multitude de services exclusifs. &lt;br&gt;&lt;br&gt;Créez votre espace sur</t>
+        </is>
+      </c>
+      <c r="T458" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U458" t="inlineStr"/>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G459" t="n">
+        <v>596028698</v>
+      </c>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>Méditel</t>
+        </is>
+      </c>
+      <c r="J459" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K459" t="n">
+        <v>0</v>
+      </c>
+      <c r="L459" t="b">
+        <v>1</v>
+      </c>
+      <c r="M459" t="n">
+        <v>3.94766</v>
+      </c>
+      <c r="N459" t="n">
+        <v>2751</v>
+      </c>
+      <c r="P459" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "MA" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R459" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S459" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l'expérience mobile réinventé
+Max it, c'est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d'une multitude de services exclusifs. 
+Créez votre espace sur mesure et bénéficiez d'</t>
+        </is>
+      </c>
+      <c r="T459" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U459" t="inlineStr"/>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>com.oml.dsi.orangemobile</t>
+        </is>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J460" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K460" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L460" t="b">
+        <v>0</v>
+      </c>
+      <c r="M460" t="n">
+        <v>2.6951187</v>
+      </c>
+      <c r="N460" t="n">
+        <v>38259</v>
+      </c>
+      <c r="P460" t="inlineStr"/>
+      <c r="Q460" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R460" t="inlineStr">
+        <is>
+          <t>6.5.0</t>
+        </is>
+      </c>
+      <c r="S460" t="inlineStr">
+        <is>
+          <t>Easily manage your Orange Mali line&lt;br&gt;● Manage your account and view all essential information, your offers, and your phone lines.&lt;br&gt;● Subscribe to call, SMS, Internet, and international call packages.&lt;br&gt;● Track your usage by checking your credit and Internet balance.&lt;br&gt;● Recharge your line by p</t>
+        </is>
+      </c>
+      <c r="T460" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U460" t="inlineStr"/>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G461" t="n">
+        <v>1494321079</v>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J461" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K461" t="n">
+        <v>0</v>
+      </c>
+      <c r="L461" t="b">
+        <v>1</v>
+      </c>
+      <c r="M461" t="n">
+        <v>2.52481</v>
+      </c>
+      <c r="N461" t="n">
+        <v>4695</v>
+      </c>
+      <c r="O461" t="n">
+        <v>3</v>
+      </c>
+      <c r="P461" t="inlineStr"/>
+      <c r="R461" t="inlineStr">
+        <is>
+          <t>6.5.2</t>
+        </is>
+      </c>
+      <c r="S461" t="inlineStr">
+        <is>
+          <t>Gérez facilement votre ligne Orange Mali 
+●        Gérez votre compte et consultez toutes les informations essentielles sur celui-ci, vos offres, ainsi que vos lignes téléphoniques.
+●        Souscrivez aux forfaits appels, SMS, Internet, et appels internationaux.
+●        Suivez votre consommation e</t>
+        </is>
+      </c>
+      <c r="T461" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U461" t="inlineStr"/>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.omg</t>
+        </is>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J462" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K462" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L462" t="b">
+        <v>0</v>
+      </c>
+      <c r="M462" t="n">
+        <v>4.152174</v>
+      </c>
+      <c r="N462" t="n">
+        <v>1359</v>
+      </c>
+      <c r="O462" t="n">
+        <v>26</v>
+      </c>
+      <c r="P462" t="inlineStr"/>
+      <c r="Q462" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R462" t="inlineStr">
+        <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="S462" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.&lt;br&gt;&lt;br&gt;Simplify Your Life with Max it&lt;br&gt;With Max It, ac</t>
+        </is>
+      </c>
+      <c r="T462" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U462" t="inlineStr"/>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G463" t="n">
+        <v>1295171817</v>
+      </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K463" t="n">
+        <v>0</v>
+      </c>
+      <c r="L463" t="b">
+        <v>1</v>
+      </c>
+      <c r="M463" t="n">
+        <v>3.08696</v>
+      </c>
+      <c r="N463" t="n">
+        <v>69</v>
+      </c>
+      <c r="O463" t="n">
+        <v>13</v>
+      </c>
+      <c r="P463" t="inlineStr"/>
+      <c r="R463" t="inlineStr">
+        <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="S463" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.
+Simplify Your Life with Max it
+With Max it, access a se</t>
+        </is>
+      </c>
+      <c r="T463" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U463" t="inlineStr"/>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.olr</t>
+        </is>
+      </c>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>Orange Max it - Liberia</t>
+        </is>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K464" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L464" t="b">
+        <v>0</v>
+      </c>
+      <c r="M464" t="n">
+        <v>4.5469255</v>
+      </c>
+      <c r="N464" t="n">
+        <v>3090</v>
+      </c>
+      <c r="O464" t="n">
+        <v>111</v>
+      </c>
+      <c r="P464" t="inlineStr"/>
+      <c r="Q464" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R464" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="S464" t="inlineStr">
+        <is>
+          <t>Max it: your personalized experience by Orange Liberia!&lt;br&gt;&lt;br&gt;Step into Max it, your all-in-one solution for telecom, marketplace, and financial services! Manage your mobile line, customize offers, pay your bills, keep&lt;br&gt;track of your usage with ease, and recharge your credit. Access exclusive eve</t>
+        </is>
+      </c>
+      <c r="T464" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U464" t="inlineStr"/>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G465" t="n">
+        <v>6746187327</v>
+      </c>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>Orange Max it – Liberia</t>
+        </is>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J465" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K465" t="n">
+        <v>0</v>
+      </c>
+      <c r="L465" t="b">
+        <v>1</v>
+      </c>
+      <c r="M465" t="n">
+        <v>4.04255</v>
+      </c>
+      <c r="N465" t="n">
+        <v>47</v>
+      </c>
+      <c r="P465" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "LR" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R465" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="S465" t="inlineStr">
+        <is>
+          <t>Max it is a free application, which allows Orange Liberia customers to:
+- Consult your account in real time: minutes, sms, internet
+- Top up your account or a friend account 
+- Buy  Bundles (voice, data, SMS, roaming, international)
+- Discover the latest offers and promotions 
+- Access to Orange se</t>
+        </is>
+      </c>
+      <c r="T465" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U465" t="inlineStr"/>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ojo</t>
+        </is>
+      </c>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K466" t="inlineStr">
+        <is>
+          <t>JOD 0.000</t>
+        </is>
+      </c>
+      <c r="L466" t="b">
+        <v>0</v>
+      </c>
+      <c r="M466" t="n">
+        <v>4.4359875</v>
+      </c>
+      <c r="N466" t="n">
+        <v>97544</v>
+      </c>
+      <c r="O466" t="n">
+        <v>46</v>
+      </c>
+      <c r="P466" t="inlineStr"/>
+      <c r="Q466" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R466" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S466" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience&lt;br&gt;Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.&lt;br&gt;Important Update:&lt;br&gt;The jood app (jood Orange) w</t>
+        </is>
+      </c>
+      <c r="T466" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U466" t="inlineStr"/>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G467" t="n">
+        <v>808824590</v>
+      </c>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K467" t="n">
+        <v>0</v>
+      </c>
+      <c r="L467" t="b">
+        <v>1</v>
+      </c>
+      <c r="M467" t="n">
+        <v>4.21232</v>
+      </c>
+      <c r="N467" t="n">
+        <v>2986</v>
+      </c>
+      <c r="O467" t="n">
+        <v>39</v>
+      </c>
+      <c r="P467" t="inlineStr"/>
+      <c r="R467" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S467" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience
+Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.
+Important Update:
+The jood app (jood Orange) will be di</t>
+        </is>
+      </c>
+      <c r="T467" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U467" t="inlineStr"/>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.oci</t>
+        </is>
+      </c>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>Orange Côte d'Ivoire S.A</t>
+        </is>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K468" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L468" t="b">
+        <v>0</v>
+      </c>
+      <c r="M468" t="n">
+        <v>4.18228</v>
+      </c>
+      <c r="N468" t="n">
+        <v>66974</v>
+      </c>
+      <c r="O468" t="n">
+        <v>13</v>
+      </c>
+      <c r="P468" t="inlineStr"/>
+      <c r="Q468" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R468" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S468" t="inlineStr">
+        <is>
+          <t>Aaaahhh, ta super app Max it, n&amp;#39;a pas fini de te surprendre... &lt;br&gt;Est-ce que tu as remarqué ? Maintenant, tu as ton QR code personnalisé en haut de ton écran d&amp;#39;accueil ! Ainsi, tu peux :&lt;br&gt;     scanner le QR code de ton ami(e) pour lui faire un transfert d&amp;#39;&amp;#39;argent&lt;br&gt;     scanner l</t>
+        </is>
+      </c>
+      <c r="T468" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U468" t="inlineStr"/>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G469" t="n">
+        <v>1061120855</v>
+      </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>Orange CI</t>
+        </is>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K469" t="n">
+        <v>0</v>
+      </c>
+      <c r="L469" t="b">
+        <v>1</v>
+      </c>
+      <c r="M469" t="n">
+        <v>3.78634</v>
+      </c>
+      <c r="N469" t="n">
+        <v>5958</v>
+      </c>
+      <c r="O469" t="n">
+        <v>3</v>
+      </c>
+      <c r="P469" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R469" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S469" t="inlineStr">
+        <is>
+          <t>Max it, la super app all-in-one te fais gagner du temps, et diminue tes soucis... Gagne plus d'espace de stockage sur ton téléphone ; plus besoin de cumuler plusieurs appli d'Orange pour avoir accès à un maximum de services. Max it est là ! Gère ta ligne (SIM) au niveau des pass, des soldes, réalise</t>
+        </is>
+      </c>
+      <c r="T469" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U469" t="inlineStr"/>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogw</t>
+        </is>
+      </c>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J470" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K470" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L470" t="b">
+        <v>0</v>
+      </c>
+      <c r="M470" t="n">
+        <v>4.4437084</v>
+      </c>
+      <c r="N470" t="n">
+        <v>1513</v>
+      </c>
+      <c r="O470" t="n">
+        <v>17</v>
+      </c>
+      <c r="P470" t="inlineStr"/>
+      <c r="Q470" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R470" t="inlineStr">
+        <is>
+          <t>4.0.18</t>
+        </is>
+      </c>
+      <c r="S470" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T470" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U470" t="inlineStr"/>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G471" t="n">
+        <v>1574668652</v>
+      </c>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K471" t="n">
+        <v>0</v>
+      </c>
+      <c r="L471" t="b">
+        <v>1</v>
+      </c>
+      <c r="M471" t="n">
+        <v>4.04054</v>
+      </c>
+      <c r="N471" t="n">
+        <v>74</v>
+      </c>
+      <c r="O471" t="n">
+        <v>5</v>
+      </c>
+      <c r="P471" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R471" t="inlineStr">
+        <is>
+          <t>6.0.35</t>
+        </is>
+      </c>
+      <c r="S471" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T471" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U471" t="inlineStr"/>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>com.orange.sugu.ocd</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K472" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L472" t="b">
+        <v>0</v>
+      </c>
+      <c r="M472" t="n">
+        <v>4.120075</v>
+      </c>
+      <c r="N472" t="n">
+        <v>5264</v>
+      </c>
+      <c r="O472" t="n">
+        <v>66</v>
+      </c>
+      <c r="P472" t="inlineStr"/>
+      <c r="Q472" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R472" t="inlineStr">
+        <is>
+          <t>9.0.12</t>
+        </is>
+      </c>
+      <c r="S472" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DRC that brings together the features of MyOrange, and Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Plans, Mobile Payments, money transfers, bill payments, subscriptions, and entertai</t>
+        </is>
+      </c>
+      <c r="T472" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U472" t="inlineStr"/>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G473" t="n">
+        <v>6447896435</v>
+      </c>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K473" t="n">
+        <v>0</v>
+      </c>
+      <c r="L473" t="b">
+        <v>1</v>
+      </c>
+      <c r="M473" t="n">
+        <v>3.55762</v>
+      </c>
+      <c r="N473" t="n">
+        <v>269</v>
+      </c>
+      <c r="P473" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "CD" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R473" t="inlineStr">
+        <is>
+          <t>9.0.6</t>
+        </is>
+      </c>
+      <c r="S473" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DR Congo. It brings together the features of Orange et Moi, as well as Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Packages, Mobile payment, money transfers, bill payment and subscri</t>
+        </is>
+      </c>
+      <c r="T473" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U473" t="inlineStr"/>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ocm</t>
+        </is>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroon</t>
+        </is>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>Orange MEA</t>
+        </is>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K474" t="inlineStr">
+        <is>
+          <t>FCFA 0</t>
+        </is>
+      </c>
+      <c r="L474" t="b">
+        <v>0</v>
+      </c>
+      <c r="M474" t="n">
+        <v>3.9435534</v>
+      </c>
+      <c r="N474" t="n">
+        <v>46767</v>
+      </c>
+      <c r="O474" t="n">
+        <v>14</v>
+      </c>
+      <c r="P474" t="inlineStr"/>
+      <c r="Q474" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R474" t="inlineStr">
+        <is>
+          <t>7.0.23</t>
+        </is>
+      </c>
+      <c r="S474" t="inlineStr">
+        <is>
+          <t>Max it brings together everything that matters to you in one app: managing your lines, money transfer, bill payment, exclusive offers, and a universe of lifestyle and entertainment. Simple, fast, and 100% secure..&lt;br&gt;&lt;br&gt;📞 My line&lt;br&gt;Manage your Orange mobile and landline bundles in a single click:</t>
+        </is>
+      </c>
+      <c r="T474" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U474" t="inlineStr"/>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G475" t="n">
+        <v>1116920093</v>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroun</t>
+        </is>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>Orange Middle East &amp; Africa</t>
+        </is>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K475" t="n">
+        <v>0</v>
+      </c>
+      <c r="L475" t="b">
+        <v>1</v>
+      </c>
+      <c r="M475" t="n">
+        <v>3.76986</v>
+      </c>
+      <c r="N475" t="n">
+        <v>16138</v>
+      </c>
+      <c r="O475" t="n">
+        <v>5</v>
+      </c>
+      <c r="P475" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R475" t="inlineStr">
+        <is>
+          <t>7.0.24</t>
+        </is>
+      </c>
+      <c r="S475" t="inlineStr">
+        <is>
+          <t>Avec Max it, Orange rassemble tout ce qui compte pour vous dans une même application : la gestion de vos lignes, les transferts d’argent, payement de vos factures, des offres exclusives et un univers lifestyle et divertissement.
+Simple, rapide et 100 % sécurisée.
+Ma ligne
+Gérez vos forfaits mobiles</t>
+        </is>
+      </c>
+      <c r="T475" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U475" t="inlineStr"/>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obf</t>
+        </is>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso</t>
+        </is>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K476" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L476" t="b">
+        <v>0</v>
+      </c>
+      <c r="M476" t="n">
+        <v>4.1448765</v>
+      </c>
+      <c r="N476" t="n">
+        <v>25382</v>
+      </c>
+      <c r="O476" t="n">
+        <v>11</v>
+      </c>
+      <c r="P476" t="inlineStr"/>
+      <c r="Q476" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R476" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S476" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.&lt;br&gt;Gérez vos lignes mobiles, effectuez des transferts d&amp;#39;argent sécurisés, réglez vos factures, profitez d&amp;#39;offres exclusives, effectuez des paiements marchands fiables, et bien plus enco</t>
+        </is>
+      </c>
+      <c r="T476" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U476" t="inlineStr"/>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G477" t="n">
+        <v>1553774707</v>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso SA</t>
+        </is>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K477" t="n">
+        <v>0</v>
+      </c>
+      <c r="L477" t="b">
+        <v>1</v>
+      </c>
+      <c r="M477" t="n">
+        <v>3.45246</v>
+      </c>
+      <c r="N477" t="n">
+        <v>1178</v>
+      </c>
+      <c r="O477" t="n">
+        <v>2</v>
+      </c>
+      <c r="P477" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R477" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S477" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.
+Gérez vos lignes mobiles, effectuez des transferts d'argent sécurisés, réglez vos factures, profitez d'offres exclusives, effectuez des paiements marchands fiables, et bien plus encore, le tout</t>
+        </is>
+      </c>
+      <c r="T477" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U477" t="inlineStr"/>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obw</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K478" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L478" t="b">
+        <v>0</v>
+      </c>
+      <c r="M478" t="n">
+        <v>3.9857652</v>
+      </c>
+      <c r="N478" t="n">
+        <v>2959</v>
+      </c>
+      <c r="O478" t="n">
+        <v>46</v>
+      </c>
+      <c r="P478" t="inlineStr"/>
+      <c r="Q478" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R478" t="inlineStr">
+        <is>
+          <t>7.3.8</t>
+        </is>
+      </c>
+      <c r="S478" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it, the brand-new Orange Botswana Super App that follows Yame and gives you access to four distinct universes for a one-of-a-kind experience!&lt;br&gt;&lt;br&gt;Manage your accounts, make quick payments using QR codes, investigate a range of online goods and services, and discover the many options provided </t>
+        </is>
+      </c>
+      <c r="T478" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U478" t="inlineStr"/>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G479" t="n">
+        <v>1195839458</v>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K479" t="n">
+        <v>0</v>
+      </c>
+      <c r="L479" t="b">
+        <v>1</v>
+      </c>
+      <c r="M479" t="n">
+        <v>3.00806</v>
+      </c>
+      <c r="N479" t="n">
+        <v>124</v>
+      </c>
+      <c r="O479" t="n">
+        <v>34</v>
+      </c>
+      <c r="P479" t="inlineStr"/>
+      <c r="R479" t="inlineStr">
+        <is>
+          <t>7.3.1</t>
+        </is>
+      </c>
+      <c r="S479" t="inlineStr">
+        <is>
+          <t>A free mobile self-care application for Orange Botswana’s mobile customers.
+Full Description :
+Max it is a free application, which allows Orange Botswana customers to:
+- Consult your account in real time: minutes, sms, internet ...
+- Top up your account or a friend account  with Orange Money
+-</t>
+        </is>
+      </c>
+      <c r="T479" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U479" t="inlineStr"/>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>com.orange.mobinilandme</t>
+        </is>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K480" t="inlineStr">
+        <is>
+          <t>EGP 0.00</t>
+        </is>
+      </c>
+      <c r="L480" t="b">
+        <v>0</v>
+      </c>
+      <c r="M480" t="n">
+        <v>4.5653305</v>
+      </c>
+      <c r="N480" t="n">
+        <v>921639</v>
+      </c>
+      <c r="O480" t="n">
+        <v>17</v>
+      </c>
+      <c r="P480" t="inlineStr"/>
+      <c r="Q480" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R480" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S480" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion&lt;br&gt;Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.&lt;br&gt;Key services include:&lt;br&gt;• Account Management: Easily manage</t>
+        </is>
+      </c>
+      <c r="T480" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U480" t="inlineStr"/>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>a65dc13d-5909-4e86-b86a-209a54293fed</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:54:16</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G481" t="n">
+        <v>942568333</v>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K481" t="n">
+        <v>0</v>
+      </c>
+      <c r="L481" t="b">
+        <v>1</v>
+      </c>
+      <c r="M481" t="n">
+        <v>4.25086</v>
+      </c>
+      <c r="N481" t="n">
+        <v>116593</v>
+      </c>
+      <c r="O481" t="n">
+        <v>62</v>
+      </c>
+      <c r="P481" t="inlineStr"/>
+      <c r="R481" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S481" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion
+Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.
+Key services include:
+• Account Management: Easily manage your Ora</t>
+        </is>
+      </c>
+      <c r="T481" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U481" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-07-23
</commit_message>
<xml_diff>
--- a/maxit_store_history.xlsx
+++ b/maxit_store_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U481"/>
+  <dimension ref="A1:U513"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38596,7 +38596,6 @@
       <c r="O450" t="n">
         <v>15</v>
       </c>
-      <c r="P450" t="inlineStr"/>
       <c r="Q450" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -38617,7 +38616,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U450" t="inlineStr"/>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
@@ -38680,7 +38678,6 @@
       <c r="N451" t="n">
         <v>319</v>
       </c>
-      <c r="P451" t="inlineStr"/>
       <c r="R451" t="inlineStr">
         <is>
           <t>6.4.8</t>
@@ -38696,7 +38693,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U451" t="inlineStr"/>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
@@ -38766,7 +38762,6 @@
       <c r="O452" t="n">
         <v>36</v>
       </c>
-      <c r="P452" t="inlineStr"/>
       <c r="Q452" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -38787,7 +38782,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U452" t="inlineStr"/>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
@@ -38853,7 +38847,6 @@
       <c r="O453" t="n">
         <v>35</v>
       </c>
-      <c r="P453" t="inlineStr"/>
       <c r="R453" t="inlineStr">
         <is>
           <t>10.0.6</t>
@@ -38871,7 +38864,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U453" t="inlineStr"/>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
@@ -38941,7 +38933,6 @@
       <c r="O454" t="n">
         <v>11</v>
       </c>
-      <c r="P454" t="inlineStr"/>
       <c r="Q454" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -38962,7 +38953,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U454" t="inlineStr"/>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
@@ -39051,7 +39041,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U455" t="inlineStr"/>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
@@ -39121,7 +39110,6 @@
       <c r="O456" t="n">
         <v>11</v>
       </c>
-      <c r="P456" t="inlineStr"/>
       <c r="Q456" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -39142,7 +39130,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U456" t="inlineStr"/>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
@@ -39208,7 +39195,6 @@
       <c r="O457" t="n">
         <v>8</v>
       </c>
-      <c r="P457" t="inlineStr"/>
       <c r="R457" t="inlineStr">
         <is>
           <t>21.1.0</t>
@@ -39226,7 +39212,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U457" t="inlineStr"/>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
@@ -39296,7 +39281,6 @@
       <c r="O458" t="n">
         <v>150</v>
       </c>
-      <c r="P458" t="inlineStr"/>
       <c r="Q458" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -39317,7 +39301,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U458" t="inlineStr"/>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
@@ -39402,7 +39385,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U459" t="inlineStr"/>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
@@ -39469,7 +39451,6 @@
       <c r="N460" t="n">
         <v>38259</v>
       </c>
-      <c r="P460" t="inlineStr"/>
       <c r="Q460" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -39490,7 +39471,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U460" t="inlineStr"/>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
@@ -39556,7 +39536,6 @@
       <c r="O461" t="n">
         <v>3</v>
       </c>
-      <c r="P461" t="inlineStr"/>
       <c r="R461" t="inlineStr">
         <is>
           <t>6.5.2</t>
@@ -39575,7 +39554,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U461" t="inlineStr"/>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
@@ -39645,7 +39623,6 @@
       <c r="O462" t="n">
         <v>26</v>
       </c>
-      <c r="P462" t="inlineStr"/>
       <c r="Q462" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -39666,7 +39643,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U462" t="inlineStr"/>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
@@ -39732,7 +39708,6 @@
       <c r="O463" t="n">
         <v>13</v>
       </c>
-      <c r="P463" t="inlineStr"/>
       <c r="R463" t="inlineStr">
         <is>
           <t>5.0.2</t>
@@ -39750,7 +39725,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U463" t="inlineStr"/>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
@@ -39820,7 +39794,6 @@
       <c r="O464" t="n">
         <v>111</v>
       </c>
-      <c r="P464" t="inlineStr"/>
       <c r="Q464" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -39841,7 +39814,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U464" t="inlineStr"/>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
@@ -39929,7 +39901,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U465" t="inlineStr"/>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
@@ -39999,7 +39970,6 @@
       <c r="O466" t="n">
         <v>46</v>
       </c>
-      <c r="P466" t="inlineStr"/>
       <c r="Q466" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -40020,7 +39990,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U466" t="inlineStr"/>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
@@ -40086,7 +40055,6 @@
       <c r="O467" t="n">
         <v>39</v>
       </c>
-      <c r="P467" t="inlineStr"/>
       <c r="R467" t="inlineStr">
         <is>
           <t>10.0.21</t>
@@ -40105,7 +40073,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U467" t="inlineStr"/>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
@@ -40175,7 +40142,6 @@
       <c r="O468" t="n">
         <v>13</v>
       </c>
-      <c r="P468" t="inlineStr"/>
       <c r="Q468" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -40196,7 +40162,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U468" t="inlineStr"/>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
@@ -40282,7 +40247,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U469" t="inlineStr"/>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
@@ -40352,7 +40316,6 @@
       <c r="O470" t="n">
         <v>17</v>
       </c>
-      <c r="P470" t="inlineStr"/>
       <c r="Q470" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -40373,7 +40336,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U470" t="inlineStr"/>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
@@ -40459,7 +40421,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U471" t="inlineStr"/>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
@@ -40529,7 +40490,6 @@
       <c r="O472" t="n">
         <v>66</v>
       </c>
-      <c r="P472" t="inlineStr"/>
       <c r="Q472" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -40550,7 +40510,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U472" t="inlineStr"/>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
@@ -40633,7 +40592,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U473" t="inlineStr"/>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
@@ -40703,7 +40661,6 @@
       <c r="O474" t="n">
         <v>14</v>
       </c>
-      <c r="P474" t="inlineStr"/>
       <c r="Q474" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -40724,7 +40681,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U474" t="inlineStr"/>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
@@ -40813,7 +40769,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U475" t="inlineStr"/>
     </row>
     <row r="476">
       <c r="A476" t="inlineStr">
@@ -40883,7 +40838,6 @@
       <c r="O476" t="n">
         <v>11</v>
       </c>
-      <c r="P476" t="inlineStr"/>
       <c r="Q476" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -40904,7 +40858,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U476" t="inlineStr"/>
     </row>
     <row r="477">
       <c r="A477" t="inlineStr">
@@ -40991,7 +40944,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U477" t="inlineStr"/>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
@@ -41061,7 +41013,6 @@
       <c r="O478" t="n">
         <v>46</v>
       </c>
-      <c r="P478" t="inlineStr"/>
       <c r="Q478" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -41082,7 +41033,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U478" t="inlineStr"/>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
@@ -41148,7 +41098,6 @@
       <c r="O479" t="n">
         <v>34</v>
       </c>
-      <c r="P479" t="inlineStr"/>
       <c r="R479" t="inlineStr">
         <is>
           <t>7.3.1</t>
@@ -41169,7 +41118,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U479" t="inlineStr"/>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
@@ -41239,7 +41187,6 @@
       <c r="O480" t="n">
         <v>17</v>
       </c>
-      <c r="P480" t="inlineStr"/>
       <c r="Q480" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -41260,7 +41207,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U480" t="inlineStr"/>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
@@ -41326,7 +41272,6 @@
       <c r="O481" t="n">
         <v>62</v>
       </c>
-      <c r="P481" t="inlineStr"/>
       <c r="R481" t="inlineStr">
         <is>
           <t>10.1.0</t>
@@ -41345,7 +41290,2825 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U481" t="inlineStr"/>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogn</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K482" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L482" t="b">
+        <v>0</v>
+      </c>
+      <c r="M482" t="n">
+        <v>4.436482</v>
+      </c>
+      <c r="N482" t="n">
+        <v>9229</v>
+      </c>
+      <c r="O482" t="n">
+        <v>18</v>
+      </c>
+      <c r="P482" t="inlineStr"/>
+      <c r="Q482" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R482" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S482" t="inlineStr">
+        <is>
+          <t>Bien plus qu&amp;#39;une application, un véritable assistant personnel pour une vie connectée et simplifiée.&lt;br&gt;Suivi de consommation: Votre tableau de bord tout-en-un pour une gestion simplifiée !&lt;br&gt;- Gestion de votre offre: Accédez à une vue détaillée de votre offre actuelle et de vos forfaits Orange</t>
+        </is>
+      </c>
+      <c r="T482" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U482" t="inlineStr"/>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G483" t="n">
+        <v>1177999485</v>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K483" t="n">
+        <v>0</v>
+      </c>
+      <c r="L483" t="b">
+        <v>1</v>
+      </c>
+      <c r="M483" t="n">
+        <v>3.90313</v>
+      </c>
+      <c r="N483" t="n">
+        <v>320</v>
+      </c>
+      <c r="P483" t="inlineStr"/>
+      <c r="R483" t="inlineStr">
+        <is>
+          <t>6.4.8</t>
+        </is>
+      </c>
+      <c r="S483" t="inlineStr">
+        <is>
+          <t>La fusion d’Orange et Moi et Orange Money donne naissance à Max it, la nouvelle Super Application Tout-en-Un. Profitez du suivi de consommation, de paiements mobiles, de toutes les fonctionnalités Orange et Moi et Money avec un large éventail de divertissements, le tout regroupé en un seul endroit !</t>
+        </is>
+      </c>
+      <c r="T483" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U483" t="inlineStr"/>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.otn</t>
+        </is>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K484" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L484" t="b">
+        <v>0</v>
+      </c>
+      <c r="M484" t="n">
+        <v>3.968983</v>
+      </c>
+      <c r="N484" t="n">
+        <v>35356</v>
+      </c>
+      <c r="O484" t="n">
+        <v>38</v>
+      </c>
+      <c r="P484" t="inlineStr"/>
+      <c r="Q484" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R484" t="inlineStr">
+        <is>
+          <t>10.0.6</t>
+        </is>
+      </c>
+      <c r="S484" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Max it par Orange Tunisie facilite votre vie au quotidien !&lt;/h2&gt;&lt;br&gt;&lt;br&gt;Welcome sur Max it !&lt;br&gt;Accédez rapidement à vos fonctionnalités Max it préférées et profitez également de contenus exclusifs, d’activités divertissantes, et de jeux interactifs pour une expérience enrichissante avec la roue</t>
+        </is>
+      </c>
+      <c r="T484" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U484" t="inlineStr"/>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G485" t="n">
+        <v>1146892088</v>
+      </c>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K485" t="n">
+        <v>0</v>
+      </c>
+      <c r="L485" t="b">
+        <v>1</v>
+      </c>
+      <c r="M485" t="n">
+        <v>3.02812</v>
+      </c>
+      <c r="N485" t="n">
+        <v>1636</v>
+      </c>
+      <c r="O485" t="n">
+        <v>39</v>
+      </c>
+      <c r="P485" t="inlineStr"/>
+      <c r="R485" t="inlineStr">
+        <is>
+          <t>10.0.6</t>
+        </is>
+      </c>
+      <c r="S485" t="inlineStr">
+        <is>
+          <t>Max it by Orange Tunisie : Votre appli incontournable pour une vie connectée
+Welcome sur Max it : Découvrez fonctionnalités, jeux &amp; contenus de divertissement by Orange Tunisie !
+Trouvez vite vos fonctionnalités Max it favorites et explorez des contenus exclusifs et des jeux pour une expérience im</t>
+        </is>
+      </c>
+      <c r="T485" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U485" t="inlineStr"/>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osl</t>
+        </is>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K486" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L486" t="b">
+        <v>0</v>
+      </c>
+      <c r="M486" t="n">
+        <v>4.423256</v>
+      </c>
+      <c r="N486" t="n">
+        <v>2110</v>
+      </c>
+      <c r="O486" t="n">
+        <v>11</v>
+      </c>
+      <c r="P486" t="inlineStr"/>
+      <c r="Q486" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R486" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S486" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it is a free application, which allows Orange Sierra Leone prepaid and postpaid customers to:&lt;br&gt;&lt;br&gt;- Consult your account in real time: minutes, sms, internet&lt;br&gt;- Top up your account or a friend account &lt;br&gt;- Buy Internet Bundles&lt;br&gt;- Discover the latest offers and promotions &lt;br&gt;- Access to </t>
+        </is>
+      </c>
+      <c r="T486" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U486" t="inlineStr"/>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G487" t="n">
+        <v>6443607903</v>
+      </c>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K487" t="n">
+        <v>0</v>
+      </c>
+      <c r="L487" t="b">
+        <v>1</v>
+      </c>
+      <c r="M487" t="n">
+        <v>3.69948</v>
+      </c>
+      <c r="N487" t="n">
+        <v>193</v>
+      </c>
+      <c r="O487" t="n">
+        <v>2</v>
+      </c>
+      <c r="P487" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R487" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S487" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The merger of My Orange &amp; Orange Money has given birth to Max it the all-in-one super app, a free application which allows all Orange Sierra Leone customers to 
+Track calls, SMS, and Data usage and monitor balance. 
+Make a secure mobile/Orange Money payment.
+Easily transfer credit to other users </t>
+        </is>
+      </c>
+      <c r="T487" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U487" t="inlineStr"/>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osn</t>
+        </is>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>Orange Sénégal</t>
+        </is>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K488" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L488" t="b">
+        <v>0</v>
+      </c>
+      <c r="M488" t="n">
+        <v>4.3138595</v>
+      </c>
+      <c r="N488" t="n">
+        <v>51121</v>
+      </c>
+      <c r="O488" t="n">
+        <v>12</v>
+      </c>
+      <c r="P488" t="inlineStr"/>
+      <c r="Q488" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R488" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S488" t="inlineStr">
+        <is>
+          <t>Lu bees ak Max it ! &lt;br&gt;Une application repensée pour être plus simple, plus rapide et adaptée à vos besoins. Une expérience optimisée pour faciliter vos usages au quotidien, avec des parcours simplifiés et un accès plus fluide à vos services. Que vous soyez client Orange ou non, Max it vous accompa</t>
+        </is>
+      </c>
+      <c r="T488" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U488" t="inlineStr"/>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G489" t="n">
+        <v>1039327980</v>
+      </c>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>Orange Senegal</t>
+        </is>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K489" t="n">
+        <v>0</v>
+      </c>
+      <c r="L489" t="b">
+        <v>1</v>
+      </c>
+      <c r="M489" t="n">
+        <v>4.16964</v>
+      </c>
+      <c r="N489" t="n">
+        <v>30205</v>
+      </c>
+      <c r="O489" t="n">
+        <v>13</v>
+      </c>
+      <c r="P489" t="inlineStr"/>
+      <c r="R489" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S489" t="inlineStr">
+        <is>
+          <t>Here is the English translation:
+Welcome to Max it!
+A redesigned app to be simpler, faster, and tailored to your needs. An optimized experience to make your daily life easier, with streamlined journeys and smoother access to your services. Whether you are an Orange customer or not, Max it is your e</t>
+        </is>
+      </c>
+      <c r="T489" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U489" t="inlineStr"/>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G490" t="inlineStr">
+        <is>
+          <t>com.orange.meditel.mediteletmoi</t>
+        </is>
+      </c>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>Orange Maroc</t>
+        </is>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K490" t="inlineStr">
+        <is>
+          <t>MAD 0.00</t>
+        </is>
+      </c>
+      <c r="L490" t="b">
+        <v>0</v>
+      </c>
+      <c r="M490" t="n">
+        <v>3.7246335</v>
+      </c>
+      <c r="N490" t="n">
+        <v>110884</v>
+      </c>
+      <c r="O490" t="n">
+        <v>141</v>
+      </c>
+      <c r="P490" t="inlineStr"/>
+      <c r="Q490" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R490" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S490" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l&amp;#39;expérience mobile réinventé&lt;br&gt;&lt;br&gt;Max it, c&amp;#39;est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d&amp;#39;une multitude de services exclusifs. &lt;br&gt;&lt;br&gt;Créez votre espace sur</t>
+        </is>
+      </c>
+      <c r="T490" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U490" t="inlineStr"/>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G491" t="n">
+        <v>596028698</v>
+      </c>
+      <c r="H491" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>Méditel</t>
+        </is>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K491" t="n">
+        <v>0</v>
+      </c>
+      <c r="L491" t="b">
+        <v>1</v>
+      </c>
+      <c r="M491" t="n">
+        <v>3.94766</v>
+      </c>
+      <c r="N491" t="n">
+        <v>2751</v>
+      </c>
+      <c r="P491" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "MA" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R491" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S491" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l'expérience mobile réinventé
+Max it, c'est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d'une multitude de services exclusifs. 
+Créez votre espace sur mesure et bénéficiez d'</t>
+        </is>
+      </c>
+      <c r="T491" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U491" t="inlineStr"/>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>com.oml.dsi.orangemobile</t>
+        </is>
+      </c>
+      <c r="H492" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K492" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L492" t="b">
+        <v>0</v>
+      </c>
+      <c r="M492" t="n">
+        <v>2.6951187</v>
+      </c>
+      <c r="N492" t="n">
+        <v>38259</v>
+      </c>
+      <c r="P492" t="inlineStr"/>
+      <c r="Q492" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R492" t="inlineStr">
+        <is>
+          <t>6.5.0</t>
+        </is>
+      </c>
+      <c r="S492" t="inlineStr">
+        <is>
+          <t>Easily manage your Orange Mali line&lt;br&gt;● Manage your account and view all essential information, your offers, and your phone lines.&lt;br&gt;● Subscribe to call, SMS, Internet, and international call packages.&lt;br&gt;● Track your usage by checking your credit and Internet balance.&lt;br&gt;● Recharge your line by p</t>
+        </is>
+      </c>
+      <c r="T492" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U492" t="inlineStr"/>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G493" t="n">
+        <v>1494321079</v>
+      </c>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K493" t="n">
+        <v>0</v>
+      </c>
+      <c r="L493" t="b">
+        <v>1</v>
+      </c>
+      <c r="M493" t="n">
+        <v>2.52109</v>
+      </c>
+      <c r="N493" t="n">
+        <v>4717</v>
+      </c>
+      <c r="O493" t="n">
+        <v>10</v>
+      </c>
+      <c r="P493" t="inlineStr"/>
+      <c r="R493" t="inlineStr">
+        <is>
+          <t>6.5.2</t>
+        </is>
+      </c>
+      <c r="S493" t="inlineStr">
+        <is>
+          <t>Gérez facilement votre ligne Orange Mali 
+●        Gérez votre compte et consultez toutes les informations essentielles sur celui-ci, vos offres, ainsi que vos lignes téléphoniques.
+●        Souscrivez aux forfaits appels, SMS, Internet, et appels internationaux.
+●        Suivez votre consommation e</t>
+        </is>
+      </c>
+      <c r="T493" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U493" t="inlineStr"/>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.omg</t>
+        </is>
+      </c>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K494" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L494" t="b">
+        <v>0</v>
+      </c>
+      <c r="M494" t="n">
+        <v>4.1760564</v>
+      </c>
+      <c r="N494" t="n">
+        <v>1363</v>
+      </c>
+      <c r="O494" t="n">
+        <v>31</v>
+      </c>
+      <c r="P494" t="inlineStr"/>
+      <c r="Q494" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R494" t="inlineStr">
+        <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="S494" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.&lt;br&gt;&lt;br&gt;Simplify Your Life with Max it&lt;br&gt;With Max It, ac</t>
+        </is>
+      </c>
+      <c r="T494" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U494" t="inlineStr"/>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G495" t="n">
+        <v>1295171817</v>
+      </c>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K495" t="n">
+        <v>0</v>
+      </c>
+      <c r="L495" t="b">
+        <v>1</v>
+      </c>
+      <c r="M495" t="n">
+        <v>3.08696</v>
+      </c>
+      <c r="N495" t="n">
+        <v>69</v>
+      </c>
+      <c r="O495" t="n">
+        <v>19</v>
+      </c>
+      <c r="P495" t="inlineStr"/>
+      <c r="R495" t="inlineStr">
+        <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="S495" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.
+Simplify Your Life with Max it
+With Max it, access a se</t>
+        </is>
+      </c>
+      <c r="T495" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U495" t="inlineStr"/>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G496" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.olr</t>
+        </is>
+      </c>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>Orange Max it - Liberia</t>
+        </is>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K496" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L496" t="b">
+        <v>0</v>
+      </c>
+      <c r="M496" t="n">
+        <v>4.5469255</v>
+      </c>
+      <c r="N496" t="n">
+        <v>3090</v>
+      </c>
+      <c r="O496" t="n">
+        <v>90</v>
+      </c>
+      <c r="P496" t="inlineStr"/>
+      <c r="Q496" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R496" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="S496" t="inlineStr">
+        <is>
+          <t>Max it: your personalized experience by Orange Liberia!&lt;br&gt;&lt;br&gt;Step into Max it, your all-in-one solution for telecom, marketplace, and financial services! Manage your mobile line, customize offers, pay your bills, keep&lt;br&gt;track of your usage with ease, and recharge your credit. Access exclusive eve</t>
+        </is>
+      </c>
+      <c r="T496" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U496" t="inlineStr"/>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G497" t="n">
+        <v>6746187327</v>
+      </c>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>Orange Max it – Liberia</t>
+        </is>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K497" t="n">
+        <v>0</v>
+      </c>
+      <c r="L497" t="b">
+        <v>1</v>
+      </c>
+      <c r="M497" t="n">
+        <v>4.04255</v>
+      </c>
+      <c r="N497" t="n">
+        <v>47</v>
+      </c>
+      <c r="P497" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "LR" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R497" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="S497" t="inlineStr">
+        <is>
+          <t>Max it is a free application, which allows Orange Liberia customers to:
+- Consult your account in real time: minutes, sms, internet
+- Top up your account or a friend account 
+- Buy  Bundles (voice, data, SMS, roaming, international)
+- Discover the latest offers and promotions 
+- Access to Orange se</t>
+        </is>
+      </c>
+      <c r="T497" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U497" t="inlineStr"/>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ojo</t>
+        </is>
+      </c>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K498" t="inlineStr">
+        <is>
+          <t>JOD 0.000</t>
+        </is>
+      </c>
+      <c r="L498" t="b">
+        <v>0</v>
+      </c>
+      <c r="M498" t="n">
+        <v>4.4348207</v>
+      </c>
+      <c r="N498" t="n">
+        <v>97574</v>
+      </c>
+      <c r="O498" t="n">
+        <v>53</v>
+      </c>
+      <c r="P498" t="inlineStr"/>
+      <c r="Q498" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R498" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S498" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience&lt;br&gt;Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.&lt;br&gt;Important Update:&lt;br&gt;The jood app (jood Orange) w</t>
+        </is>
+      </c>
+      <c r="T498" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U498" t="inlineStr"/>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G499" t="n">
+        <v>808824590</v>
+      </c>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K499" t="n">
+        <v>0</v>
+      </c>
+      <c r="L499" t="b">
+        <v>1</v>
+      </c>
+      <c r="M499" t="n">
+        <v>4.2123</v>
+      </c>
+      <c r="N499" t="n">
+        <v>2991</v>
+      </c>
+      <c r="O499" t="n">
+        <v>49</v>
+      </c>
+      <c r="P499" t="inlineStr"/>
+      <c r="R499" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S499" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience
+Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.
+Important Update:
+The jood app (jood Orange) will be di</t>
+        </is>
+      </c>
+      <c r="T499" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U499" t="inlineStr"/>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.oci</t>
+        </is>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>Orange Côte d'Ivoire S.A</t>
+        </is>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K500" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L500" t="b">
+        <v>0</v>
+      </c>
+      <c r="M500" t="n">
+        <v>4.1747413</v>
+      </c>
+      <c r="N500" t="n">
+        <v>67009</v>
+      </c>
+      <c r="O500" t="n">
+        <v>11</v>
+      </c>
+      <c r="P500" t="inlineStr"/>
+      <c r="Q500" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R500" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S500" t="inlineStr">
+        <is>
+          <t>Aaaahhh, ta super app Max it, n&amp;#39;a pas fini de te surprendre... &lt;br&gt;Est-ce que tu as remarqué ? Maintenant, tu as ton QR code personnalisé en haut de ton écran d&amp;#39;accueil ! Ainsi, tu peux :&lt;br&gt;     scanner le QR code de ton ami(e) pour lui faire un transfert d&amp;#39;&amp;#39;argent&lt;br&gt;     scanner l</t>
+        </is>
+      </c>
+      <c r="T500" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U500" t="inlineStr"/>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G501" t="n">
+        <v>1061120855</v>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>Orange CI</t>
+        </is>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K501" t="n">
+        <v>0</v>
+      </c>
+      <c r="L501" t="b">
+        <v>1</v>
+      </c>
+      <c r="M501" t="n">
+        <v>3.78647</v>
+      </c>
+      <c r="N501" t="n">
+        <v>5957</v>
+      </c>
+      <c r="O501" t="n">
+        <v>6</v>
+      </c>
+      <c r="P501" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R501" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S501" t="inlineStr">
+        <is>
+          <t>Max it, la super app all-in-one te fais gagner du temps, et diminue tes soucis... Gagne plus d'espace de stockage sur ton téléphone ; plus besoin de cumuler plusieurs appli d'Orange pour avoir accès à un maximum de services. Max it est là ! Gère ta ligne (SIM) au niveau des pass, des soldes, réalise</t>
+        </is>
+      </c>
+      <c r="T501" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U501" t="inlineStr"/>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogw</t>
+        </is>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J502" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K502" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L502" t="b">
+        <v>0</v>
+      </c>
+      <c r="M502" t="n">
+        <v>4.4437084</v>
+      </c>
+      <c r="N502" t="n">
+        <v>1513</v>
+      </c>
+      <c r="O502" t="n">
+        <v>13</v>
+      </c>
+      <c r="P502" t="inlineStr"/>
+      <c r="Q502" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R502" t="inlineStr">
+        <is>
+          <t>4.0.18</t>
+        </is>
+      </c>
+      <c r="S502" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T502" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U502" t="inlineStr"/>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G503" t="n">
+        <v>1574668652</v>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J503" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K503" t="n">
+        <v>0</v>
+      </c>
+      <c r="L503" t="b">
+        <v>1</v>
+      </c>
+      <c r="M503" t="n">
+        <v>4.04054</v>
+      </c>
+      <c r="N503" t="n">
+        <v>74</v>
+      </c>
+      <c r="O503" t="n">
+        <v>3</v>
+      </c>
+      <c r="P503" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R503" t="inlineStr">
+        <is>
+          <t>6.0.35</t>
+        </is>
+      </c>
+      <c r="S503" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T503" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U503" t="inlineStr"/>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>com.orange.sugu.ocd</t>
+        </is>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J504" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K504" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L504" t="b">
+        <v>0</v>
+      </c>
+      <c r="M504" t="n">
+        <v>4.1233644</v>
+      </c>
+      <c r="N504" t="n">
+        <v>5266</v>
+      </c>
+      <c r="O504" t="n">
+        <v>73</v>
+      </c>
+      <c r="P504" t="inlineStr"/>
+      <c r="Q504" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R504" t="inlineStr">
+        <is>
+          <t>9.0.12</t>
+        </is>
+      </c>
+      <c r="S504" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DRC that brings together the features of MyOrange, and Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Plans, Mobile Payments, money transfers, bill payments, subscriptions, and entertai</t>
+        </is>
+      </c>
+      <c r="T504" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U504" t="inlineStr"/>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G505" t="n">
+        <v>6447896435</v>
+      </c>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I505" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J505" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K505" t="n">
+        <v>0</v>
+      </c>
+      <c r="L505" t="b">
+        <v>1</v>
+      </c>
+      <c r="M505" t="n">
+        <v>3.55762</v>
+      </c>
+      <c r="N505" t="n">
+        <v>269</v>
+      </c>
+      <c r="P505" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "CD" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R505" t="inlineStr">
+        <is>
+          <t>9.0.6</t>
+        </is>
+      </c>
+      <c r="S505" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DR Congo. It brings together the features of Orange et Moi, as well as Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Packages, Mobile payment, money transfers, bill payment and subscri</t>
+        </is>
+      </c>
+      <c r="T505" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U505" t="inlineStr"/>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G506" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ocm</t>
+        </is>
+      </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroon</t>
+        </is>
+      </c>
+      <c r="I506" t="inlineStr">
+        <is>
+          <t>Orange MEA</t>
+        </is>
+      </c>
+      <c r="J506" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K506" t="inlineStr">
+        <is>
+          <t>FCFA 0</t>
+        </is>
+      </c>
+      <c r="L506" t="b">
+        <v>0</v>
+      </c>
+      <c r="M506" t="n">
+        <v>3.944788</v>
+      </c>
+      <c r="N506" t="n">
+        <v>46780</v>
+      </c>
+      <c r="O506" t="n">
+        <v>16</v>
+      </c>
+      <c r="P506" t="inlineStr"/>
+      <c r="Q506" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R506" t="inlineStr">
+        <is>
+          <t>7.0.23</t>
+        </is>
+      </c>
+      <c r="S506" t="inlineStr">
+        <is>
+          <t>Max it brings together everything that matters to you in one app: managing your lines, money transfer, bill payment, exclusive offers, and a universe of lifestyle and entertainment. Simple, fast, and 100% secure..&lt;br&gt;&lt;br&gt;📞 My line&lt;br&gt;Manage your Orange mobile and landline bundles in a single click:</t>
+        </is>
+      </c>
+      <c r="T506" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U506" t="inlineStr"/>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G507" t="n">
+        <v>1116920093</v>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroun</t>
+        </is>
+      </c>
+      <c r="I507" t="inlineStr">
+        <is>
+          <t>Orange Middle East &amp; Africa</t>
+        </is>
+      </c>
+      <c r="J507" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K507" t="n">
+        <v>0</v>
+      </c>
+      <c r="L507" t="b">
+        <v>1</v>
+      </c>
+      <c r="M507" t="n">
+        <v>3.76947</v>
+      </c>
+      <c r="N507" t="n">
+        <v>16141</v>
+      </c>
+      <c r="O507" t="n">
+        <v>3</v>
+      </c>
+      <c r="P507" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R507" t="inlineStr">
+        <is>
+          <t>7.0.24</t>
+        </is>
+      </c>
+      <c r="S507" t="inlineStr">
+        <is>
+          <t>Avec Max it, Orange rassemble tout ce qui compte pour vous dans une même application : la gestion de vos lignes, les transferts d’argent, payement de vos factures, des offres exclusives et un univers lifestyle et divertissement.
+Simple, rapide et 100 % sécurisée.
+Ma ligne
+Gérez vos forfaits mobiles</t>
+        </is>
+      </c>
+      <c r="T507" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U507" t="inlineStr"/>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G508" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obf</t>
+        </is>
+      </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso</t>
+        </is>
+      </c>
+      <c r="J508" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K508" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L508" t="b">
+        <v>0</v>
+      </c>
+      <c r="M508" t="n">
+        <v>4.1426325</v>
+      </c>
+      <c r="N508" t="n">
+        <v>25396</v>
+      </c>
+      <c r="O508" t="n">
+        <v>11</v>
+      </c>
+      <c r="P508" t="inlineStr"/>
+      <c r="Q508" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R508" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S508" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.&lt;br&gt;Gérez vos lignes mobiles, effectuez des transferts d&amp;#39;argent sécurisés, réglez vos factures, profitez d&amp;#39;offres exclusives, effectuez des paiements marchands fiables, et bien plus enco</t>
+        </is>
+      </c>
+      <c r="T508" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U508" t="inlineStr"/>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G509" t="n">
+        <v>1553774707</v>
+      </c>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I509" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso SA</t>
+        </is>
+      </c>
+      <c r="J509" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K509" t="n">
+        <v>0</v>
+      </c>
+      <c r="L509" t="b">
+        <v>1</v>
+      </c>
+      <c r="M509" t="n">
+        <v>3.45377</v>
+      </c>
+      <c r="N509" t="n">
+        <v>1179</v>
+      </c>
+      <c r="O509" t="n">
+        <v>2</v>
+      </c>
+      <c r="P509" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R509" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S509" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.
+Gérez vos lignes mobiles, effectuez des transferts d'argent sécurisés, réglez vos factures, profitez d'offres exclusives, effectuez des paiements marchands fiables, et bien plus encore, le tout</t>
+        </is>
+      </c>
+      <c r="T509" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U509" t="inlineStr"/>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obw</t>
+        </is>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I510" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J510" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K510" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L510" t="b">
+        <v>0</v>
+      </c>
+      <c r="M510" t="n">
+        <v>3.9929328</v>
+      </c>
+      <c r="N510" t="n">
+        <v>2961</v>
+      </c>
+      <c r="O510" t="n">
+        <v>44</v>
+      </c>
+      <c r="P510" t="inlineStr"/>
+      <c r="Q510" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R510" t="inlineStr">
+        <is>
+          <t>7.3.8</t>
+        </is>
+      </c>
+      <c r="S510" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it, the brand-new Orange Botswana Super App that follows Yame and gives you access to four distinct universes for a one-of-a-kind experience!&lt;br&gt;&lt;br&gt;Manage your accounts, make quick payments using QR codes, investigate a range of online goods and services, and discover the many options provided </t>
+        </is>
+      </c>
+      <c r="T510" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U510" t="inlineStr"/>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G511" t="n">
+        <v>1195839458</v>
+      </c>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I511" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J511" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K511" t="n">
+        <v>0</v>
+      </c>
+      <c r="L511" t="b">
+        <v>1</v>
+      </c>
+      <c r="M511" t="n">
+        <v>3.00806</v>
+      </c>
+      <c r="N511" t="n">
+        <v>124</v>
+      </c>
+      <c r="O511" t="n">
+        <v>34</v>
+      </c>
+      <c r="P511" t="inlineStr"/>
+      <c r="R511" t="inlineStr">
+        <is>
+          <t>7.3.1</t>
+        </is>
+      </c>
+      <c r="S511" t="inlineStr">
+        <is>
+          <t>A free mobile self-care application for Orange Botswana’s mobile customers.
+Full Description :
+Max it is a free application, which allows Orange Botswana customers to:
+- Consult your account in real time: minutes, sms, internet ...
+- Top up your account or a friend account  with Orange Money
+-</t>
+        </is>
+      </c>
+      <c r="T511" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U511" t="inlineStr"/>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G512" t="inlineStr">
+        <is>
+          <t>com.orange.mobinilandme</t>
+        </is>
+      </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I512" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J512" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K512" t="inlineStr">
+        <is>
+          <t>EGP 0.00</t>
+        </is>
+      </c>
+      <c r="L512" t="b">
+        <v>0</v>
+      </c>
+      <c r="M512" t="n">
+        <v>4.56465</v>
+      </c>
+      <c r="N512" t="n">
+        <v>922518</v>
+      </c>
+      <c r="O512" t="n">
+        <v>23</v>
+      </c>
+      <c r="P512" t="inlineStr"/>
+      <c r="Q512" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R512" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S512" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion&lt;br&gt;Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.&lt;br&gt;Key services include:&lt;br&gt;• Account Management: Easily manage</t>
+        </is>
+      </c>
+      <c r="T512" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U512" t="inlineStr"/>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>352de051-7b93-4522-aebc-ac61552e06c2</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:31:30</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G513" t="n">
+        <v>942568333</v>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I513" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J513" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K513" t="n">
+        <v>0</v>
+      </c>
+      <c r="L513" t="b">
+        <v>1</v>
+      </c>
+      <c r="M513" t="n">
+        <v>4.25103</v>
+      </c>
+      <c r="N513" t="n">
+        <v>116722</v>
+      </c>
+      <c r="O513" t="n">
+        <v>58</v>
+      </c>
+      <c r="P513" t="inlineStr"/>
+      <c r="R513" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S513" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion
+Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.
+Key services include:
+• Account Management: Easily manage your Ora</t>
+        </is>
+      </c>
+      <c r="T513" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U513" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-07-24
</commit_message>
<xml_diff>
--- a/maxit_store_history.xlsx
+++ b/maxit_store_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U513"/>
+  <dimension ref="A1:U545"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41359,7 +41359,6 @@
       <c r="O482" t="n">
         <v>18</v>
       </c>
-      <c r="P482" t="inlineStr"/>
       <c r="Q482" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -41380,7 +41379,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U482" t="inlineStr"/>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
@@ -41443,7 +41441,6 @@
       <c r="N483" t="n">
         <v>320</v>
       </c>
-      <c r="P483" t="inlineStr"/>
       <c r="R483" t="inlineStr">
         <is>
           <t>6.4.8</t>
@@ -41459,7 +41456,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U483" t="inlineStr"/>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
@@ -41529,7 +41525,6 @@
       <c r="O484" t="n">
         <v>38</v>
       </c>
-      <c r="P484" t="inlineStr"/>
       <c r="Q484" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -41550,7 +41545,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U484" t="inlineStr"/>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
@@ -41616,7 +41610,6 @@
       <c r="O485" t="n">
         <v>39</v>
       </c>
-      <c r="P485" t="inlineStr"/>
       <c r="R485" t="inlineStr">
         <is>
           <t>10.0.6</t>
@@ -41634,7 +41627,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U485" t="inlineStr"/>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
@@ -41704,7 +41696,6 @@
       <c r="O486" t="n">
         <v>11</v>
       </c>
-      <c r="P486" t="inlineStr"/>
       <c r="Q486" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -41725,7 +41716,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U486" t="inlineStr"/>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
@@ -41814,7 +41804,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U487" t="inlineStr"/>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
@@ -41884,7 +41873,6 @@
       <c r="O488" t="n">
         <v>12</v>
       </c>
-      <c r="P488" t="inlineStr"/>
       <c r="Q488" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -41905,7 +41893,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U488" t="inlineStr"/>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
@@ -41971,7 +41958,6 @@
       <c r="O489" t="n">
         <v>13</v>
       </c>
-      <c r="P489" t="inlineStr"/>
       <c r="R489" t="inlineStr">
         <is>
           <t>21.1.0</t>
@@ -41989,7 +41975,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U489" t="inlineStr"/>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
@@ -42059,7 +42044,6 @@
       <c r="O490" t="n">
         <v>141</v>
       </c>
-      <c r="P490" t="inlineStr"/>
       <c r="Q490" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -42080,7 +42064,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U490" t="inlineStr"/>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
@@ -42165,7 +42148,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U491" t="inlineStr"/>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
@@ -42232,7 +42214,6 @@
       <c r="N492" t="n">
         <v>38259</v>
       </c>
-      <c r="P492" t="inlineStr"/>
       <c r="Q492" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -42253,7 +42234,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U492" t="inlineStr"/>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
@@ -42319,7 +42299,6 @@
       <c r="O493" t="n">
         <v>10</v>
       </c>
-      <c r="P493" t="inlineStr"/>
       <c r="R493" t="inlineStr">
         <is>
           <t>6.5.2</t>
@@ -42338,7 +42317,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U493" t="inlineStr"/>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
@@ -42408,7 +42386,6 @@
       <c r="O494" t="n">
         <v>31</v>
       </c>
-      <c r="P494" t="inlineStr"/>
       <c r="Q494" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -42429,7 +42406,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U494" t="inlineStr"/>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
@@ -42495,7 +42471,6 @@
       <c r="O495" t="n">
         <v>19</v>
       </c>
-      <c r="P495" t="inlineStr"/>
       <c r="R495" t="inlineStr">
         <is>
           <t>5.0.2</t>
@@ -42513,7 +42488,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U495" t="inlineStr"/>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
@@ -42583,7 +42557,6 @@
       <c r="O496" t="n">
         <v>90</v>
       </c>
-      <c r="P496" t="inlineStr"/>
       <c r="Q496" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -42604,7 +42577,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U496" t="inlineStr"/>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
@@ -42692,7 +42664,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U497" t="inlineStr"/>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
@@ -42762,7 +42733,6 @@
       <c r="O498" t="n">
         <v>53</v>
       </c>
-      <c r="P498" t="inlineStr"/>
       <c r="Q498" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -42783,7 +42753,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U498" t="inlineStr"/>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
@@ -42849,7 +42818,6 @@
       <c r="O499" t="n">
         <v>49</v>
       </c>
-      <c r="P499" t="inlineStr"/>
       <c r="R499" t="inlineStr">
         <is>
           <t>10.0.21</t>
@@ -42868,7 +42836,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U499" t="inlineStr"/>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
@@ -42938,7 +42905,6 @@
       <c r="O500" t="n">
         <v>11</v>
       </c>
-      <c r="P500" t="inlineStr"/>
       <c r="Q500" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -42959,7 +42925,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U500" t="inlineStr"/>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
@@ -43045,7 +43010,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U501" t="inlineStr"/>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
@@ -43115,7 +43079,6 @@
       <c r="O502" t="n">
         <v>13</v>
       </c>
-      <c r="P502" t="inlineStr"/>
       <c r="Q502" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -43136,7 +43099,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U502" t="inlineStr"/>
     </row>
     <row r="503">
       <c r="A503" t="inlineStr">
@@ -43222,7 +43184,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U503" t="inlineStr"/>
     </row>
     <row r="504">
       <c r="A504" t="inlineStr">
@@ -43292,7 +43253,6 @@
       <c r="O504" t="n">
         <v>73</v>
       </c>
-      <c r="P504" t="inlineStr"/>
       <c r="Q504" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -43313,7 +43273,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U504" t="inlineStr"/>
     </row>
     <row r="505">
       <c r="A505" t="inlineStr">
@@ -43396,7 +43355,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U505" t="inlineStr"/>
     </row>
     <row r="506">
       <c r="A506" t="inlineStr">
@@ -43466,7 +43424,6 @@
       <c r="O506" t="n">
         <v>16</v>
       </c>
-      <c r="P506" t="inlineStr"/>
       <c r="Q506" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -43487,7 +43444,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U506" t="inlineStr"/>
     </row>
     <row r="507">
       <c r="A507" t="inlineStr">
@@ -43576,7 +43532,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U507" t="inlineStr"/>
     </row>
     <row r="508">
       <c r="A508" t="inlineStr">
@@ -43646,7 +43601,6 @@
       <c r="O508" t="n">
         <v>11</v>
       </c>
-      <c r="P508" t="inlineStr"/>
       <c r="Q508" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -43667,7 +43621,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U508" t="inlineStr"/>
     </row>
     <row r="509">
       <c r="A509" t="inlineStr">
@@ -43754,7 +43707,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U509" t="inlineStr"/>
     </row>
     <row r="510">
       <c r="A510" t="inlineStr">
@@ -43824,7 +43776,6 @@
       <c r="O510" t="n">
         <v>44</v>
       </c>
-      <c r="P510" t="inlineStr"/>
       <c r="Q510" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -43845,7 +43796,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U510" t="inlineStr"/>
     </row>
     <row r="511">
       <c r="A511" t="inlineStr">
@@ -43911,7 +43861,6 @@
       <c r="O511" t="n">
         <v>34</v>
       </c>
-      <c r="P511" t="inlineStr"/>
       <c r="R511" t="inlineStr">
         <is>
           <t>7.3.1</t>
@@ -43932,7 +43881,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U511" t="inlineStr"/>
     </row>
     <row r="512">
       <c r="A512" t="inlineStr">
@@ -44002,7 +43950,6 @@
       <c r="O512" t="n">
         <v>23</v>
       </c>
-      <c r="P512" t="inlineStr"/>
       <c r="Q512" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -44023,7 +43970,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U512" t="inlineStr"/>
     </row>
     <row r="513">
       <c r="A513" t="inlineStr">
@@ -44089,7 +44035,6 @@
       <c r="O513" t="n">
         <v>58</v>
       </c>
-      <c r="P513" t="inlineStr"/>
       <c r="R513" t="inlineStr">
         <is>
           <t>10.1.0</t>
@@ -44108,7 +44053,2825 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U513" t="inlineStr"/>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G514" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogn</t>
+        </is>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I514" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J514" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K514" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L514" t="b">
+        <v>0</v>
+      </c>
+      <c r="M514" t="n">
+        <v>4.4403973</v>
+      </c>
+      <c r="N514" t="n">
+        <v>9236</v>
+      </c>
+      <c r="O514" t="n">
+        <v>19</v>
+      </c>
+      <c r="P514" t="inlineStr"/>
+      <c r="Q514" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R514" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S514" t="inlineStr">
+        <is>
+          <t>Bien plus qu&amp;#39;une application, un véritable assistant personnel pour une vie connectée et simplifiée.&lt;br&gt;Suivi de consommation: Votre tableau de bord tout-en-un pour une gestion simplifiée !&lt;br&gt;- Gestion de votre offre: Accédez à une vue détaillée de votre offre actuelle et de vos forfaits Orange</t>
+        </is>
+      </c>
+      <c r="T514" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U514" t="inlineStr"/>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G515" t="n">
+        <v>1177999485</v>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I515" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J515" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K515" t="n">
+        <v>0</v>
+      </c>
+      <c r="L515" t="b">
+        <v>1</v>
+      </c>
+      <c r="M515" t="n">
+        <v>3.90343</v>
+      </c>
+      <c r="N515" t="n">
+        <v>321</v>
+      </c>
+      <c r="P515" t="inlineStr"/>
+      <c r="R515" t="inlineStr">
+        <is>
+          <t>6.4.8</t>
+        </is>
+      </c>
+      <c r="S515" t="inlineStr">
+        <is>
+          <t>La fusion d’Orange et Moi et Orange Money donne naissance à Max it, la nouvelle Super Application Tout-en-Un. Profitez du suivi de consommation, de paiements mobiles, de toutes les fonctionnalités Orange et Moi et Money avec un large éventail de divertissements, le tout regroupé en un seul endroit !</t>
+        </is>
+      </c>
+      <c r="T515" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U515" t="inlineStr"/>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G516" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.otn</t>
+        </is>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I516" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J516" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K516" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L516" t="b">
+        <v>0</v>
+      </c>
+      <c r="M516" t="n">
+        <v>3.9684052</v>
+      </c>
+      <c r="N516" t="n">
+        <v>35358</v>
+      </c>
+      <c r="O516" t="n">
+        <v>38</v>
+      </c>
+      <c r="P516" t="inlineStr"/>
+      <c r="Q516" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R516" t="inlineStr">
+        <is>
+          <t>10.0.6</t>
+        </is>
+      </c>
+      <c r="S516" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Max it par Orange Tunisie facilite votre vie au quotidien !&lt;/h2&gt;&lt;br&gt;&lt;br&gt;Welcome sur Max it !&lt;br&gt;Accédez rapidement à vos fonctionnalités Max it préférées et profitez également de contenus exclusifs, d’activités divertissantes, et de jeux interactifs pour une expérience enrichissante avec la roue</t>
+        </is>
+      </c>
+      <c r="T516" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U516" t="inlineStr"/>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G517" t="n">
+        <v>1146892088</v>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I517" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J517" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K517" t="n">
+        <v>0</v>
+      </c>
+      <c r="L517" t="b">
+        <v>1</v>
+      </c>
+      <c r="M517" t="n">
+        <v>3.02812</v>
+      </c>
+      <c r="N517" t="n">
+        <v>1636</v>
+      </c>
+      <c r="O517" t="n">
+        <v>38</v>
+      </c>
+      <c r="P517" t="inlineStr"/>
+      <c r="R517" t="inlineStr">
+        <is>
+          <t>10.0.6</t>
+        </is>
+      </c>
+      <c r="S517" t="inlineStr">
+        <is>
+          <t>Max it by Orange Tunisie : Votre appli incontournable pour une vie connectée
+Welcome sur Max it : Découvrez fonctionnalités, jeux &amp; contenus de divertissement by Orange Tunisie !
+Trouvez vite vos fonctionnalités Max it favorites et explorez des contenus exclusifs et des jeux pour une expérience im</t>
+        </is>
+      </c>
+      <c r="T517" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U517" t="inlineStr"/>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G518" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osl</t>
+        </is>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I518" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J518" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K518" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L518" t="b">
+        <v>0</v>
+      </c>
+      <c r="M518" t="n">
+        <v>4.39726</v>
+      </c>
+      <c r="N518" t="n">
+        <v>2114</v>
+      </c>
+      <c r="O518" t="n">
+        <v>11</v>
+      </c>
+      <c r="P518" t="inlineStr"/>
+      <c r="Q518" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R518" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S518" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it is a free application, which allows Orange Sierra Leone prepaid and postpaid customers to:&lt;br&gt;&lt;br&gt;- Consult your account in real time: minutes, sms, internet&lt;br&gt;- Top up your account or a friend account &lt;br&gt;- Buy Internet Bundles&lt;br&gt;- Discover the latest offers and promotions &lt;br&gt;- Access to </t>
+        </is>
+      </c>
+      <c r="T518" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U518" t="inlineStr"/>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G519" t="n">
+        <v>6443607903</v>
+      </c>
+      <c r="H519" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J519" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K519" t="n">
+        <v>0</v>
+      </c>
+      <c r="L519" t="b">
+        <v>1</v>
+      </c>
+      <c r="M519" t="n">
+        <v>3.69948</v>
+      </c>
+      <c r="N519" t="n">
+        <v>193</v>
+      </c>
+      <c r="O519" t="n">
+        <v>6</v>
+      </c>
+      <c r="P519" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R519" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S519" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The merger of My Orange &amp; Orange Money has given birth to Max it the all-in-one super app, a free application which allows all Orange Sierra Leone customers to 
+Track calls, SMS, and Data usage and monitor balance. 
+Make a secure mobile/Orange Money payment.
+Easily transfer credit to other users </t>
+        </is>
+      </c>
+      <c r="T519" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U519" t="inlineStr"/>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G520" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osn</t>
+        </is>
+      </c>
+      <c r="H520" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I520" t="inlineStr">
+        <is>
+          <t>Orange Sénégal</t>
+        </is>
+      </c>
+      <c r="J520" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K520" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L520" t="b">
+        <v>0</v>
+      </c>
+      <c r="M520" t="n">
+        <v>4.3131833</v>
+      </c>
+      <c r="N520" t="n">
+        <v>51143</v>
+      </c>
+      <c r="O520" t="n">
+        <v>12</v>
+      </c>
+      <c r="P520" t="inlineStr"/>
+      <c r="Q520" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R520" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S520" t="inlineStr">
+        <is>
+          <t>Lu bees ak Max it ! &lt;br&gt;Une application repensée pour être plus simple, plus rapide et adaptée à vos besoins. Une expérience optimisée pour faciliter vos usages au quotidien, avec des parcours simplifiés et un accès plus fluide à vos services. Que vous soyez client Orange ou non, Max it vous accompa</t>
+        </is>
+      </c>
+      <c r="T520" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U520" t="inlineStr"/>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G521" t="n">
+        <v>1039327980</v>
+      </c>
+      <c r="H521" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I521" t="inlineStr">
+        <is>
+          <t>Orange Senegal</t>
+        </is>
+      </c>
+      <c r="J521" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K521" t="n">
+        <v>0</v>
+      </c>
+      <c r="L521" t="b">
+        <v>1</v>
+      </c>
+      <c r="M521" t="n">
+        <v>4.16964</v>
+      </c>
+      <c r="N521" t="n">
+        <v>30206</v>
+      </c>
+      <c r="O521" t="n">
+        <v>15</v>
+      </c>
+      <c r="P521" t="inlineStr"/>
+      <c r="R521" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S521" t="inlineStr">
+        <is>
+          <t>Here is the English translation:
+Welcome to Max it!
+A redesigned app to be simpler, faster, and tailored to your needs. An optimized experience to make your daily life easier, with streamlined journeys and smoother access to your services. Whether you are an Orange customer or not, Max it is your e</t>
+        </is>
+      </c>
+      <c r="T521" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U521" t="inlineStr"/>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G522" t="inlineStr">
+        <is>
+          <t>com.orange.meditel.mediteletmoi</t>
+        </is>
+      </c>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I522" t="inlineStr">
+        <is>
+          <t>Orange Maroc</t>
+        </is>
+      </c>
+      <c r="J522" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K522" t="inlineStr">
+        <is>
+          <t>MAD 0.00</t>
+        </is>
+      </c>
+      <c r="L522" t="b">
+        <v>0</v>
+      </c>
+      <c r="M522" t="n">
+        <v>3.7247417</v>
+      </c>
+      <c r="N522" t="n">
+        <v>110889</v>
+      </c>
+      <c r="O522" t="n">
+        <v>149</v>
+      </c>
+      <c r="P522" t="inlineStr"/>
+      <c r="Q522" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R522" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S522" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l&amp;#39;expérience mobile réinventé&lt;br&gt;&lt;br&gt;Max it, c&amp;#39;est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d&amp;#39;une multitude de services exclusifs. &lt;br&gt;&lt;br&gt;Créez votre espace sur</t>
+        </is>
+      </c>
+      <c r="T522" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U522" t="inlineStr"/>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G523" t="n">
+        <v>596028698</v>
+      </c>
+      <c r="H523" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I523" t="inlineStr">
+        <is>
+          <t>Méditel</t>
+        </is>
+      </c>
+      <c r="J523" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K523" t="n">
+        <v>0</v>
+      </c>
+      <c r="L523" t="b">
+        <v>1</v>
+      </c>
+      <c r="M523" t="n">
+        <v>3.94766</v>
+      </c>
+      <c r="N523" t="n">
+        <v>2751</v>
+      </c>
+      <c r="P523" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "MA" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R523" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S523" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l'expérience mobile réinventé
+Max it, c'est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d'une multitude de services exclusifs. 
+Créez votre espace sur mesure et bénéficiez d'</t>
+        </is>
+      </c>
+      <c r="T523" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U523" t="inlineStr"/>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G524" t="inlineStr">
+        <is>
+          <t>com.oml.dsi.orangemobile</t>
+        </is>
+      </c>
+      <c r="H524" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I524" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J524" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K524" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L524" t="b">
+        <v>0</v>
+      </c>
+      <c r="M524" t="n">
+        <v>2.6960042</v>
+      </c>
+      <c r="N524" t="n">
+        <v>38255</v>
+      </c>
+      <c r="P524" t="inlineStr"/>
+      <c r="Q524" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R524" t="inlineStr">
+        <is>
+          <t>6.5.0</t>
+        </is>
+      </c>
+      <c r="S524" t="inlineStr">
+        <is>
+          <t>Easily manage your Orange Mali line&lt;br&gt;● Manage your account and view all essential information, your offers, and your phone lines.&lt;br&gt;● Subscribe to call, SMS, Internet, and international call packages.&lt;br&gt;● Track your usage by checking your credit and Internet balance.&lt;br&gt;● Recharge your line by p</t>
+        </is>
+      </c>
+      <c r="T524" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U524" t="inlineStr"/>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G525" t="n">
+        <v>1494321079</v>
+      </c>
+      <c r="H525" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I525" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J525" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K525" t="n">
+        <v>0</v>
+      </c>
+      <c r="L525" t="b">
+        <v>1</v>
+      </c>
+      <c r="M525" t="n">
+        <v>2.5203</v>
+      </c>
+      <c r="N525" t="n">
+        <v>4728</v>
+      </c>
+      <c r="O525" t="n">
+        <v>11</v>
+      </c>
+      <c r="P525" t="inlineStr"/>
+      <c r="R525" t="inlineStr">
+        <is>
+          <t>6.5.2</t>
+        </is>
+      </c>
+      <c r="S525" t="inlineStr">
+        <is>
+          <t>Gérez facilement votre ligne Orange Mali 
+●        Gérez votre compte et consultez toutes les informations essentielles sur celui-ci, vos offres, ainsi que vos lignes téléphoniques.
+●        Souscrivez aux forfaits appels, SMS, Internet, et appels internationaux.
+●        Suivez votre consommation e</t>
+        </is>
+      </c>
+      <c r="T525" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U525" t="inlineStr"/>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G526" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.omg</t>
+        </is>
+      </c>
+      <c r="H526" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I526" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J526" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K526" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L526" t="b">
+        <v>0</v>
+      </c>
+      <c r="M526" t="n">
+        <v>4.169231</v>
+      </c>
+      <c r="N526" t="n">
+        <v>1364</v>
+      </c>
+      <c r="O526" t="n">
+        <v>42</v>
+      </c>
+      <c r="P526" t="inlineStr"/>
+      <c r="Q526" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R526" t="inlineStr">
+        <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="S526" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.&lt;br&gt;&lt;br&gt;Simplify Your Life with Max it&lt;br&gt;With Max It, ac</t>
+        </is>
+      </c>
+      <c r="T526" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U526" t="inlineStr"/>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G527" t="n">
+        <v>1295171817</v>
+      </c>
+      <c r="H527" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I527" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J527" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K527" t="n">
+        <v>0</v>
+      </c>
+      <c r="L527" t="b">
+        <v>1</v>
+      </c>
+      <c r="M527" t="n">
+        <v>3.08696</v>
+      </c>
+      <c r="N527" t="n">
+        <v>69</v>
+      </c>
+      <c r="O527" t="n">
+        <v>26</v>
+      </c>
+      <c r="P527" t="inlineStr"/>
+      <c r="R527" t="inlineStr">
+        <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="S527" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.
+Simplify Your Life with Max it
+With Max it, access a se</t>
+        </is>
+      </c>
+      <c r="T527" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U527" t="inlineStr"/>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G528" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.olr</t>
+        </is>
+      </c>
+      <c r="H528" t="inlineStr">
+        <is>
+          <t>Orange Max it - Liberia</t>
+        </is>
+      </c>
+      <c r="I528" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J528" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K528" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L528" t="b">
+        <v>0</v>
+      </c>
+      <c r="M528" t="n">
+        <v>4.5434084</v>
+      </c>
+      <c r="N528" t="n">
+        <v>3092</v>
+      </c>
+      <c r="O528" t="n">
+        <v>75</v>
+      </c>
+      <c r="P528" t="inlineStr"/>
+      <c r="Q528" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R528" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="S528" t="inlineStr">
+        <is>
+          <t>Max it: your personalized experience by Orange Liberia!&lt;br&gt;&lt;br&gt;Step into Max it, your all-in-one solution for telecom, marketplace, and financial services! Manage your mobile line, customize offers, pay your bills, keep&lt;br&gt;track of your usage with ease, and recharge your credit. Access exclusive eve</t>
+        </is>
+      </c>
+      <c r="T528" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U528" t="inlineStr"/>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G529" t="n">
+        <v>6746187327</v>
+      </c>
+      <c r="H529" t="inlineStr">
+        <is>
+          <t>Orange Max it – Liberia</t>
+        </is>
+      </c>
+      <c r="I529" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J529" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K529" t="n">
+        <v>0</v>
+      </c>
+      <c r="L529" t="b">
+        <v>1</v>
+      </c>
+      <c r="M529" t="n">
+        <v>4.0625</v>
+      </c>
+      <c r="N529" t="n">
+        <v>48</v>
+      </c>
+      <c r="P529" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "LR" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R529" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="S529" t="inlineStr">
+        <is>
+          <t>Max it is a free application, which allows Orange Liberia customers to:
+- Consult your account in real time: minutes, sms, internet
+- Top up your account or a friend account 
+- Buy  Bundles (voice, data, SMS, roaming, international)
+- Discover the latest offers and promotions 
+- Access to Orange se</t>
+        </is>
+      </c>
+      <c r="T529" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U529" t="inlineStr"/>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G530" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ojo</t>
+        </is>
+      </c>
+      <c r="H530" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I530" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J530" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K530" t="inlineStr">
+        <is>
+          <t>JOD 0.000</t>
+        </is>
+      </c>
+      <c r="L530" t="b">
+        <v>0</v>
+      </c>
+      <c r="M530" t="n">
+        <v>4.4335265</v>
+      </c>
+      <c r="N530" t="n">
+        <v>97596</v>
+      </c>
+      <c r="O530" t="n">
+        <v>52</v>
+      </c>
+      <c r="P530" t="inlineStr"/>
+      <c r="Q530" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R530" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S530" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience&lt;br&gt;Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.&lt;br&gt;Important Update:&lt;br&gt;The jood app (jood Orange) w</t>
+        </is>
+      </c>
+      <c r="T530" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U530" t="inlineStr"/>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G531" t="n">
+        <v>808824590</v>
+      </c>
+      <c r="H531" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I531" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J531" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K531" t="n">
+        <v>0</v>
+      </c>
+      <c r="L531" t="b">
+        <v>1</v>
+      </c>
+      <c r="M531" t="n">
+        <v>4.21211</v>
+      </c>
+      <c r="N531" t="n">
+        <v>3003</v>
+      </c>
+      <c r="O531" t="n">
+        <v>48</v>
+      </c>
+      <c r="P531" t="inlineStr"/>
+      <c r="R531" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S531" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience
+Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.
+Important Update:
+The jood app (jood Orange) will be di</t>
+        </is>
+      </c>
+      <c r="T531" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U531" t="inlineStr"/>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G532" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.oci</t>
+        </is>
+      </c>
+      <c r="H532" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I532" t="inlineStr">
+        <is>
+          <t>Orange Côte d'Ivoire S.A</t>
+        </is>
+      </c>
+      <c r="J532" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K532" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L532" t="b">
+        <v>0</v>
+      </c>
+      <c r="M532" t="n">
+        <v>4.1687164</v>
+      </c>
+      <c r="N532" t="n">
+        <v>67045</v>
+      </c>
+      <c r="O532" t="n">
+        <v>10</v>
+      </c>
+      <c r="P532" t="inlineStr"/>
+      <c r="Q532" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R532" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S532" t="inlineStr">
+        <is>
+          <t>Aaaahhh, ta super app Max it, n&amp;#39;a pas fini de te surprendre... &lt;br&gt;Est-ce que tu as remarqué ? Maintenant, tu as ton QR code personnalisé en haut de ton écran d&amp;#39;accueil ! Ainsi, tu peux :&lt;br&gt;     scanner le QR code de ton ami(e) pour lui faire un transfert d&amp;#39;&amp;#39;argent&lt;br&gt;     scanner l</t>
+        </is>
+      </c>
+      <c r="T532" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U532" t="inlineStr"/>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G533" t="n">
+        <v>1061120855</v>
+      </c>
+      <c r="H533" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I533" t="inlineStr">
+        <is>
+          <t>Orange CI</t>
+        </is>
+      </c>
+      <c r="J533" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K533" t="n">
+        <v>0</v>
+      </c>
+      <c r="L533" t="b">
+        <v>1</v>
+      </c>
+      <c r="M533" t="n">
+        <v>3.78658</v>
+      </c>
+      <c r="N533" t="n">
+        <v>5960</v>
+      </c>
+      <c r="O533" t="n">
+        <v>7</v>
+      </c>
+      <c r="P533" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R533" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S533" t="inlineStr">
+        <is>
+          <t>Max it, la super app all-in-one te fais gagner du temps, et diminue tes soucis... Gagne plus d'espace de stockage sur ton téléphone ; plus besoin de cumuler plusieurs appli d'Orange pour avoir accès à un maximum de services. Max it est là ! Gère ta ligne (SIM) au niveau des pass, des soldes, réalise</t>
+        </is>
+      </c>
+      <c r="T533" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U533" t="inlineStr"/>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F534" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G534" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogw</t>
+        </is>
+      </c>
+      <c r="H534" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I534" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J534" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K534" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L534" t="b">
+        <v>0</v>
+      </c>
+      <c r="M534" t="n">
+        <v>4.4172187</v>
+      </c>
+      <c r="N534" t="n">
+        <v>1517</v>
+      </c>
+      <c r="O534" t="n">
+        <v>11</v>
+      </c>
+      <c r="P534" t="inlineStr"/>
+      <c r="Q534" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R534" t="inlineStr">
+        <is>
+          <t>4.0.18</t>
+        </is>
+      </c>
+      <c r="S534" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T534" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U534" t="inlineStr"/>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G535" t="n">
+        <v>1574668652</v>
+      </c>
+      <c r="H535" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I535" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J535" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K535" t="n">
+        <v>0</v>
+      </c>
+      <c r="L535" t="b">
+        <v>1</v>
+      </c>
+      <c r="M535" t="n">
+        <v>4.05333</v>
+      </c>
+      <c r="N535" t="n">
+        <v>75</v>
+      </c>
+      <c r="O535" t="n">
+        <v>1</v>
+      </c>
+      <c r="P535" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R535" t="inlineStr">
+        <is>
+          <t>6.0.35</t>
+        </is>
+      </c>
+      <c r="S535" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T535" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U535" t="inlineStr"/>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G536" t="inlineStr">
+        <is>
+          <t>com.orange.sugu.ocd</t>
+        </is>
+      </c>
+      <c r="H536" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I536" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J536" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K536" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L536" t="b">
+        <v>0</v>
+      </c>
+      <c r="M536" t="n">
+        <v>4.1247635</v>
+      </c>
+      <c r="N536" t="n">
+        <v>5272</v>
+      </c>
+      <c r="O536" t="n">
+        <v>83</v>
+      </c>
+      <c r="P536" t="inlineStr"/>
+      <c r="Q536" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R536" t="inlineStr">
+        <is>
+          <t>9.0.12</t>
+        </is>
+      </c>
+      <c r="S536" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DRC that brings together the features of MyOrange, and Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Plans, Mobile Payments, money transfers, bill payments, subscriptions, and entertai</t>
+        </is>
+      </c>
+      <c r="T536" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U536" t="inlineStr"/>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F537" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G537" t="n">
+        <v>6447896435</v>
+      </c>
+      <c r="H537" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I537" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J537" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K537" t="n">
+        <v>0</v>
+      </c>
+      <c r="L537" t="b">
+        <v>1</v>
+      </c>
+      <c r="M537" t="n">
+        <v>3.55762</v>
+      </c>
+      <c r="N537" t="n">
+        <v>269</v>
+      </c>
+      <c r="P537" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "CD" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R537" t="inlineStr">
+        <is>
+          <t>9.0.6</t>
+        </is>
+      </c>
+      <c r="S537" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DR Congo. It brings together the features of Orange et Moi, as well as Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Packages, Mobile payment, money transfers, bill payment and subscri</t>
+        </is>
+      </c>
+      <c r="T537" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U537" t="inlineStr"/>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F538" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G538" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ocm</t>
+        </is>
+      </c>
+      <c r="H538" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroon</t>
+        </is>
+      </c>
+      <c r="I538" t="inlineStr">
+        <is>
+          <t>Orange MEA</t>
+        </is>
+      </c>
+      <c r="J538" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K538" t="inlineStr">
+        <is>
+          <t>FCFA 0</t>
+        </is>
+      </c>
+      <c r="L538" t="b">
+        <v>0</v>
+      </c>
+      <c r="M538" t="n">
+        <v>3.9390895</v>
+      </c>
+      <c r="N538" t="n">
+        <v>46806</v>
+      </c>
+      <c r="O538" t="n">
+        <v>12</v>
+      </c>
+      <c r="P538" t="inlineStr"/>
+      <c r="Q538" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R538" t="inlineStr">
+        <is>
+          <t>7.0.23</t>
+        </is>
+      </c>
+      <c r="S538" t="inlineStr">
+        <is>
+          <t>Max it brings together everything that matters to you in one app: managing your lines, money transfer, bill payment, exclusive offers, and a universe of lifestyle and entertainment. Simple, fast, and 100% secure..&lt;br&gt;&lt;br&gt;📞 My line&lt;br&gt;Manage your Orange mobile and landline bundles in a single click:</t>
+        </is>
+      </c>
+      <c r="T538" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U538" t="inlineStr"/>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F539" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G539" t="n">
+        <v>1116920093</v>
+      </c>
+      <c r="H539" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroun</t>
+        </is>
+      </c>
+      <c r="I539" t="inlineStr">
+        <is>
+          <t>Orange Middle East &amp; Africa</t>
+        </is>
+      </c>
+      <c r="J539" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K539" t="n">
+        <v>0</v>
+      </c>
+      <c r="L539" t="b">
+        <v>1</v>
+      </c>
+      <c r="M539" t="n">
+        <v>3.76906</v>
+      </c>
+      <c r="N539" t="n">
+        <v>16143</v>
+      </c>
+      <c r="O539" t="n">
+        <v>2</v>
+      </c>
+      <c r="P539" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R539" t="inlineStr">
+        <is>
+          <t>7.0.24</t>
+        </is>
+      </c>
+      <c r="S539" t="inlineStr">
+        <is>
+          <t>Avec Max it, Orange rassemble tout ce qui compte pour vous dans une même application : la gestion de vos lignes, les transferts d’argent, payement de vos factures, des offres exclusives et un univers lifestyle et divertissement.
+Simple, rapide et 100 % sécurisée.
+Ma ligne
+Gérez vos forfaits mobiles</t>
+        </is>
+      </c>
+      <c r="T539" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U539" t="inlineStr"/>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G540" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obf</t>
+        </is>
+      </c>
+      <c r="H540" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I540" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso</t>
+        </is>
+      </c>
+      <c r="J540" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K540" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L540" t="b">
+        <v>0</v>
+      </c>
+      <c r="M540" t="n">
+        <v>4.1414537</v>
+      </c>
+      <c r="N540" t="n">
+        <v>25413</v>
+      </c>
+      <c r="O540" t="n">
+        <v>13</v>
+      </c>
+      <c r="P540" t="inlineStr"/>
+      <c r="Q540" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R540" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S540" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.&lt;br&gt;Gérez vos lignes mobiles, effectuez des transferts d&amp;#39;argent sécurisés, réglez vos factures, profitez d&amp;#39;offres exclusives, effectuez des paiements marchands fiables, et bien plus enco</t>
+        </is>
+      </c>
+      <c r="T540" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U540" t="inlineStr"/>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G541" t="n">
+        <v>1553774707</v>
+      </c>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I541" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso SA</t>
+        </is>
+      </c>
+      <c r="J541" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K541" t="n">
+        <v>0</v>
+      </c>
+      <c r="L541" t="b">
+        <v>1</v>
+      </c>
+      <c r="M541" t="n">
+        <v>3.45377</v>
+      </c>
+      <c r="N541" t="n">
+        <v>1179</v>
+      </c>
+      <c r="O541" t="n">
+        <v>3</v>
+      </c>
+      <c r="P541" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R541" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S541" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.
+Gérez vos lignes mobiles, effectuez des transferts d'argent sécurisés, réglez vos factures, profitez d'offres exclusives, effectuez des paiements marchands fiables, et bien plus encore, le tout</t>
+        </is>
+      </c>
+      <c r="T541" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U541" t="inlineStr"/>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G542" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obw</t>
+        </is>
+      </c>
+      <c r="H542" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I542" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J542" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K542" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L542" t="b">
+        <v>0</v>
+      </c>
+      <c r="M542" t="n">
+        <v>3.9929328</v>
+      </c>
+      <c r="N542" t="n">
+        <v>2962</v>
+      </c>
+      <c r="O542" t="n">
+        <v>48</v>
+      </c>
+      <c r="P542" t="inlineStr"/>
+      <c r="Q542" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R542" t="inlineStr">
+        <is>
+          <t>7.3.8</t>
+        </is>
+      </c>
+      <c r="S542" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it, the brand-new Orange Botswana Super App that follows Yame and gives you access to four distinct universes for a one-of-a-kind experience!&lt;br&gt;&lt;br&gt;Manage your accounts, make quick payments using QR codes, investigate a range of online goods and services, and discover the many options provided </t>
+        </is>
+      </c>
+      <c r="T542" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U542" t="inlineStr"/>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F543" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G543" t="n">
+        <v>1195839458</v>
+      </c>
+      <c r="H543" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I543" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J543" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K543" t="n">
+        <v>0</v>
+      </c>
+      <c r="L543" t="b">
+        <v>1</v>
+      </c>
+      <c r="M543" t="n">
+        <v>3.00806</v>
+      </c>
+      <c r="N543" t="n">
+        <v>124</v>
+      </c>
+      <c r="O543" t="n">
+        <v>30</v>
+      </c>
+      <c r="P543" t="inlineStr"/>
+      <c r="R543" t="inlineStr">
+        <is>
+          <t>7.3.1</t>
+        </is>
+      </c>
+      <c r="S543" t="inlineStr">
+        <is>
+          <t>A free mobile self-care application for Orange Botswana’s mobile customers.
+Full Description :
+Max it is a free application, which allows Orange Botswana customers to:
+- Consult your account in real time: minutes, sms, internet ...
+- Top up your account or a friend account  with Orange Money
+-</t>
+        </is>
+      </c>
+      <c r="T543" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U543" t="inlineStr"/>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F544" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G544" t="inlineStr">
+        <is>
+          <t>com.orange.mobinilandme</t>
+        </is>
+      </c>
+      <c r="H544" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I544" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J544" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K544" t="inlineStr">
+        <is>
+          <t>EGP 0.00</t>
+        </is>
+      </c>
+      <c r="L544" t="b">
+        <v>0</v>
+      </c>
+      <c r="M544" t="n">
+        <v>4.562493</v>
+      </c>
+      <c r="N544" t="n">
+        <v>923823</v>
+      </c>
+      <c r="O544" t="n">
+        <v>24</v>
+      </c>
+      <c r="P544" t="inlineStr"/>
+      <c r="Q544" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R544" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S544" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion&lt;br&gt;Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.&lt;br&gt;Key services include:&lt;br&gt;• Account Management: Easily manage</t>
+        </is>
+      </c>
+      <c r="T544" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U544" t="inlineStr"/>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>edb3c406-9106-4f9f-9993-27f2f4934642</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:27:31</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G545" t="n">
+        <v>942568333</v>
+      </c>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I545" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J545" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K545" t="n">
+        <v>0</v>
+      </c>
+      <c r="L545" t="b">
+        <v>1</v>
+      </c>
+      <c r="M545" t="n">
+        <v>4.251</v>
+      </c>
+      <c r="N545" t="n">
+        <v>116906</v>
+      </c>
+      <c r="O545" t="n">
+        <v>64</v>
+      </c>
+      <c r="P545" t="inlineStr"/>
+      <c r="R545" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S545" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion
+Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.
+Key services include:
+• Account Management: Easily manage your Ora</t>
+        </is>
+      </c>
+      <c r="T545" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U545" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-07-25
</commit_message>
<xml_diff>
--- a/maxit_store_history.xlsx
+++ b/maxit_store_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U545"/>
+  <dimension ref="A1:U577"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44122,7 +44122,6 @@
       <c r="O514" t="n">
         <v>19</v>
       </c>
-      <c r="P514" t="inlineStr"/>
       <c r="Q514" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -44143,7 +44142,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U514" t="inlineStr"/>
     </row>
     <row r="515">
       <c r="A515" t="inlineStr">
@@ -44206,7 +44204,6 @@
       <c r="N515" t="n">
         <v>321</v>
       </c>
-      <c r="P515" t="inlineStr"/>
       <c r="R515" t="inlineStr">
         <is>
           <t>6.4.8</t>
@@ -44222,7 +44219,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U515" t="inlineStr"/>
     </row>
     <row r="516">
       <c r="A516" t="inlineStr">
@@ -44292,7 +44288,6 @@
       <c r="O516" t="n">
         <v>38</v>
       </c>
-      <c r="P516" t="inlineStr"/>
       <c r="Q516" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -44313,7 +44308,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U516" t="inlineStr"/>
     </row>
     <row r="517">
       <c r="A517" t="inlineStr">
@@ -44379,7 +44373,6 @@
       <c r="O517" t="n">
         <v>38</v>
       </c>
-      <c r="P517" t="inlineStr"/>
       <c r="R517" t="inlineStr">
         <is>
           <t>10.0.6</t>
@@ -44397,7 +44390,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U517" t="inlineStr"/>
     </row>
     <row r="518">
       <c r="A518" t="inlineStr">
@@ -44467,7 +44459,6 @@
       <c r="O518" t="n">
         <v>11</v>
       </c>
-      <c r="P518" t="inlineStr"/>
       <c r="Q518" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -44488,7 +44479,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U518" t="inlineStr"/>
     </row>
     <row r="519">
       <c r="A519" t="inlineStr">
@@ -44577,7 +44567,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U519" t="inlineStr"/>
     </row>
     <row r="520">
       <c r="A520" t="inlineStr">
@@ -44647,7 +44636,6 @@
       <c r="O520" t="n">
         <v>12</v>
       </c>
-      <c r="P520" t="inlineStr"/>
       <c r="Q520" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -44668,7 +44656,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U520" t="inlineStr"/>
     </row>
     <row r="521">
       <c r="A521" t="inlineStr">
@@ -44734,7 +44721,6 @@
       <c r="O521" t="n">
         <v>15</v>
       </c>
-      <c r="P521" t="inlineStr"/>
       <c r="R521" t="inlineStr">
         <is>
           <t>21.1.0</t>
@@ -44752,7 +44738,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U521" t="inlineStr"/>
     </row>
     <row r="522">
       <c r="A522" t="inlineStr">
@@ -44822,7 +44807,6 @@
       <c r="O522" t="n">
         <v>149</v>
       </c>
-      <c r="P522" t="inlineStr"/>
       <c r="Q522" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -44843,7 +44827,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U522" t="inlineStr"/>
     </row>
     <row r="523">
       <c r="A523" t="inlineStr">
@@ -44928,7 +44911,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U523" t="inlineStr"/>
     </row>
     <row r="524">
       <c r="A524" t="inlineStr">
@@ -44995,7 +44977,6 @@
       <c r="N524" t="n">
         <v>38255</v>
       </c>
-      <c r="P524" t="inlineStr"/>
       <c r="Q524" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -45016,7 +44997,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U524" t="inlineStr"/>
     </row>
     <row r="525">
       <c r="A525" t="inlineStr">
@@ -45082,7 +45062,6 @@
       <c r="O525" t="n">
         <v>11</v>
       </c>
-      <c r="P525" t="inlineStr"/>
       <c r="R525" t="inlineStr">
         <is>
           <t>6.5.2</t>
@@ -45101,7 +45080,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U525" t="inlineStr"/>
     </row>
     <row r="526">
       <c r="A526" t="inlineStr">
@@ -45171,7 +45149,6 @@
       <c r="O526" t="n">
         <v>42</v>
       </c>
-      <c r="P526" t="inlineStr"/>
       <c r="Q526" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -45192,7 +45169,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U526" t="inlineStr"/>
     </row>
     <row r="527">
       <c r="A527" t="inlineStr">
@@ -45258,7 +45234,6 @@
       <c r="O527" t="n">
         <v>26</v>
       </c>
-      <c r="P527" t="inlineStr"/>
       <c r="R527" t="inlineStr">
         <is>
           <t>5.0.2</t>
@@ -45276,7 +45251,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U527" t="inlineStr"/>
     </row>
     <row r="528">
       <c r="A528" t="inlineStr">
@@ -45346,7 +45320,6 @@
       <c r="O528" t="n">
         <v>75</v>
       </c>
-      <c r="P528" t="inlineStr"/>
       <c r="Q528" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -45367,7 +45340,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U528" t="inlineStr"/>
     </row>
     <row r="529">
       <c r="A529" t="inlineStr">
@@ -45455,7 +45427,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U529" t="inlineStr"/>
     </row>
     <row r="530">
       <c r="A530" t="inlineStr">
@@ -45525,7 +45496,6 @@
       <c r="O530" t="n">
         <v>52</v>
       </c>
-      <c r="P530" t="inlineStr"/>
       <c r="Q530" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -45546,7 +45516,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U530" t="inlineStr"/>
     </row>
     <row r="531">
       <c r="A531" t="inlineStr">
@@ -45612,7 +45581,6 @@
       <c r="O531" t="n">
         <v>48</v>
       </c>
-      <c r="P531" t="inlineStr"/>
       <c r="R531" t="inlineStr">
         <is>
           <t>10.0.21</t>
@@ -45631,7 +45599,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U531" t="inlineStr"/>
     </row>
     <row r="532">
       <c r="A532" t="inlineStr">
@@ -45701,7 +45668,6 @@
       <c r="O532" t="n">
         <v>10</v>
       </c>
-      <c r="P532" t="inlineStr"/>
       <c r="Q532" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -45722,7 +45688,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U532" t="inlineStr"/>
     </row>
     <row r="533">
       <c r="A533" t="inlineStr">
@@ -45808,7 +45773,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U533" t="inlineStr"/>
     </row>
     <row r="534">
       <c r="A534" t="inlineStr">
@@ -45878,7 +45842,6 @@
       <c r="O534" t="n">
         <v>11</v>
       </c>
-      <c r="P534" t="inlineStr"/>
       <c r="Q534" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -45899,7 +45862,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U534" t="inlineStr"/>
     </row>
     <row r="535">
       <c r="A535" t="inlineStr">
@@ -45985,7 +45947,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U535" t="inlineStr"/>
     </row>
     <row r="536">
       <c r="A536" t="inlineStr">
@@ -46055,7 +46016,6 @@
       <c r="O536" t="n">
         <v>83</v>
       </c>
-      <c r="P536" t="inlineStr"/>
       <c r="Q536" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -46076,7 +46036,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U536" t="inlineStr"/>
     </row>
     <row r="537">
       <c r="A537" t="inlineStr">
@@ -46159,7 +46118,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U537" t="inlineStr"/>
     </row>
     <row r="538">
       <c r="A538" t="inlineStr">
@@ -46229,7 +46187,6 @@
       <c r="O538" t="n">
         <v>12</v>
       </c>
-      <c r="P538" t="inlineStr"/>
       <c r="Q538" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -46250,7 +46207,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U538" t="inlineStr"/>
     </row>
     <row r="539">
       <c r="A539" t="inlineStr">
@@ -46339,7 +46295,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U539" t="inlineStr"/>
     </row>
     <row r="540">
       <c r="A540" t="inlineStr">
@@ -46409,7 +46364,6 @@
       <c r="O540" t="n">
         <v>13</v>
       </c>
-      <c r="P540" t="inlineStr"/>
       <c r="Q540" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -46430,7 +46384,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U540" t="inlineStr"/>
     </row>
     <row r="541">
       <c r="A541" t="inlineStr">
@@ -46517,7 +46470,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U541" t="inlineStr"/>
     </row>
     <row r="542">
       <c r="A542" t="inlineStr">
@@ -46587,7 +46539,6 @@
       <c r="O542" t="n">
         <v>48</v>
       </c>
-      <c r="P542" t="inlineStr"/>
       <c r="Q542" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -46608,7 +46559,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U542" t="inlineStr"/>
     </row>
     <row r="543">
       <c r="A543" t="inlineStr">
@@ -46674,7 +46624,6 @@
       <c r="O543" t="n">
         <v>30</v>
       </c>
-      <c r="P543" t="inlineStr"/>
       <c r="R543" t="inlineStr">
         <is>
           <t>7.3.1</t>
@@ -46695,7 +46644,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U543" t="inlineStr"/>
     </row>
     <row r="544">
       <c r="A544" t="inlineStr">
@@ -46765,7 +46713,6 @@
       <c r="O544" t="n">
         <v>24</v>
       </c>
-      <c r="P544" t="inlineStr"/>
       <c r="Q544" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -46786,7 +46733,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U544" t="inlineStr"/>
     </row>
     <row r="545">
       <c r="A545" t="inlineStr">
@@ -46852,7 +46798,6 @@
       <c r="O545" t="n">
         <v>64</v>
       </c>
-      <c r="P545" t="inlineStr"/>
       <c r="R545" t="inlineStr">
         <is>
           <t>10.1.0</t>
@@ -46871,7 +46816,2825 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U545" t="inlineStr"/>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F546" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G546" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogn</t>
+        </is>
+      </c>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I546" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J546" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K546" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L546" t="b">
+        <v>0</v>
+      </c>
+      <c r="M546" t="n">
+        <v>4.4457703</v>
+      </c>
+      <c r="N546" t="n">
+        <v>9251</v>
+      </c>
+      <c r="O546" t="n">
+        <v>20</v>
+      </c>
+      <c r="P546" t="inlineStr"/>
+      <c r="Q546" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R546" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S546" t="inlineStr">
+        <is>
+          <t>Bien plus qu&amp;#39;une application, un véritable assistant personnel pour une vie connectée et simplifiée.&lt;br&gt;Suivi de consommation: Votre tableau de bord tout-en-un pour une gestion simplifiée !&lt;br&gt;- Gestion de votre offre: Accédez à une vue détaillée de votre offre actuelle et de vos forfaits Orange</t>
+        </is>
+      </c>
+      <c r="T546" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U546" t="inlineStr"/>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G547" t="n">
+        <v>1177999485</v>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I547" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J547" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K547" t="n">
+        <v>0</v>
+      </c>
+      <c r="L547" t="b">
+        <v>1</v>
+      </c>
+      <c r="M547" t="n">
+        <v>3.90343</v>
+      </c>
+      <c r="N547" t="n">
+        <v>321</v>
+      </c>
+      <c r="P547" t="inlineStr"/>
+      <c r="R547" t="inlineStr">
+        <is>
+          <t>6.4.8</t>
+        </is>
+      </c>
+      <c r="S547" t="inlineStr">
+        <is>
+          <t>La fusion d’Orange et Moi et Orange Money donne naissance à Max it, la nouvelle Super Application Tout-en-Un. Profitez du suivi de consommation, de paiements mobiles, de toutes les fonctionnalités Orange et Moi et Money avec un large éventail de divertissements, le tout regroupé en un seul endroit !</t>
+        </is>
+      </c>
+      <c r="T547" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U547" t="inlineStr"/>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F548" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G548" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.otn</t>
+        </is>
+      </c>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K548" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L548" t="b">
+        <v>0</v>
+      </c>
+      <c r="M548" t="n">
+        <v>3.9660208</v>
+      </c>
+      <c r="N548" t="n">
+        <v>35358</v>
+      </c>
+      <c r="O548" t="n">
+        <v>30</v>
+      </c>
+      <c r="P548" t="inlineStr"/>
+      <c r="Q548" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R548" t="inlineStr">
+        <is>
+          <t>10.0.6</t>
+        </is>
+      </c>
+      <c r="S548" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Max it par Orange Tunisie facilite votre vie au quotidien !&lt;/h2&gt;&lt;br&gt;&lt;br&gt;Welcome sur Max it !&lt;br&gt;Accédez rapidement à vos fonctionnalités Max it préférées et profitez également de contenus exclusifs, d’activités divertissantes, et de jeux interactifs pour une expérience enrichissante avec la roue</t>
+        </is>
+      </c>
+      <c r="T548" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U548" t="inlineStr"/>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G549" t="n">
+        <v>1146892088</v>
+      </c>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K549" t="n">
+        <v>0</v>
+      </c>
+      <c r="L549" t="b">
+        <v>1</v>
+      </c>
+      <c r="M549" t="n">
+        <v>3.02812</v>
+      </c>
+      <c r="N549" t="n">
+        <v>1636</v>
+      </c>
+      <c r="O549" t="n">
+        <v>34</v>
+      </c>
+      <c r="P549" t="inlineStr"/>
+      <c r="R549" t="inlineStr">
+        <is>
+          <t>10.0.6</t>
+        </is>
+      </c>
+      <c r="S549" t="inlineStr">
+        <is>
+          <t>Max it by Orange Tunisie : Votre appli incontournable pour une vie connectée
+Welcome sur Max it : Découvrez fonctionnalités, jeux &amp; contenus de divertissement by Orange Tunisie !
+Trouvez vite vos fonctionnalités Max it favorites et explorez des contenus exclusifs et des jeux pour une expérience im</t>
+        </is>
+      </c>
+      <c r="T549" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U549" t="inlineStr"/>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G550" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osl</t>
+        </is>
+      </c>
+      <c r="H550" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I550" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J550" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K550" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L550" t="b">
+        <v>0</v>
+      </c>
+      <c r="M550" t="n">
+        <v>4.3568077</v>
+      </c>
+      <c r="N550" t="n">
+        <v>2119</v>
+      </c>
+      <c r="O550" t="n">
+        <v>11</v>
+      </c>
+      <c r="P550" t="inlineStr"/>
+      <c r="Q550" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R550" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S550" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it is a free application, which allows Orange Sierra Leone prepaid and postpaid customers to:&lt;br&gt;&lt;br&gt;- Consult your account in real time: minutes, sms, internet&lt;br&gt;- Top up your account or a friend account &lt;br&gt;- Buy Internet Bundles&lt;br&gt;- Discover the latest offers and promotions &lt;br&gt;- Access to </t>
+        </is>
+      </c>
+      <c r="T550" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U550" t="inlineStr"/>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G551" t="n">
+        <v>6443607903</v>
+      </c>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I551" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J551" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K551" t="n">
+        <v>0</v>
+      </c>
+      <c r="L551" t="b">
+        <v>1</v>
+      </c>
+      <c r="M551" t="n">
+        <v>3.69948</v>
+      </c>
+      <c r="N551" t="n">
+        <v>193</v>
+      </c>
+      <c r="O551" t="n">
+        <v>6</v>
+      </c>
+      <c r="P551" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R551" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S551" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The merger of My Orange &amp; Orange Money has given birth to Max it the all-in-one super app, a free application which allows all Orange Sierra Leone customers to 
+Track calls, SMS, and Data usage and monitor balance. 
+Make a secure mobile/Orange Money payment.
+Easily transfer credit to other users </t>
+        </is>
+      </c>
+      <c r="T551" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U551" t="inlineStr"/>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F552" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G552" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osn</t>
+        </is>
+      </c>
+      <c r="H552" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I552" t="inlineStr">
+        <is>
+          <t>Orange Sénégal</t>
+        </is>
+      </c>
+      <c r="J552" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K552" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L552" t="b">
+        <v>0</v>
+      </c>
+      <c r="M552" t="n">
+        <v>4.312102</v>
+      </c>
+      <c r="N552" t="n">
+        <v>51160</v>
+      </c>
+      <c r="O552" t="n">
+        <v>14</v>
+      </c>
+      <c r="P552" t="inlineStr"/>
+      <c r="Q552" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R552" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S552" t="inlineStr">
+        <is>
+          <t>Lu bees ak Max it ! &lt;br&gt;Une application repensée pour être plus simple, plus rapide et adaptée à vos besoins. Une expérience optimisée pour faciliter vos usages au quotidien, avec des parcours simplifiés et un accès plus fluide à vos services. Que vous soyez client Orange ou non, Max it vous accompa</t>
+        </is>
+      </c>
+      <c r="T552" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U552" t="inlineStr"/>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F553" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G553" t="n">
+        <v>1039327980</v>
+      </c>
+      <c r="H553" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I553" t="inlineStr">
+        <is>
+          <t>Orange Senegal</t>
+        </is>
+      </c>
+      <c r="J553" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K553" t="n">
+        <v>0</v>
+      </c>
+      <c r="L553" t="b">
+        <v>1</v>
+      </c>
+      <c r="M553" t="n">
+        <v>4.16974</v>
+      </c>
+      <c r="N553" t="n">
+        <v>30210</v>
+      </c>
+      <c r="O553" t="n">
+        <v>13</v>
+      </c>
+      <c r="P553" t="inlineStr"/>
+      <c r="R553" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S553" t="inlineStr">
+        <is>
+          <t>Here is the English translation:
+Welcome to Max it!
+A redesigned app to be simpler, faster, and tailored to your needs. An optimized experience to make your daily life easier, with streamlined journeys and smoother access to your services. Whether you are an Orange customer or not, Max it is your e</t>
+        </is>
+      </c>
+      <c r="T553" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U553" t="inlineStr"/>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F554" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G554" t="inlineStr">
+        <is>
+          <t>com.orange.meditel.mediteletmoi</t>
+        </is>
+      </c>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I554" t="inlineStr">
+        <is>
+          <t>Orange Maroc</t>
+        </is>
+      </c>
+      <c r="J554" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K554" t="inlineStr">
+        <is>
+          <t>MAD 0.00</t>
+        </is>
+      </c>
+      <c r="L554" t="b">
+        <v>0</v>
+      </c>
+      <c r="M554" t="n">
+        <v>3.7243414</v>
+      </c>
+      <c r="N554" t="n">
+        <v>110895</v>
+      </c>
+      <c r="O554" t="n">
+        <v>118</v>
+      </c>
+      <c r="P554" t="inlineStr"/>
+      <c r="Q554" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R554" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S554" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l&amp;#39;expérience mobile réinventé&lt;br&gt;&lt;br&gt;Max it, c&amp;#39;est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d&amp;#39;une multitude de services exclusifs. &lt;br&gt;&lt;br&gt;Créez votre espace sur</t>
+        </is>
+      </c>
+      <c r="T554" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U554" t="inlineStr"/>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F555" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G555" t="n">
+        <v>596028698</v>
+      </c>
+      <c r="H555" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I555" t="inlineStr">
+        <is>
+          <t>Méditel</t>
+        </is>
+      </c>
+      <c r="J555" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K555" t="n">
+        <v>0</v>
+      </c>
+      <c r="L555" t="b">
+        <v>1</v>
+      </c>
+      <c r="M555" t="n">
+        <v>3.94766</v>
+      </c>
+      <c r="N555" t="n">
+        <v>2751</v>
+      </c>
+      <c r="P555" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "MA" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R555" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S555" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l'expérience mobile réinventé
+Max it, c'est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d'une multitude de services exclusifs. 
+Créez votre espace sur mesure et bénéficiez d'</t>
+        </is>
+      </c>
+      <c r="T555" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U555" t="inlineStr"/>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F556" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G556" t="inlineStr">
+        <is>
+          <t>com.oml.dsi.orangemobile</t>
+        </is>
+      </c>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J556" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K556" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L556" t="b">
+        <v>0</v>
+      </c>
+      <c r="M556" t="n">
+        <v>2.6960042</v>
+      </c>
+      <c r="N556" t="n">
+        <v>38254</v>
+      </c>
+      <c r="P556" t="inlineStr"/>
+      <c r="Q556" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R556" t="inlineStr">
+        <is>
+          <t>6.5.0</t>
+        </is>
+      </c>
+      <c r="S556" t="inlineStr">
+        <is>
+          <t>Easily manage your Orange Mali line&lt;br&gt;● Manage your account and view all essential information, your offers, and your phone lines.&lt;br&gt;● Subscribe to call, SMS, Internet, and international call packages.&lt;br&gt;● Track your usage by checking your credit and Internet balance.&lt;br&gt;● Recharge your line by p</t>
+        </is>
+      </c>
+      <c r="T556" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U556" t="inlineStr"/>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G557" t="n">
+        <v>1494321079</v>
+      </c>
+      <c r="H557" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I557" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J557" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K557" t="n">
+        <v>0</v>
+      </c>
+      <c r="L557" t="b">
+        <v>1</v>
+      </c>
+      <c r="M557" t="n">
+        <v>2.5206</v>
+      </c>
+      <c r="N557" t="n">
+        <v>4733</v>
+      </c>
+      <c r="O557" t="n">
+        <v>9</v>
+      </c>
+      <c r="P557" t="inlineStr"/>
+      <c r="R557" t="inlineStr">
+        <is>
+          <t>6.5.2</t>
+        </is>
+      </c>
+      <c r="S557" t="inlineStr">
+        <is>
+          <t>Gérez facilement votre ligne Orange Mali 
+●        Gérez votre compte et consultez toutes les informations essentielles sur celui-ci, vos offres, ainsi que vos lignes téléphoniques.
+●        Souscrivez aux forfaits appels, SMS, Internet, et appels internationaux.
+●        Suivez votre consommation e</t>
+        </is>
+      </c>
+      <c r="T557" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U557" t="inlineStr"/>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F558" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G558" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.omg</t>
+        </is>
+      </c>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I558" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J558" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K558" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L558" t="b">
+        <v>0</v>
+      </c>
+      <c r="M558" t="n">
+        <v>4.18797</v>
+      </c>
+      <c r="N558" t="n">
+        <v>1367</v>
+      </c>
+      <c r="O558" t="n">
+        <v>48</v>
+      </c>
+      <c r="P558" t="inlineStr"/>
+      <c r="Q558" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R558" t="inlineStr">
+        <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="S558" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.&lt;br&gt;&lt;br&gt;Simplify Your Life with Max it&lt;br&gt;With Max It, ac</t>
+        </is>
+      </c>
+      <c r="T558" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U558" t="inlineStr"/>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G559" t="n">
+        <v>1295171817</v>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J559" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K559" t="n">
+        <v>0</v>
+      </c>
+      <c r="L559" t="b">
+        <v>1</v>
+      </c>
+      <c r="M559" t="n">
+        <v>3.08696</v>
+      </c>
+      <c r="N559" t="n">
+        <v>69</v>
+      </c>
+      <c r="O559" t="n">
+        <v>29</v>
+      </c>
+      <c r="P559" t="inlineStr"/>
+      <c r="R559" t="inlineStr">
+        <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="S559" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.
+Simplify Your Life with Max it
+With Max it, access a se</t>
+        </is>
+      </c>
+      <c r="T559" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U559" t="inlineStr"/>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F560" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.olr</t>
+        </is>
+      </c>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>Orange Max it - Liberia</t>
+        </is>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J560" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K560" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L560" t="b">
+        <v>0</v>
+      </c>
+      <c r="M560" t="n">
+        <v>4.5434084</v>
+      </c>
+      <c r="N560" t="n">
+        <v>3092</v>
+      </c>
+      <c r="O560" t="n">
+        <v>72</v>
+      </c>
+      <c r="P560" t="inlineStr"/>
+      <c r="Q560" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R560" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="S560" t="inlineStr">
+        <is>
+          <t>Max it: your personalized experience by Orange Liberia!&lt;br&gt;&lt;br&gt;Step into Max it, your all-in-one solution for telecom, marketplace, and financial services! Manage your mobile line, customize offers, pay your bills, keep&lt;br&gt;track of your usage with ease, and recharge your credit. Access exclusive eve</t>
+        </is>
+      </c>
+      <c r="T560" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U560" t="inlineStr"/>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G561" t="n">
+        <v>6746187327</v>
+      </c>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>Orange Max it – Liberia</t>
+        </is>
+      </c>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J561" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K561" t="n">
+        <v>0</v>
+      </c>
+      <c r="L561" t="b">
+        <v>1</v>
+      </c>
+      <c r="M561" t="n">
+        <v>4.0625</v>
+      </c>
+      <c r="N561" t="n">
+        <v>48</v>
+      </c>
+      <c r="P561" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "LR" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R561" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="S561" t="inlineStr">
+        <is>
+          <t>Max it is a free application, which allows Orange Liberia customers to:
+- Consult your account in real time: minutes, sms, internet
+- Top up your account or a friend account 
+- Buy  Bundles (voice, data, SMS, roaming, international)
+- Discover the latest offers and promotions 
+- Access to Orange se</t>
+        </is>
+      </c>
+      <c r="T561" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U561" t="inlineStr"/>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ojo</t>
+        </is>
+      </c>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I562" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J562" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K562" t="inlineStr">
+        <is>
+          <t>JOD 0.000</t>
+        </is>
+      </c>
+      <c r="L562" t="b">
+        <v>0</v>
+      </c>
+      <c r="M562" t="n">
+        <v>4.4343834</v>
+      </c>
+      <c r="N562" t="n">
+        <v>97611</v>
+      </c>
+      <c r="O562" t="n">
+        <v>46</v>
+      </c>
+      <c r="P562" t="inlineStr"/>
+      <c r="Q562" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R562" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S562" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience&lt;br&gt;Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.&lt;br&gt;Important Update:&lt;br&gt;The jood app (jood Orange) w</t>
+        </is>
+      </c>
+      <c r="T562" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U562" t="inlineStr"/>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G563" t="n">
+        <v>808824590</v>
+      </c>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I563" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J563" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K563" t="n">
+        <v>0</v>
+      </c>
+      <c r="L563" t="b">
+        <v>1</v>
+      </c>
+      <c r="M563" t="n">
+        <v>4.21265</v>
+      </c>
+      <c r="N563" t="n">
+        <v>3005</v>
+      </c>
+      <c r="O563" t="n">
+        <v>53</v>
+      </c>
+      <c r="P563" t="inlineStr"/>
+      <c r="R563" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S563" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience
+Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.
+Important Update:
+The jood app (jood Orange) will be di</t>
+        </is>
+      </c>
+      <c r="T563" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U563" t="inlineStr"/>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.oci</t>
+        </is>
+      </c>
+      <c r="H564" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I564" t="inlineStr">
+        <is>
+          <t>Orange Côte d'Ivoire S.A</t>
+        </is>
+      </c>
+      <c r="J564" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K564" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L564" t="b">
+        <v>0</v>
+      </c>
+      <c r="M564" t="n">
+        <v>4.1701875</v>
+      </c>
+      <c r="N564" t="n">
+        <v>67076</v>
+      </c>
+      <c r="O564" t="n">
+        <v>10</v>
+      </c>
+      <c r="P564" t="inlineStr"/>
+      <c r="Q564" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R564" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S564" t="inlineStr">
+        <is>
+          <t>Aaaahhh, ta super app Max it, n&amp;#39;a pas fini de te surprendre... &lt;br&gt;Est-ce que tu as remarqué ? Maintenant, tu as ton QR code personnalisé en haut de ton écran d&amp;#39;accueil ! Ainsi, tu peux :&lt;br&gt;     scanner le QR code de ton ami(e) pour lui faire un transfert d&amp;#39;&amp;#39;argent&lt;br&gt;     scanner l</t>
+        </is>
+      </c>
+      <c r="T564" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U564" t="inlineStr"/>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G565" t="n">
+        <v>1061120855</v>
+      </c>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>Orange CI</t>
+        </is>
+      </c>
+      <c r="J565" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K565" t="n">
+        <v>0</v>
+      </c>
+      <c r="L565" t="b">
+        <v>1</v>
+      </c>
+      <c r="M565" t="n">
+        <v>3.78722</v>
+      </c>
+      <c r="N565" t="n">
+        <v>5964</v>
+      </c>
+      <c r="O565" t="n">
+        <v>2</v>
+      </c>
+      <c r="P565" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R565" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S565" t="inlineStr">
+        <is>
+          <t>Max it, la super app all-in-one te fais gagner du temps, et diminue tes soucis... Gagne plus d'espace de stockage sur ton téléphone ; plus besoin de cumuler plusieurs appli d'Orange pour avoir accès à un maximum de services. Max it est là ! Gère ta ligne (SIM) au niveau des pass, des soldes, réalise</t>
+        </is>
+      </c>
+      <c r="T565" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U565" t="inlineStr"/>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogw</t>
+        </is>
+      </c>
+      <c r="H566" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I566" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J566" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K566" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L566" t="b">
+        <v>0</v>
+      </c>
+      <c r="M566" t="n">
+        <v>4.3533335</v>
+      </c>
+      <c r="N566" t="n">
+        <v>1523</v>
+      </c>
+      <c r="O566" t="n">
+        <v>5</v>
+      </c>
+      <c r="P566" t="inlineStr"/>
+      <c r="Q566" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R566" t="inlineStr">
+        <is>
+          <t>4.0.18</t>
+        </is>
+      </c>
+      <c r="S566" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T566" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U566" t="inlineStr"/>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G567" t="n">
+        <v>1574668652</v>
+      </c>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J567" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K567" t="n">
+        <v>0</v>
+      </c>
+      <c r="L567" t="b">
+        <v>1</v>
+      </c>
+      <c r="M567" t="n">
+        <v>4.05333</v>
+      </c>
+      <c r="N567" t="n">
+        <v>75</v>
+      </c>
+      <c r="O567" t="n">
+        <v>2</v>
+      </c>
+      <c r="P567" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R567" t="inlineStr">
+        <is>
+          <t>6.0.35</t>
+        </is>
+      </c>
+      <c r="S567" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T567" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U567" t="inlineStr"/>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>com.orange.sugu.ocd</t>
+        </is>
+      </c>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I568" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J568" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K568" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L568" t="b">
+        <v>0</v>
+      </c>
+      <c r="M568" t="n">
+        <v>4.1148777</v>
+      </c>
+      <c r="N568" t="n">
+        <v>5272</v>
+      </c>
+      <c r="O568" t="n">
+        <v>83</v>
+      </c>
+      <c r="P568" t="inlineStr"/>
+      <c r="Q568" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R568" t="inlineStr">
+        <is>
+          <t>9.0.12</t>
+        </is>
+      </c>
+      <c r="S568" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DRC that brings together the features of MyOrange, and Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Plans, Mobile Payments, money transfers, bill payments, subscriptions, and entertai</t>
+        </is>
+      </c>
+      <c r="T568" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U568" t="inlineStr"/>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G569" t="n">
+        <v>6447896435</v>
+      </c>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J569" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K569" t="n">
+        <v>0</v>
+      </c>
+      <c r="L569" t="b">
+        <v>1</v>
+      </c>
+      <c r="M569" t="n">
+        <v>3.55762</v>
+      </c>
+      <c r="N569" t="n">
+        <v>269</v>
+      </c>
+      <c r="P569" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "CD" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R569" t="inlineStr">
+        <is>
+          <t>9.0.6</t>
+        </is>
+      </c>
+      <c r="S569" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DR Congo. It brings together the features of Orange et Moi, as well as Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Packages, Mobile payment, money transfers, bill payment and subscri</t>
+        </is>
+      </c>
+      <c r="T569" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U569" t="inlineStr"/>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G570" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ocm</t>
+        </is>
+      </c>
+      <c r="H570" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroon</t>
+        </is>
+      </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>Orange MEA</t>
+        </is>
+      </c>
+      <c r="J570" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K570" t="inlineStr">
+        <is>
+          <t>FCFA 0</t>
+        </is>
+      </c>
+      <c r="L570" t="b">
+        <v>0</v>
+      </c>
+      <c r="M570" t="n">
+        <v>3.9374335</v>
+      </c>
+      <c r="N570" t="n">
+        <v>46825</v>
+      </c>
+      <c r="O570" t="n">
+        <v>12</v>
+      </c>
+      <c r="P570" t="inlineStr"/>
+      <c r="Q570" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R570" t="inlineStr">
+        <is>
+          <t>7.0.23</t>
+        </is>
+      </c>
+      <c r="S570" t="inlineStr">
+        <is>
+          <t>Max it brings together everything that matters to you in one app: managing your lines, money transfer, bill payment, exclusive offers, and a universe of lifestyle and entertainment. Simple, fast, and 100% secure..&lt;br&gt;&lt;br&gt;📞 My line&lt;br&gt;Manage your Orange mobile and landline bundles in a single click:</t>
+        </is>
+      </c>
+      <c r="T570" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U570" t="inlineStr"/>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G571" t="n">
+        <v>1116920093</v>
+      </c>
+      <c r="H571" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroun</t>
+        </is>
+      </c>
+      <c r="I571" t="inlineStr">
+        <is>
+          <t>Orange Middle East &amp; Africa</t>
+        </is>
+      </c>
+      <c r="J571" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K571" t="n">
+        <v>0</v>
+      </c>
+      <c r="L571" t="b">
+        <v>1</v>
+      </c>
+      <c r="M571" t="n">
+        <v>3.7688</v>
+      </c>
+      <c r="N571" t="n">
+        <v>16146</v>
+      </c>
+      <c r="O571" t="n">
+        <v>2</v>
+      </c>
+      <c r="P571" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R571" t="inlineStr">
+        <is>
+          <t>7.0.24</t>
+        </is>
+      </c>
+      <c r="S571" t="inlineStr">
+        <is>
+          <t>Avec Max it, Orange rassemble tout ce qui compte pour vous dans une même application : la gestion de vos lignes, les transferts d’argent, payement de vos factures, des offres exclusives et un univers lifestyle et divertissement.
+Simple, rapide et 100 % sécurisée.
+Ma ligne
+Gérez vos forfaits mobiles</t>
+        </is>
+      </c>
+      <c r="T571" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U571" t="inlineStr"/>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G572" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obf</t>
+        </is>
+      </c>
+      <c r="H572" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso</t>
+        </is>
+      </c>
+      <c r="J572" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K572" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L572" t="b">
+        <v>0</v>
+      </c>
+      <c r="M572" t="n">
+        <v>4.147901</v>
+      </c>
+      <c r="N572" t="n">
+        <v>25430</v>
+      </c>
+      <c r="O572" t="n">
+        <v>13</v>
+      </c>
+      <c r="P572" t="inlineStr"/>
+      <c r="Q572" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R572" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S572" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.&lt;br&gt;Gérez vos lignes mobiles, effectuez des transferts d&amp;#39;argent sécurisés, réglez vos factures, profitez d&amp;#39;offres exclusives, effectuez des paiements marchands fiables, et bien plus enco</t>
+        </is>
+      </c>
+      <c r="T572" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U572" t="inlineStr"/>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G573" t="n">
+        <v>1553774707</v>
+      </c>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso SA</t>
+        </is>
+      </c>
+      <c r="J573" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K573" t="n">
+        <v>0</v>
+      </c>
+      <c r="L573" t="b">
+        <v>1</v>
+      </c>
+      <c r="M573" t="n">
+        <v>3.45377</v>
+      </c>
+      <c r="N573" t="n">
+        <v>1179</v>
+      </c>
+      <c r="O573" t="n">
+        <v>3</v>
+      </c>
+      <c r="P573" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R573" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S573" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.
+Gérez vos lignes mobiles, effectuez des transferts d'argent sécurisés, réglez vos factures, profitez d'offres exclusives, effectuez des paiements marchands fiables, et bien plus encore, le tout</t>
+        </is>
+      </c>
+      <c r="T573" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U573" t="inlineStr"/>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G574" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obw</t>
+        </is>
+      </c>
+      <c r="H574" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J574" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K574" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L574" t="b">
+        <v>0</v>
+      </c>
+      <c r="M574" t="n">
+        <v>3.9964788</v>
+      </c>
+      <c r="N574" t="n">
+        <v>2962</v>
+      </c>
+      <c r="O574" t="n">
+        <v>38</v>
+      </c>
+      <c r="P574" t="inlineStr"/>
+      <c r="Q574" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R574" t="inlineStr">
+        <is>
+          <t>7.3.8</t>
+        </is>
+      </c>
+      <c r="S574" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it, the brand-new Orange Botswana Super App that follows Yame and gives you access to four distinct universes for a one-of-a-kind experience!&lt;br&gt;&lt;br&gt;Manage your accounts, make quick payments using QR codes, investigate a range of online goods and services, and discover the many options provided </t>
+        </is>
+      </c>
+      <c r="T574" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U574" t="inlineStr"/>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G575" t="n">
+        <v>1195839458</v>
+      </c>
+      <c r="H575" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I575" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J575" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K575" t="n">
+        <v>0</v>
+      </c>
+      <c r="L575" t="b">
+        <v>1</v>
+      </c>
+      <c r="M575" t="n">
+        <v>3.00806</v>
+      </c>
+      <c r="N575" t="n">
+        <v>124</v>
+      </c>
+      <c r="O575" t="n">
+        <v>23</v>
+      </c>
+      <c r="P575" t="inlineStr"/>
+      <c r="R575" t="inlineStr">
+        <is>
+          <t>7.3.1</t>
+        </is>
+      </c>
+      <c r="S575" t="inlineStr">
+        <is>
+          <t>A free mobile self-care application for Orange Botswana’s mobile customers.
+Full Description :
+Max it is a free application, which allows Orange Botswana customers to:
+- Consult your account in real time: minutes, sms, internet ...
+- Top up your account or a friend account  with Orange Money
+-</t>
+        </is>
+      </c>
+      <c r="T575" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U575" t="inlineStr"/>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G576" t="inlineStr">
+        <is>
+          <t>com.orange.mobinilandme</t>
+        </is>
+      </c>
+      <c r="H576" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I576" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J576" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K576" t="inlineStr">
+        <is>
+          <t>EGP 0.00</t>
+        </is>
+      </c>
+      <c r="L576" t="b">
+        <v>0</v>
+      </c>
+      <c r="M576" t="n">
+        <v>4.5626144</v>
+      </c>
+      <c r="N576" t="n">
+        <v>924975</v>
+      </c>
+      <c r="O576" t="n">
+        <v>22</v>
+      </c>
+      <c r="P576" t="inlineStr"/>
+      <c r="Q576" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R576" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S576" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion&lt;br&gt;Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.&lt;br&gt;Key services include:&lt;br&gt;• Account Management: Easily manage</t>
+        </is>
+      </c>
+      <c r="T576" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U576" t="inlineStr"/>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>da77f2a3-c164-4cd0-94c1-8d25207c2f24</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>2026-07-25 06:19:50</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F577" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G577" t="n">
+        <v>942568333</v>
+      </c>
+      <c r="H577" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J577" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K577" t="n">
+        <v>0</v>
+      </c>
+      <c r="L577" t="b">
+        <v>1</v>
+      </c>
+      <c r="M577" t="n">
+        <v>4.25134</v>
+      </c>
+      <c r="N577" t="n">
+        <v>117068</v>
+      </c>
+      <c r="O577" t="n">
+        <v>65</v>
+      </c>
+      <c r="P577" t="inlineStr"/>
+      <c r="R577" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S577" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion
+Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.
+Key services include:
+• Account Management: Easily manage your Ora</t>
+        </is>
+      </c>
+      <c r="T577" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U577" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-07-26
</commit_message>
<xml_diff>
--- a/maxit_store_history.xlsx
+++ b/maxit_store_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U577"/>
+  <dimension ref="A1:U609"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46885,7 +46885,6 @@
       <c r="O546" t="n">
         <v>20</v>
       </c>
-      <c r="P546" t="inlineStr"/>
       <c r="Q546" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -46906,7 +46905,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U546" t="inlineStr"/>
     </row>
     <row r="547">
       <c r="A547" t="inlineStr">
@@ -46969,7 +46967,6 @@
       <c r="N547" t="n">
         <v>321</v>
       </c>
-      <c r="P547" t="inlineStr"/>
       <c r="R547" t="inlineStr">
         <is>
           <t>6.4.8</t>
@@ -46985,7 +46982,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U547" t="inlineStr"/>
     </row>
     <row r="548">
       <c r="A548" t="inlineStr">
@@ -47055,7 +47051,6 @@
       <c r="O548" t="n">
         <v>30</v>
       </c>
-      <c r="P548" t="inlineStr"/>
       <c r="Q548" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -47076,7 +47071,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U548" t="inlineStr"/>
     </row>
     <row r="549">
       <c r="A549" t="inlineStr">
@@ -47142,7 +47136,6 @@
       <c r="O549" t="n">
         <v>34</v>
       </c>
-      <c r="P549" t="inlineStr"/>
       <c r="R549" t="inlineStr">
         <is>
           <t>10.0.6</t>
@@ -47160,7 +47153,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U549" t="inlineStr"/>
     </row>
     <row r="550">
       <c r="A550" t="inlineStr">
@@ -47230,7 +47222,6 @@
       <c r="O550" t="n">
         <v>11</v>
       </c>
-      <c r="P550" t="inlineStr"/>
       <c r="Q550" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -47251,7 +47242,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U550" t="inlineStr"/>
     </row>
     <row r="551">
       <c r="A551" t="inlineStr">
@@ -47340,7 +47330,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U551" t="inlineStr"/>
     </row>
     <row r="552">
       <c r="A552" t="inlineStr">
@@ -47410,7 +47399,6 @@
       <c r="O552" t="n">
         <v>14</v>
       </c>
-      <c r="P552" t="inlineStr"/>
       <c r="Q552" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -47431,7 +47419,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U552" t="inlineStr"/>
     </row>
     <row r="553">
       <c r="A553" t="inlineStr">
@@ -47497,7 +47484,6 @@
       <c r="O553" t="n">
         <v>13</v>
       </c>
-      <c r="P553" t="inlineStr"/>
       <c r="R553" t="inlineStr">
         <is>
           <t>21.1.0</t>
@@ -47515,7 +47501,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U553" t="inlineStr"/>
     </row>
     <row r="554">
       <c r="A554" t="inlineStr">
@@ -47585,7 +47570,6 @@
       <c r="O554" t="n">
         <v>118</v>
       </c>
-      <c r="P554" t="inlineStr"/>
       <c r="Q554" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -47606,7 +47590,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U554" t="inlineStr"/>
     </row>
     <row r="555">
       <c r="A555" t="inlineStr">
@@ -47691,7 +47674,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U555" t="inlineStr"/>
     </row>
     <row r="556">
       <c r="A556" t="inlineStr">
@@ -47758,7 +47740,6 @@
       <c r="N556" t="n">
         <v>38254</v>
       </c>
-      <c r="P556" t="inlineStr"/>
       <c r="Q556" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -47779,7 +47760,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U556" t="inlineStr"/>
     </row>
     <row r="557">
       <c r="A557" t="inlineStr">
@@ -47845,7 +47825,6 @@
       <c r="O557" t="n">
         <v>9</v>
       </c>
-      <c r="P557" t="inlineStr"/>
       <c r="R557" t="inlineStr">
         <is>
           <t>6.5.2</t>
@@ -47864,7 +47843,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U557" t="inlineStr"/>
     </row>
     <row r="558">
       <c r="A558" t="inlineStr">
@@ -47934,7 +47912,6 @@
       <c r="O558" t="n">
         <v>48</v>
       </c>
-      <c r="P558" t="inlineStr"/>
       <c r="Q558" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -47955,7 +47932,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U558" t="inlineStr"/>
     </row>
     <row r="559">
       <c r="A559" t="inlineStr">
@@ -48021,7 +47997,6 @@
       <c r="O559" t="n">
         <v>29</v>
       </c>
-      <c r="P559" t="inlineStr"/>
       <c r="R559" t="inlineStr">
         <is>
           <t>5.0.2</t>
@@ -48039,7 +48014,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U559" t="inlineStr"/>
     </row>
     <row r="560">
       <c r="A560" t="inlineStr">
@@ -48109,7 +48083,6 @@
       <c r="O560" t="n">
         <v>72</v>
       </c>
-      <c r="P560" t="inlineStr"/>
       <c r="Q560" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -48130,7 +48103,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U560" t="inlineStr"/>
     </row>
     <row r="561">
       <c r="A561" t="inlineStr">
@@ -48218,7 +48190,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U561" t="inlineStr"/>
     </row>
     <row r="562">
       <c r="A562" t="inlineStr">
@@ -48288,7 +48259,6 @@
       <c r="O562" t="n">
         <v>46</v>
       </c>
-      <c r="P562" t="inlineStr"/>
       <c r="Q562" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -48309,7 +48279,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U562" t="inlineStr"/>
     </row>
     <row r="563">
       <c r="A563" t="inlineStr">
@@ -48375,7 +48344,6 @@
       <c r="O563" t="n">
         <v>53</v>
       </c>
-      <c r="P563" t="inlineStr"/>
       <c r="R563" t="inlineStr">
         <is>
           <t>10.0.21</t>
@@ -48394,7 +48362,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U563" t="inlineStr"/>
     </row>
     <row r="564">
       <c r="A564" t="inlineStr">
@@ -48464,7 +48431,6 @@
       <c r="O564" t="n">
         <v>10</v>
       </c>
-      <c r="P564" t="inlineStr"/>
       <c r="Q564" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -48485,7 +48451,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U564" t="inlineStr"/>
     </row>
     <row r="565">
       <c r="A565" t="inlineStr">
@@ -48571,7 +48536,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U565" t="inlineStr"/>
     </row>
     <row r="566">
       <c r="A566" t="inlineStr">
@@ -48641,7 +48605,6 @@
       <c r="O566" t="n">
         <v>5</v>
       </c>
-      <c r="P566" t="inlineStr"/>
       <c r="Q566" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -48662,7 +48625,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U566" t="inlineStr"/>
     </row>
     <row r="567">
       <c r="A567" t="inlineStr">
@@ -48748,7 +48710,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U567" t="inlineStr"/>
     </row>
     <row r="568">
       <c r="A568" t="inlineStr">
@@ -48818,7 +48779,6 @@
       <c r="O568" t="n">
         <v>83</v>
       </c>
-      <c r="P568" t="inlineStr"/>
       <c r="Q568" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -48839,7 +48799,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U568" t="inlineStr"/>
     </row>
     <row r="569">
       <c r="A569" t="inlineStr">
@@ -48922,7 +48881,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U569" t="inlineStr"/>
     </row>
     <row r="570">
       <c r="A570" t="inlineStr">
@@ -48992,7 +48950,6 @@
       <c r="O570" t="n">
         <v>12</v>
       </c>
-      <c r="P570" t="inlineStr"/>
       <c r="Q570" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -49013,7 +48970,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U570" t="inlineStr"/>
     </row>
     <row r="571">
       <c r="A571" t="inlineStr">
@@ -49102,7 +49058,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U571" t="inlineStr"/>
     </row>
     <row r="572">
       <c r="A572" t="inlineStr">
@@ -49172,7 +49127,6 @@
       <c r="O572" t="n">
         <v>13</v>
       </c>
-      <c r="P572" t="inlineStr"/>
       <c r="Q572" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -49193,7 +49147,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U572" t="inlineStr"/>
     </row>
     <row r="573">
       <c r="A573" t="inlineStr">
@@ -49280,7 +49233,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U573" t="inlineStr"/>
     </row>
     <row r="574">
       <c r="A574" t="inlineStr">
@@ -49350,7 +49302,6 @@
       <c r="O574" t="n">
         <v>38</v>
       </c>
-      <c r="P574" t="inlineStr"/>
       <c r="Q574" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -49371,7 +49322,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U574" t="inlineStr"/>
     </row>
     <row r="575">
       <c r="A575" t="inlineStr">
@@ -49437,7 +49387,6 @@
       <c r="O575" t="n">
         <v>23</v>
       </c>
-      <c r="P575" t="inlineStr"/>
       <c r="R575" t="inlineStr">
         <is>
           <t>7.3.1</t>
@@ -49458,7 +49407,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U575" t="inlineStr"/>
     </row>
     <row r="576">
       <c r="A576" t="inlineStr">
@@ -49528,7 +49476,6 @@
       <c r="O576" t="n">
         <v>22</v>
       </c>
-      <c r="P576" t="inlineStr"/>
       <c r="Q576" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -49549,7 +49496,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U576" t="inlineStr"/>
     </row>
     <row r="577">
       <c r="A577" t="inlineStr">
@@ -49615,7 +49561,6 @@
       <c r="O577" t="n">
         <v>65</v>
       </c>
-      <c r="P577" t="inlineStr"/>
       <c r="R577" t="inlineStr">
         <is>
           <t>10.1.0</t>
@@ -49634,7 +49579,2828 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U577" t="inlineStr"/>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G578" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogn</t>
+        </is>
+      </c>
+      <c r="H578" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J578" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K578" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L578" t="b">
+        <v>0</v>
+      </c>
+      <c r="M578" t="n">
+        <v>4.4517546</v>
+      </c>
+      <c r="N578" t="n">
+        <v>9261</v>
+      </c>
+      <c r="O578" t="n">
+        <v>18</v>
+      </c>
+      <c r="P578" t="inlineStr"/>
+      <c r="Q578" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R578" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S578" t="inlineStr">
+        <is>
+          <t>Bien plus qu&amp;#39;une application, un véritable assistant personnel pour une vie connectée et simplifiée.&lt;br&gt;Suivi de consommation: Votre tableau de bord tout-en-un pour une gestion simplifiée !&lt;br&gt;- Gestion de votre offre: Accédez à une vue détaillée de votre offre actuelle et de vos forfaits Orange</t>
+        </is>
+      </c>
+      <c r="T578" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U578" t="inlineStr"/>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F579" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G579" t="n">
+        <v>1177999485</v>
+      </c>
+      <c r="H579" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J579" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K579" t="n">
+        <v>0</v>
+      </c>
+      <c r="L579" t="b">
+        <v>1</v>
+      </c>
+      <c r="M579" t="n">
+        <v>3.90343</v>
+      </c>
+      <c r="N579" t="n">
+        <v>321</v>
+      </c>
+      <c r="P579" t="inlineStr"/>
+      <c r="R579" t="inlineStr">
+        <is>
+          <t>6.4.8</t>
+        </is>
+      </c>
+      <c r="S579" t="inlineStr">
+        <is>
+          <t>La fusion d’Orange et Moi et Orange Money donne naissance à Max it, la nouvelle Super Application Tout-en-Un. Profitez du suivi de consommation, de paiements mobiles, de toutes les fonctionnalités Orange et Moi et Money avec un large éventail de divertissements, le tout regroupé en un seul endroit !</t>
+        </is>
+      </c>
+      <c r="T579" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U579" t="inlineStr"/>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.otn</t>
+        </is>
+      </c>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J580" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K580" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L580" t="b">
+        <v>0</v>
+      </c>
+      <c r="M580" t="n">
+        <v>3.966399</v>
+      </c>
+      <c r="N580" t="n">
+        <v>35368</v>
+      </c>
+      <c r="O580" t="n">
+        <v>28</v>
+      </c>
+      <c r="P580" t="inlineStr"/>
+      <c r="Q580" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R580" t="inlineStr">
+        <is>
+          <t>10.0.6</t>
+        </is>
+      </c>
+      <c r="S580" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Max it par Orange Tunisie facilite votre vie au quotidien !&lt;/h2&gt;&lt;br&gt;&lt;br&gt;Welcome sur Max it !&lt;br&gt;Accédez rapidement à vos fonctionnalités Max it préférées et profitez également de contenus exclusifs, d’activités divertissantes, et de jeux interactifs pour une expérience enrichissante avec la roue</t>
+        </is>
+      </c>
+      <c r="T580" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U580" t="inlineStr"/>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G581" t="n">
+        <v>1146892088</v>
+      </c>
+      <c r="H581" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J581" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K581" t="n">
+        <v>0</v>
+      </c>
+      <c r="L581" t="b">
+        <v>1</v>
+      </c>
+      <c r="M581" t="n">
+        <v>3.03053</v>
+      </c>
+      <c r="N581" t="n">
+        <v>1638</v>
+      </c>
+      <c r="O581" t="n">
+        <v>33</v>
+      </c>
+      <c r="P581" t="inlineStr"/>
+      <c r="R581" t="inlineStr">
+        <is>
+          <t>10.0.6</t>
+        </is>
+      </c>
+      <c r="S581" t="inlineStr">
+        <is>
+          <t>Max it by Orange Tunisie : Votre appli incontournable pour une vie connectée
+Welcome sur Max it : Découvrez fonctionnalités, jeux &amp; contenus de divertissement by Orange Tunisie !
+Trouvez vite vos fonctionnalités Max it favorites et explorez des contenus exclusifs et des jeux pour une expérience im</t>
+        </is>
+      </c>
+      <c r="T581" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U581" t="inlineStr"/>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G582" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osl</t>
+        </is>
+      </c>
+      <c r="H582" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J582" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K582" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L582" t="b">
+        <v>0</v>
+      </c>
+      <c r="M582" t="n">
+        <v>4.3537736</v>
+      </c>
+      <c r="N582" t="n">
+        <v>2122</v>
+      </c>
+      <c r="O582" t="n">
+        <v>10</v>
+      </c>
+      <c r="P582" t="inlineStr"/>
+      <c r="Q582" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R582" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S582" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it is a free application, which allows Orange Sierra Leone prepaid and postpaid customers to:&lt;br&gt;&lt;br&gt;- Consult your account in real time: minutes, sms, internet&lt;br&gt;- Top up your account or a friend account &lt;br&gt;- Buy Internet Bundles&lt;br&gt;- Discover the latest offers and promotions &lt;br&gt;- Access to </t>
+        </is>
+      </c>
+      <c r="T582" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U582" t="inlineStr"/>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G583" t="n">
+        <v>6443607903</v>
+      </c>
+      <c r="H583" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I583" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J583" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K583" t="n">
+        <v>0</v>
+      </c>
+      <c r="L583" t="b">
+        <v>1</v>
+      </c>
+      <c r="M583" t="n">
+        <v>3.69948</v>
+      </c>
+      <c r="N583" t="n">
+        <v>193</v>
+      </c>
+      <c r="O583" t="n">
+        <v>11</v>
+      </c>
+      <c r="P583" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R583" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S583" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The merger of My Orange &amp; Orange Money has given birth to Max it the all-in-one super app, a free application which allows all Orange Sierra Leone customers to 
+Track calls, SMS, and Data usage and monitor balance. 
+Make a secure mobile/Orange Money payment.
+Easily transfer credit to other users </t>
+        </is>
+      </c>
+      <c r="T583" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U583" t="inlineStr"/>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G584" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osn</t>
+        </is>
+      </c>
+      <c r="H584" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>Orange Sénégal</t>
+        </is>
+      </c>
+      <c r="J584" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K584" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L584" t="b">
+        <v>0</v>
+      </c>
+      <c r="M584" t="n">
+        <v>4.3126283</v>
+      </c>
+      <c r="N584" t="n">
+        <v>51172</v>
+      </c>
+      <c r="O584" t="n">
+        <v>13</v>
+      </c>
+      <c r="P584" t="inlineStr"/>
+      <c r="Q584" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R584" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S584" t="inlineStr">
+        <is>
+          <t>Lu bees ak Max it ! &lt;br&gt;Une application repensée pour être plus simple, plus rapide et adaptée à vos besoins. Une expérience optimisée pour faciliter vos usages au quotidien, avec des parcours simplifiés et un accès plus fluide à vos services. Que vous soyez client Orange ou non, Max it vous accompa</t>
+        </is>
+      </c>
+      <c r="T584" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U584" t="inlineStr"/>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G585" t="n">
+        <v>1039327980</v>
+      </c>
+      <c r="H585" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>Orange Senegal</t>
+        </is>
+      </c>
+      <c r="J585" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K585" t="n">
+        <v>0</v>
+      </c>
+      <c r="L585" t="b">
+        <v>1</v>
+      </c>
+      <c r="M585" t="n">
+        <v>4.16983</v>
+      </c>
+      <c r="N585" t="n">
+        <v>30213</v>
+      </c>
+      <c r="O585" t="n">
+        <v>14</v>
+      </c>
+      <c r="P585" t="inlineStr"/>
+      <c r="R585" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S585" t="inlineStr">
+        <is>
+          <t>Here is the English translation:
+Welcome to Max it!
+A redesigned app to be simpler, faster, and tailored to your needs. An optimized experience to make your daily life easier, with streamlined journeys and smoother access to your services. Whether you are an Orange customer or not, Max it is your e</t>
+        </is>
+      </c>
+      <c r="T585" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U585" t="inlineStr"/>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>com.orange.meditel.mediteletmoi</t>
+        </is>
+      </c>
+      <c r="H586" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>Orange Maroc</t>
+        </is>
+      </c>
+      <c r="J586" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K586" t="inlineStr">
+        <is>
+          <t>MAD 0.00</t>
+        </is>
+      </c>
+      <c r="L586" t="b">
+        <v>0</v>
+      </c>
+      <c r="M586" t="n">
+        <v>3.7242193</v>
+      </c>
+      <c r="N586" t="n">
+        <v>110908</v>
+      </c>
+      <c r="O586" t="n">
+        <v>72</v>
+      </c>
+      <c r="P586" t="inlineStr"/>
+      <c r="Q586" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R586" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S586" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l&amp;#39;expérience mobile réinventé&lt;br&gt;&lt;br&gt;Max it, c&amp;#39;est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d&amp;#39;une multitude de services exclusifs. &lt;br&gt;&lt;br&gt;Créez votre espace sur</t>
+        </is>
+      </c>
+      <c r="T586" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U586" t="inlineStr"/>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G587" t="n">
+        <v>596028698</v>
+      </c>
+      <c r="H587" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>Méditel</t>
+        </is>
+      </c>
+      <c r="J587" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K587" t="n">
+        <v>0</v>
+      </c>
+      <c r="L587" t="b">
+        <v>1</v>
+      </c>
+      <c r="M587" t="n">
+        <v>3.94626</v>
+      </c>
+      <c r="N587" t="n">
+        <v>2754</v>
+      </c>
+      <c r="P587" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "MA" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R587" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S587" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l'expérience mobile réinventé
+Max it, c'est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d'une multitude de services exclusifs. 
+Créez votre espace sur mesure et bénéficiez d'</t>
+        </is>
+      </c>
+      <c r="T587" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U587" t="inlineStr"/>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G588" t="inlineStr">
+        <is>
+          <t>com.oml.dsi.orangemobile</t>
+        </is>
+      </c>
+      <c r="H588" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J588" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K588" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L588" t="b">
+        <v>0</v>
+      </c>
+      <c r="M588" t="n">
+        <v>2.6954024</v>
+      </c>
+      <c r="N588" t="n">
+        <v>38251</v>
+      </c>
+      <c r="P588" t="inlineStr"/>
+      <c r="Q588" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R588" t="inlineStr">
+        <is>
+          <t>6.5.0</t>
+        </is>
+      </c>
+      <c r="S588" t="inlineStr">
+        <is>
+          <t>Easily manage your Orange Mali line&lt;br&gt;● Manage your account and view all essential information, your offers, and your phone lines.&lt;br&gt;● Subscribe to call, SMS, Internet, and international call packages.&lt;br&gt;● Track your usage by checking your credit and Internet balance.&lt;br&gt;● Recharge your line by p</t>
+        </is>
+      </c>
+      <c r="T588" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U588" t="inlineStr"/>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F589" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G589" t="n">
+        <v>1494321079</v>
+      </c>
+      <c r="H589" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J589" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K589" t="n">
+        <v>0</v>
+      </c>
+      <c r="L589" t="b">
+        <v>1</v>
+      </c>
+      <c r="M589" t="n">
+        <v>2.51932</v>
+      </c>
+      <c r="N589" t="n">
+        <v>4737</v>
+      </c>
+      <c r="O589" t="n">
+        <v>14</v>
+      </c>
+      <c r="P589" t="inlineStr"/>
+      <c r="R589" t="inlineStr">
+        <is>
+          <t>6.5.2</t>
+        </is>
+      </c>
+      <c r="S589" t="inlineStr">
+        <is>
+          <t>Gérez facilement votre ligne Orange Mali 
+●        Gérez votre compte et consultez toutes les informations essentielles sur celui-ci, vos offres, ainsi que vos lignes téléphoniques.
+●        Souscrivez aux forfaits appels, SMS, Internet, et appels internationaux.
+●        Suivez votre consommation e</t>
+        </is>
+      </c>
+      <c r="T589" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U589" t="inlineStr"/>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G590" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.omg</t>
+        </is>
+      </c>
+      <c r="H590" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J590" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K590" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L590" t="b">
+        <v>0</v>
+      </c>
+      <c r="M590" t="n">
+        <v>4.154412</v>
+      </c>
+      <c r="N590" t="n">
+        <v>1370</v>
+      </c>
+      <c r="O590" t="n">
+        <v>52</v>
+      </c>
+      <c r="P590" t="inlineStr"/>
+      <c r="Q590" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R590" t="inlineStr">
+        <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="S590" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.&lt;br&gt;&lt;br&gt;Simplify Your Life with Max it&lt;br&gt;With Max It, ac</t>
+        </is>
+      </c>
+      <c r="T590" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U590" t="inlineStr"/>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G591" t="n">
+        <v>1295171817</v>
+      </c>
+      <c r="H591" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I591" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J591" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K591" t="n">
+        <v>0</v>
+      </c>
+      <c r="L591" t="b">
+        <v>1</v>
+      </c>
+      <c r="M591" t="n">
+        <v>3.08696</v>
+      </c>
+      <c r="N591" t="n">
+        <v>69</v>
+      </c>
+      <c r="O591" t="n">
+        <v>23</v>
+      </c>
+      <c r="P591" t="inlineStr"/>
+      <c r="R591" t="inlineStr">
+        <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="S591" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.
+Simplify Your Life with Max it
+With Max it, access a se</t>
+        </is>
+      </c>
+      <c r="T591" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U591" t="inlineStr"/>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G592" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.olr</t>
+        </is>
+      </c>
+      <c r="H592" t="inlineStr">
+        <is>
+          <t>Orange Max it - Liberia</t>
+        </is>
+      </c>
+      <c r="I592" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J592" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K592" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L592" t="b">
+        <v>0</v>
+      </c>
+      <c r="M592" t="n">
+        <v>4.5434084</v>
+      </c>
+      <c r="N592" t="n">
+        <v>3092</v>
+      </c>
+      <c r="O592" t="n">
+        <v>64</v>
+      </c>
+      <c r="P592" t="inlineStr"/>
+      <c r="Q592" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R592" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="S592" t="inlineStr">
+        <is>
+          <t>Max it: your personalized experience by Orange Liberia!&lt;br&gt;&lt;br&gt;Step into Max it, your all-in-one solution for telecom, marketplace, and financial services! Manage your mobile line, customize offers, pay your bills, keep&lt;br&gt;track of your usage with ease, and recharge your credit. Access exclusive eve</t>
+        </is>
+      </c>
+      <c r="T592" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U592" t="inlineStr"/>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G593" t="n">
+        <v>6746187327</v>
+      </c>
+      <c r="H593" t="inlineStr">
+        <is>
+          <t>Orange Max it – Liberia</t>
+        </is>
+      </c>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J593" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K593" t="n">
+        <v>0</v>
+      </c>
+      <c r="L593" t="b">
+        <v>1</v>
+      </c>
+      <c r="M593" t="n">
+        <v>4.0625</v>
+      </c>
+      <c r="N593" t="n">
+        <v>48</v>
+      </c>
+      <c r="O593" t="n">
+        <v>24</v>
+      </c>
+      <c r="P593" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R593" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="S593" t="inlineStr">
+        <is>
+          <t>Max it is a free application, which allows Orange Liberia customers to:
+- Consult your account in real time: minutes, sms, internet
+- Top up your account or a friend account 
+- Buy  Bundles (voice, data, SMS, roaming, international)
+- Discover the latest offers and promotions 
+- Access to Orange se</t>
+        </is>
+      </c>
+      <c r="T593" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U593" t="inlineStr"/>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ojo</t>
+        </is>
+      </c>
+      <c r="H594" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J594" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K594" t="inlineStr">
+        <is>
+          <t>JOD 0.000</t>
+        </is>
+      </c>
+      <c r="L594" t="b">
+        <v>0</v>
+      </c>
+      <c r="M594" t="n">
+        <v>4.433151</v>
+      </c>
+      <c r="N594" t="n">
+        <v>97633</v>
+      </c>
+      <c r="O594" t="n">
+        <v>51</v>
+      </c>
+      <c r="P594" t="inlineStr"/>
+      <c r="Q594" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R594" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S594" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience&lt;br&gt;Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.&lt;br&gt;Important Update:&lt;br&gt;The jood app (jood Orange) w</t>
+        </is>
+      </c>
+      <c r="T594" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U594" t="inlineStr"/>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G595" t="n">
+        <v>808824590</v>
+      </c>
+      <c r="H595" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J595" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K595" t="n">
+        <v>0</v>
+      </c>
+      <c r="L595" t="b">
+        <v>1</v>
+      </c>
+      <c r="M595" t="n">
+        <v>4.21217</v>
+      </c>
+      <c r="N595" t="n">
+        <v>3007</v>
+      </c>
+      <c r="O595" t="n">
+        <v>54</v>
+      </c>
+      <c r="P595" t="inlineStr"/>
+      <c r="R595" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S595" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience
+Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.
+Important Update:
+The jood app (jood Orange) will be di</t>
+        </is>
+      </c>
+      <c r="T595" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U595" t="inlineStr"/>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.oci</t>
+        </is>
+      </c>
+      <c r="H596" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>Orange Côte d'Ivoire S.A</t>
+        </is>
+      </c>
+      <c r="J596" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K596" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L596" t="b">
+        <v>0</v>
+      </c>
+      <c r="M596" t="n">
+        <v>4.1703935</v>
+      </c>
+      <c r="N596" t="n">
+        <v>67108</v>
+      </c>
+      <c r="O596" t="n">
+        <v>10</v>
+      </c>
+      <c r="P596" t="inlineStr"/>
+      <c r="Q596" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R596" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S596" t="inlineStr">
+        <is>
+          <t>Aaaahhh, ta super app Max it, n&amp;#39;a pas fini de te surprendre... &lt;br&gt;Est-ce que tu as remarqué ? Maintenant, tu as ton QR code personnalisé en haut de ton écran d&amp;#39;accueil ! Ainsi, tu peux :&lt;br&gt;     scanner le QR code de ton ami(e) pour lui faire un transfert d&amp;#39;&amp;#39;argent&lt;br&gt;     scanner l</t>
+        </is>
+      </c>
+      <c r="T596" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U596" t="inlineStr"/>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G597" t="n">
+        <v>1061120855</v>
+      </c>
+      <c r="H597" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>Orange CI</t>
+        </is>
+      </c>
+      <c r="J597" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K597" t="n">
+        <v>0</v>
+      </c>
+      <c r="L597" t="b">
+        <v>1</v>
+      </c>
+      <c r="M597" t="n">
+        <v>3.78702</v>
+      </c>
+      <c r="N597" t="n">
+        <v>5963</v>
+      </c>
+      <c r="O597" t="n">
+        <v>11</v>
+      </c>
+      <c r="P597" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R597" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S597" t="inlineStr">
+        <is>
+          <t>Max it, la super app all-in-one te fais gagner du temps, et diminue tes soucis... Gagne plus d'espace de stockage sur ton téléphone ; plus besoin de cumuler plusieurs appli d'Orange pour avoir accès à un maximum de services. Max it est là ! Gère ta ligne (SIM) au niveau des pass, des soldes, réalise</t>
+        </is>
+      </c>
+      <c r="T597" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U597" t="inlineStr"/>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G598" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogw</t>
+        </is>
+      </c>
+      <c r="H598" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J598" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K598" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L598" t="b">
+        <v>0</v>
+      </c>
+      <c r="M598" t="n">
+        <v>4.3636365</v>
+      </c>
+      <c r="N598" t="n">
+        <v>1527</v>
+      </c>
+      <c r="O598" t="n">
+        <v>5</v>
+      </c>
+      <c r="P598" t="inlineStr"/>
+      <c r="Q598" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R598" t="inlineStr">
+        <is>
+          <t>4.0.18</t>
+        </is>
+      </c>
+      <c r="S598" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T598" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U598" t="inlineStr"/>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G599" t="n">
+        <v>1574668652</v>
+      </c>
+      <c r="H599" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J599" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K599" t="n">
+        <v>0</v>
+      </c>
+      <c r="L599" t="b">
+        <v>1</v>
+      </c>
+      <c r="M599" t="n">
+        <v>4.05333</v>
+      </c>
+      <c r="N599" t="n">
+        <v>75</v>
+      </c>
+      <c r="O599" t="n">
+        <v>14</v>
+      </c>
+      <c r="P599" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R599" t="inlineStr">
+        <is>
+          <t>6.0.35</t>
+        </is>
+      </c>
+      <c r="S599" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T599" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U599" t="inlineStr"/>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G600" t="inlineStr">
+        <is>
+          <t>com.orange.sugu.ocd</t>
+        </is>
+      </c>
+      <c r="H600" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I600" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J600" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K600" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L600" t="b">
+        <v>0</v>
+      </c>
+      <c r="M600" t="n">
+        <v>4.1217227</v>
+      </c>
+      <c r="N600" t="n">
+        <v>5285</v>
+      </c>
+      <c r="O600" t="n">
+        <v>69</v>
+      </c>
+      <c r="P600" t="inlineStr"/>
+      <c r="Q600" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R600" t="inlineStr">
+        <is>
+          <t>9.0.12</t>
+        </is>
+      </c>
+      <c r="S600" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DRC that brings together the features of MyOrange, and Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Plans, Mobile Payments, money transfers, bill payments, subscriptions, and entertai</t>
+        </is>
+      </c>
+      <c r="T600" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U600" t="inlineStr"/>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G601" t="n">
+        <v>6447896435</v>
+      </c>
+      <c r="H601" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J601" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K601" t="n">
+        <v>0</v>
+      </c>
+      <c r="L601" t="b">
+        <v>1</v>
+      </c>
+      <c r="M601" t="n">
+        <v>3.55762</v>
+      </c>
+      <c r="N601" t="n">
+        <v>269</v>
+      </c>
+      <c r="P601" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "CD" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R601" t="inlineStr">
+        <is>
+          <t>9.0.6</t>
+        </is>
+      </c>
+      <c r="S601" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DR Congo. It brings together the features of Orange et Moi, as well as Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Packages, Mobile payment, money transfers, bill payment and subscri</t>
+        </is>
+      </c>
+      <c r="T601" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U601" t="inlineStr"/>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G602" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ocm</t>
+        </is>
+      </c>
+      <c r="H602" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroon</t>
+        </is>
+      </c>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>Orange MEA</t>
+        </is>
+      </c>
+      <c r="J602" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K602" t="inlineStr">
+        <is>
+          <t>FCFA 0</t>
+        </is>
+      </c>
+      <c r="L602" t="b">
+        <v>0</v>
+      </c>
+      <c r="M602" t="n">
+        <v>3.9349732</v>
+      </c>
+      <c r="N602" t="n">
+        <v>46856</v>
+      </c>
+      <c r="O602" t="n">
+        <v>12</v>
+      </c>
+      <c r="P602" t="inlineStr"/>
+      <c r="Q602" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R602" t="inlineStr">
+        <is>
+          <t>7.0.23</t>
+        </is>
+      </c>
+      <c r="S602" t="inlineStr">
+        <is>
+          <t>Max it brings together everything that matters to you in one app: managing your lines, money transfer, bill payment, exclusive offers, and a universe of lifestyle and entertainment. Simple, fast, and 100% secure..&lt;br&gt;&lt;br&gt;📞 My line&lt;br&gt;Manage your Orange mobile and landline bundles in a single click:</t>
+        </is>
+      </c>
+      <c r="T602" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U602" t="inlineStr"/>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G603" t="n">
+        <v>1116920093</v>
+      </c>
+      <c r="H603" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroun</t>
+        </is>
+      </c>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>Orange Middle East &amp; Africa</t>
+        </is>
+      </c>
+      <c r="J603" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K603" t="n">
+        <v>0</v>
+      </c>
+      <c r="L603" t="b">
+        <v>1</v>
+      </c>
+      <c r="M603" t="n">
+        <v>3.76879</v>
+      </c>
+      <c r="N603" t="n">
+        <v>16150</v>
+      </c>
+      <c r="O603" t="n">
+        <v>2</v>
+      </c>
+      <c r="P603" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R603" t="inlineStr">
+        <is>
+          <t>7.0.24</t>
+        </is>
+      </c>
+      <c r="S603" t="inlineStr">
+        <is>
+          <t>Avec Max it, Orange rassemble tout ce qui compte pour vous dans une même application : la gestion de vos lignes, les transferts d’argent, payement de vos factures, des offres exclusives et un univers lifestyle et divertissement.
+Simple, rapide et 100 % sécurisée.
+Ma ligne
+Gérez vos forfaits mobiles</t>
+        </is>
+      </c>
+      <c r="T603" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U603" t="inlineStr"/>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G604" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obf</t>
+        </is>
+      </c>
+      <c r="H604" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I604" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso</t>
+        </is>
+      </c>
+      <c r="J604" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K604" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L604" t="b">
+        <v>0</v>
+      </c>
+      <c r="M604" t="n">
+        <v>4.146562</v>
+      </c>
+      <c r="N604" t="n">
+        <v>25449</v>
+      </c>
+      <c r="O604" t="n">
+        <v>11</v>
+      </c>
+      <c r="P604" t="inlineStr"/>
+      <c r="Q604" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R604" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S604" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.&lt;br&gt;Gérez vos lignes mobiles, effectuez des transferts d&amp;#39;argent sécurisés, réglez vos factures, profitez d&amp;#39;offres exclusives, effectuez des paiements marchands fiables, et bien plus enco</t>
+        </is>
+      </c>
+      <c r="T604" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U604" t="inlineStr"/>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G605" t="n">
+        <v>1553774707</v>
+      </c>
+      <c r="H605" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso SA</t>
+        </is>
+      </c>
+      <c r="J605" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K605" t="n">
+        <v>0</v>
+      </c>
+      <c r="L605" t="b">
+        <v>1</v>
+      </c>
+      <c r="M605" t="n">
+        <v>3.45377</v>
+      </c>
+      <c r="N605" t="n">
+        <v>1179</v>
+      </c>
+      <c r="O605" t="n">
+        <v>9</v>
+      </c>
+      <c r="P605" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R605" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S605" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.
+Gérez vos lignes mobiles, effectuez des transferts d'argent sécurisés, réglez vos factures, profitez d'offres exclusives, effectuez des paiements marchands fiables, et bien plus encore, le tout</t>
+        </is>
+      </c>
+      <c r="T605" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U605" t="inlineStr"/>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G606" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obw</t>
+        </is>
+      </c>
+      <c r="H606" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J606" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K606" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L606" t="b">
+        <v>0</v>
+      </c>
+      <c r="M606" t="n">
+        <v>3.9929328</v>
+      </c>
+      <c r="N606" t="n">
+        <v>2961</v>
+      </c>
+      <c r="O606" t="n">
+        <v>34</v>
+      </c>
+      <c r="P606" t="inlineStr"/>
+      <c r="Q606" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R606" t="inlineStr">
+        <is>
+          <t>7.3.8</t>
+        </is>
+      </c>
+      <c r="S606" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it, the brand-new Orange Botswana Super App that follows Yame and gives you access to four distinct universes for a one-of-a-kind experience!&lt;br&gt;&lt;br&gt;Manage your accounts, make quick payments using QR codes, investigate a range of online goods and services, and discover the many options provided </t>
+        </is>
+      </c>
+      <c r="T606" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U606" t="inlineStr"/>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G607" t="n">
+        <v>1195839458</v>
+      </c>
+      <c r="H607" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I607" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J607" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K607" t="n">
+        <v>0</v>
+      </c>
+      <c r="L607" t="b">
+        <v>1</v>
+      </c>
+      <c r="M607" t="n">
+        <v>3.00806</v>
+      </c>
+      <c r="N607" t="n">
+        <v>124</v>
+      </c>
+      <c r="O607" t="n">
+        <v>32</v>
+      </c>
+      <c r="P607" t="inlineStr"/>
+      <c r="R607" t="inlineStr">
+        <is>
+          <t>7.3.1</t>
+        </is>
+      </c>
+      <c r="S607" t="inlineStr">
+        <is>
+          <t>A free mobile self-care application for Orange Botswana’s mobile customers.
+Full Description :
+Max it is a free application, which allows Orange Botswana customers to:
+- Consult your account in real time: minutes, sms, internet ...
+- Top up your account or a friend account  with Orange Money
+-</t>
+        </is>
+      </c>
+      <c r="T607" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U607" t="inlineStr"/>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G608" t="inlineStr">
+        <is>
+          <t>com.orange.mobinilandme</t>
+        </is>
+      </c>
+      <c r="H608" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I608" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J608" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K608" t="inlineStr">
+        <is>
+          <t>EGP 0.00</t>
+        </is>
+      </c>
+      <c r="L608" t="b">
+        <v>0</v>
+      </c>
+      <c r="M608" t="n">
+        <v>4.5609107</v>
+      </c>
+      <c r="N608" t="n">
+        <v>926099</v>
+      </c>
+      <c r="O608" t="n">
+        <v>23</v>
+      </c>
+      <c r="P608" t="inlineStr"/>
+      <c r="Q608" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R608" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S608" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion&lt;br&gt;Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.&lt;br&gt;Key services include:&lt;br&gt;• Account Management: Easily manage</t>
+        </is>
+      </c>
+      <c r="T608" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U608" t="inlineStr"/>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>1203a28d-a956-455a-aaa0-231b5a06d6a1</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>2026-07-26 06:38:15</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G609" t="n">
+        <v>942568333</v>
+      </c>
+      <c r="H609" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I609" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J609" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K609" t="n">
+        <v>0</v>
+      </c>
+      <c r="L609" t="b">
+        <v>1</v>
+      </c>
+      <c r="M609" t="n">
+        <v>4.25164</v>
+      </c>
+      <c r="N609" t="n">
+        <v>117221</v>
+      </c>
+      <c r="O609" t="n">
+        <v>61</v>
+      </c>
+      <c r="P609" t="inlineStr"/>
+      <c r="R609" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S609" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion
+Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.
+Key services include:
+• Account Management: Easily manage your Ora</t>
+        </is>
+      </c>
+      <c r="T609" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U609" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-07-27
</commit_message>
<xml_diff>
--- a/maxit_store_history.xlsx
+++ b/maxit_store_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U609"/>
+  <dimension ref="A1:U641"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49648,7 +49648,6 @@
       <c r="O578" t="n">
         <v>18</v>
       </c>
-      <c r="P578" t="inlineStr"/>
       <c r="Q578" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -49669,7 +49668,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U578" t="inlineStr"/>
     </row>
     <row r="579">
       <c r="A579" t="inlineStr">
@@ -49732,7 +49730,6 @@
       <c r="N579" t="n">
         <v>321</v>
       </c>
-      <c r="P579" t="inlineStr"/>
       <c r="R579" t="inlineStr">
         <is>
           <t>6.4.8</t>
@@ -49748,7 +49745,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U579" t="inlineStr"/>
     </row>
     <row r="580">
       <c r="A580" t="inlineStr">
@@ -49818,7 +49814,6 @@
       <c r="O580" t="n">
         <v>28</v>
       </c>
-      <c r="P580" t="inlineStr"/>
       <c r="Q580" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -49839,7 +49834,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U580" t="inlineStr"/>
     </row>
     <row r="581">
       <c r="A581" t="inlineStr">
@@ -49905,7 +49899,6 @@
       <c r="O581" t="n">
         <v>33</v>
       </c>
-      <c r="P581" t="inlineStr"/>
       <c r="R581" t="inlineStr">
         <is>
           <t>10.0.6</t>
@@ -49923,7 +49916,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U581" t="inlineStr"/>
     </row>
     <row r="582">
       <c r="A582" t="inlineStr">
@@ -49993,7 +49985,6 @@
       <c r="O582" t="n">
         <v>10</v>
       </c>
-      <c r="P582" t="inlineStr"/>
       <c r="Q582" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -50014,7 +50005,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U582" t="inlineStr"/>
     </row>
     <row r="583">
       <c r="A583" t="inlineStr">
@@ -50103,7 +50093,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U583" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" t="inlineStr">
@@ -50173,7 +50162,6 @@
       <c r="O584" t="n">
         <v>13</v>
       </c>
-      <c r="P584" t="inlineStr"/>
       <c r="Q584" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -50194,7 +50182,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U584" t="inlineStr"/>
     </row>
     <row r="585">
       <c r="A585" t="inlineStr">
@@ -50260,7 +50247,6 @@
       <c r="O585" t="n">
         <v>14</v>
       </c>
-      <c r="P585" t="inlineStr"/>
       <c r="R585" t="inlineStr">
         <is>
           <t>21.1.0</t>
@@ -50278,7 +50264,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U585" t="inlineStr"/>
     </row>
     <row r="586">
       <c r="A586" t="inlineStr">
@@ -50348,7 +50333,6 @@
       <c r="O586" t="n">
         <v>72</v>
       </c>
-      <c r="P586" t="inlineStr"/>
       <c r="Q586" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -50369,7 +50353,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U586" t="inlineStr"/>
     </row>
     <row r="587">
       <c r="A587" t="inlineStr">
@@ -50454,7 +50437,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U587" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" t="inlineStr">
@@ -50521,7 +50503,6 @@
       <c r="N588" t="n">
         <v>38251</v>
       </c>
-      <c r="P588" t="inlineStr"/>
       <c r="Q588" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -50542,7 +50523,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U588" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" t="inlineStr">
@@ -50608,7 +50588,6 @@
       <c r="O589" t="n">
         <v>14</v>
       </c>
-      <c r="P589" t="inlineStr"/>
       <c r="R589" t="inlineStr">
         <is>
           <t>6.5.2</t>
@@ -50627,7 +50606,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U589" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" t="inlineStr">
@@ -50697,7 +50675,6 @@
       <c r="O590" t="n">
         <v>52</v>
       </c>
-      <c r="P590" t="inlineStr"/>
       <c r="Q590" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -50718,7 +50695,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U590" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" t="inlineStr">
@@ -50784,7 +50760,6 @@
       <c r="O591" t="n">
         <v>23</v>
       </c>
-      <c r="P591" t="inlineStr"/>
       <c r="R591" t="inlineStr">
         <is>
           <t>5.0.2</t>
@@ -50802,7 +50777,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U591" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" t="inlineStr">
@@ -50872,7 +50846,6 @@
       <c r="O592" t="n">
         <v>64</v>
       </c>
-      <c r="P592" t="inlineStr"/>
       <c r="Q592" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -50893,7 +50866,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U592" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" t="inlineStr">
@@ -50984,7 +50956,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U593" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" t="inlineStr">
@@ -51054,7 +51025,6 @@
       <c r="O594" t="n">
         <v>51</v>
       </c>
-      <c r="P594" t="inlineStr"/>
       <c r="Q594" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -51075,7 +51045,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U594" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" t="inlineStr">
@@ -51141,7 +51110,6 @@
       <c r="O595" t="n">
         <v>54</v>
       </c>
-      <c r="P595" t="inlineStr"/>
       <c r="R595" t="inlineStr">
         <is>
           <t>10.0.21</t>
@@ -51160,7 +51128,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U595" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" t="inlineStr">
@@ -51230,7 +51197,6 @@
       <c r="O596" t="n">
         <v>10</v>
       </c>
-      <c r="P596" t="inlineStr"/>
       <c r="Q596" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -51251,7 +51217,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U596" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" t="inlineStr">
@@ -51337,7 +51302,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U597" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" t="inlineStr">
@@ -51407,7 +51371,6 @@
       <c r="O598" t="n">
         <v>5</v>
       </c>
-      <c r="P598" t="inlineStr"/>
       <c r="Q598" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -51428,7 +51391,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U598" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" t="inlineStr">
@@ -51514,7 +51476,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U599" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" t="inlineStr">
@@ -51584,7 +51545,6 @@
       <c r="O600" t="n">
         <v>69</v>
       </c>
-      <c r="P600" t="inlineStr"/>
       <c r="Q600" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -51605,7 +51565,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U600" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" t="inlineStr">
@@ -51688,7 +51647,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U601" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" t="inlineStr">
@@ -51758,7 +51716,6 @@
       <c r="O602" t="n">
         <v>12</v>
       </c>
-      <c r="P602" t="inlineStr"/>
       <c r="Q602" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -51779,7 +51736,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U602" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" t="inlineStr">
@@ -51868,7 +51824,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U603" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" t="inlineStr">
@@ -51938,7 +51893,6 @@
       <c r="O604" t="n">
         <v>11</v>
       </c>
-      <c r="P604" t="inlineStr"/>
       <c r="Q604" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -51959,7 +51913,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U604" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" t="inlineStr">
@@ -52046,7 +51999,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U605" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" t="inlineStr">
@@ -52116,7 +52068,6 @@
       <c r="O606" t="n">
         <v>34</v>
       </c>
-      <c r="P606" t="inlineStr"/>
       <c r="Q606" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -52137,7 +52088,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U606" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" t="inlineStr">
@@ -52203,7 +52153,6 @@
       <c r="O607" t="n">
         <v>32</v>
       </c>
-      <c r="P607" t="inlineStr"/>
       <c r="R607" t="inlineStr">
         <is>
           <t>7.3.1</t>
@@ -52224,7 +52173,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U607" t="inlineStr"/>
     </row>
     <row r="608">
       <c r="A608" t="inlineStr">
@@ -52294,7 +52242,6 @@
       <c r="O608" t="n">
         <v>23</v>
       </c>
-      <c r="P608" t="inlineStr"/>
       <c r="Q608" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -52315,7 +52262,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U608" t="inlineStr"/>
     </row>
     <row r="609">
       <c r="A609" t="inlineStr">
@@ -52381,7 +52327,6 @@
       <c r="O609" t="n">
         <v>61</v>
       </c>
-      <c r="P609" t="inlineStr"/>
       <c r="R609" t="inlineStr">
         <is>
           <t>10.1.0</t>
@@ -52400,7 +52345,2825 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U609" t="inlineStr"/>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G610" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogn</t>
+        </is>
+      </c>
+      <c r="H610" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I610" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J610" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K610" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L610" t="b">
+        <v>0</v>
+      </c>
+      <c r="M610" t="n">
+        <v>4.454846</v>
+      </c>
+      <c r="N610" t="n">
+        <v>9267</v>
+      </c>
+      <c r="O610" t="n">
+        <v>23</v>
+      </c>
+      <c r="P610" t="inlineStr"/>
+      <c r="Q610" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R610" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S610" t="inlineStr">
+        <is>
+          <t>Bien plus qu&amp;#39;une application, un véritable assistant personnel pour une vie connectée et simplifiée.&lt;br&gt;Suivi de consommation: Votre tableau de bord tout-en-un pour une gestion simplifiée !&lt;br&gt;- Gestion de votre offre: Accédez à une vue détaillée de votre offre actuelle et de vos forfaits Orange</t>
+        </is>
+      </c>
+      <c r="T610" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U610" t="inlineStr"/>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G611" t="n">
+        <v>1177999485</v>
+      </c>
+      <c r="H611" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I611" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J611" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K611" t="n">
+        <v>0</v>
+      </c>
+      <c r="L611" t="b">
+        <v>1</v>
+      </c>
+      <c r="M611" t="n">
+        <v>3.89441</v>
+      </c>
+      <c r="N611" t="n">
+        <v>322</v>
+      </c>
+      <c r="P611" t="inlineStr"/>
+      <c r="R611" t="inlineStr">
+        <is>
+          <t>6.4.8</t>
+        </is>
+      </c>
+      <c r="S611" t="inlineStr">
+        <is>
+          <t>La fusion d’Orange et Moi et Orange Money donne naissance à Max it, la nouvelle Super Application Tout-en-Un. Profitez du suivi de consommation, de paiements mobiles, de toutes les fonctionnalités Orange et Moi et Money avec un large éventail de divertissements, le tout regroupé en un seul endroit !</t>
+        </is>
+      </c>
+      <c r="T611" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U611" t="inlineStr"/>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G612" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.otn</t>
+        </is>
+      </c>
+      <c r="H612" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J612" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K612" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L612" t="b">
+        <v>0</v>
+      </c>
+      <c r="M612" t="n">
+        <v>3.967656</v>
+      </c>
+      <c r="N612" t="n">
+        <v>35375</v>
+      </c>
+      <c r="O612" t="n">
+        <v>29</v>
+      </c>
+      <c r="P612" t="inlineStr"/>
+      <c r="Q612" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R612" t="inlineStr">
+        <is>
+          <t>10.0.6</t>
+        </is>
+      </c>
+      <c r="S612" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Max it par Orange Tunisie facilite votre vie au quotidien !&lt;/h2&gt;&lt;br&gt;&lt;br&gt;Welcome sur Max it !&lt;br&gt;Accédez rapidement à vos fonctionnalités Max it préférées et profitez également de contenus exclusifs, d’activités divertissantes, et de jeux interactifs pour une expérience enrichissante avec la roue</t>
+        </is>
+      </c>
+      <c r="T612" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U612" t="inlineStr"/>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G613" t="n">
+        <v>1146892088</v>
+      </c>
+      <c r="H613" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J613" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K613" t="n">
+        <v>0</v>
+      </c>
+      <c r="L613" t="b">
+        <v>1</v>
+      </c>
+      <c r="M613" t="n">
+        <v>3.03053</v>
+      </c>
+      <c r="N613" t="n">
+        <v>1638</v>
+      </c>
+      <c r="O613" t="n">
+        <v>43</v>
+      </c>
+      <c r="P613" t="inlineStr"/>
+      <c r="R613" t="inlineStr">
+        <is>
+          <t>10.0.6</t>
+        </is>
+      </c>
+      <c r="S613" t="inlineStr">
+        <is>
+          <t>Max it by Orange Tunisie : Votre appli incontournable pour une vie connectée
+Welcome sur Max it : Découvrez fonctionnalités, jeux &amp; contenus de divertissement by Orange Tunisie !
+Trouvez vite vos fonctionnalités Max it favorites et explorez des contenus exclusifs et des jeux pour une expérience im</t>
+        </is>
+      </c>
+      <c r="T613" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U613" t="inlineStr"/>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G614" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osl</t>
+        </is>
+      </c>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J614" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K614" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L614" t="b">
+        <v>0</v>
+      </c>
+      <c r="M614" t="n">
+        <v>4.35023</v>
+      </c>
+      <c r="N614" t="n">
+        <v>2127</v>
+      </c>
+      <c r="O614" t="n">
+        <v>11</v>
+      </c>
+      <c r="P614" t="inlineStr"/>
+      <c r="Q614" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R614" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S614" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it is a free application, which allows Orange Sierra Leone prepaid and postpaid customers to:&lt;br&gt;&lt;br&gt;- Consult your account in real time: minutes, sms, internet&lt;br&gt;- Top up your account or a friend account &lt;br&gt;- Buy Internet Bundles&lt;br&gt;- Discover the latest offers and promotions &lt;br&gt;- Access to </t>
+        </is>
+      </c>
+      <c r="T614" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U614" t="inlineStr"/>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G615" t="n">
+        <v>6443607903</v>
+      </c>
+      <c r="H615" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J615" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K615" t="n">
+        <v>0</v>
+      </c>
+      <c r="L615" t="b">
+        <v>1</v>
+      </c>
+      <c r="M615" t="n">
+        <v>3.69948</v>
+      </c>
+      <c r="N615" t="n">
+        <v>193</v>
+      </c>
+      <c r="O615" t="n">
+        <v>9</v>
+      </c>
+      <c r="P615" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R615" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S615" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The merger of My Orange &amp; Orange Money has given birth to Max it the all-in-one super app, a free application which allows all Orange Sierra Leone customers to 
+Track calls, SMS, and Data usage and monitor balance. 
+Make a secure mobile/Orange Money payment.
+Easily transfer credit to other users </t>
+        </is>
+      </c>
+      <c r="T615" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U615" t="inlineStr"/>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osn</t>
+        </is>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>Orange Sénégal</t>
+        </is>
+      </c>
+      <c r="J616" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K616" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L616" t="b">
+        <v>0</v>
+      </c>
+      <c r="M616" t="n">
+        <v>4.308696</v>
+      </c>
+      <c r="N616" t="n">
+        <v>51195</v>
+      </c>
+      <c r="O616" t="n">
+        <v>13</v>
+      </c>
+      <c r="P616" t="inlineStr"/>
+      <c r="Q616" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R616" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S616" t="inlineStr">
+        <is>
+          <t>Lu bees ak Max it ! &lt;br&gt;Une application repensée pour être plus simple, plus rapide et adaptée à vos besoins. Une expérience optimisée pour faciliter vos usages au quotidien, avec des parcours simplifiés et un accès plus fluide à vos services. Que vous soyez client Orange ou non, Max it vous accompa</t>
+        </is>
+      </c>
+      <c r="T616" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U616" t="inlineStr"/>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G617" t="n">
+        <v>1039327980</v>
+      </c>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>Orange Senegal</t>
+        </is>
+      </c>
+      <c r="J617" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K617" t="n">
+        <v>0</v>
+      </c>
+      <c r="L617" t="b">
+        <v>1</v>
+      </c>
+      <c r="M617" t="n">
+        <v>4.16967</v>
+      </c>
+      <c r="N617" t="n">
+        <v>30217</v>
+      </c>
+      <c r="O617" t="n">
+        <v>8</v>
+      </c>
+      <c r="P617" t="inlineStr"/>
+      <c r="R617" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S617" t="inlineStr">
+        <is>
+          <t>Here is the English translation:
+Welcome to Max it!
+A redesigned app to be simpler, faster, and tailored to your needs. An optimized experience to make your daily life easier, with streamlined journeys and smoother access to your services. Whether you are an Orange customer or not, Max it is your e</t>
+        </is>
+      </c>
+      <c r="T617" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U617" t="inlineStr"/>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G618" t="inlineStr">
+        <is>
+          <t>com.orange.meditel.mediteletmoi</t>
+        </is>
+      </c>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I618" t="inlineStr">
+        <is>
+          <t>Orange Maroc</t>
+        </is>
+      </c>
+      <c r="J618" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K618" t="inlineStr">
+        <is>
+          <t>MAD 0.00</t>
+        </is>
+      </c>
+      <c r="L618" t="b">
+        <v>0</v>
+      </c>
+      <c r="M618" t="n">
+        <v>3.7238638</v>
+      </c>
+      <c r="N618" t="n">
+        <v>110913</v>
+      </c>
+      <c r="O618" t="n">
+        <v>82</v>
+      </c>
+      <c r="P618" t="inlineStr"/>
+      <c r="Q618" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R618" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S618" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l&amp;#39;expérience mobile réinventé&lt;br&gt;&lt;br&gt;Max it, c&amp;#39;est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d&amp;#39;une multitude de services exclusifs. &lt;br&gt;&lt;br&gt;Créez votre espace sur</t>
+        </is>
+      </c>
+      <c r="T618" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U618" t="inlineStr"/>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G619" t="n">
+        <v>596028698</v>
+      </c>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>Méditel</t>
+        </is>
+      </c>
+      <c r="J619" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K619" t="n">
+        <v>0</v>
+      </c>
+      <c r="L619" t="b">
+        <v>1</v>
+      </c>
+      <c r="M619" t="n">
+        <v>3.94626</v>
+      </c>
+      <c r="N619" t="n">
+        <v>2754</v>
+      </c>
+      <c r="P619" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "MA" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R619" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S619" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l'expérience mobile réinventé
+Max it, c'est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d'une multitude de services exclusifs. 
+Créez votre espace sur mesure et bénéficiez d'</t>
+        </is>
+      </c>
+      <c r="T619" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U619" t="inlineStr"/>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G620" t="inlineStr">
+        <is>
+          <t>com.oml.dsi.orangemobile</t>
+        </is>
+      </c>
+      <c r="H620" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I620" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J620" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K620" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L620" t="b">
+        <v>0</v>
+      </c>
+      <c r="M620" t="n">
+        <v>2.6958454</v>
+      </c>
+      <c r="N620" t="n">
+        <v>38250</v>
+      </c>
+      <c r="P620" t="inlineStr"/>
+      <c r="Q620" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R620" t="inlineStr">
+        <is>
+          <t>6.5.0</t>
+        </is>
+      </c>
+      <c r="S620" t="inlineStr">
+        <is>
+          <t>Easily manage your Orange Mali line&lt;br&gt;● Manage your account and view all essential information, your offers, and your phone lines.&lt;br&gt;● Subscribe to call, SMS, Internet, and international call packages.&lt;br&gt;● Track your usage by checking your credit and Internet balance.&lt;br&gt;● Recharge your line by p</t>
+        </is>
+      </c>
+      <c r="T620" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U620" t="inlineStr"/>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G621" t="n">
+        <v>1494321079</v>
+      </c>
+      <c r="H621" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J621" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K621" t="n">
+        <v>0</v>
+      </c>
+      <c r="L621" t="b">
+        <v>1</v>
+      </c>
+      <c r="M621" t="n">
+        <v>2.51962</v>
+      </c>
+      <c r="N621" t="n">
+        <v>4738</v>
+      </c>
+      <c r="O621" t="n">
+        <v>11</v>
+      </c>
+      <c r="P621" t="inlineStr"/>
+      <c r="R621" t="inlineStr">
+        <is>
+          <t>6.5.2</t>
+        </is>
+      </c>
+      <c r="S621" t="inlineStr">
+        <is>
+          <t>Gérez facilement votre ligne Orange Mali 
+●        Gérez votre compte et consultez toutes les informations essentielles sur celui-ci, vos offres, ainsi que vos lignes téléphoniques.
+●        Souscrivez aux forfaits appels, SMS, Internet, et appels internationaux.
+●        Suivez votre consommation e</t>
+        </is>
+      </c>
+      <c r="T621" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U621" t="inlineStr"/>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G622" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.omg</t>
+        </is>
+      </c>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J622" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K622" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L622" t="b">
+        <v>0</v>
+      </c>
+      <c r="M622" t="n">
+        <v>4.1666665</v>
+      </c>
+      <c r="N622" t="n">
+        <v>1372</v>
+      </c>
+      <c r="O622" t="n">
+        <v>55</v>
+      </c>
+      <c r="P622" t="inlineStr"/>
+      <c r="Q622" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R622" t="inlineStr">
+        <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="S622" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.&lt;br&gt;&lt;br&gt;Simplify Your Life with Max it&lt;br&gt;With Max It, ac</t>
+        </is>
+      </c>
+      <c r="T622" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U622" t="inlineStr"/>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G623" t="n">
+        <v>1295171817</v>
+      </c>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J623" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K623" t="n">
+        <v>0</v>
+      </c>
+      <c r="L623" t="b">
+        <v>1</v>
+      </c>
+      <c r="M623" t="n">
+        <v>3.08696</v>
+      </c>
+      <c r="N623" t="n">
+        <v>69</v>
+      </c>
+      <c r="O623" t="n">
+        <v>33</v>
+      </c>
+      <c r="P623" t="inlineStr"/>
+      <c r="R623" t="inlineStr">
+        <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="S623" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.
+Simplify Your Life with Max it
+With Max it, access a se</t>
+        </is>
+      </c>
+      <c r="T623" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U623" t="inlineStr"/>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.olr</t>
+        </is>
+      </c>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>Orange Max it - Liberia</t>
+        </is>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J624" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K624" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L624" t="b">
+        <v>0</v>
+      </c>
+      <c r="M624" t="n">
+        <v>4.551282</v>
+      </c>
+      <c r="N624" t="n">
+        <v>3096</v>
+      </c>
+      <c r="O624" t="n">
+        <v>62</v>
+      </c>
+      <c r="P624" t="inlineStr"/>
+      <c r="Q624" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R624" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="S624" t="inlineStr">
+        <is>
+          <t>Max it: your personalized experience by Orange Liberia!&lt;br&gt;&lt;br&gt;Step into Max it, your all-in-one solution for telecom, marketplace, and financial services! Manage your mobile line, customize offers, pay your bills, keep&lt;br&gt;track of your usage with ease, and recharge your credit. Access exclusive eve</t>
+        </is>
+      </c>
+      <c r="T624" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U624" t="inlineStr"/>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G625" t="n">
+        <v>6746187327</v>
+      </c>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>Orange Max it – Liberia</t>
+        </is>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J625" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K625" t="n">
+        <v>0</v>
+      </c>
+      <c r="L625" t="b">
+        <v>1</v>
+      </c>
+      <c r="M625" t="n">
+        <v>4.0625</v>
+      </c>
+      <c r="N625" t="n">
+        <v>48</v>
+      </c>
+      <c r="P625" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "LR" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R625" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="S625" t="inlineStr">
+        <is>
+          <t>Max it is a free application, which allows Orange Liberia customers to:
+- Consult your account in real time: minutes, sms, internet
+- Top up your account or a friend account 
+- Buy  Bundles (voice, data, SMS, roaming, international)
+- Discover the latest offers and promotions 
+- Access to Orange se</t>
+        </is>
+      </c>
+      <c r="T625" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U625" t="inlineStr"/>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G626" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ojo</t>
+        </is>
+      </c>
+      <c r="H626" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J626" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K626" t="inlineStr">
+        <is>
+          <t>JOD 0.000</t>
+        </is>
+      </c>
+      <c r="L626" t="b">
+        <v>0</v>
+      </c>
+      <c r="M626" t="n">
+        <v>4.4331293</v>
+      </c>
+      <c r="N626" t="n">
+        <v>97659</v>
+      </c>
+      <c r="O626" t="n">
+        <v>51</v>
+      </c>
+      <c r="P626" t="inlineStr"/>
+      <c r="Q626" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R626" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S626" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience&lt;br&gt;Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.&lt;br&gt;Important Update:&lt;br&gt;The jood app (jood Orange) w</t>
+        </is>
+      </c>
+      <c r="T626" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U626" t="inlineStr"/>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G627" t="n">
+        <v>808824590</v>
+      </c>
+      <c r="H627" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J627" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K627" t="n">
+        <v>0</v>
+      </c>
+      <c r="L627" t="b">
+        <v>1</v>
+      </c>
+      <c r="M627" t="n">
+        <v>4.21056</v>
+      </c>
+      <c r="N627" t="n">
+        <v>3011</v>
+      </c>
+      <c r="O627" t="n">
+        <v>47</v>
+      </c>
+      <c r="P627" t="inlineStr"/>
+      <c r="R627" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S627" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience
+Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.
+Important Update:
+The jood app (jood Orange) will be di</t>
+        </is>
+      </c>
+      <c r="T627" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U627" t="inlineStr"/>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G628" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.oci</t>
+        </is>
+      </c>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>Orange Côte d'Ivoire S.A</t>
+        </is>
+      </c>
+      <c r="J628" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K628" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L628" t="b">
+        <v>0</v>
+      </c>
+      <c r="M628" t="n">
+        <v>4.166269</v>
+      </c>
+      <c r="N628" t="n">
+        <v>67145</v>
+      </c>
+      <c r="O628" t="n">
+        <v>13</v>
+      </c>
+      <c r="P628" t="inlineStr"/>
+      <c r="Q628" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R628" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S628" t="inlineStr">
+        <is>
+          <t>Aaaahhh, ta super app Max it, n&amp;#39;a pas fini de te surprendre... &lt;br&gt;Est-ce que tu as remarqué ? Maintenant, tu as ton QR code personnalisé en haut de ton écran d&amp;#39;accueil ! Ainsi, tu peux :&lt;br&gt;     scanner le QR code de ton ami(e) pour lui faire un transfert d&amp;#39;&amp;#39;argent&lt;br&gt;     scanner l</t>
+        </is>
+      </c>
+      <c r="T628" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U628" t="inlineStr"/>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G629" t="n">
+        <v>1061120855</v>
+      </c>
+      <c r="H629" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>Orange CI</t>
+        </is>
+      </c>
+      <c r="J629" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K629" t="n">
+        <v>0</v>
+      </c>
+      <c r="L629" t="b">
+        <v>1</v>
+      </c>
+      <c r="M629" t="n">
+        <v>3.78743</v>
+      </c>
+      <c r="N629" t="n">
+        <v>5965</v>
+      </c>
+      <c r="O629" t="n">
+        <v>9</v>
+      </c>
+      <c r="P629" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R629" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S629" t="inlineStr">
+        <is>
+          <t>Max it, la super app all-in-one te fais gagner du temps, et diminue tes soucis... Gagne plus d'espace de stockage sur ton téléphone ; plus besoin de cumuler plusieurs appli d'Orange pour avoir accès à un maximum de services. Max it est là ! Gère ta ligne (SIM) au niveau des pass, des soldes, réalise</t>
+        </is>
+      </c>
+      <c r="T629" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U629" t="inlineStr"/>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G630" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogw</t>
+        </is>
+      </c>
+      <c r="H630" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J630" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K630" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L630" t="b">
+        <v>0</v>
+      </c>
+      <c r="M630" t="n">
+        <v>4.350993</v>
+      </c>
+      <c r="N630" t="n">
+        <v>1530</v>
+      </c>
+      <c r="O630" t="n">
+        <v>3</v>
+      </c>
+      <c r="P630" t="inlineStr"/>
+      <c r="Q630" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R630" t="inlineStr">
+        <is>
+          <t>4.0.18</t>
+        </is>
+      </c>
+      <c r="S630" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T630" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U630" t="inlineStr"/>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G631" t="n">
+        <v>1574668652</v>
+      </c>
+      <c r="H631" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I631" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J631" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K631" t="n">
+        <v>0</v>
+      </c>
+      <c r="L631" t="b">
+        <v>1</v>
+      </c>
+      <c r="M631" t="n">
+        <v>4.05333</v>
+      </c>
+      <c r="N631" t="n">
+        <v>75</v>
+      </c>
+      <c r="O631" t="n">
+        <v>15</v>
+      </c>
+      <c r="P631" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R631" t="inlineStr">
+        <is>
+          <t>6.0.35</t>
+        </is>
+      </c>
+      <c r="S631" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T631" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U631" t="inlineStr"/>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G632" t="inlineStr">
+        <is>
+          <t>com.orange.sugu.ocd</t>
+        </is>
+      </c>
+      <c r="H632" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I632" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J632" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K632" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L632" t="b">
+        <v>0</v>
+      </c>
+      <c r="M632" t="n">
+        <v>4.121212</v>
+      </c>
+      <c r="N632" t="n">
+        <v>5288</v>
+      </c>
+      <c r="O632" t="n">
+        <v>62</v>
+      </c>
+      <c r="P632" t="inlineStr"/>
+      <c r="Q632" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R632" t="inlineStr">
+        <is>
+          <t>9.0.12</t>
+        </is>
+      </c>
+      <c r="S632" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DRC that brings together the features of MyOrange, and Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Plans, Mobile Payments, money transfers, bill payments, subscriptions, and entertai</t>
+        </is>
+      </c>
+      <c r="T632" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U632" t="inlineStr"/>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G633" t="n">
+        <v>6447896435</v>
+      </c>
+      <c r="H633" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I633" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J633" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K633" t="n">
+        <v>0</v>
+      </c>
+      <c r="L633" t="b">
+        <v>1</v>
+      </c>
+      <c r="M633" t="n">
+        <v>3.55762</v>
+      </c>
+      <c r="N633" t="n">
+        <v>269</v>
+      </c>
+      <c r="P633" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "CD" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R633" t="inlineStr">
+        <is>
+          <t>9.0.6</t>
+        </is>
+      </c>
+      <c r="S633" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DR Congo. It brings together the features of Orange et Moi, as well as Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Packages, Mobile payment, money transfers, bill payment and subscri</t>
+        </is>
+      </c>
+      <c r="T633" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U633" t="inlineStr"/>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G634" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ocm</t>
+        </is>
+      </c>
+      <c r="H634" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroon</t>
+        </is>
+      </c>
+      <c r="I634" t="inlineStr">
+        <is>
+          <t>Orange MEA</t>
+        </is>
+      </c>
+      <c r="J634" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K634" t="inlineStr">
+        <is>
+          <t>FCFA 0</t>
+        </is>
+      </c>
+      <c r="L634" t="b">
+        <v>0</v>
+      </c>
+      <c r="M634" t="n">
+        <v>3.9318182</v>
+      </c>
+      <c r="N634" t="n">
+        <v>46888</v>
+      </c>
+      <c r="O634" t="n">
+        <v>8</v>
+      </c>
+      <c r="P634" t="inlineStr"/>
+      <c r="Q634" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R634" t="inlineStr">
+        <is>
+          <t>7.0.23</t>
+        </is>
+      </c>
+      <c r="S634" t="inlineStr">
+        <is>
+          <t>Max it brings together everything that matters to you in one app: managing your lines, money transfer, bill payment, exclusive offers, and a universe of lifestyle and entertainment. Simple, fast, and 100% secure..&lt;br&gt;&lt;br&gt;📞 My line&lt;br&gt;Manage your Orange mobile and landline bundles in a single click:</t>
+        </is>
+      </c>
+      <c r="T634" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U634" t="inlineStr"/>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G635" t="n">
+        <v>1116920093</v>
+      </c>
+      <c r="H635" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroun</t>
+        </is>
+      </c>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>Orange Middle East &amp; Africa</t>
+        </is>
+      </c>
+      <c r="J635" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K635" t="n">
+        <v>0</v>
+      </c>
+      <c r="L635" t="b">
+        <v>1</v>
+      </c>
+      <c r="M635" t="n">
+        <v>3.76878</v>
+      </c>
+      <c r="N635" t="n">
+        <v>16149</v>
+      </c>
+      <c r="O635" t="n">
+        <v>2</v>
+      </c>
+      <c r="P635" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R635" t="inlineStr">
+        <is>
+          <t>7.0.24</t>
+        </is>
+      </c>
+      <c r="S635" t="inlineStr">
+        <is>
+          <t>Avec Max it, Orange rassemble tout ce qui compte pour vous dans une même application : la gestion de vos lignes, les transferts d’argent, payement de vos factures, des offres exclusives et un univers lifestyle et divertissement.
+Simple, rapide et 100 % sécurisée.
+Ma ligne
+Gérez vos forfaits mobiles</t>
+        </is>
+      </c>
+      <c r="T635" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U635" t="inlineStr"/>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G636" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obf</t>
+        </is>
+      </c>
+      <c r="H636" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso</t>
+        </is>
+      </c>
+      <c r="J636" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K636" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L636" t="b">
+        <v>0</v>
+      </c>
+      <c r="M636" t="n">
+        <v>4.143025</v>
+      </c>
+      <c r="N636" t="n">
+        <v>25456</v>
+      </c>
+      <c r="O636" t="n">
+        <v>11</v>
+      </c>
+      <c r="P636" t="inlineStr"/>
+      <c r="Q636" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R636" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S636" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.&lt;br&gt;Gérez vos lignes mobiles, effectuez des transferts d&amp;#39;argent sécurisés, réglez vos factures, profitez d&amp;#39;offres exclusives, effectuez des paiements marchands fiables, et bien plus enco</t>
+        </is>
+      </c>
+      <c r="T636" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U636" t="inlineStr"/>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G637" t="n">
+        <v>1553774707</v>
+      </c>
+      <c r="H637" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso SA</t>
+        </is>
+      </c>
+      <c r="J637" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K637" t="n">
+        <v>0</v>
+      </c>
+      <c r="L637" t="b">
+        <v>1</v>
+      </c>
+      <c r="M637" t="n">
+        <v>3.45377</v>
+      </c>
+      <c r="N637" t="n">
+        <v>1179</v>
+      </c>
+      <c r="O637" t="n">
+        <v>7</v>
+      </c>
+      <c r="P637" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R637" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S637" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.
+Gérez vos lignes mobiles, effectuez des transferts d'argent sécurisés, réglez vos factures, profitez d'offres exclusives, effectuez des paiements marchands fiables, et bien plus encore, le tout</t>
+        </is>
+      </c>
+      <c r="T637" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U637" t="inlineStr"/>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G638" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obw</t>
+        </is>
+      </c>
+      <c r="H638" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J638" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K638" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L638" t="b">
+        <v>0</v>
+      </c>
+      <c r="M638" t="n">
+        <v>3.9964788</v>
+      </c>
+      <c r="N638" t="n">
+        <v>2962</v>
+      </c>
+      <c r="O638" t="n">
+        <v>36</v>
+      </c>
+      <c r="P638" t="inlineStr"/>
+      <c r="Q638" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R638" t="inlineStr">
+        <is>
+          <t>7.3.8</t>
+        </is>
+      </c>
+      <c r="S638" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it, the brand-new Orange Botswana Super App that follows Yame and gives you access to four distinct universes for a one-of-a-kind experience!&lt;br&gt;&lt;br&gt;Manage your accounts, make quick payments using QR codes, investigate a range of online goods and services, and discover the many options provided </t>
+        </is>
+      </c>
+      <c r="T638" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U638" t="inlineStr"/>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G639" t="n">
+        <v>1195839458</v>
+      </c>
+      <c r="H639" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J639" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K639" t="n">
+        <v>0</v>
+      </c>
+      <c r="L639" t="b">
+        <v>1</v>
+      </c>
+      <c r="M639" t="n">
+        <v>3.00806</v>
+      </c>
+      <c r="N639" t="n">
+        <v>124</v>
+      </c>
+      <c r="O639" t="n">
+        <v>11</v>
+      </c>
+      <c r="P639" t="inlineStr"/>
+      <c r="R639" t="inlineStr">
+        <is>
+          <t>7.3.1</t>
+        </is>
+      </c>
+      <c r="S639" t="inlineStr">
+        <is>
+          <t>A free mobile self-care application for Orange Botswana’s mobile customers.
+Full Description :
+Max it is a free application, which allows Orange Botswana customers to:
+- Consult your account in real time: minutes, sms, internet ...
+- Top up your account or a friend account  with Orange Money
+-</t>
+        </is>
+      </c>
+      <c r="T639" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U639" t="inlineStr"/>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G640" t="inlineStr">
+        <is>
+          <t>com.orange.mobinilandme</t>
+        </is>
+      </c>
+      <c r="H640" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J640" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K640" t="inlineStr">
+        <is>
+          <t>EGP 0.00</t>
+        </is>
+      </c>
+      <c r="L640" t="b">
+        <v>0</v>
+      </c>
+      <c r="M640" t="n">
+        <v>4.5600924</v>
+      </c>
+      <c r="N640" t="n">
+        <v>927252</v>
+      </c>
+      <c r="O640" t="n">
+        <v>23</v>
+      </c>
+      <c r="P640" t="inlineStr"/>
+      <c r="Q640" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R640" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S640" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion&lt;br&gt;Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.&lt;br&gt;Key services include:&lt;br&gt;• Account Management: Easily manage</t>
+        </is>
+      </c>
+      <c r="T640" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U640" t="inlineStr"/>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>4e0f2882-0359-4bb5-812d-fa8bbb7a6337</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>2026-07-27 07:34:37</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G641" t="n">
+        <v>942568333</v>
+      </c>
+      <c r="H641" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J641" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K641" t="n">
+        <v>0</v>
+      </c>
+      <c r="L641" t="b">
+        <v>1</v>
+      </c>
+      <c r="M641" t="n">
+        <v>4.25182</v>
+      </c>
+      <c r="N641" t="n">
+        <v>117381</v>
+      </c>
+      <c r="O641" t="n">
+        <v>67</v>
+      </c>
+      <c r="P641" t="inlineStr"/>
+      <c r="R641" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S641" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion
+Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.
+Key services include:
+• Account Management: Easily manage your Ora</t>
+        </is>
+      </c>
+      <c r="T641" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U641" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-07-28
</commit_message>
<xml_diff>
--- a/maxit_store_history.xlsx
+++ b/maxit_store_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U641"/>
+  <dimension ref="A1:U673"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52414,7 +52414,6 @@
       <c r="O610" t="n">
         <v>23</v>
       </c>
-      <c r="P610" t="inlineStr"/>
       <c r="Q610" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -52435,7 +52434,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U610" t="inlineStr"/>
     </row>
     <row r="611">
       <c r="A611" t="inlineStr">
@@ -52498,7 +52496,6 @@
       <c r="N611" t="n">
         <v>322</v>
       </c>
-      <c r="P611" t="inlineStr"/>
       <c r="R611" t="inlineStr">
         <is>
           <t>6.4.8</t>
@@ -52514,7 +52511,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U611" t="inlineStr"/>
     </row>
     <row r="612">
       <c r="A612" t="inlineStr">
@@ -52584,7 +52580,6 @@
       <c r="O612" t="n">
         <v>29</v>
       </c>
-      <c r="P612" t="inlineStr"/>
       <c r="Q612" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -52605,7 +52600,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U612" t="inlineStr"/>
     </row>
     <row r="613">
       <c r="A613" t="inlineStr">
@@ -52671,7 +52665,6 @@
       <c r="O613" t="n">
         <v>43</v>
       </c>
-      <c r="P613" t="inlineStr"/>
       <c r="R613" t="inlineStr">
         <is>
           <t>10.0.6</t>
@@ -52689,7 +52682,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U613" t="inlineStr"/>
     </row>
     <row r="614">
       <c r="A614" t="inlineStr">
@@ -52759,7 +52751,6 @@
       <c r="O614" t="n">
         <v>11</v>
       </c>
-      <c r="P614" t="inlineStr"/>
       <c r="Q614" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -52780,7 +52771,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U614" t="inlineStr"/>
     </row>
     <row r="615">
       <c r="A615" t="inlineStr">
@@ -52869,7 +52859,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U615" t="inlineStr"/>
     </row>
     <row r="616">
       <c r="A616" t="inlineStr">
@@ -52939,7 +52928,6 @@
       <c r="O616" t="n">
         <v>13</v>
       </c>
-      <c r="P616" t="inlineStr"/>
       <c r="Q616" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -52960,7 +52948,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U616" t="inlineStr"/>
     </row>
     <row r="617">
       <c r="A617" t="inlineStr">
@@ -53026,7 +53013,6 @@
       <c r="O617" t="n">
         <v>8</v>
       </c>
-      <c r="P617" t="inlineStr"/>
       <c r="R617" t="inlineStr">
         <is>
           <t>21.1.0</t>
@@ -53044,7 +53030,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U617" t="inlineStr"/>
     </row>
     <row r="618">
       <c r="A618" t="inlineStr">
@@ -53114,7 +53099,6 @@
       <c r="O618" t="n">
         <v>82</v>
       </c>
-      <c r="P618" t="inlineStr"/>
       <c r="Q618" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -53135,7 +53119,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U618" t="inlineStr"/>
     </row>
     <row r="619">
       <c r="A619" t="inlineStr">
@@ -53220,7 +53203,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U619" t="inlineStr"/>
     </row>
     <row r="620">
       <c r="A620" t="inlineStr">
@@ -53287,7 +53269,6 @@
       <c r="N620" t="n">
         <v>38250</v>
       </c>
-      <c r="P620" t="inlineStr"/>
       <c r="Q620" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -53308,7 +53289,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U620" t="inlineStr"/>
     </row>
     <row r="621">
       <c r="A621" t="inlineStr">
@@ -53374,7 +53354,6 @@
       <c r="O621" t="n">
         <v>11</v>
       </c>
-      <c r="P621" t="inlineStr"/>
       <c r="R621" t="inlineStr">
         <is>
           <t>6.5.2</t>
@@ -53393,7 +53372,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U621" t="inlineStr"/>
     </row>
     <row r="622">
       <c r="A622" t="inlineStr">
@@ -53463,7 +53441,6 @@
       <c r="O622" t="n">
         <v>55</v>
       </c>
-      <c r="P622" t="inlineStr"/>
       <c r="Q622" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -53484,7 +53461,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U622" t="inlineStr"/>
     </row>
     <row r="623">
       <c r="A623" t="inlineStr">
@@ -53550,7 +53526,6 @@
       <c r="O623" t="n">
         <v>33</v>
       </c>
-      <c r="P623" t="inlineStr"/>
       <c r="R623" t="inlineStr">
         <is>
           <t>5.0.2</t>
@@ -53568,7 +53543,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U623" t="inlineStr"/>
     </row>
     <row r="624">
       <c r="A624" t="inlineStr">
@@ -53638,7 +53612,6 @@
       <c r="O624" t="n">
         <v>62</v>
       </c>
-      <c r="P624" t="inlineStr"/>
       <c r="Q624" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -53659,7 +53632,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U624" t="inlineStr"/>
     </row>
     <row r="625">
       <c r="A625" t="inlineStr">
@@ -53747,7 +53719,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U625" t="inlineStr"/>
     </row>
     <row r="626">
       <c r="A626" t="inlineStr">
@@ -53817,7 +53788,6 @@
       <c r="O626" t="n">
         <v>51</v>
       </c>
-      <c r="P626" t="inlineStr"/>
       <c r="Q626" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -53838,7 +53808,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U626" t="inlineStr"/>
     </row>
     <row r="627">
       <c r="A627" t="inlineStr">
@@ -53904,7 +53873,6 @@
       <c r="O627" t="n">
         <v>47</v>
       </c>
-      <c r="P627" t="inlineStr"/>
       <c r="R627" t="inlineStr">
         <is>
           <t>10.0.21</t>
@@ -53923,7 +53891,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U627" t="inlineStr"/>
     </row>
     <row r="628">
       <c r="A628" t="inlineStr">
@@ -53993,7 +53960,6 @@
       <c r="O628" t="n">
         <v>13</v>
       </c>
-      <c r="P628" t="inlineStr"/>
       <c r="Q628" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -54014,7 +53980,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U628" t="inlineStr"/>
     </row>
     <row r="629">
       <c r="A629" t="inlineStr">
@@ -54100,7 +54065,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U629" t="inlineStr"/>
     </row>
     <row r="630">
       <c r="A630" t="inlineStr">
@@ -54170,7 +54134,6 @@
       <c r="O630" t="n">
         <v>3</v>
       </c>
-      <c r="P630" t="inlineStr"/>
       <c r="Q630" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -54191,7 +54154,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U630" t="inlineStr"/>
     </row>
     <row r="631">
       <c r="A631" t="inlineStr">
@@ -54277,7 +54239,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U631" t="inlineStr"/>
     </row>
     <row r="632">
       <c r="A632" t="inlineStr">
@@ -54347,7 +54308,6 @@
       <c r="O632" t="n">
         <v>62</v>
       </c>
-      <c r="P632" t="inlineStr"/>
       <c r="Q632" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -54368,7 +54328,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U632" t="inlineStr"/>
     </row>
     <row r="633">
       <c r="A633" t="inlineStr">
@@ -54451,7 +54410,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U633" t="inlineStr"/>
     </row>
     <row r="634">
       <c r="A634" t="inlineStr">
@@ -54521,7 +54479,6 @@
       <c r="O634" t="n">
         <v>8</v>
       </c>
-      <c r="P634" t="inlineStr"/>
       <c r="Q634" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -54542,7 +54499,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U634" t="inlineStr"/>
     </row>
     <row r="635">
       <c r="A635" t="inlineStr">
@@ -54631,7 +54587,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U635" t="inlineStr"/>
     </row>
     <row r="636">
       <c r="A636" t="inlineStr">
@@ -54701,7 +54656,6 @@
       <c r="O636" t="n">
         <v>11</v>
       </c>
-      <c r="P636" t="inlineStr"/>
       <c r="Q636" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -54722,7 +54676,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U636" t="inlineStr"/>
     </row>
     <row r="637">
       <c r="A637" t="inlineStr">
@@ -54809,7 +54762,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U637" t="inlineStr"/>
     </row>
     <row r="638">
       <c r="A638" t="inlineStr">
@@ -54879,7 +54831,6 @@
       <c r="O638" t="n">
         <v>36</v>
       </c>
-      <c r="P638" t="inlineStr"/>
       <c r="Q638" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -54900,7 +54851,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U638" t="inlineStr"/>
     </row>
     <row r="639">
       <c r="A639" t="inlineStr">
@@ -54966,7 +54916,6 @@
       <c r="O639" t="n">
         <v>11</v>
       </c>
-      <c r="P639" t="inlineStr"/>
       <c r="R639" t="inlineStr">
         <is>
           <t>7.3.1</t>
@@ -54987,7 +54936,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U639" t="inlineStr"/>
     </row>
     <row r="640">
       <c r="A640" t="inlineStr">
@@ -55057,7 +55005,6 @@
       <c r="O640" t="n">
         <v>23</v>
       </c>
-      <c r="P640" t="inlineStr"/>
       <c r="Q640" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -55078,7 +55025,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U640" t="inlineStr"/>
     </row>
     <row r="641">
       <c r="A641" t="inlineStr">
@@ -55144,7 +55090,6 @@
       <c r="O641" t="n">
         <v>67</v>
       </c>
-      <c r="P641" t="inlineStr"/>
       <c r="R641" t="inlineStr">
         <is>
           <t>10.1.0</t>
@@ -55163,7 +55108,2825 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U641" t="inlineStr"/>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G642" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogn</t>
+        </is>
+      </c>
+      <c r="H642" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J642" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K642" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L642" t="b">
+        <v>0</v>
+      </c>
+      <c r="M642" t="n">
+        <v>4.453245</v>
+      </c>
+      <c r="N642" t="n">
+        <v>9279</v>
+      </c>
+      <c r="O642" t="n">
+        <v>20</v>
+      </c>
+      <c r="P642" t="inlineStr"/>
+      <c r="Q642" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R642" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S642" t="inlineStr">
+        <is>
+          <t>Bien plus qu&amp;#39;une application, un véritable assistant personnel pour une vie connectée et simplifiée.&lt;br&gt;Suivi de consommation: Votre tableau de bord tout-en-un pour une gestion simplifiée !&lt;br&gt;- Gestion de votre offre: Accédez à une vue détaillée de votre offre actuelle et de vos forfaits Orange</t>
+        </is>
+      </c>
+      <c r="T642" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U642" t="inlineStr"/>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G643" t="n">
+        <v>1177999485</v>
+      </c>
+      <c r="H643" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J643" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K643" t="n">
+        <v>0</v>
+      </c>
+      <c r="L643" t="b">
+        <v>1</v>
+      </c>
+      <c r="M643" t="n">
+        <v>3.89441</v>
+      </c>
+      <c r="N643" t="n">
+        <v>322</v>
+      </c>
+      <c r="P643" t="inlineStr"/>
+      <c r="R643" t="inlineStr">
+        <is>
+          <t>6.4.8</t>
+        </is>
+      </c>
+      <c r="S643" t="inlineStr">
+        <is>
+          <t>La fusion d’Orange et Moi et Orange Money donne naissance à Max it, la nouvelle Super Application Tout-en-Un. Profitez du suivi de consommation, de paiements mobiles, de toutes les fonctionnalités Orange et Moi et Money avec un large éventail de divertissements, le tout regroupé en un seul endroit !</t>
+        </is>
+      </c>
+      <c r="T643" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U643" t="inlineStr"/>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G644" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.otn</t>
+        </is>
+      </c>
+      <c r="H644" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J644" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K644" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L644" t="b">
+        <v>0</v>
+      </c>
+      <c r="M644" t="n">
+        <v>3.967962</v>
+      </c>
+      <c r="N644" t="n">
+        <v>35374</v>
+      </c>
+      <c r="O644" t="n">
+        <v>28</v>
+      </c>
+      <c r="P644" t="inlineStr"/>
+      <c r="Q644" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R644" t="inlineStr">
+        <is>
+          <t>10.0.6</t>
+        </is>
+      </c>
+      <c r="S644" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Max it par Orange Tunisie facilite votre vie au quotidien !&lt;/h2&gt;&lt;br&gt;&lt;br&gt;Welcome sur Max it !&lt;br&gt;Accédez rapidement à vos fonctionnalités Max it préférées et profitez également de contenus exclusifs, d’activités divertissantes, et de jeux interactifs pour une expérience enrichissante avec la roue</t>
+        </is>
+      </c>
+      <c r="T644" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U644" t="inlineStr"/>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G645" t="n">
+        <v>1146892088</v>
+      </c>
+      <c r="H645" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J645" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K645" t="n">
+        <v>0</v>
+      </c>
+      <c r="L645" t="b">
+        <v>1</v>
+      </c>
+      <c r="M645" t="n">
+        <v>3.03173</v>
+      </c>
+      <c r="N645" t="n">
+        <v>1639</v>
+      </c>
+      <c r="O645" t="n">
+        <v>35</v>
+      </c>
+      <c r="P645" t="inlineStr"/>
+      <c r="R645" t="inlineStr">
+        <is>
+          <t>10.0.6</t>
+        </is>
+      </c>
+      <c r="S645" t="inlineStr">
+        <is>
+          <t>Max it by Orange Tunisie : Votre appli incontournable pour une vie connectée
+Welcome sur Max it : Découvrez fonctionnalités, jeux &amp; contenus de divertissement by Orange Tunisie !
+Trouvez vite vos fonctionnalités Max it favorites et explorez des contenus exclusifs et des jeux pour une expérience im</t>
+        </is>
+      </c>
+      <c r="T645" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U645" t="inlineStr"/>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G646" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osl</t>
+        </is>
+      </c>
+      <c r="H646" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J646" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K646" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L646" t="b">
+        <v>0</v>
+      </c>
+      <c r="M646" t="n">
+        <v>4.361991</v>
+      </c>
+      <c r="N646" t="n">
+        <v>2131</v>
+      </c>
+      <c r="O646" t="n">
+        <v>9</v>
+      </c>
+      <c r="P646" t="inlineStr"/>
+      <c r="Q646" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R646" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S646" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it is a free application, which allows Orange Sierra Leone prepaid and postpaid customers to:&lt;br&gt;&lt;br&gt;- Consult your account in real time: minutes, sms, internet&lt;br&gt;- Top up your account or a friend account &lt;br&gt;- Buy Internet Bundles&lt;br&gt;- Discover the latest offers and promotions &lt;br&gt;- Access to </t>
+        </is>
+      </c>
+      <c r="T646" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U646" t="inlineStr"/>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G647" t="n">
+        <v>6443607903</v>
+      </c>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J647" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K647" t="n">
+        <v>0</v>
+      </c>
+      <c r="L647" t="b">
+        <v>1</v>
+      </c>
+      <c r="M647" t="n">
+        <v>3.69948</v>
+      </c>
+      <c r="N647" t="n">
+        <v>193</v>
+      </c>
+      <c r="O647" t="n">
+        <v>8</v>
+      </c>
+      <c r="P647" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R647" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S647" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The merger of My Orange &amp; Orange Money has given birth to Max it the all-in-one super app, a free application which allows all Orange Sierra Leone customers to 
+Track calls, SMS, and Data usage and monitor balance. 
+Make a secure mobile/Orange Money payment.
+Easily transfer credit to other users </t>
+        </is>
+      </c>
+      <c r="T647" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U647" t="inlineStr"/>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G648" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osn</t>
+        </is>
+      </c>
+      <c r="H648" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>Orange Sénégal</t>
+        </is>
+      </c>
+      <c r="J648" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K648" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L648" t="b">
+        <v>0</v>
+      </c>
+      <c r="M648" t="n">
+        <v>4.3026533</v>
+      </c>
+      <c r="N648" t="n">
+        <v>51221</v>
+      </c>
+      <c r="O648" t="n">
+        <v>13</v>
+      </c>
+      <c r="P648" t="inlineStr"/>
+      <c r="Q648" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R648" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S648" t="inlineStr">
+        <is>
+          <t>Lu bees ak Max it ! &lt;br&gt;Une application repensée pour être plus simple, plus rapide et adaptée à vos besoins. Une expérience optimisée pour faciliter vos usages au quotidien, avec des parcours simplifiés et un accès plus fluide à vos services. Que vous soyez client Orange ou non, Max it vous accompa</t>
+        </is>
+      </c>
+      <c r="T648" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U648" t="inlineStr"/>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G649" t="n">
+        <v>1039327980</v>
+      </c>
+      <c r="H649" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>Orange Senegal</t>
+        </is>
+      </c>
+      <c r="J649" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K649" t="n">
+        <v>0</v>
+      </c>
+      <c r="L649" t="b">
+        <v>1</v>
+      </c>
+      <c r="M649" t="n">
+        <v>4.16941</v>
+      </c>
+      <c r="N649" t="n">
+        <v>30221</v>
+      </c>
+      <c r="O649" t="n">
+        <v>4</v>
+      </c>
+      <c r="P649" t="inlineStr"/>
+      <c r="R649" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S649" t="inlineStr">
+        <is>
+          <t>Here is the English translation:
+Welcome to Max it!
+A redesigned app to be simpler, faster, and tailored to your needs. An optimized experience to make your daily life easier, with streamlined journeys and smoother access to your services. Whether you are an Orange customer or not, Max it is your e</t>
+        </is>
+      </c>
+      <c r="T649" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U649" t="inlineStr"/>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G650" t="inlineStr">
+        <is>
+          <t>com.orange.meditel.mediteletmoi</t>
+        </is>
+      </c>
+      <c r="H650" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>Orange Maroc</t>
+        </is>
+      </c>
+      <c r="J650" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K650" t="inlineStr">
+        <is>
+          <t>MAD 0.00</t>
+        </is>
+      </c>
+      <c r="L650" t="b">
+        <v>0</v>
+      </c>
+      <c r="M650" t="n">
+        <v>3.7194004</v>
+      </c>
+      <c r="N650" t="n">
+        <v>110913</v>
+      </c>
+      <c r="O650" t="n">
+        <v>77</v>
+      </c>
+      <c r="P650" t="inlineStr"/>
+      <c r="Q650" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R650" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S650" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l&amp;#39;expérience mobile réinventé&lt;br&gt;&lt;br&gt;Max it, c&amp;#39;est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d&amp;#39;une multitude de services exclusifs. &lt;br&gt;&lt;br&gt;Créez votre espace sur</t>
+        </is>
+      </c>
+      <c r="T650" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U650" t="inlineStr"/>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G651" t="n">
+        <v>596028698</v>
+      </c>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>Méditel</t>
+        </is>
+      </c>
+      <c r="J651" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K651" t="n">
+        <v>0</v>
+      </c>
+      <c r="L651" t="b">
+        <v>1</v>
+      </c>
+      <c r="M651" t="n">
+        <v>3.94664</v>
+      </c>
+      <c r="N651" t="n">
+        <v>2755</v>
+      </c>
+      <c r="P651" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "MA" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R651" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S651" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l'expérience mobile réinventé
+Max it, c'est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d'une multitude de services exclusifs. 
+Créez votre espace sur mesure et bénéficiez d'</t>
+        </is>
+      </c>
+      <c r="T651" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U651" t="inlineStr"/>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G652" t="inlineStr">
+        <is>
+          <t>com.oml.dsi.orangemobile</t>
+        </is>
+      </c>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J652" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K652" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L652" t="b">
+        <v>0</v>
+      </c>
+      <c r="M652" t="n">
+        <v>2.6958454</v>
+      </c>
+      <c r="N652" t="n">
+        <v>38249</v>
+      </c>
+      <c r="P652" t="inlineStr"/>
+      <c r="Q652" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R652" t="inlineStr">
+        <is>
+          <t>6.5.0</t>
+        </is>
+      </c>
+      <c r="S652" t="inlineStr">
+        <is>
+          <t>Easily manage your Orange Mali line&lt;br&gt;● Manage your account and view all essential information, your offers, and your phone lines.&lt;br&gt;● Subscribe to call, SMS, Internet, and international call packages.&lt;br&gt;● Track your usage by checking your credit and Internet balance.&lt;br&gt;● Recharge your line by p</t>
+        </is>
+      </c>
+      <c r="T652" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U652" t="inlineStr"/>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G653" t="n">
+        <v>1494321079</v>
+      </c>
+      <c r="H653" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J653" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K653" t="n">
+        <v>0</v>
+      </c>
+      <c r="L653" t="b">
+        <v>1</v>
+      </c>
+      <c r="M653" t="n">
+        <v>2.51948</v>
+      </c>
+      <c r="N653" t="n">
+        <v>4745</v>
+      </c>
+      <c r="O653" t="n">
+        <v>12</v>
+      </c>
+      <c r="P653" t="inlineStr"/>
+      <c r="R653" t="inlineStr">
+        <is>
+          <t>6.5.2</t>
+        </is>
+      </c>
+      <c r="S653" t="inlineStr">
+        <is>
+          <t>Gérez facilement votre ligne Orange Mali 
+●        Gérez votre compte et consultez toutes les informations essentielles sur celui-ci, vos offres, ainsi que vos lignes téléphoniques.
+●        Souscrivez aux forfaits appels, SMS, Internet, et appels internationaux.
+●        Suivez votre consommation e</t>
+        </is>
+      </c>
+      <c r="T653" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U653" t="inlineStr"/>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G654" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.omg</t>
+        </is>
+      </c>
+      <c r="H654" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I654" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J654" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K654" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L654" t="b">
+        <v>0</v>
+      </c>
+      <c r="M654" t="n">
+        <v>4.151515</v>
+      </c>
+      <c r="N654" t="n">
+        <v>1375</v>
+      </c>
+      <c r="O654" t="n">
+        <v>51</v>
+      </c>
+      <c r="P654" t="inlineStr"/>
+      <c r="Q654" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R654" t="inlineStr">
+        <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="S654" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.&lt;br&gt;&lt;br&gt;Simplify Your Life with Max it&lt;br&gt;With Max It, ac</t>
+        </is>
+      </c>
+      <c r="T654" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U654" t="inlineStr"/>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G655" t="n">
+        <v>1295171817</v>
+      </c>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J655" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K655" t="n">
+        <v>0</v>
+      </c>
+      <c r="L655" t="b">
+        <v>1</v>
+      </c>
+      <c r="M655" t="n">
+        <v>3.08696</v>
+      </c>
+      <c r="N655" t="n">
+        <v>69</v>
+      </c>
+      <c r="O655" t="n">
+        <v>16</v>
+      </c>
+      <c r="P655" t="inlineStr"/>
+      <c r="R655" t="inlineStr">
+        <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="S655" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.
+Simplify Your Life with Max it
+With Max it, access a se</t>
+        </is>
+      </c>
+      <c r="T655" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U655" t="inlineStr"/>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G656" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.olr</t>
+        </is>
+      </c>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>Orange Max it - Liberia</t>
+        </is>
+      </c>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J656" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K656" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L656" t="b">
+        <v>0</v>
+      </c>
+      <c r="M656" t="n">
+        <v>4.5451612</v>
+      </c>
+      <c r="N656" t="n">
+        <v>3099</v>
+      </c>
+      <c r="O656" t="n">
+        <v>76</v>
+      </c>
+      <c r="P656" t="inlineStr"/>
+      <c r="Q656" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R656" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="S656" t="inlineStr">
+        <is>
+          <t>Max it: your personalized experience by Orange Liberia!&lt;br&gt;&lt;br&gt;Step into Max it, your all-in-one solution for telecom, marketplace, and financial services! Manage your mobile line, customize offers, pay your bills, keep&lt;br&gt;track of your usage with ease, and recharge your credit. Access exclusive eve</t>
+        </is>
+      </c>
+      <c r="T656" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U656" t="inlineStr"/>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G657" t="n">
+        <v>6746187327</v>
+      </c>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>Orange Max it – Liberia</t>
+        </is>
+      </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J657" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K657" t="n">
+        <v>0</v>
+      </c>
+      <c r="L657" t="b">
+        <v>1</v>
+      </c>
+      <c r="M657" t="n">
+        <v>4.0625</v>
+      </c>
+      <c r="N657" t="n">
+        <v>48</v>
+      </c>
+      <c r="P657" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "LR" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R657" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="S657" t="inlineStr">
+        <is>
+          <t>Max it is a free application, which allows Orange Liberia customers to:
+- Consult your account in real time: minutes, sms, internet
+- Top up your account or a friend account 
+- Buy  Bundles (voice, data, SMS, roaming, international)
+- Discover the latest offers and promotions 
+- Access to Orange se</t>
+        </is>
+      </c>
+      <c r="T657" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U657" t="inlineStr"/>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G658" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ojo</t>
+        </is>
+      </c>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J658" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K658" t="inlineStr">
+        <is>
+          <t>JOD 0.000</t>
+        </is>
+      </c>
+      <c r="L658" t="b">
+        <v>0</v>
+      </c>
+      <c r="M658" t="n">
+        <v>4.430946</v>
+      </c>
+      <c r="N658" t="n">
+        <v>97672</v>
+      </c>
+      <c r="O658" t="n">
+        <v>43</v>
+      </c>
+      <c r="P658" t="inlineStr"/>
+      <c r="Q658" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R658" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S658" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience&lt;br&gt;Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.&lt;br&gt;Important Update:&lt;br&gt;The jood app (jood Orange) w</t>
+        </is>
+      </c>
+      <c r="T658" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U658" t="inlineStr"/>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G659" t="n">
+        <v>808824590</v>
+      </c>
+      <c r="H659" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J659" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K659" t="n">
+        <v>0</v>
+      </c>
+      <c r="L659" t="b">
+        <v>1</v>
+      </c>
+      <c r="M659" t="n">
+        <v>4.21067</v>
+      </c>
+      <c r="N659" t="n">
+        <v>3019</v>
+      </c>
+      <c r="O659" t="n">
+        <v>44</v>
+      </c>
+      <c r="P659" t="inlineStr"/>
+      <c r="R659" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S659" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience
+Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.
+Important Update:
+The jood app (jood Orange) will be di</t>
+        </is>
+      </c>
+      <c r="T659" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U659" t="inlineStr"/>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G660" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.oci</t>
+        </is>
+      </c>
+      <c r="H660" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I660" t="inlineStr">
+        <is>
+          <t>Orange Côte d'Ivoire S.A</t>
+        </is>
+      </c>
+      <c r="J660" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K660" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L660" t="b">
+        <v>0</v>
+      </c>
+      <c r="M660" t="n">
+        <v>4.165109</v>
+      </c>
+      <c r="N660" t="n">
+        <v>67183</v>
+      </c>
+      <c r="O660" t="n">
+        <v>12</v>
+      </c>
+      <c r="P660" t="inlineStr"/>
+      <c r="Q660" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R660" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S660" t="inlineStr">
+        <is>
+          <t>Aaaahhh, ta super app Max it, n&amp;#39;a pas fini de te surprendre... &lt;br&gt;Est-ce que tu as remarqué ? Maintenant, tu as ton QR code personnalisé en haut de ton écran d&amp;#39;accueil ! Ainsi, tu peux :&lt;br&gt;     scanner le QR code de ton ami(e) pour lui faire un transfert d&amp;#39;&amp;#39;argent&lt;br&gt;     scanner l</t>
+        </is>
+      </c>
+      <c r="T660" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U660" t="inlineStr"/>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G661" t="n">
+        <v>1061120855</v>
+      </c>
+      <c r="H661" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>Orange CI</t>
+        </is>
+      </c>
+      <c r="J661" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K661" t="n">
+        <v>0</v>
+      </c>
+      <c r="L661" t="b">
+        <v>1</v>
+      </c>
+      <c r="M661" t="n">
+        <v>3.78636</v>
+      </c>
+      <c r="N661" t="n">
+        <v>5968</v>
+      </c>
+      <c r="O661" t="n">
+        <v>13</v>
+      </c>
+      <c r="P661" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R661" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S661" t="inlineStr">
+        <is>
+          <t>Max it, la super app all-in-one te fais gagner du temps, et diminue tes soucis... Gagne plus d'espace de stockage sur ton téléphone ; plus besoin de cumuler plusieurs appli d'Orange pour avoir accès à un maximum de services. Max it est là ! Gère ta ligne (SIM) au niveau des pass, des soldes, réalise</t>
+        </is>
+      </c>
+      <c r="T661" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U661" t="inlineStr"/>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogw</t>
+        </is>
+      </c>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J662" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K662" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L662" t="b">
+        <v>0</v>
+      </c>
+      <c r="M662" t="n">
+        <v>4.350993</v>
+      </c>
+      <c r="N662" t="n">
+        <v>1533</v>
+      </c>
+      <c r="O662" t="n">
+        <v>4</v>
+      </c>
+      <c r="P662" t="inlineStr"/>
+      <c r="Q662" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R662" t="inlineStr">
+        <is>
+          <t>4.0.18</t>
+        </is>
+      </c>
+      <c r="S662" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T662" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U662" t="inlineStr"/>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G663" t="n">
+        <v>1574668652</v>
+      </c>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J663" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K663" t="n">
+        <v>0</v>
+      </c>
+      <c r="L663" t="b">
+        <v>1</v>
+      </c>
+      <c r="M663" t="n">
+        <v>4.05333</v>
+      </c>
+      <c r="N663" t="n">
+        <v>75</v>
+      </c>
+      <c r="O663" t="n">
+        <v>18</v>
+      </c>
+      <c r="P663" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R663" t="inlineStr">
+        <is>
+          <t>6.0.35</t>
+        </is>
+      </c>
+      <c r="S663" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T663" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U663" t="inlineStr"/>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G664" t="inlineStr">
+        <is>
+          <t>com.orange.sugu.ocd</t>
+        </is>
+      </c>
+      <c r="H664" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J664" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K664" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L664" t="b">
+        <v>0</v>
+      </c>
+      <c r="M664" t="n">
+        <v>4.1257033</v>
+      </c>
+      <c r="N664" t="n">
+        <v>5298</v>
+      </c>
+      <c r="O664" t="n">
+        <v>64</v>
+      </c>
+      <c r="P664" t="inlineStr"/>
+      <c r="Q664" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R664" t="inlineStr">
+        <is>
+          <t>9.0.12</t>
+        </is>
+      </c>
+      <c r="S664" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DRC that brings together the features of MyOrange, and Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Plans, Mobile Payments, money transfers, bill payments, subscriptions, and entertai</t>
+        </is>
+      </c>
+      <c r="T664" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U664" t="inlineStr"/>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G665" t="n">
+        <v>6447896435</v>
+      </c>
+      <c r="H665" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J665" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K665" t="n">
+        <v>0</v>
+      </c>
+      <c r="L665" t="b">
+        <v>1</v>
+      </c>
+      <c r="M665" t="n">
+        <v>3.55762</v>
+      </c>
+      <c r="N665" t="n">
+        <v>269</v>
+      </c>
+      <c r="P665" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "CD" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R665" t="inlineStr">
+        <is>
+          <t>9.0.6</t>
+        </is>
+      </c>
+      <c r="S665" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DR Congo. It brings together the features of Orange et Moi, as well as Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Packages, Mobile payment, money transfers, bill payment and subscri</t>
+        </is>
+      </c>
+      <c r="T665" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U665" t="inlineStr"/>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G666" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ocm</t>
+        </is>
+      </c>
+      <c r="H666" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroon</t>
+        </is>
+      </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>Orange MEA</t>
+        </is>
+      </c>
+      <c r="J666" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K666" t="inlineStr">
+        <is>
+          <t>FCFA 0</t>
+        </is>
+      </c>
+      <c r="L666" t="b">
+        <v>0</v>
+      </c>
+      <c r="M666" t="n">
+        <v>3.9292653</v>
+      </c>
+      <c r="N666" t="n">
+        <v>46914</v>
+      </c>
+      <c r="O666" t="n">
+        <v>10</v>
+      </c>
+      <c r="P666" t="inlineStr"/>
+      <c r="Q666" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R666" t="inlineStr">
+        <is>
+          <t>7.0.23</t>
+        </is>
+      </c>
+      <c r="S666" t="inlineStr">
+        <is>
+          <t>Max it brings together everything that matters to you in one app: managing your lines, money transfer, bill payment, exclusive offers, and a universe of lifestyle and entertainment. Simple, fast, and 100% secure..&lt;br&gt;&lt;br&gt;📞 My line&lt;br&gt;Manage your Orange mobile and landline bundles in a single click:</t>
+        </is>
+      </c>
+      <c r="T666" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U666" t="inlineStr"/>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G667" t="n">
+        <v>1116920093</v>
+      </c>
+      <c r="H667" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroun</t>
+        </is>
+      </c>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>Orange Middle East &amp; Africa</t>
+        </is>
+      </c>
+      <c r="J667" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K667" t="n">
+        <v>0</v>
+      </c>
+      <c r="L667" t="b">
+        <v>1</v>
+      </c>
+      <c r="M667" t="n">
+        <v>3.76843</v>
+      </c>
+      <c r="N667" t="n">
+        <v>16155</v>
+      </c>
+      <c r="O667" t="n">
+        <v>1</v>
+      </c>
+      <c r="P667" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R667" t="inlineStr">
+        <is>
+          <t>7.0.24</t>
+        </is>
+      </c>
+      <c r="S667" t="inlineStr">
+        <is>
+          <t>Avec Max it, Orange rassemble tout ce qui compte pour vous dans une même application : la gestion de vos lignes, les transferts d’argent, payement de vos factures, des offres exclusives et un univers lifestyle et divertissement.
+Simple, rapide et 100 % sécurisée.
+Ma ligne
+Gérez vos forfaits mobiles</t>
+        </is>
+      </c>
+      <c r="T667" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U667" t="inlineStr"/>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G668" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obf</t>
+        </is>
+      </c>
+      <c r="H668" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso</t>
+        </is>
+      </c>
+      <c r="J668" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K668" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L668" t="b">
+        <v>0</v>
+      </c>
+      <c r="M668" t="n">
+        <v>4.139608</v>
+      </c>
+      <c r="N668" t="n">
+        <v>25475</v>
+      </c>
+      <c r="O668" t="n">
+        <v>9</v>
+      </c>
+      <c r="P668" t="inlineStr"/>
+      <c r="Q668" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R668" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S668" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.&lt;br&gt;Gérez vos lignes mobiles, effectuez des transferts d&amp;#39;argent sécurisés, réglez vos factures, profitez d&amp;#39;offres exclusives, effectuez des paiements marchands fiables, et bien plus enco</t>
+        </is>
+      </c>
+      <c r="T668" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U668" t="inlineStr"/>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G669" t="n">
+        <v>1553774707</v>
+      </c>
+      <c r="H669" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso SA</t>
+        </is>
+      </c>
+      <c r="J669" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K669" t="n">
+        <v>0</v>
+      </c>
+      <c r="L669" t="b">
+        <v>1</v>
+      </c>
+      <c r="M669" t="n">
+        <v>3.45377</v>
+      </c>
+      <c r="N669" t="n">
+        <v>1179</v>
+      </c>
+      <c r="O669" t="n">
+        <v>6</v>
+      </c>
+      <c r="P669" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R669" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S669" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.
+Gérez vos lignes mobiles, effectuez des transferts d'argent sécurisés, réglez vos factures, profitez d'offres exclusives, effectuez des paiements marchands fiables, et bien plus encore, le tout</t>
+        </is>
+      </c>
+      <c r="T669" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U669" t="inlineStr"/>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G670" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obw</t>
+        </is>
+      </c>
+      <c r="H670" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J670" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K670" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L670" t="b">
+        <v>0</v>
+      </c>
+      <c r="M670" t="n">
+        <v>3.9782608</v>
+      </c>
+      <c r="N670" t="n">
+        <v>2964</v>
+      </c>
+      <c r="O670" t="n">
+        <v>29</v>
+      </c>
+      <c r="P670" t="inlineStr"/>
+      <c r="Q670" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R670" t="inlineStr">
+        <is>
+          <t>7.3.8</t>
+        </is>
+      </c>
+      <c r="S670" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it, the brand-new Orange Botswana Super App that follows Yame and gives you access to four distinct universes for a one-of-a-kind experience!&lt;br&gt;&lt;br&gt;Manage your accounts, make quick payments using QR codes, investigate a range of online goods and services, and discover the many options provided </t>
+        </is>
+      </c>
+      <c r="T670" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U670" t="inlineStr"/>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G671" t="n">
+        <v>1195839458</v>
+      </c>
+      <c r="H671" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J671" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K671" t="n">
+        <v>0</v>
+      </c>
+      <c r="L671" t="b">
+        <v>1</v>
+      </c>
+      <c r="M671" t="n">
+        <v>3.00806</v>
+      </c>
+      <c r="N671" t="n">
+        <v>124</v>
+      </c>
+      <c r="O671" t="n">
+        <v>28</v>
+      </c>
+      <c r="P671" t="inlineStr"/>
+      <c r="R671" t="inlineStr">
+        <is>
+          <t>7.3.1</t>
+        </is>
+      </c>
+      <c r="S671" t="inlineStr">
+        <is>
+          <t>A free mobile self-care application for Orange Botswana’s mobile customers.
+Full Description :
+Max it is a free application, which allows Orange Botswana customers to:
+- Consult your account in real time: minutes, sms, internet ...
+- Top up your account or a friend account  with Orange Money
+-</t>
+        </is>
+      </c>
+      <c r="T671" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U671" t="inlineStr"/>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G672" t="inlineStr">
+        <is>
+          <t>com.orange.mobinilandme</t>
+        </is>
+      </c>
+      <c r="H672" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I672" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J672" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K672" t="inlineStr">
+        <is>
+          <t>EGP 0.00</t>
+        </is>
+      </c>
+      <c r="L672" t="b">
+        <v>0</v>
+      </c>
+      <c r="M672" t="n">
+        <v>4.5593715</v>
+      </c>
+      <c r="N672" t="n">
+        <v>928443</v>
+      </c>
+      <c r="O672" t="n">
+        <v>19</v>
+      </c>
+      <c r="P672" t="inlineStr"/>
+      <c r="Q672" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R672" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S672" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion&lt;br&gt;Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.&lt;br&gt;Key services include:&lt;br&gt;• Account Management: Easily manage</t>
+        </is>
+      </c>
+      <c r="T672" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U672" t="inlineStr"/>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>d445bac1-444e-4fc1-98b6-726b017b168e</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>2026-07-28 06:28:21</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G673" t="n">
+        <v>942568333</v>
+      </c>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I673" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J673" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K673" t="n">
+        <v>0</v>
+      </c>
+      <c r="L673" t="b">
+        <v>1</v>
+      </c>
+      <c r="M673" t="n">
+        <v>4.25202</v>
+      </c>
+      <c r="N673" t="n">
+        <v>117563</v>
+      </c>
+      <c r="O673" t="n">
+        <v>55</v>
+      </c>
+      <c r="P673" t="inlineStr"/>
+      <c r="R673" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S673" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion
+Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.
+Key services include:
+• Account Management: Easily manage your Ora</t>
+        </is>
+      </c>
+      <c r="T673" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U673" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-07-29
</commit_message>
<xml_diff>
--- a/maxit_store_history.xlsx
+++ b/maxit_store_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U673"/>
+  <dimension ref="A1:U705"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55177,7 +55177,6 @@
       <c r="O642" t="n">
         <v>20</v>
       </c>
-      <c r="P642" t="inlineStr"/>
       <c r="Q642" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -55198,7 +55197,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U642" t="inlineStr"/>
     </row>
     <row r="643">
       <c r="A643" t="inlineStr">
@@ -55261,7 +55259,6 @@
       <c r="N643" t="n">
         <v>322</v>
       </c>
-      <c r="P643" t="inlineStr"/>
       <c r="R643" t="inlineStr">
         <is>
           <t>6.4.8</t>
@@ -55277,7 +55274,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U643" t="inlineStr"/>
     </row>
     <row r="644">
       <c r="A644" t="inlineStr">
@@ -55347,7 +55343,6 @@
       <c r="O644" t="n">
         <v>28</v>
       </c>
-      <c r="P644" t="inlineStr"/>
       <c r="Q644" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -55368,7 +55363,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U644" t="inlineStr"/>
     </row>
     <row r="645">
       <c r="A645" t="inlineStr">
@@ -55434,7 +55428,6 @@
       <c r="O645" t="n">
         <v>35</v>
       </c>
-      <c r="P645" t="inlineStr"/>
       <c r="R645" t="inlineStr">
         <is>
           <t>10.0.6</t>
@@ -55452,7 +55445,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U645" t="inlineStr"/>
     </row>
     <row r="646">
       <c r="A646" t="inlineStr">
@@ -55522,7 +55514,6 @@
       <c r="O646" t="n">
         <v>9</v>
       </c>
-      <c r="P646" t="inlineStr"/>
       <c r="Q646" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -55543,7 +55534,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U646" t="inlineStr"/>
     </row>
     <row r="647">
       <c r="A647" t="inlineStr">
@@ -55632,7 +55622,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U647" t="inlineStr"/>
     </row>
     <row r="648">
       <c r="A648" t="inlineStr">
@@ -55702,7 +55691,6 @@
       <c r="O648" t="n">
         <v>13</v>
       </c>
-      <c r="P648" t="inlineStr"/>
       <c r="Q648" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -55723,7 +55711,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U648" t="inlineStr"/>
     </row>
     <row r="649">
       <c r="A649" t="inlineStr">
@@ -55789,7 +55776,6 @@
       <c r="O649" t="n">
         <v>4</v>
       </c>
-      <c r="P649" t="inlineStr"/>
       <c r="R649" t="inlineStr">
         <is>
           <t>21.1.0</t>
@@ -55807,7 +55793,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U649" t="inlineStr"/>
     </row>
     <row r="650">
       <c r="A650" t="inlineStr">
@@ -55877,7 +55862,6 @@
       <c r="O650" t="n">
         <v>77</v>
       </c>
-      <c r="P650" t="inlineStr"/>
       <c r="Q650" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -55898,7 +55882,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U650" t="inlineStr"/>
     </row>
     <row r="651">
       <c r="A651" t="inlineStr">
@@ -55983,7 +55966,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U651" t="inlineStr"/>
     </row>
     <row r="652">
       <c r="A652" t="inlineStr">
@@ -56050,7 +56032,6 @@
       <c r="N652" t="n">
         <v>38249</v>
       </c>
-      <c r="P652" t="inlineStr"/>
       <c r="Q652" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -56071,7 +56052,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U652" t="inlineStr"/>
     </row>
     <row r="653">
       <c r="A653" t="inlineStr">
@@ -56137,7 +56117,6 @@
       <c r="O653" t="n">
         <v>12</v>
       </c>
-      <c r="P653" t="inlineStr"/>
       <c r="R653" t="inlineStr">
         <is>
           <t>6.5.2</t>
@@ -56156,7 +56135,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U653" t="inlineStr"/>
     </row>
     <row r="654">
       <c r="A654" t="inlineStr">
@@ -56226,7 +56204,6 @@
       <c r="O654" t="n">
         <v>51</v>
       </c>
-      <c r="P654" t="inlineStr"/>
       <c r="Q654" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -56247,7 +56224,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U654" t="inlineStr"/>
     </row>
     <row r="655">
       <c r="A655" t="inlineStr">
@@ -56313,7 +56289,6 @@
       <c r="O655" t="n">
         <v>16</v>
       </c>
-      <c r="P655" t="inlineStr"/>
       <c r="R655" t="inlineStr">
         <is>
           <t>5.0.2</t>
@@ -56331,7 +56306,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U655" t="inlineStr"/>
     </row>
     <row r="656">
       <c r="A656" t="inlineStr">
@@ -56401,7 +56375,6 @@
       <c r="O656" t="n">
         <v>76</v>
       </c>
-      <c r="P656" t="inlineStr"/>
       <c r="Q656" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -56422,7 +56395,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U656" t="inlineStr"/>
     </row>
     <row r="657">
       <c r="A657" t="inlineStr">
@@ -56510,7 +56482,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U657" t="inlineStr"/>
     </row>
     <row r="658">
       <c r="A658" t="inlineStr">
@@ -56580,7 +56551,6 @@
       <c r="O658" t="n">
         <v>43</v>
       </c>
-      <c r="P658" t="inlineStr"/>
       <c r="Q658" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -56601,7 +56571,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U658" t="inlineStr"/>
     </row>
     <row r="659">
       <c r="A659" t="inlineStr">
@@ -56667,7 +56636,6 @@
       <c r="O659" t="n">
         <v>44</v>
       </c>
-      <c r="P659" t="inlineStr"/>
       <c r="R659" t="inlineStr">
         <is>
           <t>10.0.21</t>
@@ -56686,7 +56654,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U659" t="inlineStr"/>
     </row>
     <row r="660">
       <c r="A660" t="inlineStr">
@@ -56756,7 +56723,6 @@
       <c r="O660" t="n">
         <v>12</v>
       </c>
-      <c r="P660" t="inlineStr"/>
       <c r="Q660" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -56777,7 +56743,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U660" t="inlineStr"/>
     </row>
     <row r="661">
       <c r="A661" t="inlineStr">
@@ -56863,7 +56828,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U661" t="inlineStr"/>
     </row>
     <row r="662">
       <c r="A662" t="inlineStr">
@@ -56933,7 +56897,6 @@
       <c r="O662" t="n">
         <v>4</v>
       </c>
-      <c r="P662" t="inlineStr"/>
       <c r="Q662" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -56954,7 +56917,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U662" t="inlineStr"/>
     </row>
     <row r="663">
       <c r="A663" t="inlineStr">
@@ -57040,7 +57002,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U663" t="inlineStr"/>
     </row>
     <row r="664">
       <c r="A664" t="inlineStr">
@@ -57110,7 +57071,6 @@
       <c r="O664" t="n">
         <v>64</v>
       </c>
-      <c r="P664" t="inlineStr"/>
       <c r="Q664" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -57131,7 +57091,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U664" t="inlineStr"/>
     </row>
     <row r="665">
       <c r="A665" t="inlineStr">
@@ -57214,7 +57173,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U665" t="inlineStr"/>
     </row>
     <row r="666">
       <c r="A666" t="inlineStr">
@@ -57284,7 +57242,6 @@
       <c r="O666" t="n">
         <v>10</v>
       </c>
-      <c r="P666" t="inlineStr"/>
       <c r="Q666" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -57305,7 +57262,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U666" t="inlineStr"/>
     </row>
     <row r="667">
       <c r="A667" t="inlineStr">
@@ -57394,7 +57350,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U667" t="inlineStr"/>
     </row>
     <row r="668">
       <c r="A668" t="inlineStr">
@@ -57464,7 +57419,6 @@
       <c r="O668" t="n">
         <v>9</v>
       </c>
-      <c r="P668" t="inlineStr"/>
       <c r="Q668" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -57485,7 +57439,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U668" t="inlineStr"/>
     </row>
     <row r="669">
       <c r="A669" t="inlineStr">
@@ -57572,7 +57525,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U669" t="inlineStr"/>
     </row>
     <row r="670">
       <c r="A670" t="inlineStr">
@@ -57642,7 +57594,6 @@
       <c r="O670" t="n">
         <v>29</v>
       </c>
-      <c r="P670" t="inlineStr"/>
       <c r="Q670" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -57663,7 +57614,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U670" t="inlineStr"/>
     </row>
     <row r="671">
       <c r="A671" t="inlineStr">
@@ -57729,7 +57679,6 @@
       <c r="O671" t="n">
         <v>28</v>
       </c>
-      <c r="P671" t="inlineStr"/>
       <c r="R671" t="inlineStr">
         <is>
           <t>7.3.1</t>
@@ -57750,7 +57699,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U671" t="inlineStr"/>
     </row>
     <row r="672">
       <c r="A672" t="inlineStr">
@@ -57820,7 +57768,6 @@
       <c r="O672" t="n">
         <v>19</v>
       </c>
-      <c r="P672" t="inlineStr"/>
       <c r="Q672" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -57841,7 +57788,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U672" t="inlineStr"/>
     </row>
     <row r="673">
       <c r="A673" t="inlineStr">
@@ -57907,7 +57853,6 @@
       <c r="O673" t="n">
         <v>55</v>
       </c>
-      <c r="P673" t="inlineStr"/>
       <c r="R673" t="inlineStr">
         <is>
           <t>10.1.0</t>
@@ -57926,7 +57871,2825 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U673" t="inlineStr"/>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G674" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogn</t>
+        </is>
+      </c>
+      <c r="H674" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J674" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K674" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L674" t="b">
+        <v>0</v>
+      </c>
+      <c r="M674" t="n">
+        <v>4.45733</v>
+      </c>
+      <c r="N674" t="n">
+        <v>9296</v>
+      </c>
+      <c r="O674" t="n">
+        <v>28</v>
+      </c>
+      <c r="P674" t="inlineStr"/>
+      <c r="Q674" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R674" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S674" t="inlineStr">
+        <is>
+          <t>Bien plus qu&amp;#39;une application, un véritable assistant personnel pour une vie connectée et simplifiée.&lt;br&gt;Suivi de consommation: Votre tableau de bord tout-en-un pour une gestion simplifiée !&lt;br&gt;- Gestion de votre offre: Accédez à une vue détaillée de votre offre actuelle et de vos forfaits Orange</t>
+        </is>
+      </c>
+      <c r="T674" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U674" t="inlineStr"/>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G675" t="n">
+        <v>1177999485</v>
+      </c>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J675" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K675" t="n">
+        <v>0</v>
+      </c>
+      <c r="L675" t="b">
+        <v>1</v>
+      </c>
+      <c r="M675" t="n">
+        <v>3.88272</v>
+      </c>
+      <c r="N675" t="n">
+        <v>324</v>
+      </c>
+      <c r="P675" t="inlineStr"/>
+      <c r="R675" t="inlineStr">
+        <is>
+          <t>6.4.8</t>
+        </is>
+      </c>
+      <c r="S675" t="inlineStr">
+        <is>
+          <t>La fusion d’Orange et Moi et Orange Money donne naissance à Max it, la nouvelle Super Application Tout-en-Un. Profitez du suivi de consommation, de paiements mobiles, de toutes les fonctionnalités Orange et Moi et Money avec un large éventail de divertissements, le tout regroupé en un seul endroit !</t>
+        </is>
+      </c>
+      <c r="T675" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U675" t="inlineStr"/>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G676" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.otn</t>
+        </is>
+      </c>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J676" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K676" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L676" t="b">
+        <v>0</v>
+      </c>
+      <c r="M676" t="n">
+        <v>3.967694</v>
+      </c>
+      <c r="N676" t="n">
+        <v>35377</v>
+      </c>
+      <c r="O676" t="n">
+        <v>28</v>
+      </c>
+      <c r="P676" t="inlineStr"/>
+      <c r="Q676" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R676" t="inlineStr">
+        <is>
+          <t>10.0.6</t>
+        </is>
+      </c>
+      <c r="S676" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Max it par Orange Tunisie facilite votre vie au quotidien !&lt;/h2&gt;&lt;br&gt;&lt;br&gt;Welcome sur Max it !&lt;br&gt;Accédez rapidement à vos fonctionnalités Max it préférées et profitez également de contenus exclusifs, d’activités divertissantes, et de jeux interactifs pour une expérience enrichissante avec la roue</t>
+        </is>
+      </c>
+      <c r="T676" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U676" t="inlineStr"/>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G677" t="n">
+        <v>1146892088</v>
+      </c>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J677" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K677" t="n">
+        <v>0</v>
+      </c>
+      <c r="L677" t="b">
+        <v>1</v>
+      </c>
+      <c r="M677" t="n">
+        <v>3.03049</v>
+      </c>
+      <c r="N677" t="n">
+        <v>1640</v>
+      </c>
+      <c r="O677" t="n">
+        <v>45</v>
+      </c>
+      <c r="P677" t="inlineStr"/>
+      <c r="R677" t="inlineStr">
+        <is>
+          <t>10.0.6</t>
+        </is>
+      </c>
+      <c r="S677" t="inlineStr">
+        <is>
+          <t>Max it by Orange Tunisie : Votre appli incontournable pour une vie connectée
+Welcome sur Max it : Découvrez fonctionnalités, jeux &amp; contenus de divertissement by Orange Tunisie !
+Trouvez vite vos fonctionnalités Max it favorites et explorez des contenus exclusifs et des jeux pour une expérience im</t>
+        </is>
+      </c>
+      <c r="T677" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U677" t="inlineStr"/>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G678" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osl</t>
+        </is>
+      </c>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J678" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K678" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L678" t="b">
+        <v>0</v>
+      </c>
+      <c r="M678" t="n">
+        <v>4.361991</v>
+      </c>
+      <c r="N678" t="n">
+        <v>2131</v>
+      </c>
+      <c r="O678" t="n">
+        <v>10</v>
+      </c>
+      <c r="P678" t="inlineStr"/>
+      <c r="Q678" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R678" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S678" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it is a free application, which allows Orange Sierra Leone prepaid and postpaid customers to:&lt;br&gt;&lt;br&gt;- Consult your account in real time: minutes, sms, internet&lt;br&gt;- Top up your account or a friend account &lt;br&gt;- Buy Internet Bundles&lt;br&gt;- Discover the latest offers and promotions &lt;br&gt;- Access to </t>
+        </is>
+      </c>
+      <c r="T678" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U678" t="inlineStr"/>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G679" t="n">
+        <v>6443607903</v>
+      </c>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J679" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K679" t="n">
+        <v>0</v>
+      </c>
+      <c r="L679" t="b">
+        <v>1</v>
+      </c>
+      <c r="M679" t="n">
+        <v>3.69948</v>
+      </c>
+      <c r="N679" t="n">
+        <v>193</v>
+      </c>
+      <c r="O679" t="n">
+        <v>9</v>
+      </c>
+      <c r="P679" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R679" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S679" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The merger of My Orange &amp; Orange Money has given birth to Max it the all-in-one super app, a free application which allows all Orange Sierra Leone customers to 
+Track calls, SMS, and Data usage and monitor balance. 
+Make a secure mobile/Orange Money payment.
+Easily transfer credit to other users </t>
+        </is>
+      </c>
+      <c r="T679" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U679" t="inlineStr"/>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G680" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osn</t>
+        </is>
+      </c>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>Orange Sénégal</t>
+        </is>
+      </c>
+      <c r="J680" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K680" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L680" t="b">
+        <v>0</v>
+      </c>
+      <c r="M680" t="n">
+        <v>4.3002076</v>
+      </c>
+      <c r="N680" t="n">
+        <v>51247</v>
+      </c>
+      <c r="O680" t="n">
+        <v>11</v>
+      </c>
+      <c r="P680" t="inlineStr"/>
+      <c r="Q680" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R680" t="inlineStr">
+        <is>
+          <t>22.0.0</t>
+        </is>
+      </c>
+      <c r="S680" t="inlineStr">
+        <is>
+          <t>Lu bees ak Max it ! &lt;br&gt;Une application repensée pour être plus simple, plus rapide et adaptée à vos besoins. Une expérience optimisée pour faciliter vos usages au quotidien, avec des parcours simplifiés et un accès plus fluide à vos services. Que vous soyez client Orange ou non, Max it vous accompa</t>
+        </is>
+      </c>
+      <c r="T680" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U680" t="inlineStr"/>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G681" t="n">
+        <v>1039327980</v>
+      </c>
+      <c r="H681" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>Orange Senegal</t>
+        </is>
+      </c>
+      <c r="J681" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K681" t="n">
+        <v>0</v>
+      </c>
+      <c r="L681" t="b">
+        <v>1</v>
+      </c>
+      <c r="M681" t="n">
+        <v>4.16941</v>
+      </c>
+      <c r="N681" t="n">
+        <v>30223</v>
+      </c>
+      <c r="O681" t="n">
+        <v>3</v>
+      </c>
+      <c r="P681" t="inlineStr"/>
+      <c r="R681" t="inlineStr">
+        <is>
+          <t>22.0.0</t>
+        </is>
+      </c>
+      <c r="S681" t="inlineStr">
+        <is>
+          <t>Here is the English translation:
+Welcome to Max it!
+A redesigned app to be simpler, faster, and tailored to your needs. An optimized experience to make your daily life easier, with streamlined journeys and smoother access to your services. Whether you are an Orange customer or not, Max it is your e</t>
+        </is>
+      </c>
+      <c r="T681" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U681" t="inlineStr"/>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G682" t="inlineStr">
+        <is>
+          <t>com.orange.meditel.mediteletmoi</t>
+        </is>
+      </c>
+      <c r="H682" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>Orange Maroc</t>
+        </is>
+      </c>
+      <c r="J682" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K682" t="inlineStr">
+        <is>
+          <t>MAD 0.00</t>
+        </is>
+      </c>
+      <c r="L682" t="b">
+        <v>0</v>
+      </c>
+      <c r="M682" t="n">
+        <v>3.7189627</v>
+      </c>
+      <c r="N682" t="n">
+        <v>110915</v>
+      </c>
+      <c r="O682" t="n">
+        <v>110</v>
+      </c>
+      <c r="P682" t="inlineStr"/>
+      <c r="Q682" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R682" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S682" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l&amp;#39;expérience mobile réinventé&lt;br&gt;&lt;br&gt;Max it, c&amp;#39;est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d&amp;#39;une multitude de services exclusifs. &lt;br&gt;&lt;br&gt;Créez votre espace sur</t>
+        </is>
+      </c>
+      <c r="T682" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U682" t="inlineStr"/>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G683" t="n">
+        <v>596028698</v>
+      </c>
+      <c r="H683" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I683" t="inlineStr">
+        <is>
+          <t>Méditel</t>
+        </is>
+      </c>
+      <c r="J683" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K683" t="n">
+        <v>0</v>
+      </c>
+      <c r="L683" t="b">
+        <v>1</v>
+      </c>
+      <c r="M683" t="n">
+        <v>3.94557</v>
+      </c>
+      <c r="N683" t="n">
+        <v>2756</v>
+      </c>
+      <c r="P683" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "MA" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R683" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S683" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l'expérience mobile réinventé
+Max it, c'est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d'une multitude de services exclusifs. 
+Créez votre espace sur mesure et bénéficiez d'</t>
+        </is>
+      </c>
+      <c r="T683" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U683" t="inlineStr"/>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>com.oml.dsi.orangemobile</t>
+        </is>
+      </c>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J684" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K684" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L684" t="b">
+        <v>0</v>
+      </c>
+      <c r="M684" t="n">
+        <v>2.6958454</v>
+      </c>
+      <c r="N684" t="n">
+        <v>38249</v>
+      </c>
+      <c r="P684" t="inlineStr"/>
+      <c r="Q684" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R684" t="inlineStr">
+        <is>
+          <t>6.5.0</t>
+        </is>
+      </c>
+      <c r="S684" t="inlineStr">
+        <is>
+          <t>Easily manage your Orange Mali line&lt;br&gt;● Manage your account and view all essential information, your offers, and your phone lines.&lt;br&gt;● Subscribe to call, SMS, Internet, and international call packages.&lt;br&gt;● Track your usage by checking your credit and Internet balance.&lt;br&gt;● Recharge your line by p</t>
+        </is>
+      </c>
+      <c r="T684" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U684" t="inlineStr"/>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G685" t="n">
+        <v>1494321079</v>
+      </c>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J685" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K685" t="n">
+        <v>0</v>
+      </c>
+      <c r="L685" t="b">
+        <v>1</v>
+      </c>
+      <c r="M685" t="n">
+        <v>2.52147</v>
+      </c>
+      <c r="N685" t="n">
+        <v>4750</v>
+      </c>
+      <c r="O685" t="n">
+        <v>14</v>
+      </c>
+      <c r="P685" t="inlineStr"/>
+      <c r="R685" t="inlineStr">
+        <is>
+          <t>6.5.2</t>
+        </is>
+      </c>
+      <c r="S685" t="inlineStr">
+        <is>
+          <t>Gérez facilement votre ligne Orange Mali 
+●        Gérez votre compte et consultez toutes les informations essentielles sur celui-ci, vos offres, ainsi que vos lignes téléphoniques.
+●        Souscrivez aux forfaits appels, SMS, Internet, et appels internationaux.
+●        Suivez votre consommation e</t>
+        </is>
+      </c>
+      <c r="T685" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U685" t="inlineStr"/>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G686" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.omg</t>
+        </is>
+      </c>
+      <c r="H686" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J686" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K686" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L686" t="b">
+        <v>0</v>
+      </c>
+      <c r="M686" t="n">
+        <v>4.145038</v>
+      </c>
+      <c r="N686" t="n">
+        <v>1374</v>
+      </c>
+      <c r="O686" t="n">
+        <v>53</v>
+      </c>
+      <c r="P686" t="inlineStr"/>
+      <c r="Q686" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R686" t="inlineStr">
+        <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="S686" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.&lt;br&gt;&lt;br&gt;Simplify Your Life with Max it&lt;br&gt;With Max It, ac</t>
+        </is>
+      </c>
+      <c r="T686" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U686" t="inlineStr"/>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G687" t="n">
+        <v>1295171817</v>
+      </c>
+      <c r="H687" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I687" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J687" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K687" t="n">
+        <v>0</v>
+      </c>
+      <c r="L687" t="b">
+        <v>1</v>
+      </c>
+      <c r="M687" t="n">
+        <v>3.08696</v>
+      </c>
+      <c r="N687" t="n">
+        <v>69</v>
+      </c>
+      <c r="O687" t="n">
+        <v>19</v>
+      </c>
+      <c r="P687" t="inlineStr"/>
+      <c r="R687" t="inlineStr">
+        <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="S687" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.
+Simplify Your Life with Max it
+With Max it, access a se</t>
+        </is>
+      </c>
+      <c r="T687" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U687" t="inlineStr"/>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G688" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.olr</t>
+        </is>
+      </c>
+      <c r="H688" t="inlineStr">
+        <is>
+          <t>Orange Max it - Liberia</t>
+        </is>
+      </c>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J688" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K688" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L688" t="b">
+        <v>0</v>
+      </c>
+      <c r="M688" t="n">
+        <v>4.5451612</v>
+      </c>
+      <c r="N688" t="n">
+        <v>3099</v>
+      </c>
+      <c r="O688" t="n">
+        <v>94</v>
+      </c>
+      <c r="P688" t="inlineStr"/>
+      <c r="Q688" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R688" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="S688" t="inlineStr">
+        <is>
+          <t>Max it: your personalized experience by Orange Liberia!&lt;br&gt;&lt;br&gt;Step into Max it, your all-in-one solution for telecom, marketplace, and financial services! Manage your mobile line, customize offers, pay your bills, keep&lt;br&gt;track of your usage with ease, and recharge your credit. Access exclusive eve</t>
+        </is>
+      </c>
+      <c r="T688" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U688" t="inlineStr"/>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G689" t="n">
+        <v>6746187327</v>
+      </c>
+      <c r="H689" t="inlineStr">
+        <is>
+          <t>Orange Max it – Liberia</t>
+        </is>
+      </c>
+      <c r="I689" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J689" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K689" t="n">
+        <v>0</v>
+      </c>
+      <c r="L689" t="b">
+        <v>1</v>
+      </c>
+      <c r="M689" t="n">
+        <v>4.0625</v>
+      </c>
+      <c r="N689" t="n">
+        <v>48</v>
+      </c>
+      <c r="P689" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "LR" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R689" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="S689" t="inlineStr">
+        <is>
+          <t>Max it is a free application, which allows Orange Liberia customers to:
+- Consult your account in real time: minutes, sms, internet
+- Top up your account or a friend account 
+- Buy  Bundles (voice, data, SMS, roaming, international)
+- Discover the latest offers and promotions 
+- Access to Orange se</t>
+        </is>
+      </c>
+      <c r="T689" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U689" t="inlineStr"/>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G690" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ojo</t>
+        </is>
+      </c>
+      <c r="H690" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J690" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K690" t="inlineStr">
+        <is>
+          <t>JOD 0.000</t>
+        </is>
+      </c>
+      <c r="L690" t="b">
+        <v>0</v>
+      </c>
+      <c r="M690" t="n">
+        <v>4.4316044</v>
+      </c>
+      <c r="N690" t="n">
+        <v>97715</v>
+      </c>
+      <c r="O690" t="n">
+        <v>46</v>
+      </c>
+      <c r="P690" t="inlineStr"/>
+      <c r="Q690" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R690" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S690" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience&lt;br&gt;Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.&lt;br&gt;Important Update:&lt;br&gt;The jood app (jood Orange) w</t>
+        </is>
+      </c>
+      <c r="T690" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U690" t="inlineStr"/>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G691" t="n">
+        <v>808824590</v>
+      </c>
+      <c r="H691" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I691" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J691" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K691" t="n">
+        <v>0</v>
+      </c>
+      <c r="L691" t="b">
+        <v>1</v>
+      </c>
+      <c r="M691" t="n">
+        <v>4.21157</v>
+      </c>
+      <c r="N691" t="n">
+        <v>3025</v>
+      </c>
+      <c r="O691" t="n">
+        <v>42</v>
+      </c>
+      <c r="P691" t="inlineStr"/>
+      <c r="R691" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S691" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience
+Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.
+Important Update:
+The jood app (jood Orange) will be di</t>
+        </is>
+      </c>
+      <c r="T691" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U691" t="inlineStr"/>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F692" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G692" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.oci</t>
+        </is>
+      </c>
+      <c r="H692" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I692" t="inlineStr">
+        <is>
+          <t>Orange Côte d'Ivoire S.A</t>
+        </is>
+      </c>
+      <c r="J692" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K692" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L692" t="b">
+        <v>0</v>
+      </c>
+      <c r="M692" t="n">
+        <v>4.161401</v>
+      </c>
+      <c r="N692" t="n">
+        <v>67223</v>
+      </c>
+      <c r="O692" t="n">
+        <v>13</v>
+      </c>
+      <c r="P692" t="inlineStr"/>
+      <c r="Q692" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R692" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S692" t="inlineStr">
+        <is>
+          <t>Aaaahhh, ta super app Max it, n&amp;#39;a pas fini de te surprendre... &lt;br&gt;Est-ce que tu as remarqué ? Maintenant, tu as ton QR code personnalisé en haut de ton écran d&amp;#39;accueil ! Ainsi, tu peux :&lt;br&gt;     scanner le QR code de ton ami(e) pour lui faire un transfert d&amp;#39;&amp;#39;argent&lt;br&gt;     scanner l</t>
+        </is>
+      </c>
+      <c r="T692" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U692" t="inlineStr"/>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G693" t="n">
+        <v>1061120855</v>
+      </c>
+      <c r="H693" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>Orange CI</t>
+        </is>
+      </c>
+      <c r="J693" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K693" t="n">
+        <v>0</v>
+      </c>
+      <c r="L693" t="b">
+        <v>1</v>
+      </c>
+      <c r="M693" t="n">
+        <v>3.78576</v>
+      </c>
+      <c r="N693" t="n">
+        <v>5970</v>
+      </c>
+      <c r="O693" t="n">
+        <v>3</v>
+      </c>
+      <c r="P693" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R693" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S693" t="inlineStr">
+        <is>
+          <t>Max it, la super app all-in-one te fais gagner du temps, et diminue tes soucis... Gagne plus d'espace de stockage sur ton téléphone ; plus besoin de cumuler plusieurs appli d'Orange pour avoir accès à un maximum de services. Max it est là ! Gère ta ligne (SIM) au niveau des pass, des soldes, réalise</t>
+        </is>
+      </c>
+      <c r="T693" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U693" t="inlineStr"/>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G694" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogw</t>
+        </is>
+      </c>
+      <c r="H694" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I694" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J694" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K694" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L694" t="b">
+        <v>0</v>
+      </c>
+      <c r="M694" t="n">
+        <v>4.350993</v>
+      </c>
+      <c r="N694" t="n">
+        <v>1533</v>
+      </c>
+      <c r="O694" t="n">
+        <v>4</v>
+      </c>
+      <c r="P694" t="inlineStr"/>
+      <c r="Q694" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R694" t="inlineStr">
+        <is>
+          <t>4.0.18</t>
+        </is>
+      </c>
+      <c r="S694" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T694" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U694" t="inlineStr"/>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G695" t="n">
+        <v>1574668652</v>
+      </c>
+      <c r="H695" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J695" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K695" t="n">
+        <v>0</v>
+      </c>
+      <c r="L695" t="b">
+        <v>1</v>
+      </c>
+      <c r="M695" t="n">
+        <v>4.05333</v>
+      </c>
+      <c r="N695" t="n">
+        <v>75</v>
+      </c>
+      <c r="O695" t="n">
+        <v>16</v>
+      </c>
+      <c r="P695" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R695" t="inlineStr">
+        <is>
+          <t>6.0.35</t>
+        </is>
+      </c>
+      <c r="S695" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T695" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U695" t="inlineStr"/>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G696" t="inlineStr">
+        <is>
+          <t>com.orange.sugu.ocd</t>
+        </is>
+      </c>
+      <c r="H696" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J696" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K696" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L696" t="b">
+        <v>0</v>
+      </c>
+      <c r="M696" t="n">
+        <v>4.1301117</v>
+      </c>
+      <c r="N696" t="n">
+        <v>5303</v>
+      </c>
+      <c r="O696" t="n">
+        <v>74</v>
+      </c>
+      <c r="P696" t="inlineStr"/>
+      <c r="Q696" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R696" t="inlineStr">
+        <is>
+          <t>9.0.12</t>
+        </is>
+      </c>
+      <c r="S696" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DRC that brings together the features of MyOrange, and Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Plans, Mobile Payments, money transfers, bill payments, subscriptions, and entertai</t>
+        </is>
+      </c>
+      <c r="T696" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U696" t="inlineStr"/>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G697" t="n">
+        <v>6447896435</v>
+      </c>
+      <c r="H697" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I697" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J697" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K697" t="n">
+        <v>0</v>
+      </c>
+      <c r="L697" t="b">
+        <v>1</v>
+      </c>
+      <c r="M697" t="n">
+        <v>3.55762</v>
+      </c>
+      <c r="N697" t="n">
+        <v>269</v>
+      </c>
+      <c r="P697" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "CD" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R697" t="inlineStr">
+        <is>
+          <t>9.0.6</t>
+        </is>
+      </c>
+      <c r="S697" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DR Congo. It brings together the features of Orange et Moi, as well as Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Packages, Mobile payment, money transfers, bill payment and subscri</t>
+        </is>
+      </c>
+      <c r="T697" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U697" t="inlineStr"/>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G698" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ocm</t>
+        </is>
+      </c>
+      <c r="H698" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroon</t>
+        </is>
+      </c>
+      <c r="I698" t="inlineStr">
+        <is>
+          <t>Orange MEA</t>
+        </is>
+      </c>
+      <c r="J698" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K698" t="inlineStr">
+        <is>
+          <t>FCFA 0</t>
+        </is>
+      </c>
+      <c r="L698" t="b">
+        <v>0</v>
+      </c>
+      <c r="M698" t="n">
+        <v>3.924713</v>
+      </c>
+      <c r="N698" t="n">
+        <v>46937</v>
+      </c>
+      <c r="O698" t="n">
+        <v>8</v>
+      </c>
+      <c r="P698" t="inlineStr"/>
+      <c r="Q698" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R698" t="inlineStr">
+        <is>
+          <t>7.0.23</t>
+        </is>
+      </c>
+      <c r="S698" t="inlineStr">
+        <is>
+          <t>Max it brings together everything that matters to you in one app: managing your lines, money transfer, bill payment, exclusive offers, and a universe of lifestyle and entertainment. Simple, fast, and 100% secure..&lt;br&gt;&lt;br&gt;📞 My line&lt;br&gt;Manage your Orange mobile and landline bundles in a single click:</t>
+        </is>
+      </c>
+      <c r="T698" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U698" t="inlineStr"/>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F699" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G699" t="n">
+        <v>1116920093</v>
+      </c>
+      <c r="H699" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroun</t>
+        </is>
+      </c>
+      <c r="I699" t="inlineStr">
+        <is>
+          <t>Orange Middle East &amp; Africa</t>
+        </is>
+      </c>
+      <c r="J699" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K699" t="n">
+        <v>0</v>
+      </c>
+      <c r="L699" t="b">
+        <v>1</v>
+      </c>
+      <c r="M699" t="n">
+        <v>3.76841</v>
+      </c>
+      <c r="N699" t="n">
+        <v>16158</v>
+      </c>
+      <c r="O699" t="n">
+        <v>1</v>
+      </c>
+      <c r="P699" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R699" t="inlineStr">
+        <is>
+          <t>7.0.24</t>
+        </is>
+      </c>
+      <c r="S699" t="inlineStr">
+        <is>
+          <t>Avec Max it, Orange rassemble tout ce qui compte pour vous dans une même application : la gestion de vos lignes, les transferts d’argent, payement de vos factures, des offres exclusives et un univers lifestyle et divertissement.
+Simple, rapide et 100 % sécurisée.
+Ma ligne
+Gérez vos forfaits mobiles</t>
+        </is>
+      </c>
+      <c r="T699" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U699" t="inlineStr"/>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F700" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G700" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obf</t>
+        </is>
+      </c>
+      <c r="H700" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I700" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso</t>
+        </is>
+      </c>
+      <c r="J700" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K700" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L700" t="b">
+        <v>0</v>
+      </c>
+      <c r="M700" t="n">
+        <v>4.1368628</v>
+      </c>
+      <c r="N700" t="n">
+        <v>25479</v>
+      </c>
+      <c r="O700" t="n">
+        <v>11</v>
+      </c>
+      <c r="P700" t="inlineStr"/>
+      <c r="Q700" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R700" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S700" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.&lt;br&gt;Gérez vos lignes mobiles, effectuez des transferts d&amp;#39;argent sécurisés, réglez vos factures, profitez d&amp;#39;offres exclusives, effectuez des paiements marchands fiables, et bien plus enco</t>
+        </is>
+      </c>
+      <c r="T700" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U700" t="inlineStr"/>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F701" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G701" t="n">
+        <v>1553774707</v>
+      </c>
+      <c r="H701" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I701" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso SA</t>
+        </is>
+      </c>
+      <c r="J701" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K701" t="n">
+        <v>0</v>
+      </c>
+      <c r="L701" t="b">
+        <v>1</v>
+      </c>
+      <c r="M701" t="n">
+        <v>3.45377</v>
+      </c>
+      <c r="N701" t="n">
+        <v>1179</v>
+      </c>
+      <c r="O701" t="n">
+        <v>5</v>
+      </c>
+      <c r="P701" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R701" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S701" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.
+Gérez vos lignes mobiles, effectuez des transferts d'argent sécurisés, réglez vos factures, profitez d'offres exclusives, effectuez des paiements marchands fiables, et bien plus encore, le tout</t>
+        </is>
+      </c>
+      <c r="T701" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U701" t="inlineStr"/>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F702" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G702" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obw</t>
+        </is>
+      </c>
+      <c r="H702" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I702" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J702" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K702" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L702" t="b">
+        <v>0</v>
+      </c>
+      <c r="M702" t="n">
+        <v>3.9819496</v>
+      </c>
+      <c r="N702" t="n">
+        <v>2965</v>
+      </c>
+      <c r="O702" t="n">
+        <v>30</v>
+      </c>
+      <c r="P702" t="inlineStr"/>
+      <c r="Q702" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R702" t="inlineStr">
+        <is>
+          <t>7.3.8</t>
+        </is>
+      </c>
+      <c r="S702" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it, the brand-new Orange Botswana Super App that follows Yame and gives you access to four distinct universes for a one-of-a-kind experience!&lt;br&gt;&lt;br&gt;Manage your accounts, make quick payments using QR codes, investigate a range of online goods and services, and discover the many options provided </t>
+        </is>
+      </c>
+      <c r="T702" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U702" t="inlineStr"/>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F703" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G703" t="n">
+        <v>1195839458</v>
+      </c>
+      <c r="H703" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I703" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J703" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K703" t="n">
+        <v>0</v>
+      </c>
+      <c r="L703" t="b">
+        <v>1</v>
+      </c>
+      <c r="M703" t="n">
+        <v>3.00806</v>
+      </c>
+      <c r="N703" t="n">
+        <v>124</v>
+      </c>
+      <c r="O703" t="n">
+        <v>12</v>
+      </c>
+      <c r="P703" t="inlineStr"/>
+      <c r="R703" t="inlineStr">
+        <is>
+          <t>7.3.1</t>
+        </is>
+      </c>
+      <c r="S703" t="inlineStr">
+        <is>
+          <t>A free mobile self-care application for Orange Botswana’s mobile customers.
+Full Description :
+Max it is a free application, which allows Orange Botswana customers to:
+- Consult your account in real time: minutes, sms, internet ...
+- Top up your account or a friend account  with Orange Money
+-</t>
+        </is>
+      </c>
+      <c r="T703" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U703" t="inlineStr"/>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G704" t="inlineStr">
+        <is>
+          <t>com.orange.mobinilandme</t>
+        </is>
+      </c>
+      <c r="H704" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I704" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J704" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K704" t="inlineStr">
+        <is>
+          <t>EGP 0.00</t>
+        </is>
+      </c>
+      <c r="L704" t="b">
+        <v>0</v>
+      </c>
+      <c r="M704" t="n">
+        <v>4.5589232</v>
+      </c>
+      <c r="N704" t="n">
+        <v>929771</v>
+      </c>
+      <c r="O704" t="n">
+        <v>19</v>
+      </c>
+      <c r="P704" t="inlineStr"/>
+      <c r="Q704" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R704" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S704" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion&lt;br&gt;Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.&lt;br&gt;Key services include:&lt;br&gt;• Account Management: Easily manage</t>
+        </is>
+      </c>
+      <c r="T704" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U704" t="inlineStr"/>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>fc3e35ab-dc20-4feb-90f8-e24f9b094347</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>2026-07-29 06:32:33</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F705" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G705" t="n">
+        <v>942568333</v>
+      </c>
+      <c r="H705" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I705" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J705" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K705" t="n">
+        <v>0</v>
+      </c>
+      <c r="L705" t="b">
+        <v>1</v>
+      </c>
+      <c r="M705" t="n">
+        <v>4.25193</v>
+      </c>
+      <c r="N705" t="n">
+        <v>117725</v>
+      </c>
+      <c r="O705" t="n">
+        <v>53</v>
+      </c>
+      <c r="P705" t="inlineStr"/>
+      <c r="R705" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S705" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion
+Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.
+Key services include:
+• Account Management: Easily manage your Ora</t>
+        </is>
+      </c>
+      <c r="T705" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U705" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-07-30
</commit_message>
<xml_diff>
--- a/maxit_store_history.xlsx
+++ b/maxit_store_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U705"/>
+  <dimension ref="A1:U737"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57940,7 +57940,6 @@
       <c r="O674" t="n">
         <v>28</v>
       </c>
-      <c r="P674" t="inlineStr"/>
       <c r="Q674" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -57961,7 +57960,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U674" t="inlineStr"/>
     </row>
     <row r="675">
       <c r="A675" t="inlineStr">
@@ -58024,7 +58022,6 @@
       <c r="N675" t="n">
         <v>324</v>
       </c>
-      <c r="P675" t="inlineStr"/>
       <c r="R675" t="inlineStr">
         <is>
           <t>6.4.8</t>
@@ -58040,7 +58037,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U675" t="inlineStr"/>
     </row>
     <row r="676">
       <c r="A676" t="inlineStr">
@@ -58110,7 +58106,6 @@
       <c r="O676" t="n">
         <v>28</v>
       </c>
-      <c r="P676" t="inlineStr"/>
       <c r="Q676" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -58131,7 +58126,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U676" t="inlineStr"/>
     </row>
     <row r="677">
       <c r="A677" t="inlineStr">
@@ -58197,7 +58191,6 @@
       <c r="O677" t="n">
         <v>45</v>
       </c>
-      <c r="P677" t="inlineStr"/>
       <c r="R677" t="inlineStr">
         <is>
           <t>10.0.6</t>
@@ -58215,7 +58208,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U677" t="inlineStr"/>
     </row>
     <row r="678">
       <c r="A678" t="inlineStr">
@@ -58285,7 +58277,6 @@
       <c r="O678" t="n">
         <v>10</v>
       </c>
-      <c r="P678" t="inlineStr"/>
       <c r="Q678" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -58306,7 +58297,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U678" t="inlineStr"/>
     </row>
     <row r="679">
       <c r="A679" t="inlineStr">
@@ -58395,7 +58385,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U679" t="inlineStr"/>
     </row>
     <row r="680">
       <c r="A680" t="inlineStr">
@@ -58465,7 +58454,6 @@
       <c r="O680" t="n">
         <v>11</v>
       </c>
-      <c r="P680" t="inlineStr"/>
       <c r="Q680" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -58486,7 +58474,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U680" t="inlineStr"/>
     </row>
     <row r="681">
       <c r="A681" t="inlineStr">
@@ -58552,7 +58539,6 @@
       <c r="O681" t="n">
         <v>3</v>
       </c>
-      <c r="P681" t="inlineStr"/>
       <c r="R681" t="inlineStr">
         <is>
           <t>22.0.0</t>
@@ -58570,7 +58556,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U681" t="inlineStr"/>
     </row>
     <row r="682">
       <c r="A682" t="inlineStr">
@@ -58640,7 +58625,6 @@
       <c r="O682" t="n">
         <v>110</v>
       </c>
-      <c r="P682" t="inlineStr"/>
       <c r="Q682" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -58661,7 +58645,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U682" t="inlineStr"/>
     </row>
     <row r="683">
       <c r="A683" t="inlineStr">
@@ -58746,7 +58729,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U683" t="inlineStr"/>
     </row>
     <row r="684">
       <c r="A684" t="inlineStr">
@@ -58813,7 +58795,6 @@
       <c r="N684" t="n">
         <v>38249</v>
       </c>
-      <c r="P684" t="inlineStr"/>
       <c r="Q684" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -58834,7 +58815,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U684" t="inlineStr"/>
     </row>
     <row r="685">
       <c r="A685" t="inlineStr">
@@ -58900,7 +58880,6 @@
       <c r="O685" t="n">
         <v>14</v>
       </c>
-      <c r="P685" t="inlineStr"/>
       <c r="R685" t="inlineStr">
         <is>
           <t>6.5.2</t>
@@ -58919,7 +58898,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U685" t="inlineStr"/>
     </row>
     <row r="686">
       <c r="A686" t="inlineStr">
@@ -58989,7 +58967,6 @@
       <c r="O686" t="n">
         <v>53</v>
       </c>
-      <c r="P686" t="inlineStr"/>
       <c r="Q686" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -59010,7 +58987,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U686" t="inlineStr"/>
     </row>
     <row r="687">
       <c r="A687" t="inlineStr">
@@ -59076,7 +59052,6 @@
       <c r="O687" t="n">
         <v>19</v>
       </c>
-      <c r="P687" t="inlineStr"/>
       <c r="R687" t="inlineStr">
         <is>
           <t>5.0.2</t>
@@ -59094,7 +59069,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U687" t="inlineStr"/>
     </row>
     <row r="688">
       <c r="A688" t="inlineStr">
@@ -59164,7 +59138,6 @@
       <c r="O688" t="n">
         <v>94</v>
       </c>
-      <c r="P688" t="inlineStr"/>
       <c r="Q688" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -59185,7 +59158,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U688" t="inlineStr"/>
     </row>
     <row r="689">
       <c r="A689" t="inlineStr">
@@ -59273,7 +59245,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U689" t="inlineStr"/>
     </row>
     <row r="690">
       <c r="A690" t="inlineStr">
@@ -59343,7 +59314,6 @@
       <c r="O690" t="n">
         <v>46</v>
       </c>
-      <c r="P690" t="inlineStr"/>
       <c r="Q690" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -59364,7 +59334,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U690" t="inlineStr"/>
     </row>
     <row r="691">
       <c r="A691" t="inlineStr">
@@ -59430,7 +59399,6 @@
       <c r="O691" t="n">
         <v>42</v>
       </c>
-      <c r="P691" t="inlineStr"/>
       <c r="R691" t="inlineStr">
         <is>
           <t>10.0.21</t>
@@ -59449,7 +59417,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U691" t="inlineStr"/>
     </row>
     <row r="692">
       <c r="A692" t="inlineStr">
@@ -59519,7 +59486,6 @@
       <c r="O692" t="n">
         <v>13</v>
       </c>
-      <c r="P692" t="inlineStr"/>
       <c r="Q692" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -59540,7 +59506,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U692" t="inlineStr"/>
     </row>
     <row r="693">
       <c r="A693" t="inlineStr">
@@ -59626,7 +59591,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U693" t="inlineStr"/>
     </row>
     <row r="694">
       <c r="A694" t="inlineStr">
@@ -59696,7 +59660,6 @@
       <c r="O694" t="n">
         <v>4</v>
       </c>
-      <c r="P694" t="inlineStr"/>
       <c r="Q694" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -59717,7 +59680,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U694" t="inlineStr"/>
     </row>
     <row r="695">
       <c r="A695" t="inlineStr">
@@ -59803,7 +59765,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U695" t="inlineStr"/>
     </row>
     <row r="696">
       <c r="A696" t="inlineStr">
@@ -59873,7 +59834,6 @@
       <c r="O696" t="n">
         <v>74</v>
       </c>
-      <c r="P696" t="inlineStr"/>
       <c r="Q696" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -59894,7 +59854,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U696" t="inlineStr"/>
     </row>
     <row r="697">
       <c r="A697" t="inlineStr">
@@ -59977,7 +59936,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U697" t="inlineStr"/>
     </row>
     <row r="698">
       <c r="A698" t="inlineStr">
@@ -60047,7 +60005,6 @@
       <c r="O698" t="n">
         <v>8</v>
       </c>
-      <c r="P698" t="inlineStr"/>
       <c r="Q698" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -60068,7 +60025,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U698" t="inlineStr"/>
     </row>
     <row r="699">
       <c r="A699" t="inlineStr">
@@ -60157,7 +60113,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U699" t="inlineStr"/>
     </row>
     <row r="700">
       <c r="A700" t="inlineStr">
@@ -60227,7 +60182,6 @@
       <c r="O700" t="n">
         <v>11</v>
       </c>
-      <c r="P700" t="inlineStr"/>
       <c r="Q700" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -60248,7 +60202,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U700" t="inlineStr"/>
     </row>
     <row r="701">
       <c r="A701" t="inlineStr">
@@ -60335,7 +60288,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U701" t="inlineStr"/>
     </row>
     <row r="702">
       <c r="A702" t="inlineStr">
@@ -60405,7 +60357,6 @@
       <c r="O702" t="n">
         <v>30</v>
       </c>
-      <c r="P702" t="inlineStr"/>
       <c r="Q702" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -60426,7 +60377,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U702" t="inlineStr"/>
     </row>
     <row r="703">
       <c r="A703" t="inlineStr">
@@ -60492,7 +60442,6 @@
       <c r="O703" t="n">
         <v>12</v>
       </c>
-      <c r="P703" t="inlineStr"/>
       <c r="R703" t="inlineStr">
         <is>
           <t>7.3.1</t>
@@ -60513,7 +60462,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U703" t="inlineStr"/>
     </row>
     <row r="704">
       <c r="A704" t="inlineStr">
@@ -60583,7 +60531,6 @@
       <c r="O704" t="n">
         <v>19</v>
       </c>
-      <c r="P704" t="inlineStr"/>
       <c r="Q704" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -60604,7 +60551,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U704" t="inlineStr"/>
     </row>
     <row r="705">
       <c r="A705" t="inlineStr">
@@ -60670,7 +60616,6 @@
       <c r="O705" t="n">
         <v>53</v>
       </c>
-      <c r="P705" t="inlineStr"/>
       <c r="R705" t="inlineStr">
         <is>
           <t>10.1.0</t>
@@ -60689,7 +60634,2825 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U705" t="inlineStr"/>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F706" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G706" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogn</t>
+        </is>
+      </c>
+      <c r="H706" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I706" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J706" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K706" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L706" t="b">
+        <v>0</v>
+      </c>
+      <c r="M706" t="n">
+        <v>4.4421396</v>
+      </c>
+      <c r="N706" t="n">
+        <v>9311</v>
+      </c>
+      <c r="O706" t="n">
+        <v>35</v>
+      </c>
+      <c r="P706" t="inlineStr"/>
+      <c r="Q706" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R706" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S706" t="inlineStr">
+        <is>
+          <t>Bien plus qu&amp;#39;une application, un véritable assistant personnel pour une vie connectée et simplifiée.&lt;br&gt;Suivi de consommation: Votre tableau de bord tout-en-un pour une gestion simplifiée !&lt;br&gt;- Gestion de votre offre: Accédez à une vue détaillée de votre offre actuelle et de vos forfaits Orange</t>
+        </is>
+      </c>
+      <c r="T706" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U706" t="inlineStr"/>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F707" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G707" t="n">
+        <v>1177999485</v>
+      </c>
+      <c r="H707" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I707" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J707" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K707" t="n">
+        <v>0</v>
+      </c>
+      <c r="L707" t="b">
+        <v>1</v>
+      </c>
+      <c r="M707" t="n">
+        <v>3.88272</v>
+      </c>
+      <c r="N707" t="n">
+        <v>324</v>
+      </c>
+      <c r="P707" t="inlineStr"/>
+      <c r="R707" t="inlineStr">
+        <is>
+          <t>6.4.8</t>
+        </is>
+      </c>
+      <c r="S707" t="inlineStr">
+        <is>
+          <t>La fusion d’Orange et Moi et Orange Money donne naissance à Max it, la nouvelle Super Application Tout-en-Un. Profitez du suivi de consommation, de paiements mobiles, de toutes les fonctionnalités Orange et Moi et Money avec un large éventail de divertissements, le tout regroupé en un seul endroit !</t>
+        </is>
+      </c>
+      <c r="T707" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U707" t="inlineStr"/>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F708" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G708" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.otn</t>
+        </is>
+      </c>
+      <c r="H708" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I708" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J708" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K708" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L708" t="b">
+        <v>0</v>
+      </c>
+      <c r="M708" t="n">
+        <v>3.968889</v>
+      </c>
+      <c r="N708" t="n">
+        <v>35375</v>
+      </c>
+      <c r="O708" t="n">
+        <v>31</v>
+      </c>
+      <c r="P708" t="inlineStr"/>
+      <c r="Q708" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R708" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S708" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Max it par Orange Tunisie facilite votre vie au quotidien !&lt;/h2&gt;&lt;br&gt;&lt;br&gt;Welcome sur Max it !&lt;br&gt;Accédez rapidement à vos fonctionnalités Max it préférées et profitez également de contenus exclusifs, d’activités divertissantes, et de jeux interactifs pour une expérience enrichissante avec la roue</t>
+        </is>
+      </c>
+      <c r="T708" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U708" t="inlineStr"/>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F709" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G709" t="n">
+        <v>1146892088</v>
+      </c>
+      <c r="H709" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I709" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J709" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K709" t="n">
+        <v>0</v>
+      </c>
+      <c r="L709" t="b">
+        <v>1</v>
+      </c>
+      <c r="M709" t="n">
+        <v>3.03049</v>
+      </c>
+      <c r="N709" t="n">
+        <v>1640</v>
+      </c>
+      <c r="O709" t="n">
+        <v>47</v>
+      </c>
+      <c r="P709" t="inlineStr"/>
+      <c r="R709" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S709" t="inlineStr">
+        <is>
+          <t>Max it by Orange Tunisie : Votre appli incontournable pour une vie connectée
+Welcome sur Max it : Découvrez fonctionnalités, jeux &amp; contenus de divertissement by Orange Tunisie !
+Trouvez vite vos fonctionnalités Max it favorites et explorez des contenus exclusifs et des jeux pour une expérience im</t>
+        </is>
+      </c>
+      <c r="T709" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U709" t="inlineStr"/>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F710" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G710" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osl</t>
+        </is>
+      </c>
+      <c r="H710" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I710" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J710" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K710" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L710" t="b">
+        <v>0</v>
+      </c>
+      <c r="M710" t="n">
+        <v>4.384259</v>
+      </c>
+      <c r="N710" t="n">
+        <v>2139</v>
+      </c>
+      <c r="O710" t="n">
+        <v>10</v>
+      </c>
+      <c r="P710" t="inlineStr"/>
+      <c r="Q710" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R710" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S710" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it is a free application, which allows Orange Sierra Leone prepaid and postpaid customers to:&lt;br&gt;&lt;br&gt;- Consult your account in real time: minutes, sms, internet&lt;br&gt;- Top up your account or a friend account &lt;br&gt;- Buy Internet Bundles&lt;br&gt;- Discover the latest offers and promotions &lt;br&gt;- Access to </t>
+        </is>
+      </c>
+      <c r="T710" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U710" t="inlineStr"/>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F711" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G711" t="n">
+        <v>6443607903</v>
+      </c>
+      <c r="H711" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I711" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J711" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K711" t="n">
+        <v>0</v>
+      </c>
+      <c r="L711" t="b">
+        <v>1</v>
+      </c>
+      <c r="M711" t="n">
+        <v>3.69948</v>
+      </c>
+      <c r="N711" t="n">
+        <v>193</v>
+      </c>
+      <c r="O711" t="n">
+        <v>8</v>
+      </c>
+      <c r="P711" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R711" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S711" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The merger of My Orange &amp; Orange Money has given birth to Max it the all-in-one super app, a free application which allows all Orange Sierra Leone customers to 
+Track calls, SMS, and Data usage and monitor balance. 
+Make a secure mobile/Orange Money payment.
+Easily transfer credit to other users </t>
+        </is>
+      </c>
+      <c r="T711" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U711" t="inlineStr"/>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F712" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G712" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osn</t>
+        </is>
+      </c>
+      <c r="H712" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I712" t="inlineStr">
+        <is>
+          <t>Orange Sénégal</t>
+        </is>
+      </c>
+      <c r="J712" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K712" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L712" t="b">
+        <v>0</v>
+      </c>
+      <c r="M712" t="n">
+        <v>4.3007255</v>
+      </c>
+      <c r="N712" t="n">
+        <v>51260</v>
+      </c>
+      <c r="O712" t="n">
+        <v>10</v>
+      </c>
+      <c r="P712" t="inlineStr"/>
+      <c r="Q712" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R712" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S712" t="inlineStr">
+        <is>
+          <t>Lu bees ak Max it ! &lt;br&gt;Une application repensée pour être plus simple, plus rapide et adaptée à vos besoins. Une expérience optimisée pour faciliter vos usages au quotidien, avec des parcours simplifiés et un accès plus fluide à vos services. Que vous soyez client Orange ou non, Max it vous accompa</t>
+        </is>
+      </c>
+      <c r="T712" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U712" t="inlineStr"/>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F713" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G713" t="n">
+        <v>1039327980</v>
+      </c>
+      <c r="H713" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I713" t="inlineStr">
+        <is>
+          <t>Orange Senegal</t>
+        </is>
+      </c>
+      <c r="J713" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K713" t="n">
+        <v>0</v>
+      </c>
+      <c r="L713" t="b">
+        <v>1</v>
+      </c>
+      <c r="M713" t="n">
+        <v>4.16929</v>
+      </c>
+      <c r="N713" t="n">
+        <v>30226</v>
+      </c>
+      <c r="O713" t="n">
+        <v>2</v>
+      </c>
+      <c r="P713" t="inlineStr"/>
+      <c r="R713" t="inlineStr">
+        <is>
+          <t>22.0.0</t>
+        </is>
+      </c>
+      <c r="S713" t="inlineStr">
+        <is>
+          <t>Here is the English translation:
+Welcome to Max it!
+A redesigned app to be simpler, faster, and tailored to your needs. An optimized experience to make your daily life easier, with streamlined journeys and smoother access to your services. Whether you are an Orange customer or not, Max it is your e</t>
+        </is>
+      </c>
+      <c r="T713" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U713" t="inlineStr"/>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F714" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G714" t="inlineStr">
+        <is>
+          <t>com.orange.meditel.mediteletmoi</t>
+        </is>
+      </c>
+      <c r="H714" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I714" t="inlineStr">
+        <is>
+          <t>Orange Maroc</t>
+        </is>
+      </c>
+      <c r="J714" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K714" t="inlineStr">
+        <is>
+          <t>MAD 0.00</t>
+        </is>
+      </c>
+      <c r="L714" t="b">
+        <v>0</v>
+      </c>
+      <c r="M714" t="n">
+        <v>3.719018</v>
+      </c>
+      <c r="N714" t="n">
+        <v>110915</v>
+      </c>
+      <c r="O714" t="n">
+        <v>104</v>
+      </c>
+      <c r="P714" t="inlineStr"/>
+      <c r="Q714" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R714" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S714" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l&amp;#39;expérience mobile réinventé&lt;br&gt;&lt;br&gt;Max it, c&amp;#39;est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d&amp;#39;une multitude de services exclusifs. &lt;br&gt;&lt;br&gt;Créez votre espace sur</t>
+        </is>
+      </c>
+      <c r="T714" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U714" t="inlineStr"/>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F715" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G715" t="n">
+        <v>596028698</v>
+      </c>
+      <c r="H715" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I715" t="inlineStr">
+        <is>
+          <t>Méditel</t>
+        </is>
+      </c>
+      <c r="J715" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K715" t="n">
+        <v>0</v>
+      </c>
+      <c r="L715" t="b">
+        <v>1</v>
+      </c>
+      <c r="M715" t="n">
+        <v>3.94557</v>
+      </c>
+      <c r="N715" t="n">
+        <v>2756</v>
+      </c>
+      <c r="P715" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "MA" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R715" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S715" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l'expérience mobile réinventé
+Max it, c'est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d'une multitude de services exclusifs. 
+Créez votre espace sur mesure et bénéficiez d'</t>
+        </is>
+      </c>
+      <c r="T715" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U715" t="inlineStr"/>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F716" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G716" t="inlineStr">
+        <is>
+          <t>com.oml.dsi.orangemobile</t>
+        </is>
+      </c>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I716" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J716" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K716" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L716" t="b">
+        <v>0</v>
+      </c>
+      <c r="M716" t="n">
+        <v>2.6952431</v>
+      </c>
+      <c r="N716" t="n">
+        <v>38250</v>
+      </c>
+      <c r="P716" t="inlineStr"/>
+      <c r="Q716" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R716" t="inlineStr">
+        <is>
+          <t>6.5.0</t>
+        </is>
+      </c>
+      <c r="S716" t="inlineStr">
+        <is>
+          <t>Easily manage your Orange Mali line&lt;br&gt;● Manage your account and view all essential information, your offers, and your phone lines.&lt;br&gt;● Subscribe to call, SMS, Internet, and international call packages.&lt;br&gt;● Track your usage by checking your credit and Internet balance.&lt;br&gt;● Recharge your line by p</t>
+        </is>
+      </c>
+      <c r="T716" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U716" t="inlineStr"/>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F717" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G717" t="n">
+        <v>1494321079</v>
+      </c>
+      <c r="H717" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I717" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J717" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K717" t="n">
+        <v>0</v>
+      </c>
+      <c r="L717" t="b">
+        <v>1</v>
+      </c>
+      <c r="M717" t="n">
+        <v>2.52147</v>
+      </c>
+      <c r="N717" t="n">
+        <v>4750</v>
+      </c>
+      <c r="O717" t="n">
+        <v>14</v>
+      </c>
+      <c r="P717" t="inlineStr"/>
+      <c r="R717" t="inlineStr">
+        <is>
+          <t>6.5.2</t>
+        </is>
+      </c>
+      <c r="S717" t="inlineStr">
+        <is>
+          <t>Gérez facilement votre ligne Orange Mali 
+●        Gérez votre compte et consultez toutes les informations essentielles sur celui-ci, vos offres, ainsi que vos lignes téléphoniques.
+●        Souscrivez aux forfaits appels, SMS, Internet, et appels internationaux.
+●        Suivez votre consommation e</t>
+        </is>
+      </c>
+      <c r="T717" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U717" t="inlineStr"/>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F718" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G718" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.omg</t>
+        </is>
+      </c>
+      <c r="H718" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I718" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J718" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K718" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L718" t="b">
+        <v>0</v>
+      </c>
+      <c r="M718" t="n">
+        <v>4.151515</v>
+      </c>
+      <c r="N718" t="n">
+        <v>1377</v>
+      </c>
+      <c r="O718" t="n">
+        <v>55</v>
+      </c>
+      <c r="P718" t="inlineStr"/>
+      <c r="Q718" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R718" t="inlineStr">
+        <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="S718" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.&lt;br&gt;&lt;br&gt;Simplify Your Life with Max it&lt;br&gt;With Max It, ac</t>
+        </is>
+      </c>
+      <c r="T718" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U718" t="inlineStr"/>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F719" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G719" t="n">
+        <v>1295171817</v>
+      </c>
+      <c r="H719" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I719" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J719" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K719" t="n">
+        <v>0</v>
+      </c>
+      <c r="L719" t="b">
+        <v>1</v>
+      </c>
+      <c r="M719" t="n">
+        <v>3.08696</v>
+      </c>
+      <c r="N719" t="n">
+        <v>69</v>
+      </c>
+      <c r="O719" t="n">
+        <v>20</v>
+      </c>
+      <c r="P719" t="inlineStr"/>
+      <c r="R719" t="inlineStr">
+        <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="S719" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.
+Simplify Your Life with Max it
+With Max it, access a se</t>
+        </is>
+      </c>
+      <c r="T719" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U719" t="inlineStr"/>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F720" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G720" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.olr</t>
+        </is>
+      </c>
+      <c r="H720" t="inlineStr">
+        <is>
+          <t>Orange Max it - Liberia</t>
+        </is>
+      </c>
+      <c r="I720" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J720" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K720" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L720" t="b">
+        <v>0</v>
+      </c>
+      <c r="M720" t="n">
+        <v>4.5466237</v>
+      </c>
+      <c r="N720" t="n">
+        <v>3100</v>
+      </c>
+      <c r="O720" t="n">
+        <v>108</v>
+      </c>
+      <c r="P720" t="inlineStr"/>
+      <c r="Q720" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R720" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="S720" t="inlineStr">
+        <is>
+          <t>Max it: your personalized experience by Orange Liberia!&lt;br&gt;&lt;br&gt;Step into Max it, your all-in-one solution for telecom, marketplace, and financial services! Manage your mobile line, customize offers, pay your bills, keep&lt;br&gt;track of your usage with ease, and recharge your credit. Access exclusive eve</t>
+        </is>
+      </c>
+      <c r="T720" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U720" t="inlineStr"/>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F721" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G721" t="n">
+        <v>6746187327</v>
+      </c>
+      <c r="H721" t="inlineStr">
+        <is>
+          <t>Orange Max it – Liberia</t>
+        </is>
+      </c>
+      <c r="I721" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J721" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K721" t="n">
+        <v>0</v>
+      </c>
+      <c r="L721" t="b">
+        <v>1</v>
+      </c>
+      <c r="M721" t="n">
+        <v>4.0625</v>
+      </c>
+      <c r="N721" t="n">
+        <v>48</v>
+      </c>
+      <c r="P721" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "LR" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R721" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="S721" t="inlineStr">
+        <is>
+          <t>Max it is a free application, which allows Orange Liberia customers to:
+- Consult your account in real time: minutes, sms, internet
+- Top up your account or a friend account 
+- Buy  Bundles (voice, data, SMS, roaming, international)
+- Discover the latest offers and promotions 
+- Access to Orange se</t>
+        </is>
+      </c>
+      <c r="T721" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U721" t="inlineStr"/>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F722" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G722" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ojo</t>
+        </is>
+      </c>
+      <c r="H722" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I722" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J722" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K722" t="inlineStr">
+        <is>
+          <t>JOD 0.000</t>
+        </is>
+      </c>
+      <c r="L722" t="b">
+        <v>0</v>
+      </c>
+      <c r="M722" t="n">
+        <v>4.4311795</v>
+      </c>
+      <c r="N722" t="n">
+        <v>97742</v>
+      </c>
+      <c r="O722" t="n">
+        <v>41</v>
+      </c>
+      <c r="P722" t="inlineStr"/>
+      <c r="Q722" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R722" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S722" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience&lt;br&gt;Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.&lt;br&gt;Important Update:&lt;br&gt;The jood app (jood Orange) w</t>
+        </is>
+      </c>
+      <c r="T722" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U722" t="inlineStr"/>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F723" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G723" t="n">
+        <v>808824590</v>
+      </c>
+      <c r="H723" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I723" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J723" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K723" t="n">
+        <v>0</v>
+      </c>
+      <c r="L723" t="b">
+        <v>1</v>
+      </c>
+      <c r="M723" t="n">
+        <v>4.20995</v>
+      </c>
+      <c r="N723" t="n">
+        <v>3034</v>
+      </c>
+      <c r="O723" t="n">
+        <v>42</v>
+      </c>
+      <c r="P723" t="inlineStr"/>
+      <c r="R723" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S723" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience
+Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.
+Important Update:
+The jood app (jood Orange) will be di</t>
+        </is>
+      </c>
+      <c r="T723" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U723" t="inlineStr"/>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F724" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G724" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.oci</t>
+        </is>
+      </c>
+      <c r="H724" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I724" t="inlineStr">
+        <is>
+          <t>Orange Côte d'Ivoire S.A</t>
+        </is>
+      </c>
+      <c r="J724" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K724" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L724" t="b">
+        <v>0</v>
+      </c>
+      <c r="M724" t="n">
+        <v>4.1540875</v>
+      </c>
+      <c r="N724" t="n">
+        <v>67256</v>
+      </c>
+      <c r="O724" t="n">
+        <v>11</v>
+      </c>
+      <c r="P724" t="inlineStr"/>
+      <c r="Q724" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R724" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S724" t="inlineStr">
+        <is>
+          <t>Aaaahhh, ta super app Max it, n&amp;#39;a pas fini de te surprendre... &lt;br&gt;Est-ce que tu as remarqué ? Maintenant, tu as ton QR code personnalisé en haut de ton écran d&amp;#39;accueil ! Ainsi, tu peux :&lt;br&gt;     scanner le QR code de ton ami(e) pour lui faire un transfert d&amp;#39;&amp;#39;argent&lt;br&gt;     scanner l</t>
+        </is>
+      </c>
+      <c r="T724" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U724" t="inlineStr"/>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D725" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F725" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G725" t="n">
+        <v>1061120855</v>
+      </c>
+      <c r="H725" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I725" t="inlineStr">
+        <is>
+          <t>Orange CI</t>
+        </is>
+      </c>
+      <c r="J725" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K725" t="n">
+        <v>0</v>
+      </c>
+      <c r="L725" t="b">
+        <v>1</v>
+      </c>
+      <c r="M725" t="n">
+        <v>3.78583</v>
+      </c>
+      <c r="N725" t="n">
+        <v>5972</v>
+      </c>
+      <c r="O725" t="n">
+        <v>9</v>
+      </c>
+      <c r="P725" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R725" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S725" t="inlineStr">
+        <is>
+          <t>Max it, la super app all-in-one te fais gagner du temps, et diminue tes soucis... Gagne plus d'espace de stockage sur ton téléphone ; plus besoin de cumuler plusieurs appli d'Orange pour avoir accès à un maximum de services. Max it est là ! Gère ta ligne (SIM) au niveau des pass, des soldes, réalise</t>
+        </is>
+      </c>
+      <c r="T725" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U725" t="inlineStr"/>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F726" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G726" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogw</t>
+        </is>
+      </c>
+      <c r="H726" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I726" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J726" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K726" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L726" t="b">
+        <v>0</v>
+      </c>
+      <c r="M726" t="n">
+        <v>4.385621</v>
+      </c>
+      <c r="N726" t="n">
+        <v>1538</v>
+      </c>
+      <c r="O726" t="n">
+        <v>4</v>
+      </c>
+      <c r="P726" t="inlineStr"/>
+      <c r="Q726" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R726" t="inlineStr">
+        <is>
+          <t>4.0.18</t>
+        </is>
+      </c>
+      <c r="S726" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T726" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U726" t="inlineStr"/>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F727" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G727" t="n">
+        <v>1574668652</v>
+      </c>
+      <c r="H727" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I727" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J727" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K727" t="n">
+        <v>0</v>
+      </c>
+      <c r="L727" t="b">
+        <v>1</v>
+      </c>
+      <c r="M727" t="n">
+        <v>4.05333</v>
+      </c>
+      <c r="N727" t="n">
+        <v>75</v>
+      </c>
+      <c r="O727" t="n">
+        <v>13</v>
+      </c>
+      <c r="P727" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R727" t="inlineStr">
+        <is>
+          <t>6.0.35</t>
+        </is>
+      </c>
+      <c r="S727" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T727" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U727" t="inlineStr"/>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F728" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G728" t="inlineStr">
+        <is>
+          <t>com.orange.sugu.ocd</t>
+        </is>
+      </c>
+      <c r="H728" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I728" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J728" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K728" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L728" t="b">
+        <v>0</v>
+      </c>
+      <c r="M728" t="n">
+        <v>4.13371</v>
+      </c>
+      <c r="N728" t="n">
+        <v>5309</v>
+      </c>
+      <c r="O728" t="n">
+        <v>79</v>
+      </c>
+      <c r="P728" t="inlineStr"/>
+      <c r="Q728" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R728" t="inlineStr">
+        <is>
+          <t>9.0.12</t>
+        </is>
+      </c>
+      <c r="S728" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DRC that brings together the features of MyOrange, and Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Plans, Mobile Payments, money transfers, bill payments, subscriptions, and entertai</t>
+        </is>
+      </c>
+      <c r="T728" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U728" t="inlineStr"/>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F729" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G729" t="n">
+        <v>6447896435</v>
+      </c>
+      <c r="H729" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I729" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J729" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K729" t="n">
+        <v>0</v>
+      </c>
+      <c r="L729" t="b">
+        <v>1</v>
+      </c>
+      <c r="M729" t="n">
+        <v>3.55762</v>
+      </c>
+      <c r="N729" t="n">
+        <v>269</v>
+      </c>
+      <c r="P729" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "CD" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R729" t="inlineStr">
+        <is>
+          <t>9.0.6</t>
+        </is>
+      </c>
+      <c r="S729" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DR Congo. It brings together the features of Orange et Moi, as well as Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Packages, Mobile payment, money transfers, bill payment and subscri</t>
+        </is>
+      </c>
+      <c r="T729" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U729" t="inlineStr"/>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F730" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G730" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ocm</t>
+        </is>
+      </c>
+      <c r="H730" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroon</t>
+        </is>
+      </c>
+      <c r="I730" t="inlineStr">
+        <is>
+          <t>Orange MEA</t>
+        </is>
+      </c>
+      <c r="J730" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K730" t="inlineStr">
+        <is>
+          <t>FCFA 0</t>
+        </is>
+      </c>
+      <c r="L730" t="b">
+        <v>0</v>
+      </c>
+      <c r="M730" t="n">
+        <v>3.9275208</v>
+      </c>
+      <c r="N730" t="n">
+        <v>46956</v>
+      </c>
+      <c r="O730" t="n">
+        <v>12</v>
+      </c>
+      <c r="P730" t="inlineStr"/>
+      <c r="Q730" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R730" t="inlineStr">
+        <is>
+          <t>7.0.23</t>
+        </is>
+      </c>
+      <c r="S730" t="inlineStr">
+        <is>
+          <t>Max it brings together everything that matters to you in one app: managing your lines, money transfer, bill payment, exclusive offers, and a universe of lifestyle and entertainment. Simple, fast, and 100% secure..&lt;br&gt;&lt;br&gt;📞 My line&lt;br&gt;Manage your Orange mobile and landline bundles in a single click:</t>
+        </is>
+      </c>
+      <c r="T730" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U730" t="inlineStr"/>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F731" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G731" t="n">
+        <v>1116920093</v>
+      </c>
+      <c r="H731" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroun</t>
+        </is>
+      </c>
+      <c r="I731" t="inlineStr">
+        <is>
+          <t>Orange Middle East &amp; Africa</t>
+        </is>
+      </c>
+      <c r="J731" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K731" t="n">
+        <v>0</v>
+      </c>
+      <c r="L731" t="b">
+        <v>1</v>
+      </c>
+      <c r="M731" t="n">
+        <v>3.76859</v>
+      </c>
+      <c r="N731" t="n">
+        <v>16162</v>
+      </c>
+      <c r="O731" t="n">
+        <v>3</v>
+      </c>
+      <c r="P731" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R731" t="inlineStr">
+        <is>
+          <t>7.0.24</t>
+        </is>
+      </c>
+      <c r="S731" t="inlineStr">
+        <is>
+          <t>Avec Max it, Orange rassemble tout ce qui compte pour vous dans une même application : la gestion de vos lignes, les transferts d’argent, payement de vos factures, des offres exclusives et un univers lifestyle et divertissement.
+Simple, rapide et 100 % sécurisée.
+Ma ligne
+Gérez vos forfaits mobiles</t>
+        </is>
+      </c>
+      <c r="T731" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U731" t="inlineStr"/>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F732" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G732" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obf</t>
+        </is>
+      </c>
+      <c r="H732" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I732" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso</t>
+        </is>
+      </c>
+      <c r="J732" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K732" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L732" t="b">
+        <v>0</v>
+      </c>
+      <c r="M732" t="n">
+        <v>4.1388345</v>
+      </c>
+      <c r="N732" t="n">
+        <v>25497</v>
+      </c>
+      <c r="O732" t="n">
+        <v>10</v>
+      </c>
+      <c r="P732" t="inlineStr"/>
+      <c r="Q732" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R732" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S732" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.&lt;br&gt;Gérez vos lignes mobiles, effectuez des transferts d&amp;#39;argent sécurisés, réglez vos factures, profitez d&amp;#39;offres exclusives, effectuez des paiements marchands fiables, et bien plus enco</t>
+        </is>
+      </c>
+      <c r="T732" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U732" t="inlineStr"/>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F733" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G733" t="n">
+        <v>1553774707</v>
+      </c>
+      <c r="H733" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I733" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso SA</t>
+        </is>
+      </c>
+      <c r="J733" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K733" t="n">
+        <v>0</v>
+      </c>
+      <c r="L733" t="b">
+        <v>1</v>
+      </c>
+      <c r="M733" t="n">
+        <v>3.45377</v>
+      </c>
+      <c r="N733" t="n">
+        <v>1179</v>
+      </c>
+      <c r="O733" t="n">
+        <v>3</v>
+      </c>
+      <c r="P733" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R733" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S733" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.
+Gérez vos lignes mobiles, effectuez des transferts d'argent sécurisés, réglez vos factures, profitez d'offres exclusives, effectuez des paiements marchands fiables, et bien plus encore, le tout</t>
+        </is>
+      </c>
+      <c r="T733" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U733" t="inlineStr"/>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F734" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G734" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obw</t>
+        </is>
+      </c>
+      <c r="H734" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I734" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J734" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K734" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L734" t="b">
+        <v>0</v>
+      </c>
+      <c r="M734" t="n">
+        <v>3.9819496</v>
+      </c>
+      <c r="N734" t="n">
+        <v>2964</v>
+      </c>
+      <c r="O734" t="n">
+        <v>32</v>
+      </c>
+      <c r="P734" t="inlineStr"/>
+      <c r="Q734" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R734" t="inlineStr">
+        <is>
+          <t>7.3.8</t>
+        </is>
+      </c>
+      <c r="S734" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it, the brand-new Orange Botswana Super App that follows Yame and gives you access to four distinct universes for a one-of-a-kind experience!&lt;br&gt;&lt;br&gt;Manage your accounts, make quick payments using QR codes, investigate a range of online goods and services, and discover the many options provided </t>
+        </is>
+      </c>
+      <c r="T734" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U734" t="inlineStr"/>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F735" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G735" t="n">
+        <v>1195839458</v>
+      </c>
+      <c r="H735" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I735" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J735" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K735" t="n">
+        <v>0</v>
+      </c>
+      <c r="L735" t="b">
+        <v>1</v>
+      </c>
+      <c r="M735" t="n">
+        <v>3.00806</v>
+      </c>
+      <c r="N735" t="n">
+        <v>124</v>
+      </c>
+      <c r="O735" t="n">
+        <v>22</v>
+      </c>
+      <c r="P735" t="inlineStr"/>
+      <c r="R735" t="inlineStr">
+        <is>
+          <t>7.3.1</t>
+        </is>
+      </c>
+      <c r="S735" t="inlineStr">
+        <is>
+          <t>A free mobile self-care application for Orange Botswana’s mobile customers.
+Full Description :
+Max it is a free application, which allows Orange Botswana customers to:
+- Consult your account in real time: minutes, sms, internet ...
+- Top up your account or a friend account  with Orange Money
+-</t>
+        </is>
+      </c>
+      <c r="T735" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U735" t="inlineStr"/>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F736" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G736" t="inlineStr">
+        <is>
+          <t>com.orange.mobinilandme</t>
+        </is>
+      </c>
+      <c r="H736" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I736" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J736" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K736" t="inlineStr">
+        <is>
+          <t>EGP 0.00</t>
+        </is>
+      </c>
+      <c r="L736" t="b">
+        <v>0</v>
+      </c>
+      <c r="M736" t="n">
+        <v>4.5589666</v>
+      </c>
+      <c r="N736" t="n">
+        <v>931170</v>
+      </c>
+      <c r="O736" t="n">
+        <v>17</v>
+      </c>
+      <c r="P736" t="inlineStr"/>
+      <c r="Q736" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R736" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S736" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion&lt;br&gt;Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.&lt;br&gt;Key services include:&lt;br&gt;• Account Management: Easily manage</t>
+        </is>
+      </c>
+      <c r="T736" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U736" t="inlineStr"/>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>1e5467ff-3c7b-4fc3-9436-44547d5dc06a</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>2026-07-30 06:29:56</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F737" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G737" t="n">
+        <v>942568333</v>
+      </c>
+      <c r="H737" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I737" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J737" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K737" t="n">
+        <v>0</v>
+      </c>
+      <c r="L737" t="b">
+        <v>1</v>
+      </c>
+      <c r="M737" t="n">
+        <v>4.25253</v>
+      </c>
+      <c r="N737" t="n">
+        <v>117917</v>
+      </c>
+      <c r="O737" t="n">
+        <v>53</v>
+      </c>
+      <c r="P737" t="inlineStr"/>
+      <c r="R737" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S737" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion
+Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.
+Key services include:
+• Account Management: Easily manage your Ora</t>
+        </is>
+      </c>
+      <c r="T737" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U737" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-07-31
</commit_message>
<xml_diff>
--- a/maxit_store_history.xlsx
+++ b/maxit_store_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U737"/>
+  <dimension ref="A1:U769"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -60703,7 +60703,6 @@
       <c r="O706" t="n">
         <v>35</v>
       </c>
-      <c r="P706" t="inlineStr"/>
       <c r="Q706" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -60724,7 +60723,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U706" t="inlineStr"/>
     </row>
     <row r="707">
       <c r="A707" t="inlineStr">
@@ -60787,7 +60785,6 @@
       <c r="N707" t="n">
         <v>324</v>
       </c>
-      <c r="P707" t="inlineStr"/>
       <c r="R707" t="inlineStr">
         <is>
           <t>6.4.8</t>
@@ -60803,7 +60800,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U707" t="inlineStr"/>
     </row>
     <row r="708">
       <c r="A708" t="inlineStr">
@@ -60873,7 +60869,6 @@
       <c r="O708" t="n">
         <v>31</v>
       </c>
-      <c r="P708" t="inlineStr"/>
       <c r="Q708" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -60894,7 +60889,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U708" t="inlineStr"/>
     </row>
     <row r="709">
       <c r="A709" t="inlineStr">
@@ -60960,7 +60954,6 @@
       <c r="O709" t="n">
         <v>47</v>
       </c>
-      <c r="P709" t="inlineStr"/>
       <c r="R709" t="inlineStr">
         <is>
           <t>10.0.7</t>
@@ -60978,7 +60971,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U709" t="inlineStr"/>
     </row>
     <row r="710">
       <c r="A710" t="inlineStr">
@@ -61048,7 +61040,6 @@
       <c r="O710" t="n">
         <v>10</v>
       </c>
-      <c r="P710" t="inlineStr"/>
       <c r="Q710" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -61069,7 +61060,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U710" t="inlineStr"/>
     </row>
     <row r="711">
       <c r="A711" t="inlineStr">
@@ -61158,7 +61148,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U711" t="inlineStr"/>
     </row>
     <row r="712">
       <c r="A712" t="inlineStr">
@@ -61228,7 +61217,6 @@
       <c r="O712" t="n">
         <v>10</v>
       </c>
-      <c r="P712" t="inlineStr"/>
       <c r="Q712" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -61249,7 +61237,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U712" t="inlineStr"/>
     </row>
     <row r="713">
       <c r="A713" t="inlineStr">
@@ -61315,7 +61302,6 @@
       <c r="O713" t="n">
         <v>2</v>
       </c>
-      <c r="P713" t="inlineStr"/>
       <c r="R713" t="inlineStr">
         <is>
           <t>22.0.0</t>
@@ -61333,7 +61319,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U713" t="inlineStr"/>
     </row>
     <row r="714">
       <c r="A714" t="inlineStr">
@@ -61403,7 +61388,6 @@
       <c r="O714" t="n">
         <v>104</v>
       </c>
-      <c r="P714" t="inlineStr"/>
       <c r="Q714" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -61424,7 +61408,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U714" t="inlineStr"/>
     </row>
     <row r="715">
       <c r="A715" t="inlineStr">
@@ -61509,7 +61492,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U715" t="inlineStr"/>
     </row>
     <row r="716">
       <c r="A716" t="inlineStr">
@@ -61576,7 +61558,6 @@
       <c r="N716" t="n">
         <v>38250</v>
       </c>
-      <c r="P716" t="inlineStr"/>
       <c r="Q716" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -61597,7 +61578,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U716" t="inlineStr"/>
     </row>
     <row r="717">
       <c r="A717" t="inlineStr">
@@ -61663,7 +61643,6 @@
       <c r="O717" t="n">
         <v>14</v>
       </c>
-      <c r="P717" t="inlineStr"/>
       <c r="R717" t="inlineStr">
         <is>
           <t>6.5.2</t>
@@ -61682,7 +61661,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U717" t="inlineStr"/>
     </row>
     <row r="718">
       <c r="A718" t="inlineStr">
@@ -61752,7 +61730,6 @@
       <c r="O718" t="n">
         <v>55</v>
       </c>
-      <c r="P718" t="inlineStr"/>
       <c r="Q718" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -61773,7 +61750,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U718" t="inlineStr"/>
     </row>
     <row r="719">
       <c r="A719" t="inlineStr">
@@ -61839,7 +61815,6 @@
       <c r="O719" t="n">
         <v>20</v>
       </c>
-      <c r="P719" t="inlineStr"/>
       <c r="R719" t="inlineStr">
         <is>
           <t>5.0.2</t>
@@ -61857,7 +61832,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U719" t="inlineStr"/>
     </row>
     <row r="720">
       <c r="A720" t="inlineStr">
@@ -61927,7 +61901,6 @@
       <c r="O720" t="n">
         <v>108</v>
       </c>
-      <c r="P720" t="inlineStr"/>
       <c r="Q720" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -61948,7 +61921,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U720" t="inlineStr"/>
     </row>
     <row r="721">
       <c r="A721" t="inlineStr">
@@ -62036,7 +62008,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U721" t="inlineStr"/>
     </row>
     <row r="722">
       <c r="A722" t="inlineStr">
@@ -62106,7 +62077,6 @@
       <c r="O722" t="n">
         <v>41</v>
       </c>
-      <c r="P722" t="inlineStr"/>
       <c r="Q722" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -62127,7 +62097,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U722" t="inlineStr"/>
     </row>
     <row r="723">
       <c r="A723" t="inlineStr">
@@ -62193,7 +62162,6 @@
       <c r="O723" t="n">
         <v>42</v>
       </c>
-      <c r="P723" t="inlineStr"/>
       <c r="R723" t="inlineStr">
         <is>
           <t>10.0.21</t>
@@ -62212,7 +62180,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U723" t="inlineStr"/>
     </row>
     <row r="724">
       <c r="A724" t="inlineStr">
@@ -62282,7 +62249,6 @@
       <c r="O724" t="n">
         <v>11</v>
       </c>
-      <c r="P724" t="inlineStr"/>
       <c r="Q724" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -62303,7 +62269,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U724" t="inlineStr"/>
     </row>
     <row r="725">
       <c r="A725" t="inlineStr">
@@ -62389,7 +62354,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U725" t="inlineStr"/>
     </row>
     <row r="726">
       <c r="A726" t="inlineStr">
@@ -62459,7 +62423,6 @@
       <c r="O726" t="n">
         <v>4</v>
       </c>
-      <c r="P726" t="inlineStr"/>
       <c r="Q726" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -62480,7 +62443,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U726" t="inlineStr"/>
     </row>
     <row r="727">
       <c r="A727" t="inlineStr">
@@ -62566,7 +62528,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U727" t="inlineStr"/>
     </row>
     <row r="728">
       <c r="A728" t="inlineStr">
@@ -62636,7 +62597,6 @@
       <c r="O728" t="n">
         <v>79</v>
       </c>
-      <c r="P728" t="inlineStr"/>
       <c r="Q728" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -62657,7 +62617,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U728" t="inlineStr"/>
     </row>
     <row r="729">
       <c r="A729" t="inlineStr">
@@ -62740,7 +62699,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U729" t="inlineStr"/>
     </row>
     <row r="730">
       <c r="A730" t="inlineStr">
@@ -62810,7 +62768,6 @@
       <c r="O730" t="n">
         <v>12</v>
       </c>
-      <c r="P730" t="inlineStr"/>
       <c r="Q730" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -62831,7 +62788,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U730" t="inlineStr"/>
     </row>
     <row r="731">
       <c r="A731" t="inlineStr">
@@ -62920,7 +62876,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U731" t="inlineStr"/>
     </row>
     <row r="732">
       <c r="A732" t="inlineStr">
@@ -62990,7 +62945,6 @@
       <c r="O732" t="n">
         <v>10</v>
       </c>
-      <c r="P732" t="inlineStr"/>
       <c r="Q732" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -63011,7 +62965,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U732" t="inlineStr"/>
     </row>
     <row r="733">
       <c r="A733" t="inlineStr">
@@ -63098,7 +63051,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U733" t="inlineStr"/>
     </row>
     <row r="734">
       <c r="A734" t="inlineStr">
@@ -63168,7 +63120,6 @@
       <c r="O734" t="n">
         <v>32</v>
       </c>
-      <c r="P734" t="inlineStr"/>
       <c r="Q734" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -63189,7 +63140,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U734" t="inlineStr"/>
     </row>
     <row r="735">
       <c r="A735" t="inlineStr">
@@ -63255,7 +63205,6 @@
       <c r="O735" t="n">
         <v>22</v>
       </c>
-      <c r="P735" t="inlineStr"/>
       <c r="R735" t="inlineStr">
         <is>
           <t>7.3.1</t>
@@ -63276,7 +63225,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U735" t="inlineStr"/>
     </row>
     <row r="736">
       <c r="A736" t="inlineStr">
@@ -63346,7 +63294,6 @@
       <c r="O736" t="n">
         <v>17</v>
       </c>
-      <c r="P736" t="inlineStr"/>
       <c r="Q736" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -63367,7 +63314,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U736" t="inlineStr"/>
     </row>
     <row r="737">
       <c r="A737" t="inlineStr">
@@ -63433,7 +63379,6 @@
       <c r="O737" t="n">
         <v>53</v>
       </c>
-      <c r="P737" t="inlineStr"/>
       <c r="R737" t="inlineStr">
         <is>
           <t>10.1.0</t>
@@ -63452,7 +63397,2825 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U737" t="inlineStr"/>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F738" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G738" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogn</t>
+        </is>
+      </c>
+      <c r="H738" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I738" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J738" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K738" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L738" t="b">
+        <v>0</v>
+      </c>
+      <c r="M738" t="n">
+        <v>4.4438386</v>
+      </c>
+      <c r="N738" t="n">
+        <v>9330</v>
+      </c>
+      <c r="O738" t="n">
+        <v>34</v>
+      </c>
+      <c r="P738" t="inlineStr"/>
+      <c r="Q738" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R738" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S738" t="inlineStr">
+        <is>
+          <t>Bien plus qu&amp;#39;une application, un véritable assistant personnel pour une vie connectée et simplifiée.&lt;br&gt;Suivi de consommation: Votre tableau de bord tout-en-un pour une gestion simplifiée !&lt;br&gt;- Gestion de votre offre: Accédez à une vue détaillée de votre offre actuelle et de vos forfaits Orange</t>
+        </is>
+      </c>
+      <c r="T738" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U738" t="inlineStr"/>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D739" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E739" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F739" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G739" t="n">
+        <v>1177999485</v>
+      </c>
+      <c r="H739" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I739" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J739" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K739" t="n">
+        <v>0</v>
+      </c>
+      <c r="L739" t="b">
+        <v>1</v>
+      </c>
+      <c r="M739" t="n">
+        <v>3.88272</v>
+      </c>
+      <c r="N739" t="n">
+        <v>324</v>
+      </c>
+      <c r="P739" t="inlineStr"/>
+      <c r="R739" t="inlineStr">
+        <is>
+          <t>6.4.8</t>
+        </is>
+      </c>
+      <c r="S739" t="inlineStr">
+        <is>
+          <t>La fusion d’Orange et Moi et Orange Money donne naissance à Max it, la nouvelle Super Application Tout-en-Un. Profitez du suivi de consommation, de paiements mobiles, de toutes les fonctionnalités Orange et Moi et Money avec un large éventail de divertissements, le tout regroupé en un seul endroit !</t>
+        </is>
+      </c>
+      <c r="T739" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U739" t="inlineStr"/>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E740" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F740" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G740" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.otn</t>
+        </is>
+      </c>
+      <c r="H740" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I740" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J740" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K740" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L740" t="b">
+        <v>0</v>
+      </c>
+      <c r="M740" t="n">
+        <v>3.9660614</v>
+      </c>
+      <c r="N740" t="n">
+        <v>35386</v>
+      </c>
+      <c r="O740" t="n">
+        <v>30</v>
+      </c>
+      <c r="P740" t="inlineStr"/>
+      <c r="Q740" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R740" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S740" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Max it par Orange Tunisie facilite votre vie au quotidien !&lt;/h2&gt;&lt;br&gt;&lt;br&gt;Welcome sur Max it !&lt;br&gt;Accédez rapidement à vos fonctionnalités Max it préférées et profitez également de contenus exclusifs, d’activités divertissantes, et de jeux interactifs pour une expérience enrichissante avec la roue</t>
+        </is>
+      </c>
+      <c r="T740" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U740" t="inlineStr"/>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D741" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E741" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F741" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G741" t="n">
+        <v>1146892088</v>
+      </c>
+      <c r="H741" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I741" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J741" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K741" t="n">
+        <v>0</v>
+      </c>
+      <c r="L741" t="b">
+        <v>1</v>
+      </c>
+      <c r="M741" t="n">
+        <v>3.03049</v>
+      </c>
+      <c r="N741" t="n">
+        <v>1640</v>
+      </c>
+      <c r="O741" t="n">
+        <v>42</v>
+      </c>
+      <c r="P741" t="inlineStr"/>
+      <c r="R741" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S741" t="inlineStr">
+        <is>
+          <t>Max it by Orange Tunisie : Votre appli incontournable pour une vie connectée
+Welcome sur Max it : Découvrez fonctionnalités, jeux &amp; contenus de divertissement by Orange Tunisie !
+Trouvez vite vos fonctionnalités Max it favorites et explorez des contenus exclusifs et des jeux pour une expérience im</t>
+        </is>
+      </c>
+      <c r="T741" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U741" t="inlineStr"/>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E742" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F742" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G742" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osl</t>
+        </is>
+      </c>
+      <c r="H742" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I742" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J742" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K742" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L742" t="b">
+        <v>0</v>
+      </c>
+      <c r="M742" t="n">
+        <v>4.4139533</v>
+      </c>
+      <c r="N742" t="n">
+        <v>2142</v>
+      </c>
+      <c r="O742" t="n">
+        <v>10</v>
+      </c>
+      <c r="P742" t="inlineStr"/>
+      <c r="Q742" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R742" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S742" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it is a free application, which allows Orange Sierra Leone prepaid and postpaid customers to:&lt;br&gt;&lt;br&gt;- Consult your account in real time: minutes, sms, internet&lt;br&gt;- Top up your account or a friend account &lt;br&gt;- Buy Internet Bundles&lt;br&gt;- Discover the latest offers and promotions &lt;br&gt;- Access to </t>
+        </is>
+      </c>
+      <c r="T742" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U742" t="inlineStr"/>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E743" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F743" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G743" t="n">
+        <v>6443607903</v>
+      </c>
+      <c r="H743" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I743" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J743" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K743" t="n">
+        <v>0</v>
+      </c>
+      <c r="L743" t="b">
+        <v>1</v>
+      </c>
+      <c r="M743" t="n">
+        <v>3.69948</v>
+      </c>
+      <c r="N743" t="n">
+        <v>193</v>
+      </c>
+      <c r="O743" t="n">
+        <v>6</v>
+      </c>
+      <c r="P743" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R743" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S743" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The merger of My Orange &amp; Orange Money has given birth to Max it the all-in-one super app, a free application which allows all Orange Sierra Leone customers to 
+Track calls, SMS, and Data usage and monitor balance. 
+Make a secure mobile/Orange Money payment.
+Easily transfer credit to other users </t>
+        </is>
+      </c>
+      <c r="T743" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U743" t="inlineStr"/>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E744" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F744" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G744" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osn</t>
+        </is>
+      </c>
+      <c r="H744" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I744" t="inlineStr">
+        <is>
+          <t>Orange Sénégal</t>
+        </is>
+      </c>
+      <c r="J744" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K744" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L744" t="b">
+        <v>0</v>
+      </c>
+      <c r="M744" t="n">
+        <v>4.2990885</v>
+      </c>
+      <c r="N744" t="n">
+        <v>51289</v>
+      </c>
+      <c r="O744" t="n">
+        <v>10</v>
+      </c>
+      <c r="P744" t="inlineStr"/>
+      <c r="Q744" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R744" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S744" t="inlineStr">
+        <is>
+          <t>Lu bees ak Max it ! &lt;br&gt;Une application repensée pour être plus simple, plus rapide et adaptée à vos besoins. Une expérience optimisée pour faciliter vos usages au quotidien, avec des parcours simplifiés et un accès plus fluide à vos services. Que vous soyez client Orange ou non, Max it vous accompa</t>
+        </is>
+      </c>
+      <c r="T744" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U744" t="inlineStr"/>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E745" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F745" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G745" t="n">
+        <v>1039327980</v>
+      </c>
+      <c r="H745" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I745" t="inlineStr">
+        <is>
+          <t>Orange Senegal</t>
+        </is>
+      </c>
+      <c r="J745" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K745" t="n">
+        <v>0</v>
+      </c>
+      <c r="L745" t="b">
+        <v>1</v>
+      </c>
+      <c r="M745" t="n">
+        <v>4.16932</v>
+      </c>
+      <c r="N745" t="n">
+        <v>30227</v>
+      </c>
+      <c r="O745" t="n">
+        <v>2</v>
+      </c>
+      <c r="P745" t="inlineStr"/>
+      <c r="R745" t="inlineStr">
+        <is>
+          <t>22.0.0</t>
+        </is>
+      </c>
+      <c r="S745" t="inlineStr">
+        <is>
+          <t>Here is the English translation:
+Welcome to Max it!
+A redesigned app to be simpler, faster, and tailored to your needs. An optimized experience to make your daily life easier, with streamlined journeys and smoother access to your services. Whether you are an Orange customer or not, Max it is your e</t>
+        </is>
+      </c>
+      <c r="T745" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U745" t="inlineStr"/>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E746" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F746" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G746" t="inlineStr">
+        <is>
+          <t>com.orange.meditel.mediteletmoi</t>
+        </is>
+      </c>
+      <c r="H746" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I746" t="inlineStr">
+        <is>
+          <t>Orange Maroc</t>
+        </is>
+      </c>
+      <c r="J746" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K746" t="inlineStr">
+        <is>
+          <t>MAD 0.00</t>
+        </is>
+      </c>
+      <c r="L746" t="b">
+        <v>0</v>
+      </c>
+      <c r="M746" t="n">
+        <v>3.719255</v>
+      </c>
+      <c r="N746" t="n">
+        <v>110919</v>
+      </c>
+      <c r="O746" t="n">
+        <v>80</v>
+      </c>
+      <c r="P746" t="inlineStr"/>
+      <c r="Q746" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R746" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S746" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l&amp;#39;expérience mobile réinventé&lt;br&gt;&lt;br&gt;Max it, c&amp;#39;est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d&amp;#39;une multitude de services exclusifs. &lt;br&gt;&lt;br&gt;Créez votre espace sur</t>
+        </is>
+      </c>
+      <c r="T746" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U746" t="inlineStr"/>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E747" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F747" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G747" t="n">
+        <v>596028698</v>
+      </c>
+      <c r="H747" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I747" t="inlineStr">
+        <is>
+          <t>Méditel</t>
+        </is>
+      </c>
+      <c r="J747" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K747" t="n">
+        <v>0</v>
+      </c>
+      <c r="L747" t="b">
+        <v>1</v>
+      </c>
+      <c r="M747" t="n">
+        <v>3.94561</v>
+      </c>
+      <c r="N747" t="n">
+        <v>2758</v>
+      </c>
+      <c r="P747" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "MA" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R747" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S747" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l'expérience mobile réinventé
+Max it, c'est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d'une multitude de services exclusifs. 
+Créez votre espace sur mesure et bénéficiez d'</t>
+        </is>
+      </c>
+      <c r="T747" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U747" t="inlineStr"/>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E748" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F748" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G748" t="inlineStr">
+        <is>
+          <t>com.oml.dsi.orangemobile</t>
+        </is>
+      </c>
+      <c r="H748" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I748" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J748" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K748" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L748" t="b">
+        <v>0</v>
+      </c>
+      <c r="M748" t="n">
+        <v>2.7071838</v>
+      </c>
+      <c r="N748" t="n">
+        <v>38243</v>
+      </c>
+      <c r="P748" t="inlineStr"/>
+      <c r="Q748" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R748" t="inlineStr">
+        <is>
+          <t>6.5.0</t>
+        </is>
+      </c>
+      <c r="S748" t="inlineStr">
+        <is>
+          <t>Easily manage your Orange Mali line&lt;br&gt;● Manage your account and view all essential information, your offers, and your phone lines.&lt;br&gt;● Subscribe to call, SMS, Internet, and international call packages.&lt;br&gt;● Track your usage by checking your credit and Internet balance.&lt;br&gt;● Recharge your line by p</t>
+        </is>
+      </c>
+      <c r="T748" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U748" t="inlineStr"/>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F749" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G749" t="n">
+        <v>1494321079</v>
+      </c>
+      <c r="H749" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I749" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J749" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K749" t="n">
+        <v>0</v>
+      </c>
+      <c r="L749" t="b">
+        <v>1</v>
+      </c>
+      <c r="M749" t="n">
+        <v>2.5224</v>
+      </c>
+      <c r="N749" t="n">
+        <v>4755</v>
+      </c>
+      <c r="O749" t="n">
+        <v>14</v>
+      </c>
+      <c r="P749" t="inlineStr"/>
+      <c r="R749" t="inlineStr">
+        <is>
+          <t>6.5.2</t>
+        </is>
+      </c>
+      <c r="S749" t="inlineStr">
+        <is>
+          <t>Gérez facilement votre ligne Orange Mali 
+●        Gérez votre compte et consultez toutes les informations essentielles sur celui-ci, vos offres, ainsi que vos lignes téléphoniques.
+●        Souscrivez aux forfaits appels, SMS, Internet, et appels internationaux.
+●        Suivez votre consommation e</t>
+        </is>
+      </c>
+      <c r="T749" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U749" t="inlineStr"/>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F750" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G750" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.omg</t>
+        </is>
+      </c>
+      <c r="H750" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I750" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J750" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K750" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L750" t="b">
+        <v>0</v>
+      </c>
+      <c r="M750" t="n">
+        <v>4.126866</v>
+      </c>
+      <c r="N750" t="n">
+        <v>1378</v>
+      </c>
+      <c r="O750" t="n">
+        <v>51</v>
+      </c>
+      <c r="P750" t="inlineStr"/>
+      <c r="Q750" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R750" t="inlineStr">
+        <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="S750" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.&lt;br&gt;&lt;br&gt;Simplify Your Life with Max it&lt;br&gt;With Max It, ac</t>
+        </is>
+      </c>
+      <c r="T750" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U750" t="inlineStr"/>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E751" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F751" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G751" t="n">
+        <v>1295171817</v>
+      </c>
+      <c r="H751" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I751" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J751" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K751" t="n">
+        <v>0</v>
+      </c>
+      <c r="L751" t="b">
+        <v>1</v>
+      </c>
+      <c r="M751" t="n">
+        <v>3.08696</v>
+      </c>
+      <c r="N751" t="n">
+        <v>69</v>
+      </c>
+      <c r="O751" t="n">
+        <v>21</v>
+      </c>
+      <c r="P751" t="inlineStr"/>
+      <c r="R751" t="inlineStr">
+        <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="S751" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.
+Simplify Your Life with Max it
+With Max it, access a se</t>
+        </is>
+      </c>
+      <c r="T751" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U751" t="inlineStr"/>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F752" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G752" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.olr</t>
+        </is>
+      </c>
+      <c r="H752" t="inlineStr">
+        <is>
+          <t>Orange Max it - Liberia</t>
+        </is>
+      </c>
+      <c r="I752" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J752" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K752" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L752" t="b">
+        <v>0</v>
+      </c>
+      <c r="M752" t="n">
+        <v>4.5352564</v>
+      </c>
+      <c r="N752" t="n">
+        <v>3101</v>
+      </c>
+      <c r="O752" t="n">
+        <v>81</v>
+      </c>
+      <c r="P752" t="inlineStr"/>
+      <c r="Q752" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R752" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="S752" t="inlineStr">
+        <is>
+          <t>Max it: your personalized experience by Orange Liberia!&lt;br&gt;&lt;br&gt;Step into Max it, your all-in-one solution for telecom, marketplace, and financial services! Manage your mobile line, customize offers, pay your bills, keep&lt;br&gt;track of your usage with ease, and recharge your credit. Access exclusive eve</t>
+        </is>
+      </c>
+      <c r="T752" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U752" t="inlineStr"/>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F753" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G753" t="n">
+        <v>6746187327</v>
+      </c>
+      <c r="H753" t="inlineStr">
+        <is>
+          <t>Orange Max it – Liberia</t>
+        </is>
+      </c>
+      <c r="I753" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J753" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K753" t="n">
+        <v>0</v>
+      </c>
+      <c r="L753" t="b">
+        <v>1</v>
+      </c>
+      <c r="M753" t="n">
+        <v>4.0625</v>
+      </c>
+      <c r="N753" t="n">
+        <v>48</v>
+      </c>
+      <c r="P753" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "LR" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R753" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="S753" t="inlineStr">
+        <is>
+          <t>Max it is a free application, which allows Orange Liberia customers to:
+- Consult your account in real time: minutes, sms, internet
+- Top up your account or a friend account 
+- Buy  Bundles (voice, data, SMS, roaming, international)
+- Discover the latest offers and promotions 
+- Access to Orange se</t>
+        </is>
+      </c>
+      <c r="T753" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U753" t="inlineStr"/>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F754" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G754" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ojo</t>
+        </is>
+      </c>
+      <c r="H754" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I754" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J754" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K754" t="inlineStr">
+        <is>
+          <t>JOD 0.000</t>
+        </is>
+      </c>
+      <c r="L754" t="b">
+        <v>0</v>
+      </c>
+      <c r="M754" t="n">
+        <v>4.4322906</v>
+      </c>
+      <c r="N754" t="n">
+        <v>97777</v>
+      </c>
+      <c r="O754" t="n">
+        <v>45</v>
+      </c>
+      <c r="P754" t="inlineStr"/>
+      <c r="Q754" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R754" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S754" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience&lt;br&gt;Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.&lt;br&gt;Important Update:&lt;br&gt;The jood app (jood Orange) w</t>
+        </is>
+      </c>
+      <c r="T754" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U754" t="inlineStr"/>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F755" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G755" t="n">
+        <v>808824590</v>
+      </c>
+      <c r="H755" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I755" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J755" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K755" t="n">
+        <v>0</v>
+      </c>
+      <c r="L755" t="b">
+        <v>1</v>
+      </c>
+      <c r="M755" t="n">
+        <v>4.20638</v>
+      </c>
+      <c r="N755" t="n">
+        <v>3043</v>
+      </c>
+      <c r="O755" t="n">
+        <v>47</v>
+      </c>
+      <c r="P755" t="inlineStr"/>
+      <c r="R755" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S755" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience
+Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.
+Important Update:
+The jood app (jood Orange) will be di</t>
+        </is>
+      </c>
+      <c r="T755" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U755" t="inlineStr"/>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E756" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F756" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G756" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.oci</t>
+        </is>
+      </c>
+      <c r="H756" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I756" t="inlineStr">
+        <is>
+          <t>Orange Côte d'Ivoire S.A</t>
+        </is>
+      </c>
+      <c r="J756" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K756" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L756" t="b">
+        <v>0</v>
+      </c>
+      <c r="M756" t="n">
+        <v>4.1529884</v>
+      </c>
+      <c r="N756" t="n">
+        <v>67291</v>
+      </c>
+      <c r="O756" t="n">
+        <v>10</v>
+      </c>
+      <c r="P756" t="inlineStr"/>
+      <c r="Q756" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R756" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S756" t="inlineStr">
+        <is>
+          <t>Aaaahhh, ta super app Max it, n&amp;#39;a pas fini de te surprendre... &lt;br&gt;Est-ce que tu as remarqué ? Maintenant, tu as ton QR code personnalisé en haut de ton écran d&amp;#39;accueil ! Ainsi, tu peux :&lt;br&gt;     scanner le QR code de ton ami(e) pour lui faire un transfert d&amp;#39;&amp;#39;argent&lt;br&gt;     scanner l</t>
+        </is>
+      </c>
+      <c r="T756" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U756" t="inlineStr"/>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E757" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F757" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G757" t="n">
+        <v>1061120855</v>
+      </c>
+      <c r="H757" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I757" t="inlineStr">
+        <is>
+          <t>Orange CI</t>
+        </is>
+      </c>
+      <c r="J757" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K757" t="n">
+        <v>0</v>
+      </c>
+      <c r="L757" t="b">
+        <v>1</v>
+      </c>
+      <c r="M757" t="n">
+        <v>3.78557</v>
+      </c>
+      <c r="N757" t="n">
+        <v>5974</v>
+      </c>
+      <c r="O757" t="n">
+        <v>13</v>
+      </c>
+      <c r="P757" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R757" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S757" t="inlineStr">
+        <is>
+          <t>Max it, la super app all-in-one te fais gagner du temps, et diminue tes soucis... Gagne plus d'espace de stockage sur ton téléphone ; plus besoin de cumuler plusieurs appli d'Orange pour avoir accès à un maximum de services. Max it est là ! Gère ta ligne (SIM) au niveau des pass, des soldes, réalise</t>
+        </is>
+      </c>
+      <c r="T757" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U757" t="inlineStr"/>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D758" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E758" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F758" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G758" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogw</t>
+        </is>
+      </c>
+      <c r="H758" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I758" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J758" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K758" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L758" t="b">
+        <v>0</v>
+      </c>
+      <c r="M758" t="n">
+        <v>4.3896103</v>
+      </c>
+      <c r="N758" t="n">
+        <v>1539</v>
+      </c>
+      <c r="O758" t="n">
+        <v>4</v>
+      </c>
+      <c r="P758" t="inlineStr"/>
+      <c r="Q758" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R758" t="inlineStr">
+        <is>
+          <t>4.0.18</t>
+        </is>
+      </c>
+      <c r="S758" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T758" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U758" t="inlineStr"/>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D759" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E759" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F759" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G759" t="n">
+        <v>1574668652</v>
+      </c>
+      <c r="H759" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I759" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J759" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K759" t="n">
+        <v>0</v>
+      </c>
+      <c r="L759" t="b">
+        <v>1</v>
+      </c>
+      <c r="M759" t="n">
+        <v>4.05333</v>
+      </c>
+      <c r="N759" t="n">
+        <v>75</v>
+      </c>
+      <c r="O759" t="n">
+        <v>10</v>
+      </c>
+      <c r="P759" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R759" t="inlineStr">
+        <is>
+          <t>6.0.35</t>
+        </is>
+      </c>
+      <c r="S759" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T759" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U759" t="inlineStr"/>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D760" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E760" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F760" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G760" t="inlineStr">
+        <is>
+          <t>com.orange.sugu.ocd</t>
+        </is>
+      </c>
+      <c r="H760" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I760" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J760" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K760" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L760" t="b">
+        <v>0</v>
+      </c>
+      <c r="M760" t="n">
+        <v>4.1348314</v>
+      </c>
+      <c r="N760" t="n">
+        <v>5312</v>
+      </c>
+      <c r="O760" t="n">
+        <v>91</v>
+      </c>
+      <c r="P760" t="inlineStr"/>
+      <c r="Q760" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R760" t="inlineStr">
+        <is>
+          <t>9.0.12</t>
+        </is>
+      </c>
+      <c r="S760" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DRC that brings together the features of MyOrange, and Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Plans, Mobile Payments, money transfers, bill payments, subscriptions, and entertai</t>
+        </is>
+      </c>
+      <c r="T760" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U760" t="inlineStr"/>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D761" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E761" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F761" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G761" t="n">
+        <v>6447896435</v>
+      </c>
+      <c r="H761" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I761" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J761" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K761" t="n">
+        <v>0</v>
+      </c>
+      <c r="L761" t="b">
+        <v>1</v>
+      </c>
+      <c r="M761" t="n">
+        <v>3.56296</v>
+      </c>
+      <c r="N761" t="n">
+        <v>270</v>
+      </c>
+      <c r="P761" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "CD" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R761" t="inlineStr">
+        <is>
+          <t>9.0.6</t>
+        </is>
+      </c>
+      <c r="S761" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DR Congo. It brings together the features of Orange et Moi, as well as Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Packages, Mobile payment, money transfers, bill payment and subscri</t>
+        </is>
+      </c>
+      <c r="T761" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U761" t="inlineStr"/>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D762" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E762" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F762" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G762" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ocm</t>
+        </is>
+      </c>
+      <c r="H762" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroon</t>
+        </is>
+      </c>
+      <c r="I762" t="inlineStr">
+        <is>
+          <t>Orange MEA</t>
+        </is>
+      </c>
+      <c r="J762" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K762" t="inlineStr">
+        <is>
+          <t>FCFA 0</t>
+        </is>
+      </c>
+      <c r="L762" t="b">
+        <v>0</v>
+      </c>
+      <c r="M762" t="n">
+        <v>3.9252396</v>
+      </c>
+      <c r="N762" t="n">
+        <v>46987</v>
+      </c>
+      <c r="O762" t="n">
+        <v>11</v>
+      </c>
+      <c r="P762" t="inlineStr"/>
+      <c r="Q762" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R762" t="inlineStr">
+        <is>
+          <t>7.0.23</t>
+        </is>
+      </c>
+      <c r="S762" t="inlineStr">
+        <is>
+          <t>Max it brings together everything that matters to you in one app: managing your lines, money transfer, bill payment, exclusive offers, and a universe of lifestyle and entertainment. Simple, fast, and 100% secure..&lt;br&gt;&lt;br&gt;📞 My line&lt;br&gt;Manage your Orange mobile and landline bundles in a single click:</t>
+        </is>
+      </c>
+      <c r="T762" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U762" t="inlineStr"/>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D763" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E763" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F763" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G763" t="n">
+        <v>1116920093</v>
+      </c>
+      <c r="H763" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroun</t>
+        </is>
+      </c>
+      <c r="I763" t="inlineStr">
+        <is>
+          <t>Orange Middle East &amp; Africa</t>
+        </is>
+      </c>
+      <c r="J763" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K763" t="n">
+        <v>0</v>
+      </c>
+      <c r="L763" t="b">
+        <v>1</v>
+      </c>
+      <c r="M763" t="n">
+        <v>3.76839</v>
+      </c>
+      <c r="N763" t="n">
+        <v>16165</v>
+      </c>
+      <c r="O763" t="n">
+        <v>1</v>
+      </c>
+      <c r="P763" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R763" t="inlineStr">
+        <is>
+          <t>7.0.24</t>
+        </is>
+      </c>
+      <c r="S763" t="inlineStr">
+        <is>
+          <t>Avec Max it, Orange rassemble tout ce qui compte pour vous dans une même application : la gestion de vos lignes, les transferts d’argent, payement de vos factures, des offres exclusives et un univers lifestyle et divertissement.
+Simple, rapide et 100 % sécurisée.
+Ma ligne
+Gérez vos forfaits mobiles</t>
+        </is>
+      </c>
+      <c r="T763" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U763" t="inlineStr"/>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D764" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E764" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F764" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G764" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obf</t>
+        </is>
+      </c>
+      <c r="H764" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I764" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso</t>
+        </is>
+      </c>
+      <c r="J764" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K764" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L764" t="b">
+        <v>0</v>
+      </c>
+      <c r="M764" t="n">
+        <v>4.137324</v>
+      </c>
+      <c r="N764" t="n">
+        <v>25504</v>
+      </c>
+      <c r="O764" t="n">
+        <v>12</v>
+      </c>
+      <c r="P764" t="inlineStr"/>
+      <c r="Q764" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R764" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S764" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.&lt;br&gt;Gérez vos lignes mobiles, effectuez des transferts d&amp;#39;argent sécurisés, réglez vos factures, profitez d&amp;#39;offres exclusives, effectuez des paiements marchands fiables, et bien plus enco</t>
+        </is>
+      </c>
+      <c r="T764" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U764" t="inlineStr"/>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E765" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F765" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G765" t="n">
+        <v>1553774707</v>
+      </c>
+      <c r="H765" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I765" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso SA</t>
+        </is>
+      </c>
+      <c r="J765" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K765" t="n">
+        <v>0</v>
+      </c>
+      <c r="L765" t="b">
+        <v>1</v>
+      </c>
+      <c r="M765" t="n">
+        <v>3.45377</v>
+      </c>
+      <c r="N765" t="n">
+        <v>1179</v>
+      </c>
+      <c r="O765" t="n">
+        <v>9</v>
+      </c>
+      <c r="P765" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R765" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S765" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.
+Gérez vos lignes mobiles, effectuez des transferts d'argent sécurisés, réglez vos factures, profitez d'offres exclusives, effectuez des paiements marchands fiables, et bien plus encore, le tout</t>
+        </is>
+      </c>
+      <c r="T765" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U765" t="inlineStr"/>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D766" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E766" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F766" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G766" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obw</t>
+        </is>
+      </c>
+      <c r="H766" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I766" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J766" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K766" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L766" t="b">
+        <v>0</v>
+      </c>
+      <c r="M766" t="n">
+        <v>3.9784172</v>
+      </c>
+      <c r="N766" t="n">
+        <v>2965</v>
+      </c>
+      <c r="O766" t="n">
+        <v>25</v>
+      </c>
+      <c r="P766" t="inlineStr"/>
+      <c r="Q766" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R766" t="inlineStr">
+        <is>
+          <t>7.3.8</t>
+        </is>
+      </c>
+      <c r="S766" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it, the brand-new Orange Botswana Super App that follows Yame and gives you access to four distinct universes for a one-of-a-kind experience!&lt;br&gt;&lt;br&gt;Manage your accounts, make quick payments using QR codes, investigate a range of online goods and services, and discover the many options provided </t>
+        </is>
+      </c>
+      <c r="T766" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U766" t="inlineStr"/>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D767" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E767" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F767" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G767" t="n">
+        <v>1195839458</v>
+      </c>
+      <c r="H767" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I767" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J767" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K767" t="n">
+        <v>0</v>
+      </c>
+      <c r="L767" t="b">
+        <v>1</v>
+      </c>
+      <c r="M767" t="n">
+        <v>3.00806</v>
+      </c>
+      <c r="N767" t="n">
+        <v>124</v>
+      </c>
+      <c r="O767" t="n">
+        <v>23</v>
+      </c>
+      <c r="P767" t="inlineStr"/>
+      <c r="R767" t="inlineStr">
+        <is>
+          <t>7.3.1</t>
+        </is>
+      </c>
+      <c r="S767" t="inlineStr">
+        <is>
+          <t>A free mobile self-care application for Orange Botswana’s mobile customers.
+Full Description :
+Max it is a free application, which allows Orange Botswana customers to:
+- Consult your account in real time: minutes, sms, internet ...
+- Top up your account or a friend account  with Orange Money
+-</t>
+        </is>
+      </c>
+      <c r="T767" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U767" t="inlineStr"/>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D768" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E768" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F768" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G768" t="inlineStr">
+        <is>
+          <t>com.orange.mobinilandme</t>
+        </is>
+      </c>
+      <c r="H768" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I768" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J768" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K768" t="inlineStr">
+        <is>
+          <t>EGP 0.00</t>
+        </is>
+      </c>
+      <c r="L768" t="b">
+        <v>0</v>
+      </c>
+      <c r="M768" t="n">
+        <v>4.5586658</v>
+      </c>
+      <c r="N768" t="n">
+        <v>932357</v>
+      </c>
+      <c r="O768" t="n">
+        <v>19</v>
+      </c>
+      <c r="P768" t="inlineStr"/>
+      <c r="Q768" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R768" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S768" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion&lt;br&gt;Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.&lt;br&gt;Key services include:&lt;br&gt;• Account Management: Easily manage</t>
+        </is>
+      </c>
+      <c r="T768" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U768" t="inlineStr"/>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>a8ddc271-0a37-436d-9198-6e15dca53119</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>2026-07-31 06:45:20</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D769" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E769" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F769" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G769" t="n">
+        <v>942568333</v>
+      </c>
+      <c r="H769" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I769" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J769" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K769" t="n">
+        <v>0</v>
+      </c>
+      <c r="L769" t="b">
+        <v>1</v>
+      </c>
+      <c r="M769" t="n">
+        <v>4.25251</v>
+      </c>
+      <c r="N769" t="n">
+        <v>118120</v>
+      </c>
+      <c r="O769" t="n">
+        <v>50</v>
+      </c>
+      <c r="P769" t="inlineStr"/>
+      <c r="R769" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S769" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion
+Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.
+Key services include:
+• Account Management: Easily manage your Ora</t>
+        </is>
+      </c>
+      <c r="T769" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U769" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-08-01
</commit_message>
<xml_diff>
--- a/maxit_store_history.xlsx
+++ b/maxit_store_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U769"/>
+  <dimension ref="A1:U801"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63466,7 +63466,6 @@
       <c r="O738" t="n">
         <v>34</v>
       </c>
-      <c r="P738" t="inlineStr"/>
       <c r="Q738" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -63487,7 +63486,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U738" t="inlineStr"/>
     </row>
     <row r="739">
       <c r="A739" t="inlineStr">
@@ -63550,7 +63548,6 @@
       <c r="N739" t="n">
         <v>324</v>
       </c>
-      <c r="P739" t="inlineStr"/>
       <c r="R739" t="inlineStr">
         <is>
           <t>6.4.8</t>
@@ -63566,7 +63563,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U739" t="inlineStr"/>
     </row>
     <row r="740">
       <c r="A740" t="inlineStr">
@@ -63636,7 +63632,6 @@
       <c r="O740" t="n">
         <v>30</v>
       </c>
-      <c r="P740" t="inlineStr"/>
       <c r="Q740" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -63657,7 +63652,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U740" t="inlineStr"/>
     </row>
     <row r="741">
       <c r="A741" t="inlineStr">
@@ -63723,7 +63717,6 @@
       <c r="O741" t="n">
         <v>42</v>
       </c>
-      <c r="P741" t="inlineStr"/>
       <c r="R741" t="inlineStr">
         <is>
           <t>10.0.7</t>
@@ -63741,7 +63734,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U741" t="inlineStr"/>
     </row>
     <row r="742">
       <c r="A742" t="inlineStr">
@@ -63811,7 +63803,6 @@
       <c r="O742" t="n">
         <v>10</v>
       </c>
-      <c r="P742" t="inlineStr"/>
       <c r="Q742" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -63832,7 +63823,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U742" t="inlineStr"/>
     </row>
     <row r="743">
       <c r="A743" t="inlineStr">
@@ -63921,7 +63911,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U743" t="inlineStr"/>
     </row>
     <row r="744">
       <c r="A744" t="inlineStr">
@@ -63991,7 +63980,6 @@
       <c r="O744" t="n">
         <v>10</v>
       </c>
-      <c r="P744" t="inlineStr"/>
       <c r="Q744" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -64012,7 +64000,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U744" t="inlineStr"/>
     </row>
     <row r="745">
       <c r="A745" t="inlineStr">
@@ -64078,7 +64065,6 @@
       <c r="O745" t="n">
         <v>2</v>
       </c>
-      <c r="P745" t="inlineStr"/>
       <c r="R745" t="inlineStr">
         <is>
           <t>22.0.0</t>
@@ -64096,7 +64082,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U745" t="inlineStr"/>
     </row>
     <row r="746">
       <c r="A746" t="inlineStr">
@@ -64166,7 +64151,6 @@
       <c r="O746" t="n">
         <v>80</v>
       </c>
-      <c r="P746" t="inlineStr"/>
       <c r="Q746" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -64187,7 +64171,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U746" t="inlineStr"/>
     </row>
     <row r="747">
       <c r="A747" t="inlineStr">
@@ -64272,7 +64255,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U747" t="inlineStr"/>
     </row>
     <row r="748">
       <c r="A748" t="inlineStr">
@@ -64339,7 +64321,6 @@
       <c r="N748" t="n">
         <v>38243</v>
       </c>
-      <c r="P748" t="inlineStr"/>
       <c r="Q748" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -64360,7 +64341,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U748" t="inlineStr"/>
     </row>
     <row r="749">
       <c r="A749" t="inlineStr">
@@ -64426,7 +64406,6 @@
       <c r="O749" t="n">
         <v>14</v>
       </c>
-      <c r="P749" t="inlineStr"/>
       <c r="R749" t="inlineStr">
         <is>
           <t>6.5.2</t>
@@ -64445,7 +64424,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U749" t="inlineStr"/>
     </row>
     <row r="750">
       <c r="A750" t="inlineStr">
@@ -64515,7 +64493,6 @@
       <c r="O750" t="n">
         <v>51</v>
       </c>
-      <c r="P750" t="inlineStr"/>
       <c r="Q750" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -64536,7 +64513,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U750" t="inlineStr"/>
     </row>
     <row r="751">
       <c r="A751" t="inlineStr">
@@ -64602,7 +64578,6 @@
       <c r="O751" t="n">
         <v>21</v>
       </c>
-      <c r="P751" t="inlineStr"/>
       <c r="R751" t="inlineStr">
         <is>
           <t>5.0.2</t>
@@ -64620,7 +64595,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U751" t="inlineStr"/>
     </row>
     <row r="752">
       <c r="A752" t="inlineStr">
@@ -64690,7 +64664,6 @@
       <c r="O752" t="n">
         <v>81</v>
       </c>
-      <c r="P752" t="inlineStr"/>
       <c r="Q752" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -64711,7 +64684,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U752" t="inlineStr"/>
     </row>
     <row r="753">
       <c r="A753" t="inlineStr">
@@ -64799,7 +64771,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U753" t="inlineStr"/>
     </row>
     <row r="754">
       <c r="A754" t="inlineStr">
@@ -64869,7 +64840,6 @@
       <c r="O754" t="n">
         <v>45</v>
       </c>
-      <c r="P754" t="inlineStr"/>
       <c r="Q754" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -64890,7 +64860,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U754" t="inlineStr"/>
     </row>
     <row r="755">
       <c r="A755" t="inlineStr">
@@ -64956,7 +64925,6 @@
       <c r="O755" t="n">
         <v>47</v>
       </c>
-      <c r="P755" t="inlineStr"/>
       <c r="R755" t="inlineStr">
         <is>
           <t>10.0.21</t>
@@ -64975,7 +64943,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U755" t="inlineStr"/>
     </row>
     <row r="756">
       <c r="A756" t="inlineStr">
@@ -65045,7 +65012,6 @@
       <c r="O756" t="n">
         <v>10</v>
       </c>
-      <c r="P756" t="inlineStr"/>
       <c r="Q756" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -65066,7 +65032,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U756" t="inlineStr"/>
     </row>
     <row r="757">
       <c r="A757" t="inlineStr">
@@ -65152,7 +65117,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U757" t="inlineStr"/>
     </row>
     <row r="758">
       <c r="A758" t="inlineStr">
@@ -65222,7 +65186,6 @@
       <c r="O758" t="n">
         <v>4</v>
       </c>
-      <c r="P758" t="inlineStr"/>
       <c r="Q758" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -65243,7 +65206,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U758" t="inlineStr"/>
     </row>
     <row r="759">
       <c r="A759" t="inlineStr">
@@ -65329,7 +65291,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U759" t="inlineStr"/>
     </row>
     <row r="760">
       <c r="A760" t="inlineStr">
@@ -65399,7 +65360,6 @@
       <c r="O760" t="n">
         <v>91</v>
       </c>
-      <c r="P760" t="inlineStr"/>
       <c r="Q760" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -65420,7 +65380,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U760" t="inlineStr"/>
     </row>
     <row r="761">
       <c r="A761" t="inlineStr">
@@ -65503,7 +65462,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U761" t="inlineStr"/>
     </row>
     <row r="762">
       <c r="A762" t="inlineStr">
@@ -65573,7 +65531,6 @@
       <c r="O762" t="n">
         <v>11</v>
       </c>
-      <c r="P762" t="inlineStr"/>
       <c r="Q762" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -65594,7 +65551,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U762" t="inlineStr"/>
     </row>
     <row r="763">
       <c r="A763" t="inlineStr">
@@ -65683,7 +65639,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U763" t="inlineStr"/>
     </row>
     <row r="764">
       <c r="A764" t="inlineStr">
@@ -65753,7 +65708,6 @@
       <c r="O764" t="n">
         <v>12</v>
       </c>
-      <c r="P764" t="inlineStr"/>
       <c r="Q764" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -65774,7 +65728,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U764" t="inlineStr"/>
     </row>
     <row r="765">
       <c r="A765" t="inlineStr">
@@ -65861,7 +65814,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U765" t="inlineStr"/>
     </row>
     <row r="766">
       <c r="A766" t="inlineStr">
@@ -65931,7 +65883,6 @@
       <c r="O766" t="n">
         <v>25</v>
       </c>
-      <c r="P766" t="inlineStr"/>
       <c r="Q766" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -65952,7 +65903,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U766" t="inlineStr"/>
     </row>
     <row r="767">
       <c r="A767" t="inlineStr">
@@ -66018,7 +65968,6 @@
       <c r="O767" t="n">
         <v>23</v>
       </c>
-      <c r="P767" t="inlineStr"/>
       <c r="R767" t="inlineStr">
         <is>
           <t>7.3.1</t>
@@ -66039,7 +65988,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U767" t="inlineStr"/>
     </row>
     <row r="768">
       <c r="A768" t="inlineStr">
@@ -66109,7 +66057,6 @@
       <c r="O768" t="n">
         <v>19</v>
       </c>
-      <c r="P768" t="inlineStr"/>
       <c r="Q768" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -66130,7 +66077,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U768" t="inlineStr"/>
     </row>
     <row r="769">
       <c r="A769" t="inlineStr">
@@ -66196,7 +66142,6 @@
       <c r="O769" t="n">
         <v>50</v>
       </c>
-      <c r="P769" t="inlineStr"/>
       <c r="R769" t="inlineStr">
         <is>
           <t>10.1.0</t>
@@ -66215,7 +66160,2825 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U769" t="inlineStr"/>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E770" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F770" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G770" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogn</t>
+        </is>
+      </c>
+      <c r="H770" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I770" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J770" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K770" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L770" t="b">
+        <v>0</v>
+      </c>
+      <c r="M770" t="n">
+        <v>4.445652</v>
+      </c>
+      <c r="N770" t="n">
+        <v>9333</v>
+      </c>
+      <c r="O770" t="n">
+        <v>35</v>
+      </c>
+      <c r="P770" t="inlineStr"/>
+      <c r="Q770" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R770" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S770" t="inlineStr">
+        <is>
+          <t>Bien plus qu&amp;#39;une application, un véritable assistant personnel pour une vie connectée et simplifiée.&lt;br&gt;Suivi de consommation: Votre tableau de bord tout-en-un pour une gestion simplifiée !&lt;br&gt;- Gestion de votre offre: Accédez à une vue détaillée de votre offre actuelle et de vos forfaits Orange</t>
+        </is>
+      </c>
+      <c r="T770" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U770" t="inlineStr"/>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E771" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F771" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G771" t="n">
+        <v>1177999485</v>
+      </c>
+      <c r="H771" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I771" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J771" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K771" t="n">
+        <v>0</v>
+      </c>
+      <c r="L771" t="b">
+        <v>1</v>
+      </c>
+      <c r="M771" t="n">
+        <v>3.88272</v>
+      </c>
+      <c r="N771" t="n">
+        <v>324</v>
+      </c>
+      <c r="P771" t="inlineStr"/>
+      <c r="R771" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S771" t="inlineStr">
+        <is>
+          <t>La fusion d’Orange et Moi et Orange Money donne naissance à Max it, la nouvelle Super Application Tout-en-Un. Profitez du suivi de consommation, de paiements mobiles, de toutes les fonctionnalités Orange et Moi et Money avec un large éventail de divertissements, le tout regroupé en un seul endroit !</t>
+        </is>
+      </c>
+      <c r="T771" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U771" t="inlineStr"/>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E772" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F772" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G772" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.otn</t>
+        </is>
+      </c>
+      <c r="H772" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I772" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J772" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K772" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L772" t="b">
+        <v>0</v>
+      </c>
+      <c r="M772" t="n">
+        <v>3.9654968</v>
+      </c>
+      <c r="N772" t="n">
+        <v>35388</v>
+      </c>
+      <c r="O772" t="n">
+        <v>37</v>
+      </c>
+      <c r="P772" t="inlineStr"/>
+      <c r="Q772" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R772" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S772" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Max it par Orange Tunisie facilite votre vie au quotidien !&lt;/h2&gt;&lt;br&gt;&lt;br&gt;Welcome sur Max it !&lt;br&gt;Accédez rapidement à vos fonctionnalités Max it préférées et profitez également de contenus exclusifs, d’activités divertissantes, et de jeux interactifs pour une expérience enrichissante avec la roue</t>
+        </is>
+      </c>
+      <c r="T772" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U772" t="inlineStr"/>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E773" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F773" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G773" t="n">
+        <v>1146892088</v>
+      </c>
+      <c r="H773" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I773" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J773" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K773" t="n">
+        <v>0</v>
+      </c>
+      <c r="L773" t="b">
+        <v>1</v>
+      </c>
+      <c r="M773" t="n">
+        <v>3.02862</v>
+      </c>
+      <c r="N773" t="n">
+        <v>1642</v>
+      </c>
+      <c r="O773" t="n">
+        <v>41</v>
+      </c>
+      <c r="P773" t="inlineStr"/>
+      <c r="R773" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S773" t="inlineStr">
+        <is>
+          <t>Max it by Orange Tunisie : Votre appli incontournable pour une vie connectée
+Welcome sur Max it : Découvrez fonctionnalités, jeux &amp; contenus de divertissement by Orange Tunisie !
+Trouvez vite vos fonctionnalités Max it favorites et explorez des contenus exclusifs et des jeux pour une expérience im</t>
+        </is>
+      </c>
+      <c r="T773" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U773" t="inlineStr"/>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E774" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F774" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G774" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osl</t>
+        </is>
+      </c>
+      <c r="H774" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I774" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J774" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K774" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L774" t="b">
+        <v>0</v>
+      </c>
+      <c r="M774" t="n">
+        <v>4.4439254</v>
+      </c>
+      <c r="N774" t="n">
+        <v>2146</v>
+      </c>
+      <c r="O774" t="n">
+        <v>10</v>
+      </c>
+      <c r="P774" t="inlineStr"/>
+      <c r="Q774" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R774" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S774" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it is a free application, which allows Orange Sierra Leone prepaid and postpaid customers to:&lt;br&gt;&lt;br&gt;- Consult your account in real time: minutes, sms, internet&lt;br&gt;- Top up your account or a friend account &lt;br&gt;- Buy Internet Bundles&lt;br&gt;- Discover the latest offers and promotions &lt;br&gt;- Access to </t>
+        </is>
+      </c>
+      <c r="T774" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U774" t="inlineStr"/>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E775" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F775" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G775" t="n">
+        <v>6443607903</v>
+      </c>
+      <c r="H775" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I775" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J775" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K775" t="n">
+        <v>0</v>
+      </c>
+      <c r="L775" t="b">
+        <v>1</v>
+      </c>
+      <c r="M775" t="n">
+        <v>3.69948</v>
+      </c>
+      <c r="N775" t="n">
+        <v>193</v>
+      </c>
+      <c r="O775" t="n">
+        <v>5</v>
+      </c>
+      <c r="P775" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R775" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S775" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The merger of My Orange &amp; Orange Money has given birth to Max it the all-in-one super app, a free application which allows all Orange Sierra Leone customers to 
+Track calls, SMS, and Data usage and monitor balance. 
+Make a secure mobile/Orange Money payment.
+Easily transfer credit to other users </t>
+        </is>
+      </c>
+      <c r="T775" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U775" t="inlineStr"/>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E776" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F776" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G776" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osn</t>
+        </is>
+      </c>
+      <c r="H776" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I776" t="inlineStr">
+        <is>
+          <t>Orange Sénégal</t>
+        </is>
+      </c>
+      <c r="J776" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K776" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L776" t="b">
+        <v>0</v>
+      </c>
+      <c r="M776" t="n">
+        <v>4.299279</v>
+      </c>
+      <c r="N776" t="n">
+        <v>51315</v>
+      </c>
+      <c r="O776" t="n">
+        <v>8</v>
+      </c>
+      <c r="P776" t="inlineStr"/>
+      <c r="Q776" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R776" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S776" t="inlineStr">
+        <is>
+          <t>Lu bees ak Max it ! &lt;br&gt;Une application repensée pour être plus simple, plus rapide et adaptée à vos besoins. Une expérience optimisée pour faciliter vos usages au quotidien, avec des parcours simplifiés et un accès plus fluide à vos services. Que vous soyez client Orange ou non, Max it vous accompa</t>
+        </is>
+      </c>
+      <c r="T776" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U776" t="inlineStr"/>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E777" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F777" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G777" t="n">
+        <v>1039327980</v>
+      </c>
+      <c r="H777" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I777" t="inlineStr">
+        <is>
+          <t>Orange Senegal</t>
+        </is>
+      </c>
+      <c r="J777" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K777" t="n">
+        <v>0</v>
+      </c>
+      <c r="L777" t="b">
+        <v>1</v>
+      </c>
+      <c r="M777" t="n">
+        <v>4.1693</v>
+      </c>
+      <c r="N777" t="n">
+        <v>30230</v>
+      </c>
+      <c r="O777" t="n">
+        <v>2</v>
+      </c>
+      <c r="P777" t="inlineStr"/>
+      <c r="R777" t="inlineStr">
+        <is>
+          <t>22.0.0</t>
+        </is>
+      </c>
+      <c r="S777" t="inlineStr">
+        <is>
+          <t>Here is the English translation:
+Welcome to Max it!
+A redesigned app to be simpler, faster, and tailored to your needs. An optimized experience to make your daily life easier, with streamlined journeys and smoother access to your services. Whether you are an Orange customer or not, Max it is your e</t>
+        </is>
+      </c>
+      <c r="T777" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U777" t="inlineStr"/>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E778" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F778" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G778" t="inlineStr">
+        <is>
+          <t>com.orange.meditel.mediteletmoi</t>
+        </is>
+      </c>
+      <c r="H778" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I778" t="inlineStr">
+        <is>
+          <t>Orange Maroc</t>
+        </is>
+      </c>
+      <c r="J778" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K778" t="inlineStr">
+        <is>
+          <t>MAD 0.00</t>
+        </is>
+      </c>
+      <c r="L778" t="b">
+        <v>0</v>
+      </c>
+      <c r="M778" t="n">
+        <v>3.7192206</v>
+      </c>
+      <c r="N778" t="n">
+        <v>110932</v>
+      </c>
+      <c r="O778" t="n">
+        <v>57</v>
+      </c>
+      <c r="P778" t="inlineStr"/>
+      <c r="Q778" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R778" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S778" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l&amp;#39;expérience mobile réinventé&lt;br&gt;&lt;br&gt;Max it, c&amp;#39;est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d&amp;#39;une multitude de services exclusifs. &lt;br&gt;&lt;br&gt;Créez votre espace sur</t>
+        </is>
+      </c>
+      <c r="T778" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U778" t="inlineStr"/>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E779" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F779" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G779" t="n">
+        <v>596028698</v>
+      </c>
+      <c r="H779" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I779" t="inlineStr">
+        <is>
+          <t>Méditel</t>
+        </is>
+      </c>
+      <c r="J779" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K779" t="n">
+        <v>0</v>
+      </c>
+      <c r="L779" t="b">
+        <v>1</v>
+      </c>
+      <c r="M779" t="n">
+        <v>3.94601</v>
+      </c>
+      <c r="N779" t="n">
+        <v>2760</v>
+      </c>
+      <c r="P779" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "MA" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R779" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S779" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l'expérience mobile réinventé
+Max it, c'est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d'une multitude de services exclusifs. 
+Créez votre espace sur mesure et bénéficiez d'</t>
+        </is>
+      </c>
+      <c r="T779" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U779" t="inlineStr"/>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E780" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F780" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G780" t="inlineStr">
+        <is>
+          <t>com.oml.dsi.orangemobile</t>
+        </is>
+      </c>
+      <c r="H780" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I780" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J780" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K780" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L780" t="b">
+        <v>0</v>
+      </c>
+      <c r="M780" t="n">
+        <v>2.7071838</v>
+      </c>
+      <c r="N780" t="n">
+        <v>38243</v>
+      </c>
+      <c r="P780" t="inlineStr"/>
+      <c r="Q780" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R780" t="inlineStr">
+        <is>
+          <t>6.5.0</t>
+        </is>
+      </c>
+      <c r="S780" t="inlineStr">
+        <is>
+          <t>Easily manage your Orange Mali line&lt;br&gt;● Manage your account and view all essential information, your offers, and your phone lines.&lt;br&gt;● Subscribe to call, SMS, Internet, and international call packages.&lt;br&gt;● Track your usage by checking your credit and Internet balance.&lt;br&gt;● Recharge your line by p</t>
+        </is>
+      </c>
+      <c r="T780" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U780" t="inlineStr"/>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E781" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F781" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G781" t="n">
+        <v>1494321079</v>
+      </c>
+      <c r="H781" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I781" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J781" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K781" t="n">
+        <v>0</v>
+      </c>
+      <c r="L781" t="b">
+        <v>1</v>
+      </c>
+      <c r="M781" t="n">
+        <v>2.52176</v>
+      </c>
+      <c r="N781" t="n">
+        <v>4757</v>
+      </c>
+      <c r="O781" t="n">
+        <v>10</v>
+      </c>
+      <c r="P781" t="inlineStr"/>
+      <c r="R781" t="inlineStr">
+        <is>
+          <t>6.5.2</t>
+        </is>
+      </c>
+      <c r="S781" t="inlineStr">
+        <is>
+          <t>Gérez facilement votre ligne Orange Mali 
+●        Gérez votre compte et consultez toutes les informations essentielles sur celui-ci, vos offres, ainsi que vos lignes téléphoniques.
+●        Souscrivez aux forfaits appels, SMS, Internet, et appels internationaux.
+●        Suivez votre consommation e</t>
+        </is>
+      </c>
+      <c r="T781" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U781" t="inlineStr"/>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E782" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F782" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G782" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.omg</t>
+        </is>
+      </c>
+      <c r="H782" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I782" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J782" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K782" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L782" t="b">
+        <v>0</v>
+      </c>
+      <c r="M782" t="n">
+        <v>4.1353383</v>
+      </c>
+      <c r="N782" t="n">
+        <v>1389</v>
+      </c>
+      <c r="O782" t="n">
+        <v>51</v>
+      </c>
+      <c r="P782" t="inlineStr"/>
+      <c r="Q782" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R782" t="inlineStr">
+        <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="S782" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.&lt;br&gt;&lt;br&gt;Simplify Your Life with Max it&lt;br&gt;With Max It, ac</t>
+        </is>
+      </c>
+      <c r="T782" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U782" t="inlineStr"/>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E783" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F783" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G783" t="n">
+        <v>1295171817</v>
+      </c>
+      <c r="H783" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I783" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J783" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K783" t="n">
+        <v>0</v>
+      </c>
+      <c r="L783" t="b">
+        <v>1</v>
+      </c>
+      <c r="M783" t="n">
+        <v>3.05714</v>
+      </c>
+      <c r="N783" t="n">
+        <v>70</v>
+      </c>
+      <c r="O783" t="n">
+        <v>15</v>
+      </c>
+      <c r="P783" t="inlineStr"/>
+      <c r="R783" t="inlineStr">
+        <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="S783" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.
+Simplify Your Life with Max it
+With Max it, access a se</t>
+        </is>
+      </c>
+      <c r="T783" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U783" t="inlineStr"/>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E784" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F784" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G784" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.olr</t>
+        </is>
+      </c>
+      <c r="H784" t="inlineStr">
+        <is>
+          <t>Orange Max it - Liberia</t>
+        </is>
+      </c>
+      <c r="I784" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J784" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K784" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L784" t="b">
+        <v>0</v>
+      </c>
+      <c r="M784" t="n">
+        <v>4.5301585</v>
+      </c>
+      <c r="N784" t="n">
+        <v>3104</v>
+      </c>
+      <c r="O784" t="n">
+        <v>69</v>
+      </c>
+      <c r="P784" t="inlineStr"/>
+      <c r="Q784" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R784" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="S784" t="inlineStr">
+        <is>
+          <t>Max it: your personalized experience by Orange Liberia!&lt;br&gt;&lt;br&gt;Step into Max it, your all-in-one solution for telecom, marketplace, and financial services! Manage your mobile line, customize offers, pay your bills, keep&lt;br&gt;track of your usage with ease, and recharge your credit. Access exclusive eve</t>
+        </is>
+      </c>
+      <c r="T784" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U784" t="inlineStr"/>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E785" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F785" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G785" t="n">
+        <v>6746187327</v>
+      </c>
+      <c r="H785" t="inlineStr">
+        <is>
+          <t>Orange Max it – Liberia</t>
+        </is>
+      </c>
+      <c r="I785" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J785" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K785" t="n">
+        <v>0</v>
+      </c>
+      <c r="L785" t="b">
+        <v>1</v>
+      </c>
+      <c r="M785" t="n">
+        <v>4.0625</v>
+      </c>
+      <c r="N785" t="n">
+        <v>48</v>
+      </c>
+      <c r="P785" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "LR" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R785" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="S785" t="inlineStr">
+        <is>
+          <t>Max it is a free application, which allows Orange Liberia customers to:
+- Consult your account in real time: minutes, sms, internet
+- Top up your account or a friend account 
+- Buy  Bundles (voice, data, SMS, roaming, international)
+- Discover the latest offers and promotions 
+- Access to Orange se</t>
+        </is>
+      </c>
+      <c r="T785" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U785" t="inlineStr"/>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D786" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E786" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F786" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G786" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ojo</t>
+        </is>
+      </c>
+      <c r="H786" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I786" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J786" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K786" t="inlineStr">
+        <is>
+          <t>JOD 0.000</t>
+        </is>
+      </c>
+      <c r="L786" t="b">
+        <v>0</v>
+      </c>
+      <c r="M786" t="n">
+        <v>4.431287</v>
+      </c>
+      <c r="N786" t="n">
+        <v>97819</v>
+      </c>
+      <c r="O786" t="n">
+        <v>43</v>
+      </c>
+      <c r="P786" t="inlineStr"/>
+      <c r="Q786" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R786" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S786" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience&lt;br&gt;Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.&lt;br&gt;Important Update:&lt;br&gt;The jood app (jood Orange) w</t>
+        </is>
+      </c>
+      <c r="T786" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U786" t="inlineStr"/>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E787" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F787" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G787" t="n">
+        <v>808824590</v>
+      </c>
+      <c r="H787" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I787" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J787" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K787" t="n">
+        <v>0</v>
+      </c>
+      <c r="L787" t="b">
+        <v>1</v>
+      </c>
+      <c r="M787" t="n">
+        <v>4.20622</v>
+      </c>
+      <c r="N787" t="n">
+        <v>3050</v>
+      </c>
+      <c r="O787" t="n">
+        <v>51</v>
+      </c>
+      <c r="P787" t="inlineStr"/>
+      <c r="R787" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S787" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience
+Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.
+Important Update:
+The jood app (jood Orange) will be di</t>
+        </is>
+      </c>
+      <c r="T787" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U787" t="inlineStr"/>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E788" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F788" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G788" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.oci</t>
+        </is>
+      </c>
+      <c r="H788" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I788" t="inlineStr">
+        <is>
+          <t>Orange Côte d'Ivoire S.A</t>
+        </is>
+      </c>
+      <c r="J788" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K788" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L788" t="b">
+        <v>0</v>
+      </c>
+      <c r="M788" t="n">
+        <v>4.1514387</v>
+      </c>
+      <c r="N788" t="n">
+        <v>67307</v>
+      </c>
+      <c r="O788" t="n">
+        <v>13</v>
+      </c>
+      <c r="P788" t="inlineStr"/>
+      <c r="Q788" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R788" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S788" t="inlineStr">
+        <is>
+          <t>Aaaahhh, ta super app Max it, n&amp;#39;a pas fini de te surprendre... &lt;br&gt;Est-ce que tu as remarqué ? Maintenant, tu as ton QR code personnalisé en haut de ton écran d&amp;#39;accueil ! Ainsi, tu peux :&lt;br&gt;     scanner le QR code de ton ami(e) pour lui faire un transfert d&amp;#39;&amp;#39;argent&lt;br&gt;     scanner l</t>
+        </is>
+      </c>
+      <c r="T788" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U788" t="inlineStr"/>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D789" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E789" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F789" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G789" t="n">
+        <v>1061120855</v>
+      </c>
+      <c r="H789" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I789" t="inlineStr">
+        <is>
+          <t>Orange CI</t>
+        </is>
+      </c>
+      <c r="J789" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K789" t="n">
+        <v>0</v>
+      </c>
+      <c r="L789" t="b">
+        <v>1</v>
+      </c>
+      <c r="M789" t="n">
+        <v>3.78577</v>
+      </c>
+      <c r="N789" t="n">
+        <v>5975</v>
+      </c>
+      <c r="O789" t="n">
+        <v>2</v>
+      </c>
+      <c r="P789" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R789" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S789" t="inlineStr">
+        <is>
+          <t>Max it, la super app all-in-one te fais gagner du temps, et diminue tes soucis... Gagne plus d'espace de stockage sur ton téléphone ; plus besoin de cumuler plusieurs appli d'Orange pour avoir accès à un maximum de services. Max it est là ! Gère ta ligne (SIM) au niveau des pass, des soldes, réalise</t>
+        </is>
+      </c>
+      <c r="T789" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U789" t="inlineStr"/>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E790" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F790" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G790" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogw</t>
+        </is>
+      </c>
+      <c r="H790" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I790" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J790" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K790" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L790" t="b">
+        <v>0</v>
+      </c>
+      <c r="M790" t="n">
+        <v>4.3896103</v>
+      </c>
+      <c r="N790" t="n">
+        <v>1545</v>
+      </c>
+      <c r="O790" t="n">
+        <v>4</v>
+      </c>
+      <c r="P790" t="inlineStr"/>
+      <c r="Q790" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R790" t="inlineStr">
+        <is>
+          <t>4.0.18</t>
+        </is>
+      </c>
+      <c r="S790" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T790" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U790" t="inlineStr"/>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E791" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F791" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G791" t="n">
+        <v>1574668652</v>
+      </c>
+      <c r="H791" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I791" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J791" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K791" t="n">
+        <v>0</v>
+      </c>
+      <c r="L791" t="b">
+        <v>1</v>
+      </c>
+      <c r="M791" t="n">
+        <v>4.05333</v>
+      </c>
+      <c r="N791" t="n">
+        <v>75</v>
+      </c>
+      <c r="O791" t="n">
+        <v>4</v>
+      </c>
+      <c r="P791" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R791" t="inlineStr">
+        <is>
+          <t>6.0.35</t>
+        </is>
+      </c>
+      <c r="S791" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T791" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U791" t="inlineStr"/>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E792" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F792" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G792" t="inlineStr">
+        <is>
+          <t>com.orange.sugu.ocd</t>
+        </is>
+      </c>
+      <c r="H792" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I792" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J792" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K792" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L792" t="b">
+        <v>0</v>
+      </c>
+      <c r="M792" t="n">
+        <v>4.1327105</v>
+      </c>
+      <c r="N792" t="n">
+        <v>5313</v>
+      </c>
+      <c r="O792" t="n">
+        <v>91</v>
+      </c>
+      <c r="P792" t="inlineStr"/>
+      <c r="Q792" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R792" t="inlineStr">
+        <is>
+          <t>9.0.12</t>
+        </is>
+      </c>
+      <c r="S792" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DRC that brings together the features of MyOrange, and Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Plans, Mobile Payments, money transfers, bill payments, subscriptions, and entertai</t>
+        </is>
+      </c>
+      <c r="T792" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U792" t="inlineStr"/>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E793" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F793" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G793" t="n">
+        <v>6447896435</v>
+      </c>
+      <c r="H793" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I793" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J793" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K793" t="n">
+        <v>0</v>
+      </c>
+      <c r="L793" t="b">
+        <v>1</v>
+      </c>
+      <c r="M793" t="n">
+        <v>3.55351</v>
+      </c>
+      <c r="N793" t="n">
+        <v>271</v>
+      </c>
+      <c r="P793" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "CD" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R793" t="inlineStr">
+        <is>
+          <t>9.0.6</t>
+        </is>
+      </c>
+      <c r="S793" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DR Congo. It brings together the features of Orange et Moi, as well as Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Packages, Mobile payment, money transfers, bill payment and subscri</t>
+        </is>
+      </c>
+      <c r="T793" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U793" t="inlineStr"/>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E794" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F794" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G794" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ocm</t>
+        </is>
+      </c>
+      <c r="H794" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroon</t>
+        </is>
+      </c>
+      <c r="I794" t="inlineStr">
+        <is>
+          <t>Orange MEA</t>
+        </is>
+      </c>
+      <c r="J794" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K794" t="inlineStr">
+        <is>
+          <t>FCFA 0</t>
+        </is>
+      </c>
+      <c r="L794" t="b">
+        <v>0</v>
+      </c>
+      <c r="M794" t="n">
+        <v>3.9172325</v>
+      </c>
+      <c r="N794" t="n">
+        <v>47024</v>
+      </c>
+      <c r="O794" t="n">
+        <v>10</v>
+      </c>
+      <c r="P794" t="inlineStr"/>
+      <c r="Q794" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R794" t="inlineStr">
+        <is>
+          <t>7.0.23</t>
+        </is>
+      </c>
+      <c r="S794" t="inlineStr">
+        <is>
+          <t>Max it brings together everything that matters to you in one app: managing your lines, money transfer, bill payment, exclusive offers, and a universe of lifestyle and entertainment. Simple, fast, and 100% secure..&lt;br&gt;&lt;br&gt;📞 My line&lt;br&gt;Manage your Orange mobile and landline bundles in a single click:</t>
+        </is>
+      </c>
+      <c r="T794" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U794" t="inlineStr"/>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E795" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F795" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G795" t="n">
+        <v>1116920093</v>
+      </c>
+      <c r="H795" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroun</t>
+        </is>
+      </c>
+      <c r="I795" t="inlineStr">
+        <is>
+          <t>Orange Middle East &amp; Africa</t>
+        </is>
+      </c>
+      <c r="J795" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K795" t="n">
+        <v>0</v>
+      </c>
+      <c r="L795" t="b">
+        <v>1</v>
+      </c>
+      <c r="M795" t="n">
+        <v>3.76823</v>
+      </c>
+      <c r="N795" t="n">
+        <v>16167</v>
+      </c>
+      <c r="O795" t="n">
+        <v>3</v>
+      </c>
+      <c r="P795" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R795" t="inlineStr">
+        <is>
+          <t>7.0.24</t>
+        </is>
+      </c>
+      <c r="S795" t="inlineStr">
+        <is>
+          <t>Avec Max it, Orange rassemble tout ce qui compte pour vous dans une même application : la gestion de vos lignes, les transferts d’argent, payement de vos factures, des offres exclusives et un univers lifestyle et divertissement.
+Simple, rapide et 100 % sécurisée.
+Ma ligne
+Gérez vos forfaits mobiles</t>
+        </is>
+      </c>
+      <c r="T795" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U795" t="inlineStr"/>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E796" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F796" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G796" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obf</t>
+        </is>
+      </c>
+      <c r="H796" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I796" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso</t>
+        </is>
+      </c>
+      <c r="J796" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K796" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L796" t="b">
+        <v>0</v>
+      </c>
+      <c r="M796" t="n">
+        <v>4.139444</v>
+      </c>
+      <c r="N796" t="n">
+        <v>25521</v>
+      </c>
+      <c r="O796" t="n">
+        <v>11</v>
+      </c>
+      <c r="P796" t="inlineStr"/>
+      <c r="Q796" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R796" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S796" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.&lt;br&gt;Gérez vos lignes mobiles, effectuez des transferts d&amp;#39;argent sécurisés, réglez vos factures, profitez d&amp;#39;offres exclusives, effectuez des paiements marchands fiables, et bien plus enco</t>
+        </is>
+      </c>
+      <c r="T796" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U796" t="inlineStr"/>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E797" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F797" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G797" t="n">
+        <v>1553774707</v>
+      </c>
+      <c r="H797" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I797" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso SA</t>
+        </is>
+      </c>
+      <c r="J797" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K797" t="n">
+        <v>0</v>
+      </c>
+      <c r="L797" t="b">
+        <v>1</v>
+      </c>
+      <c r="M797" t="n">
+        <v>3.45508</v>
+      </c>
+      <c r="N797" t="n">
+        <v>1180</v>
+      </c>
+      <c r="O797" t="n">
+        <v>3</v>
+      </c>
+      <c r="P797" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R797" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S797" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.
+Gérez vos lignes mobiles, effectuez des transferts d'argent sécurisés, réglez vos factures, profitez d'offres exclusives, effectuez des paiements marchands fiables, et bien plus encore, le tout</t>
+        </is>
+      </c>
+      <c r="T797" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U797" t="inlineStr"/>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E798" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F798" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G798" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obw</t>
+        </is>
+      </c>
+      <c r="H798" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I798" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J798" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K798" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L798" t="b">
+        <v>0</v>
+      </c>
+      <c r="M798" t="n">
+        <v>3.967742</v>
+      </c>
+      <c r="N798" t="n">
+        <v>2966</v>
+      </c>
+      <c r="O798" t="n">
+        <v>29</v>
+      </c>
+      <c r="P798" t="inlineStr"/>
+      <c r="Q798" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R798" t="inlineStr">
+        <is>
+          <t>7.3.8</t>
+        </is>
+      </c>
+      <c r="S798" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it, the brand-new Orange Botswana Super App that follows Yame and gives you access to four distinct universes for a one-of-a-kind experience!&lt;br&gt;&lt;br&gt;Manage your accounts, make quick payments using QR codes, investigate a range of online goods and services, and discover the many options provided </t>
+        </is>
+      </c>
+      <c r="T798" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U798" t="inlineStr"/>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E799" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F799" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G799" t="n">
+        <v>1195839458</v>
+      </c>
+      <c r="H799" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I799" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J799" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K799" t="n">
+        <v>0</v>
+      </c>
+      <c r="L799" t="b">
+        <v>1</v>
+      </c>
+      <c r="M799" t="n">
+        <v>3.00806</v>
+      </c>
+      <c r="N799" t="n">
+        <v>124</v>
+      </c>
+      <c r="O799" t="n">
+        <v>26</v>
+      </c>
+      <c r="P799" t="inlineStr"/>
+      <c r="R799" t="inlineStr">
+        <is>
+          <t>7.3.1</t>
+        </is>
+      </c>
+      <c r="S799" t="inlineStr">
+        <is>
+          <t>A free mobile self-care application for Orange Botswana’s mobile customers.
+Full Description :
+Max it is a free application, which allows Orange Botswana customers to:
+- Consult your account in real time: minutes, sms, internet ...
+- Top up your account or a friend account  with Orange Money
+-</t>
+        </is>
+      </c>
+      <c r="T799" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U799" t="inlineStr"/>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E800" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F800" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G800" t="inlineStr">
+        <is>
+          <t>com.orange.mobinilandme</t>
+        </is>
+      </c>
+      <c r="H800" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I800" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J800" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K800" t="inlineStr">
+        <is>
+          <t>EGP 0.00</t>
+        </is>
+      </c>
+      <c r="L800" t="b">
+        <v>0</v>
+      </c>
+      <c r="M800" t="n">
+        <v>4.5573454</v>
+      </c>
+      <c r="N800" t="n">
+        <v>933561</v>
+      </c>
+      <c r="O800" t="n">
+        <v>19</v>
+      </c>
+      <c r="P800" t="inlineStr"/>
+      <c r="Q800" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R800" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S800" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion&lt;br&gt;Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.&lt;br&gt;Key services include:&lt;br&gt;• Account Management: Easily manage</t>
+        </is>
+      </c>
+      <c r="T800" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U800" t="inlineStr"/>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>767f8f69-ce61-426a-936f-f53f46109381</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>2026-08-01 06:30:58</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E801" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F801" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G801" t="n">
+        <v>942568333</v>
+      </c>
+      <c r="H801" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I801" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J801" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K801" t="n">
+        <v>0</v>
+      </c>
+      <c r="L801" t="b">
+        <v>1</v>
+      </c>
+      <c r="M801" t="n">
+        <v>4.2524</v>
+      </c>
+      <c r="N801" t="n">
+        <v>118307</v>
+      </c>
+      <c r="O801" t="n">
+        <v>54</v>
+      </c>
+      <c r="P801" t="inlineStr"/>
+      <c r="R801" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S801" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion
+Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.
+Key services include:
+• Account Management: Easily manage your Ora</t>
+        </is>
+      </c>
+      <c r="T801" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U801" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-08-02
</commit_message>
<xml_diff>
--- a/maxit_store_history.xlsx
+++ b/maxit_store_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U801"/>
+  <dimension ref="A1:U833"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -66229,7 +66229,6 @@
       <c r="O770" t="n">
         <v>35</v>
       </c>
-      <c r="P770" t="inlineStr"/>
       <c r="Q770" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -66250,7 +66249,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U770" t="inlineStr"/>
     </row>
     <row r="771">
       <c r="A771" t="inlineStr">
@@ -66313,7 +66311,6 @@
       <c r="N771" t="n">
         <v>324</v>
       </c>
-      <c r="P771" t="inlineStr"/>
       <c r="R771" t="inlineStr">
         <is>
           <t>6.4.12</t>
@@ -66329,7 +66326,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U771" t="inlineStr"/>
     </row>
     <row r="772">
       <c r="A772" t="inlineStr">
@@ -66399,7 +66395,6 @@
       <c r="O772" t="n">
         <v>37</v>
       </c>
-      <c r="P772" t="inlineStr"/>
       <c r="Q772" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -66420,7 +66415,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U772" t="inlineStr"/>
     </row>
     <row r="773">
       <c r="A773" t="inlineStr">
@@ -66486,7 +66480,6 @@
       <c r="O773" t="n">
         <v>41</v>
       </c>
-      <c r="P773" t="inlineStr"/>
       <c r="R773" t="inlineStr">
         <is>
           <t>10.0.7</t>
@@ -66504,7 +66497,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U773" t="inlineStr"/>
     </row>
     <row r="774">
       <c r="A774" t="inlineStr">
@@ -66574,7 +66566,6 @@
       <c r="O774" t="n">
         <v>10</v>
       </c>
-      <c r="P774" t="inlineStr"/>
       <c r="Q774" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -66595,7 +66586,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U774" t="inlineStr"/>
     </row>
     <row r="775">
       <c r="A775" t="inlineStr">
@@ -66684,7 +66674,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U775" t="inlineStr"/>
     </row>
     <row r="776">
       <c r="A776" t="inlineStr">
@@ -66754,7 +66743,6 @@
       <c r="O776" t="n">
         <v>8</v>
       </c>
-      <c r="P776" t="inlineStr"/>
       <c r="Q776" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -66775,7 +66763,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U776" t="inlineStr"/>
     </row>
     <row r="777">
       <c r="A777" t="inlineStr">
@@ -66841,7 +66828,6 @@
       <c r="O777" t="n">
         <v>2</v>
       </c>
-      <c r="P777" t="inlineStr"/>
       <c r="R777" t="inlineStr">
         <is>
           <t>22.0.0</t>
@@ -66859,7 +66845,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U777" t="inlineStr"/>
     </row>
     <row r="778">
       <c r="A778" t="inlineStr">
@@ -66929,7 +66914,6 @@
       <c r="O778" t="n">
         <v>57</v>
       </c>
-      <c r="P778" t="inlineStr"/>
       <c r="Q778" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -66950,7 +66934,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U778" t="inlineStr"/>
     </row>
     <row r="779">
       <c r="A779" t="inlineStr">
@@ -67035,7 +67018,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U779" t="inlineStr"/>
     </row>
     <row r="780">
       <c r="A780" t="inlineStr">
@@ -67102,7 +67084,6 @@
       <c r="N780" t="n">
         <v>38243</v>
       </c>
-      <c r="P780" t="inlineStr"/>
       <c r="Q780" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -67123,7 +67104,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U780" t="inlineStr"/>
     </row>
     <row r="781">
       <c r="A781" t="inlineStr">
@@ -67189,7 +67169,6 @@
       <c r="O781" t="n">
         <v>10</v>
       </c>
-      <c r="P781" t="inlineStr"/>
       <c r="R781" t="inlineStr">
         <is>
           <t>6.5.2</t>
@@ -67208,7 +67187,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U781" t="inlineStr"/>
     </row>
     <row r="782">
       <c r="A782" t="inlineStr">
@@ -67278,7 +67256,6 @@
       <c r="O782" t="n">
         <v>51</v>
       </c>
-      <c r="P782" t="inlineStr"/>
       <c r="Q782" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -67299,7 +67276,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U782" t="inlineStr"/>
     </row>
     <row r="783">
       <c r="A783" t="inlineStr">
@@ -67365,7 +67341,6 @@
       <c r="O783" t="n">
         <v>15</v>
       </c>
-      <c r="P783" t="inlineStr"/>
       <c r="R783" t="inlineStr">
         <is>
           <t>5.0.2</t>
@@ -67383,7 +67358,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U783" t="inlineStr"/>
     </row>
     <row r="784">
       <c r="A784" t="inlineStr">
@@ -67453,7 +67427,6 @@
       <c r="O784" t="n">
         <v>69</v>
       </c>
-      <c r="P784" t="inlineStr"/>
       <c r="Q784" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -67474,7 +67447,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U784" t="inlineStr"/>
     </row>
     <row r="785">
       <c r="A785" t="inlineStr">
@@ -67562,7 +67534,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U785" t="inlineStr"/>
     </row>
     <row r="786">
       <c r="A786" t="inlineStr">
@@ -67632,7 +67603,6 @@
       <c r="O786" t="n">
         <v>43</v>
       </c>
-      <c r="P786" t="inlineStr"/>
       <c r="Q786" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -67653,7 +67623,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U786" t="inlineStr"/>
     </row>
     <row r="787">
       <c r="A787" t="inlineStr">
@@ -67719,7 +67688,6 @@
       <c r="O787" t="n">
         <v>51</v>
       </c>
-      <c r="P787" t="inlineStr"/>
       <c r="R787" t="inlineStr">
         <is>
           <t>10.0.21</t>
@@ -67738,7 +67706,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U787" t="inlineStr"/>
     </row>
     <row r="788">
       <c r="A788" t="inlineStr">
@@ -67808,7 +67775,6 @@
       <c r="O788" t="n">
         <v>13</v>
       </c>
-      <c r="P788" t="inlineStr"/>
       <c r="Q788" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -67829,7 +67795,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U788" t="inlineStr"/>
     </row>
     <row r="789">
       <c r="A789" t="inlineStr">
@@ -67915,7 +67880,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U789" t="inlineStr"/>
     </row>
     <row r="790">
       <c r="A790" t="inlineStr">
@@ -67985,7 +67949,6 @@
       <c r="O790" t="n">
         <v>4</v>
       </c>
-      <c r="P790" t="inlineStr"/>
       <c r="Q790" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -68006,7 +67969,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U790" t="inlineStr"/>
     </row>
     <row r="791">
       <c r="A791" t="inlineStr">
@@ -68092,7 +68054,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U791" t="inlineStr"/>
     </row>
     <row r="792">
       <c r="A792" t="inlineStr">
@@ -68162,7 +68123,6 @@
       <c r="O792" t="n">
         <v>91</v>
       </c>
-      <c r="P792" t="inlineStr"/>
       <c r="Q792" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -68183,7 +68143,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U792" t="inlineStr"/>
     </row>
     <row r="793">
       <c r="A793" t="inlineStr">
@@ -68266,7 +68225,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U793" t="inlineStr"/>
     </row>
     <row r="794">
       <c r="A794" t="inlineStr">
@@ -68336,7 +68294,6 @@
       <c r="O794" t="n">
         <v>10</v>
       </c>
-      <c r="P794" t="inlineStr"/>
       <c r="Q794" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -68357,7 +68314,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U794" t="inlineStr"/>
     </row>
     <row r="795">
       <c r="A795" t="inlineStr">
@@ -68446,7 +68402,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U795" t="inlineStr"/>
     </row>
     <row r="796">
       <c r="A796" t="inlineStr">
@@ -68516,7 +68471,6 @@
       <c r="O796" t="n">
         <v>11</v>
       </c>
-      <c r="P796" t="inlineStr"/>
       <c r="Q796" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -68537,7 +68491,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U796" t="inlineStr"/>
     </row>
     <row r="797">
       <c r="A797" t="inlineStr">
@@ -68624,7 +68577,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U797" t="inlineStr"/>
     </row>
     <row r="798">
       <c r="A798" t="inlineStr">
@@ -68694,7 +68646,6 @@
       <c r="O798" t="n">
         <v>29</v>
       </c>
-      <c r="P798" t="inlineStr"/>
       <c r="Q798" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -68715,7 +68666,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U798" t="inlineStr"/>
     </row>
     <row r="799">
       <c r="A799" t="inlineStr">
@@ -68781,7 +68731,6 @@
       <c r="O799" t="n">
         <v>26</v>
       </c>
-      <c r="P799" t="inlineStr"/>
       <c r="R799" t="inlineStr">
         <is>
           <t>7.3.1</t>
@@ -68802,7 +68751,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U799" t="inlineStr"/>
     </row>
     <row r="800">
       <c r="A800" t="inlineStr">
@@ -68872,7 +68820,6 @@
       <c r="O800" t="n">
         <v>19</v>
       </c>
-      <c r="P800" t="inlineStr"/>
       <c r="Q800" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -68893,7 +68840,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U800" t="inlineStr"/>
     </row>
     <row r="801">
       <c r="A801" t="inlineStr">
@@ -68959,7 +68905,6 @@
       <c r="O801" t="n">
         <v>54</v>
       </c>
-      <c r="P801" t="inlineStr"/>
       <c r="R801" t="inlineStr">
         <is>
           <t>10.1.0</t>
@@ -68978,7 +68923,2825 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U801" t="inlineStr"/>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E802" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F802" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G802" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogn</t>
+        </is>
+      </c>
+      <c r="H802" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I802" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J802" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K802" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L802" t="b">
+        <v>0</v>
+      </c>
+      <c r="M802" t="n">
+        <v>4.4490237</v>
+      </c>
+      <c r="N802" t="n">
+        <v>9346</v>
+      </c>
+      <c r="O802" t="n">
+        <v>39</v>
+      </c>
+      <c r="P802" t="inlineStr"/>
+      <c r="Q802" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R802" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S802" t="inlineStr">
+        <is>
+          <t>Bien plus qu&amp;#39;une application, un véritable assistant personnel pour une vie connectée et simplifiée.&lt;br&gt;Suivi de consommation: Votre tableau de bord tout-en-un pour une gestion simplifiée !&lt;br&gt;- Gestion de votre offre: Accédez à une vue détaillée de votre offre actuelle et de vos forfaits Orange</t>
+        </is>
+      </c>
+      <c r="T802" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U802" t="inlineStr"/>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E803" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F803" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G803" t="n">
+        <v>1177999485</v>
+      </c>
+      <c r="H803" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I803" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J803" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K803" t="n">
+        <v>0</v>
+      </c>
+      <c r="L803" t="b">
+        <v>1</v>
+      </c>
+      <c r="M803" t="n">
+        <v>3.88615</v>
+      </c>
+      <c r="N803" t="n">
+        <v>325</v>
+      </c>
+      <c r="P803" t="inlineStr"/>
+      <c r="R803" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S803" t="inlineStr">
+        <is>
+          <t>La fusion d’Orange et Moi et Orange Money donne naissance à Max it, la nouvelle Super Application Tout-en-Un. Profitez du suivi de consommation, de paiements mobiles, de toutes les fonctionnalités Orange et Moi et Money avec un large éventail de divertissements, le tout regroupé en un seul endroit !</t>
+        </is>
+      </c>
+      <c r="T803" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U803" t="inlineStr"/>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E804" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F804" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G804" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.otn</t>
+        </is>
+      </c>
+      <c r="H804" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I804" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J804" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K804" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L804" t="b">
+        <v>0</v>
+      </c>
+      <c r="M804" t="n">
+        <v>3.9654968</v>
+      </c>
+      <c r="N804" t="n">
+        <v>35389</v>
+      </c>
+      <c r="O804" t="n">
+        <v>27</v>
+      </c>
+      <c r="P804" t="inlineStr"/>
+      <c r="Q804" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R804" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S804" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Max it par Orange Tunisie facilite votre vie au quotidien !&lt;/h2&gt;&lt;br&gt;&lt;br&gt;Welcome sur Max it !&lt;br&gt;Accédez rapidement à vos fonctionnalités Max it préférées et profitez également de contenus exclusifs, d’activités divertissantes, et de jeux interactifs pour une expérience enrichissante avec la roue</t>
+        </is>
+      </c>
+      <c r="T804" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U804" t="inlineStr"/>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D805" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E805" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F805" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G805" t="n">
+        <v>1146892088</v>
+      </c>
+      <c r="H805" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I805" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J805" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K805" t="n">
+        <v>0</v>
+      </c>
+      <c r="L805" t="b">
+        <v>1</v>
+      </c>
+      <c r="M805" t="n">
+        <v>3.02862</v>
+      </c>
+      <c r="N805" t="n">
+        <v>1642</v>
+      </c>
+      <c r="O805" t="n">
+        <v>35</v>
+      </c>
+      <c r="P805" t="inlineStr"/>
+      <c r="R805" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S805" t="inlineStr">
+        <is>
+          <t>Max it by Orange Tunisie : Votre appli incontournable pour une vie connectée
+Welcome sur Max it : Découvrez fonctionnalités, jeux &amp; contenus de divertissement by Orange Tunisie !
+Trouvez vite vos fonctionnalités Max it favorites et explorez des contenus exclusifs et des jeux pour une expérience im</t>
+        </is>
+      </c>
+      <c r="T805" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U805" t="inlineStr"/>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E806" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F806" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G806" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osl</t>
+        </is>
+      </c>
+      <c r="H806" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I806" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J806" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K806" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L806" t="b">
+        <v>0</v>
+      </c>
+      <c r="M806" t="n">
+        <v>4.4429226</v>
+      </c>
+      <c r="N806" t="n">
+        <v>2152</v>
+      </c>
+      <c r="O806" t="n">
+        <v>10</v>
+      </c>
+      <c r="P806" t="inlineStr"/>
+      <c r="Q806" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R806" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S806" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it is a free application, which allows Orange Sierra Leone prepaid and postpaid customers to:&lt;br&gt;&lt;br&gt;- Consult your account in real time: minutes, sms, internet&lt;br&gt;- Top up your account or a friend account &lt;br&gt;- Buy Internet Bundles&lt;br&gt;- Discover the latest offers and promotions &lt;br&gt;- Access to </t>
+        </is>
+      </c>
+      <c r="T806" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U806" t="inlineStr"/>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E807" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F807" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G807" t="n">
+        <v>6443607903</v>
+      </c>
+      <c r="H807" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I807" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J807" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K807" t="n">
+        <v>0</v>
+      </c>
+      <c r="L807" t="b">
+        <v>1</v>
+      </c>
+      <c r="M807" t="n">
+        <v>3.69948</v>
+      </c>
+      <c r="N807" t="n">
+        <v>193</v>
+      </c>
+      <c r="O807" t="n">
+        <v>7</v>
+      </c>
+      <c r="P807" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R807" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S807" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The merger of My Orange &amp; Orange Money has given birth to Max it the all-in-one super app, a free application which allows all Orange Sierra Leone customers to 
+Track calls, SMS, and Data usage and monitor balance. 
+Make a secure mobile/Orange Money payment.
+Easily transfer credit to other users </t>
+        </is>
+      </c>
+      <c r="T807" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U807" t="inlineStr"/>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E808" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F808" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G808" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osn</t>
+        </is>
+      </c>
+      <c r="H808" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I808" t="inlineStr">
+        <is>
+          <t>Orange Sénégal</t>
+        </is>
+      </c>
+      <c r="J808" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K808" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L808" t="b">
+        <v>0</v>
+      </c>
+      <c r="M808" t="n">
+        <v>4.295431</v>
+      </c>
+      <c r="N808" t="n">
+        <v>51345</v>
+      </c>
+      <c r="O808" t="n">
+        <v>8</v>
+      </c>
+      <c r="P808" t="inlineStr"/>
+      <c r="Q808" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R808" t="inlineStr">
+        <is>
+          <t>21.1.0</t>
+        </is>
+      </c>
+      <c r="S808" t="inlineStr">
+        <is>
+          <t>Lu bees ak Max it ! &lt;br&gt;Une application repensée pour être plus simple, plus rapide et adaptée à vos besoins. Une expérience optimisée pour faciliter vos usages au quotidien, avec des parcours simplifiés et un accès plus fluide à vos services. Que vous soyez client Orange ou non, Max it vous accompa</t>
+        </is>
+      </c>
+      <c r="T808" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U808" t="inlineStr"/>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E809" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F809" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G809" t="n">
+        <v>1039327980</v>
+      </c>
+      <c r="H809" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I809" t="inlineStr">
+        <is>
+          <t>Orange Senegal</t>
+        </is>
+      </c>
+      <c r="J809" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K809" t="n">
+        <v>0</v>
+      </c>
+      <c r="L809" t="b">
+        <v>1</v>
+      </c>
+      <c r="M809" t="n">
+        <v>4.16931</v>
+      </c>
+      <c r="N809" t="n">
+        <v>30234</v>
+      </c>
+      <c r="O809" t="n">
+        <v>11</v>
+      </c>
+      <c r="P809" t="inlineStr"/>
+      <c r="R809" t="inlineStr">
+        <is>
+          <t>22.0.0</t>
+        </is>
+      </c>
+      <c r="S809" t="inlineStr">
+        <is>
+          <t>Here is the English translation:
+Welcome to Max it!
+A redesigned app to be simpler, faster, and tailored to your needs. An optimized experience to make your daily life easier, with streamlined journeys and smoother access to your services. Whether you are an Orange customer or not, Max it is your e</t>
+        </is>
+      </c>
+      <c r="T809" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U809" t="inlineStr"/>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E810" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F810" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G810" t="inlineStr">
+        <is>
+          <t>com.orange.meditel.mediteletmoi</t>
+        </is>
+      </c>
+      <c r="H810" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I810" t="inlineStr">
+        <is>
+          <t>Orange Maroc</t>
+        </is>
+      </c>
+      <c r="J810" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K810" t="inlineStr">
+        <is>
+          <t>MAD 0.00</t>
+        </is>
+      </c>
+      <c r="L810" t="b">
+        <v>0</v>
+      </c>
+      <c r="M810" t="n">
+        <v>3.719186</v>
+      </c>
+      <c r="N810" t="n">
+        <v>110945</v>
+      </c>
+      <c r="O810" t="n">
+        <v>53</v>
+      </c>
+      <c r="P810" t="inlineStr"/>
+      <c r="Q810" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R810" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S810" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l&amp;#39;expérience mobile réinventé&lt;br&gt;&lt;br&gt;Max it, c&amp;#39;est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d&amp;#39;une multitude de services exclusifs. &lt;br&gt;&lt;br&gt;Créez votre espace sur</t>
+        </is>
+      </c>
+      <c r="T810" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U810" t="inlineStr"/>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E811" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F811" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G811" t="n">
+        <v>596028698</v>
+      </c>
+      <c r="H811" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I811" t="inlineStr">
+        <is>
+          <t>Méditel</t>
+        </is>
+      </c>
+      <c r="J811" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K811" t="n">
+        <v>0</v>
+      </c>
+      <c r="L811" t="b">
+        <v>1</v>
+      </c>
+      <c r="M811" t="n">
+        <v>3.94495</v>
+      </c>
+      <c r="N811" t="n">
+        <v>2761</v>
+      </c>
+      <c r="P811" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "MA" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R811" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S811" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l'expérience mobile réinventé
+Max it, c'est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d'une multitude de services exclusifs. 
+Créez votre espace sur mesure et bénéficiez d'</t>
+        </is>
+      </c>
+      <c r="T811" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U811" t="inlineStr"/>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E812" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F812" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G812" t="inlineStr">
+        <is>
+          <t>com.oml.dsi.orangemobile</t>
+        </is>
+      </c>
+      <c r="H812" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I812" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J812" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K812" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L812" t="b">
+        <v>0</v>
+      </c>
+      <c r="M812" t="n">
+        <v>2.7071838</v>
+      </c>
+      <c r="N812" t="n">
+        <v>38242</v>
+      </c>
+      <c r="P812" t="inlineStr"/>
+      <c r="Q812" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R812" t="inlineStr">
+        <is>
+          <t>6.5.0</t>
+        </is>
+      </c>
+      <c r="S812" t="inlineStr">
+        <is>
+          <t>Easily manage your Orange Mali line&lt;br&gt;● Manage your account and view all essential information, your offers, and your phone lines.&lt;br&gt;● Subscribe to call, SMS, Internet, and international call packages.&lt;br&gt;● Track your usage by checking your credit and Internet balance.&lt;br&gt;● Recharge your line by p</t>
+        </is>
+      </c>
+      <c r="T812" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U812" t="inlineStr"/>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E813" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F813" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G813" t="n">
+        <v>1494321079</v>
+      </c>
+      <c r="H813" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I813" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J813" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K813" t="n">
+        <v>0</v>
+      </c>
+      <c r="L813" t="b">
+        <v>1</v>
+      </c>
+      <c r="M813" t="n">
+        <v>2.52122</v>
+      </c>
+      <c r="N813" t="n">
+        <v>4760</v>
+      </c>
+      <c r="O813" t="n">
+        <v>12</v>
+      </c>
+      <c r="P813" t="inlineStr"/>
+      <c r="R813" t="inlineStr">
+        <is>
+          <t>6.5.2</t>
+        </is>
+      </c>
+      <c r="S813" t="inlineStr">
+        <is>
+          <t>Gérez facilement votre ligne Orange Mali 
+●        Gérez votre compte et consultez toutes les informations essentielles sur celui-ci, vos offres, ainsi que vos lignes téléphoniques.
+●        Souscrivez aux forfaits appels, SMS, Internet, et appels internationaux.
+●        Suivez votre consommation e</t>
+        </is>
+      </c>
+      <c r="T813" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U813" t="inlineStr"/>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E814" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F814" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G814" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.omg</t>
+        </is>
+      </c>
+      <c r="H814" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I814" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J814" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K814" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L814" t="b">
+        <v>0</v>
+      </c>
+      <c r="M814" t="n">
+        <v>4.141791</v>
+      </c>
+      <c r="N814" t="n">
+        <v>1390</v>
+      </c>
+      <c r="O814" t="n">
+        <v>52</v>
+      </c>
+      <c r="P814" t="inlineStr"/>
+      <c r="Q814" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R814" t="inlineStr">
+        <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="S814" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.&lt;br&gt;&lt;br&gt;Simplify Your Life with Max it&lt;br&gt;With Max It, ac</t>
+        </is>
+      </c>
+      <c r="T814" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U814" t="inlineStr"/>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E815" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F815" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G815" t="n">
+        <v>1295171817</v>
+      </c>
+      <c r="H815" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I815" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J815" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K815" t="n">
+        <v>0</v>
+      </c>
+      <c r="L815" t="b">
+        <v>1</v>
+      </c>
+      <c r="M815" t="n">
+        <v>3.05714</v>
+      </c>
+      <c r="N815" t="n">
+        <v>70</v>
+      </c>
+      <c r="O815" t="n">
+        <v>26</v>
+      </c>
+      <c r="P815" t="inlineStr"/>
+      <c r="R815" t="inlineStr">
+        <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="S815" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.
+Simplify Your Life with Max it
+With Max it, access a se</t>
+        </is>
+      </c>
+      <c r="T815" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U815" t="inlineStr"/>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E816" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F816" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G816" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.olr</t>
+        </is>
+      </c>
+      <c r="H816" t="inlineStr">
+        <is>
+          <t>Orange Max it - Liberia</t>
+        </is>
+      </c>
+      <c r="I816" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J816" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K816" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L816" t="b">
+        <v>0</v>
+      </c>
+      <c r="M816" t="n">
+        <v>4.517685</v>
+      </c>
+      <c r="N816" t="n">
+        <v>3106</v>
+      </c>
+      <c r="O816" t="n">
+        <v>82</v>
+      </c>
+      <c r="P816" t="inlineStr"/>
+      <c r="Q816" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R816" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="S816" t="inlineStr">
+        <is>
+          <t>Max it: your personalized experience by Orange Liberia!&lt;br&gt;&lt;br&gt;Step into Max it, your all-in-one solution for telecom, marketplace, and financial services! Manage your mobile line, customize offers, pay your bills, keep&lt;br&gt;track of your usage with ease, and recharge your credit. Access exclusive eve</t>
+        </is>
+      </c>
+      <c r="T816" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U816" t="inlineStr"/>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E817" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F817" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G817" t="n">
+        <v>6746187327</v>
+      </c>
+      <c r="H817" t="inlineStr">
+        <is>
+          <t>Orange Max it – Liberia</t>
+        </is>
+      </c>
+      <c r="I817" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J817" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K817" t="n">
+        <v>0</v>
+      </c>
+      <c r="L817" t="b">
+        <v>1</v>
+      </c>
+      <c r="M817" t="n">
+        <v>4.0625</v>
+      </c>
+      <c r="N817" t="n">
+        <v>48</v>
+      </c>
+      <c r="P817" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "LR" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R817" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="S817" t="inlineStr">
+        <is>
+          <t>Max it is a free application, which allows Orange Liberia customers to:
+- Consult your account in real time: minutes, sms, internet
+- Top up your account or a friend account 
+- Buy  Bundles (voice, data, SMS, roaming, international)
+- Discover the latest offers and promotions 
+- Access to Orange se</t>
+        </is>
+      </c>
+      <c r="T817" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U817" t="inlineStr"/>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E818" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F818" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G818" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ojo</t>
+        </is>
+      </c>
+      <c r="H818" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I818" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J818" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K818" t="inlineStr">
+        <is>
+          <t>JOD 0.000</t>
+        </is>
+      </c>
+      <c r="L818" t="b">
+        <v>0</v>
+      </c>
+      <c r="M818" t="n">
+        <v>4.4311304</v>
+      </c>
+      <c r="N818" t="n">
+        <v>97841</v>
+      </c>
+      <c r="O818" t="n">
+        <v>41</v>
+      </c>
+      <c r="P818" t="inlineStr"/>
+      <c r="Q818" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R818" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S818" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience&lt;br&gt;Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.&lt;br&gt;Important Update:&lt;br&gt;The jood app (jood Orange) w</t>
+        </is>
+      </c>
+      <c r="T818" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U818" t="inlineStr"/>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E819" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F819" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G819" t="n">
+        <v>808824590</v>
+      </c>
+      <c r="H819" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I819" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J819" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K819" t="n">
+        <v>0</v>
+      </c>
+      <c r="L819" t="b">
+        <v>1</v>
+      </c>
+      <c r="M819" t="n">
+        <v>4.20399</v>
+      </c>
+      <c r="N819" t="n">
+        <v>3054</v>
+      </c>
+      <c r="O819" t="n">
+        <v>44</v>
+      </c>
+      <c r="P819" t="inlineStr"/>
+      <c r="R819" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S819" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience
+Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.
+Important Update:
+The jood app (jood Orange) will be di</t>
+        </is>
+      </c>
+      <c r="T819" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U819" t="inlineStr"/>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E820" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F820" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G820" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.oci</t>
+        </is>
+      </c>
+      <c r="H820" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I820" t="inlineStr">
+        <is>
+          <t>Orange Côte d'Ivoire S.A</t>
+        </is>
+      </c>
+      <c r="J820" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K820" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L820" t="b">
+        <v>0</v>
+      </c>
+      <c r="M820" t="n">
+        <v>4.1485014</v>
+      </c>
+      <c r="N820" t="n">
+        <v>67331</v>
+      </c>
+      <c r="O820" t="n">
+        <v>15</v>
+      </c>
+      <c r="P820" t="inlineStr"/>
+      <c r="Q820" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R820" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S820" t="inlineStr">
+        <is>
+          <t>Aaaahhh, ta super app Max it, n&amp;#39;a pas fini de te surprendre... &lt;br&gt;Est-ce que tu as remarqué ? Maintenant, tu as ton QR code personnalisé en haut de ton écran d&amp;#39;accueil ! Ainsi, tu peux :&lt;br&gt;     scanner le QR code de ton ami(e) pour lui faire un transfert d&amp;#39;&amp;#39;argent&lt;br&gt;     scanner l</t>
+        </is>
+      </c>
+      <c r="T820" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U820" t="inlineStr"/>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E821" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F821" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G821" t="n">
+        <v>1061120855</v>
+      </c>
+      <c r="H821" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I821" t="inlineStr">
+        <is>
+          <t>Orange CI</t>
+        </is>
+      </c>
+      <c r="J821" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K821" t="n">
+        <v>0</v>
+      </c>
+      <c r="L821" t="b">
+        <v>1</v>
+      </c>
+      <c r="M821" t="n">
+        <v>3.78585</v>
+      </c>
+      <c r="N821" t="n">
+        <v>5977</v>
+      </c>
+      <c r="O821" t="n">
+        <v>11</v>
+      </c>
+      <c r="P821" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R821" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S821" t="inlineStr">
+        <is>
+          <t>Max it, la super app all-in-one te fais gagner du temps, et diminue tes soucis... Gagne plus d'espace de stockage sur ton téléphone ; plus besoin de cumuler plusieurs appli d'Orange pour avoir accès à un maximum de services. Max it est là ! Gère ta ligne (SIM) au niveau des pass, des soldes, réalise</t>
+        </is>
+      </c>
+      <c r="T821" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U821" t="inlineStr"/>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E822" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F822" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G822" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogw</t>
+        </is>
+      </c>
+      <c r="H822" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I822" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J822" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K822" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L822" t="b">
+        <v>0</v>
+      </c>
+      <c r="M822" t="n">
+        <v>4.3896103</v>
+      </c>
+      <c r="N822" t="n">
+        <v>1545</v>
+      </c>
+      <c r="O822" t="n">
+        <v>4</v>
+      </c>
+      <c r="P822" t="inlineStr"/>
+      <c r="Q822" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R822" t="inlineStr">
+        <is>
+          <t>4.0.18</t>
+        </is>
+      </c>
+      <c r="S822" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T822" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U822" t="inlineStr"/>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E823" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F823" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G823" t="n">
+        <v>1574668652</v>
+      </c>
+      <c r="H823" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I823" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J823" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K823" t="n">
+        <v>0</v>
+      </c>
+      <c r="L823" t="b">
+        <v>1</v>
+      </c>
+      <c r="M823" t="n">
+        <v>4.05333</v>
+      </c>
+      <c r="N823" t="n">
+        <v>75</v>
+      </c>
+      <c r="O823" t="n">
+        <v>1</v>
+      </c>
+      <c r="P823" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R823" t="inlineStr">
+        <is>
+          <t>6.0.35</t>
+        </is>
+      </c>
+      <c r="S823" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T823" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U823" t="inlineStr"/>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E824" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F824" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G824" t="inlineStr">
+        <is>
+          <t>com.orange.sugu.ocd</t>
+        </is>
+      </c>
+      <c r="H824" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I824" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J824" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K824" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L824" t="b">
+        <v>0</v>
+      </c>
+      <c r="M824" t="n">
+        <v>4.137218</v>
+      </c>
+      <c r="N824" t="n">
+        <v>5320</v>
+      </c>
+      <c r="O824" t="n">
+        <v>91</v>
+      </c>
+      <c r="P824" t="inlineStr"/>
+      <c r="Q824" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R824" t="inlineStr">
+        <is>
+          <t>9.0.12</t>
+        </is>
+      </c>
+      <c r="S824" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DRC that brings together the features of MyOrange, and Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Plans, Mobile Payments, money transfers, bill payments, subscriptions, and entertai</t>
+        </is>
+      </c>
+      <c r="T824" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U824" t="inlineStr"/>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E825" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F825" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G825" t="n">
+        <v>6447896435</v>
+      </c>
+      <c r="H825" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I825" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J825" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K825" t="n">
+        <v>0</v>
+      </c>
+      <c r="L825" t="b">
+        <v>1</v>
+      </c>
+      <c r="M825" t="n">
+        <v>3.55351</v>
+      </c>
+      <c r="N825" t="n">
+        <v>271</v>
+      </c>
+      <c r="P825" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "CD" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R825" t="inlineStr">
+        <is>
+          <t>9.0.6</t>
+        </is>
+      </c>
+      <c r="S825" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DR Congo. It brings together the features of Orange et Moi, as well as Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Packages, Mobile payment, money transfers, bill payment and subscri</t>
+        </is>
+      </c>
+      <c r="T825" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U825" t="inlineStr"/>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E826" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F826" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G826" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ocm</t>
+        </is>
+      </c>
+      <c r="H826" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroon</t>
+        </is>
+      </c>
+      <c r="I826" t="inlineStr">
+        <is>
+          <t>Orange MEA</t>
+        </is>
+      </c>
+      <c r="J826" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K826" t="inlineStr">
+        <is>
+          <t>FCFA 0</t>
+        </is>
+      </c>
+      <c r="L826" t="b">
+        <v>0</v>
+      </c>
+      <c r="M826" t="n">
+        <v>3.9211142</v>
+      </c>
+      <c r="N826" t="n">
+        <v>47044</v>
+      </c>
+      <c r="O826" t="n">
+        <v>12</v>
+      </c>
+      <c r="P826" t="inlineStr"/>
+      <c r="Q826" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R826" t="inlineStr">
+        <is>
+          <t>7.0.23</t>
+        </is>
+      </c>
+      <c r="S826" t="inlineStr">
+        <is>
+          <t>Max it brings together everything that matters to you in one app: managing your lines, money transfer, bill payment, exclusive offers, and a universe of lifestyle and entertainment. Simple, fast, and 100% secure..&lt;br&gt;&lt;br&gt;📞 My line&lt;br&gt;Manage your Orange mobile and landline bundles in a single click:</t>
+        </is>
+      </c>
+      <c r="T826" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U826" t="inlineStr"/>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E827" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F827" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G827" t="n">
+        <v>1116920093</v>
+      </c>
+      <c r="H827" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroun</t>
+        </is>
+      </c>
+      <c r="I827" t="inlineStr">
+        <is>
+          <t>Orange Middle East &amp; Africa</t>
+        </is>
+      </c>
+      <c r="J827" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K827" t="n">
+        <v>0</v>
+      </c>
+      <c r="L827" t="b">
+        <v>1</v>
+      </c>
+      <c r="M827" t="n">
+        <v>3.76834</v>
+      </c>
+      <c r="N827" t="n">
+        <v>16170</v>
+      </c>
+      <c r="O827" t="n">
+        <v>7</v>
+      </c>
+      <c r="P827" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R827" t="inlineStr">
+        <is>
+          <t>7.0.24</t>
+        </is>
+      </c>
+      <c r="S827" t="inlineStr">
+        <is>
+          <t>Avec Max it, Orange rassemble tout ce qui compte pour vous dans une même application : la gestion de vos lignes, les transferts d’argent, payement de vos factures, des offres exclusives et un univers lifestyle et divertissement.
+Simple, rapide et 100 % sécurisée.
+Ma ligne
+Gérez vos forfaits mobiles</t>
+        </is>
+      </c>
+      <c r="T827" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U827" t="inlineStr"/>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E828" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F828" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G828" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obf</t>
+        </is>
+      </c>
+      <c r="H828" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I828" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso</t>
+        </is>
+      </c>
+      <c r="J828" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K828" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L828" t="b">
+        <v>0</v>
+      </c>
+      <c r="M828" t="n">
+        <v>4.136772</v>
+      </c>
+      <c r="N828" t="n">
+        <v>25535</v>
+      </c>
+      <c r="O828" t="n">
+        <v>12</v>
+      </c>
+      <c r="P828" t="inlineStr"/>
+      <c r="Q828" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R828" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S828" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.&lt;br&gt;Gérez vos lignes mobiles, effectuez des transferts d&amp;#39;argent sécurisés, réglez vos factures, profitez d&amp;#39;offres exclusives, effectuez des paiements marchands fiables, et bien plus enco</t>
+        </is>
+      </c>
+      <c r="T828" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U828" t="inlineStr"/>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F829" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G829" t="n">
+        <v>1553774707</v>
+      </c>
+      <c r="H829" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I829" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso SA</t>
+        </is>
+      </c>
+      <c r="J829" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K829" t="n">
+        <v>0</v>
+      </c>
+      <c r="L829" t="b">
+        <v>1</v>
+      </c>
+      <c r="M829" t="n">
+        <v>3.45508</v>
+      </c>
+      <c r="N829" t="n">
+        <v>1180</v>
+      </c>
+      <c r="O829" t="n">
+        <v>5</v>
+      </c>
+      <c r="P829" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R829" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S829" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.
+Gérez vos lignes mobiles, effectuez des transferts d'argent sécurisés, réglez vos factures, profitez d'offres exclusives, effectuez des paiements marchands fiables, et bien plus encore, le tout</t>
+        </is>
+      </c>
+      <c r="T829" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U829" t="inlineStr"/>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E830" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F830" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G830" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obw</t>
+        </is>
+      </c>
+      <c r="H830" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I830" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J830" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K830" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L830" t="b">
+        <v>0</v>
+      </c>
+      <c r="M830" t="n">
+        <v>3.9714286</v>
+      </c>
+      <c r="N830" t="n">
+        <v>2967</v>
+      </c>
+      <c r="O830" t="n">
+        <v>31</v>
+      </c>
+      <c r="P830" t="inlineStr"/>
+      <c r="Q830" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R830" t="inlineStr">
+        <is>
+          <t>7.3.8</t>
+        </is>
+      </c>
+      <c r="S830" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it, the brand-new Orange Botswana Super App that follows Yame and gives you access to four distinct universes for a one-of-a-kind experience!&lt;br&gt;&lt;br&gt;Manage your accounts, make quick payments using QR codes, investigate a range of online goods and services, and discover the many options provided </t>
+        </is>
+      </c>
+      <c r="T830" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U830" t="inlineStr"/>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E831" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F831" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G831" t="n">
+        <v>1195839458</v>
+      </c>
+      <c r="H831" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I831" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J831" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K831" t="n">
+        <v>0</v>
+      </c>
+      <c r="L831" t="b">
+        <v>1</v>
+      </c>
+      <c r="M831" t="n">
+        <v>3.00806</v>
+      </c>
+      <c r="N831" t="n">
+        <v>124</v>
+      </c>
+      <c r="O831" t="n">
+        <v>29</v>
+      </c>
+      <c r="P831" t="inlineStr"/>
+      <c r="R831" t="inlineStr">
+        <is>
+          <t>7.3.1</t>
+        </is>
+      </c>
+      <c r="S831" t="inlineStr">
+        <is>
+          <t>A free mobile self-care application for Orange Botswana’s mobile customers.
+Full Description :
+Max it is a free application, which allows Orange Botswana customers to:
+- Consult your account in real time: minutes, sms, internet ...
+- Top up your account or a friend account  with Orange Money
+-</t>
+        </is>
+      </c>
+      <c r="T831" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U831" t="inlineStr"/>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E832" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F832" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G832" t="inlineStr">
+        <is>
+          <t>com.orange.mobinilandme</t>
+        </is>
+      </c>
+      <c r="H832" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I832" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J832" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K832" t="inlineStr">
+        <is>
+          <t>EGP 0.00</t>
+        </is>
+      </c>
+      <c r="L832" t="b">
+        <v>0</v>
+      </c>
+      <c r="M832" t="n">
+        <v>4.5574694</v>
+      </c>
+      <c r="N832" t="n">
+        <v>934777</v>
+      </c>
+      <c r="O832" t="n">
+        <v>19</v>
+      </c>
+      <c r="P832" t="inlineStr"/>
+      <c r="Q832" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R832" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S832" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion&lt;br&gt;Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.&lt;br&gt;Key services include:&lt;br&gt;• Account Management: Easily manage</t>
+        </is>
+      </c>
+      <c r="T832" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U832" t="inlineStr"/>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>18e813d7-f0ee-40cc-b226-20ffe5f60cfe</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>2026-08-02 06:34:31</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E833" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F833" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G833" t="n">
+        <v>942568333</v>
+      </c>
+      <c r="H833" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I833" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J833" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K833" t="n">
+        <v>0</v>
+      </c>
+      <c r="L833" t="b">
+        <v>1</v>
+      </c>
+      <c r="M833" t="n">
+        <v>4.2526</v>
+      </c>
+      <c r="N833" t="n">
+        <v>118420</v>
+      </c>
+      <c r="O833" t="n">
+        <v>54</v>
+      </c>
+      <c r="P833" t="inlineStr"/>
+      <c r="R833" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S833" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion
+Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.
+Key services include:
+• Account Management: Easily manage your Ora</t>
+        </is>
+      </c>
+      <c r="T833" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U833" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-08-03
</commit_message>
<xml_diff>
--- a/maxit_store_history.xlsx
+++ b/maxit_store_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U833"/>
+  <dimension ref="A1:U865"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -68992,7 +68992,6 @@
       <c r="O802" t="n">
         <v>39</v>
       </c>
-      <c r="P802" t="inlineStr"/>
       <c r="Q802" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -69013,7 +69012,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U802" t="inlineStr"/>
     </row>
     <row r="803">
       <c r="A803" t="inlineStr">
@@ -69076,7 +69074,6 @@
       <c r="N803" t="n">
         <v>325</v>
       </c>
-      <c r="P803" t="inlineStr"/>
       <c r="R803" t="inlineStr">
         <is>
           <t>6.4.12</t>
@@ -69092,7 +69089,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U803" t="inlineStr"/>
     </row>
     <row r="804">
       <c r="A804" t="inlineStr">
@@ -69162,7 +69158,6 @@
       <c r="O804" t="n">
         <v>27</v>
       </c>
-      <c r="P804" t="inlineStr"/>
       <c r="Q804" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -69183,7 +69178,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U804" t="inlineStr"/>
     </row>
     <row r="805">
       <c r="A805" t="inlineStr">
@@ -69249,7 +69243,6 @@
       <c r="O805" t="n">
         <v>35</v>
       </c>
-      <c r="P805" t="inlineStr"/>
       <c r="R805" t="inlineStr">
         <is>
           <t>10.0.7</t>
@@ -69267,7 +69260,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U805" t="inlineStr"/>
     </row>
     <row r="806">
       <c r="A806" t="inlineStr">
@@ -69337,7 +69329,6 @@
       <c r="O806" t="n">
         <v>10</v>
       </c>
-      <c r="P806" t="inlineStr"/>
       <c r="Q806" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -69358,7 +69349,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U806" t="inlineStr"/>
     </row>
     <row r="807">
       <c r="A807" t="inlineStr">
@@ -69447,7 +69437,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U807" t="inlineStr"/>
     </row>
     <row r="808">
       <c r="A808" t="inlineStr">
@@ -69517,7 +69506,6 @@
       <c r="O808" t="n">
         <v>8</v>
       </c>
-      <c r="P808" t="inlineStr"/>
       <c r="Q808" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -69538,7 +69526,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U808" t="inlineStr"/>
     </row>
     <row r="809">
       <c r="A809" t="inlineStr">
@@ -69604,7 +69591,6 @@
       <c r="O809" t="n">
         <v>11</v>
       </c>
-      <c r="P809" t="inlineStr"/>
       <c r="R809" t="inlineStr">
         <is>
           <t>22.0.0</t>
@@ -69622,7 +69608,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U809" t="inlineStr"/>
     </row>
     <row r="810">
       <c r="A810" t="inlineStr">
@@ -69692,7 +69677,6 @@
       <c r="O810" t="n">
         <v>53</v>
       </c>
-      <c r="P810" t="inlineStr"/>
       <c r="Q810" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -69713,7 +69697,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U810" t="inlineStr"/>
     </row>
     <row r="811">
       <c r="A811" t="inlineStr">
@@ -69798,7 +69781,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U811" t="inlineStr"/>
     </row>
     <row r="812">
       <c r="A812" t="inlineStr">
@@ -69865,7 +69847,6 @@
       <c r="N812" t="n">
         <v>38242</v>
       </c>
-      <c r="P812" t="inlineStr"/>
       <c r="Q812" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -69886,7 +69867,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U812" t="inlineStr"/>
     </row>
     <row r="813">
       <c r="A813" t="inlineStr">
@@ -69952,7 +69932,6 @@
       <c r="O813" t="n">
         <v>12</v>
       </c>
-      <c r="P813" t="inlineStr"/>
       <c r="R813" t="inlineStr">
         <is>
           <t>6.5.2</t>
@@ -69971,7 +69950,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U813" t="inlineStr"/>
     </row>
     <row r="814">
       <c r="A814" t="inlineStr">
@@ -70041,7 +70019,6 @@
       <c r="O814" t="n">
         <v>52</v>
       </c>
-      <c r="P814" t="inlineStr"/>
       <c r="Q814" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -70062,7 +70039,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U814" t="inlineStr"/>
     </row>
     <row r="815">
       <c r="A815" t="inlineStr">
@@ -70128,7 +70104,6 @@
       <c r="O815" t="n">
         <v>26</v>
       </c>
-      <c r="P815" t="inlineStr"/>
       <c r="R815" t="inlineStr">
         <is>
           <t>5.0.2</t>
@@ -70146,7 +70121,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U815" t="inlineStr"/>
     </row>
     <row r="816">
       <c r="A816" t="inlineStr">
@@ -70216,7 +70190,6 @@
       <c r="O816" t="n">
         <v>82</v>
       </c>
-      <c r="P816" t="inlineStr"/>
       <c r="Q816" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -70237,7 +70210,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U816" t="inlineStr"/>
     </row>
     <row r="817">
       <c r="A817" t="inlineStr">
@@ -70325,7 +70297,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U817" t="inlineStr"/>
     </row>
     <row r="818">
       <c r="A818" t="inlineStr">
@@ -70395,7 +70366,6 @@
       <c r="O818" t="n">
         <v>41</v>
       </c>
-      <c r="P818" t="inlineStr"/>
       <c r="Q818" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -70416,7 +70386,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U818" t="inlineStr"/>
     </row>
     <row r="819">
       <c r="A819" t="inlineStr">
@@ -70482,7 +70451,6 @@
       <c r="O819" t="n">
         <v>44</v>
       </c>
-      <c r="P819" t="inlineStr"/>
       <c r="R819" t="inlineStr">
         <is>
           <t>10.0.21</t>
@@ -70501,7 +70469,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U819" t="inlineStr"/>
     </row>
     <row r="820">
       <c r="A820" t="inlineStr">
@@ -70571,7 +70538,6 @@
       <c r="O820" t="n">
         <v>15</v>
       </c>
-      <c r="P820" t="inlineStr"/>
       <c r="Q820" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -70592,7 +70558,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U820" t="inlineStr"/>
     </row>
     <row r="821">
       <c r="A821" t="inlineStr">
@@ -70678,7 +70643,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U821" t="inlineStr"/>
     </row>
     <row r="822">
       <c r="A822" t="inlineStr">
@@ -70748,7 +70712,6 @@
       <c r="O822" t="n">
         <v>4</v>
       </c>
-      <c r="P822" t="inlineStr"/>
       <c r="Q822" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -70769,7 +70732,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U822" t="inlineStr"/>
     </row>
     <row r="823">
       <c r="A823" t="inlineStr">
@@ -70855,7 +70817,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U823" t="inlineStr"/>
     </row>
     <row r="824">
       <c r="A824" t="inlineStr">
@@ -70925,7 +70886,6 @@
       <c r="O824" t="n">
         <v>91</v>
       </c>
-      <c r="P824" t="inlineStr"/>
       <c r="Q824" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -70946,7 +70906,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U824" t="inlineStr"/>
     </row>
     <row r="825">
       <c r="A825" t="inlineStr">
@@ -71029,7 +70988,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U825" t="inlineStr"/>
     </row>
     <row r="826">
       <c r="A826" t="inlineStr">
@@ -71099,7 +71057,6 @@
       <c r="O826" t="n">
         <v>12</v>
       </c>
-      <c r="P826" t="inlineStr"/>
       <c r="Q826" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -71120,7 +71077,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U826" t="inlineStr"/>
     </row>
     <row r="827">
       <c r="A827" t="inlineStr">
@@ -71209,7 +71165,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U827" t="inlineStr"/>
     </row>
     <row r="828">
       <c r="A828" t="inlineStr">
@@ -71279,7 +71234,6 @@
       <c r="O828" t="n">
         <v>12</v>
       </c>
-      <c r="P828" t="inlineStr"/>
       <c r="Q828" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -71300,7 +71254,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U828" t="inlineStr"/>
     </row>
     <row r="829">
       <c r="A829" t="inlineStr">
@@ -71387,7 +71340,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U829" t="inlineStr"/>
     </row>
     <row r="830">
       <c r="A830" t="inlineStr">
@@ -71457,7 +71409,6 @@
       <c r="O830" t="n">
         <v>31</v>
       </c>
-      <c r="P830" t="inlineStr"/>
       <c r="Q830" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -71478,7 +71429,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U830" t="inlineStr"/>
     </row>
     <row r="831">
       <c r="A831" t="inlineStr">
@@ -71544,7 +71494,6 @@
       <c r="O831" t="n">
         <v>29</v>
       </c>
-      <c r="P831" t="inlineStr"/>
       <c r="R831" t="inlineStr">
         <is>
           <t>7.3.1</t>
@@ -71565,7 +71514,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U831" t="inlineStr"/>
     </row>
     <row r="832">
       <c r="A832" t="inlineStr">
@@ -71635,7 +71583,6 @@
       <c r="O832" t="n">
         <v>19</v>
       </c>
-      <c r="P832" t="inlineStr"/>
       <c r="Q832" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -71656,7 +71603,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U832" t="inlineStr"/>
     </row>
     <row r="833">
       <c r="A833" t="inlineStr">
@@ -71722,7 +71668,6 @@
       <c r="O833" t="n">
         <v>54</v>
       </c>
-      <c r="P833" t="inlineStr"/>
       <c r="R833" t="inlineStr">
         <is>
           <t>10.1.0</t>
@@ -71741,7 +71686,2825 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U833" t="inlineStr"/>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E834" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F834" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G834" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogn</t>
+        </is>
+      </c>
+      <c r="H834" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I834" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J834" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K834" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L834" t="b">
+        <v>0</v>
+      </c>
+      <c r="M834" t="n">
+        <v>4.4479394</v>
+      </c>
+      <c r="N834" t="n">
+        <v>9363</v>
+      </c>
+      <c r="O834" t="n">
+        <v>40</v>
+      </c>
+      <c r="P834" t="inlineStr"/>
+      <c r="Q834" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R834" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S834" t="inlineStr">
+        <is>
+          <t>Bien plus qu&amp;#39;une application, un véritable assistant personnel pour une vie connectée et simplifiée.&lt;br&gt;Suivi de consommation: Votre tableau de bord tout-en-un pour une gestion simplifiée !&lt;br&gt;- Gestion de votre offre: Accédez à une vue détaillée de votre offre actuelle et de vos forfaits Orange</t>
+        </is>
+      </c>
+      <c r="T834" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U834" t="inlineStr"/>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E835" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F835" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G835" t="n">
+        <v>1177999485</v>
+      </c>
+      <c r="H835" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I835" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J835" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K835" t="n">
+        <v>0</v>
+      </c>
+      <c r="L835" t="b">
+        <v>1</v>
+      </c>
+      <c r="M835" t="n">
+        <v>3.88073</v>
+      </c>
+      <c r="N835" t="n">
+        <v>327</v>
+      </c>
+      <c r="P835" t="inlineStr"/>
+      <c r="R835" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S835" t="inlineStr">
+        <is>
+          <t>La fusion d’Orange et Moi et Orange Money donne naissance à Max it, la nouvelle Super Application Tout-en-Un. Profitez du suivi de consommation, de paiements mobiles, de toutes les fonctionnalités Orange et Moi et Money avec un large éventail de divertissements, le tout regroupé en un seul endroit !</t>
+        </is>
+      </c>
+      <c r="T835" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U835" t="inlineStr"/>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E836" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F836" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G836" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.otn</t>
+        </is>
+      </c>
+      <c r="H836" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I836" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J836" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K836" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L836" t="b">
+        <v>0</v>
+      </c>
+      <c r="M836" t="n">
+        <v>3.9658146</v>
+      </c>
+      <c r="N836" t="n">
+        <v>35392</v>
+      </c>
+      <c r="O836" t="n">
+        <v>26</v>
+      </c>
+      <c r="P836" t="inlineStr"/>
+      <c r="Q836" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R836" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S836" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Max it par Orange Tunisie facilite votre vie au quotidien !&lt;/h2&gt;&lt;br&gt;&lt;br&gt;Welcome sur Max it !&lt;br&gt;Accédez rapidement à vos fonctionnalités Max it préférées et profitez également de contenus exclusifs, d’activités divertissantes, et de jeux interactifs pour une expérience enrichissante avec la roue</t>
+        </is>
+      </c>
+      <c r="T836" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U836" t="inlineStr"/>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E837" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F837" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G837" t="n">
+        <v>1146892088</v>
+      </c>
+      <c r="H837" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I837" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J837" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K837" t="n">
+        <v>0</v>
+      </c>
+      <c r="L837" t="b">
+        <v>1</v>
+      </c>
+      <c r="M837" t="n">
+        <v>3.02862</v>
+      </c>
+      <c r="N837" t="n">
+        <v>1642</v>
+      </c>
+      <c r="O837" t="n">
+        <v>43</v>
+      </c>
+      <c r="P837" t="inlineStr"/>
+      <c r="R837" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S837" t="inlineStr">
+        <is>
+          <t>Max it by Orange Tunisie : Votre appli incontournable pour une vie connectée
+Welcome sur Max it : Découvrez fonctionnalités, jeux &amp; contenus de divertissement by Orange Tunisie !
+Trouvez vite vos fonctionnalités Max it favorites et explorez des contenus exclusifs et des jeux pour une expérience im</t>
+        </is>
+      </c>
+      <c r="T837" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U837" t="inlineStr"/>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E838" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F838" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G838" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osl</t>
+        </is>
+      </c>
+      <c r="H838" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I838" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J838" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K838" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L838" t="b">
+        <v>0</v>
+      </c>
+      <c r="M838" t="n">
+        <v>4.4444447</v>
+      </c>
+      <c r="N838" t="n">
+        <v>2155</v>
+      </c>
+      <c r="O838" t="n">
+        <v>10</v>
+      </c>
+      <c r="P838" t="inlineStr"/>
+      <c r="Q838" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R838" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S838" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it is a free application, which allows Orange Sierra Leone prepaid and postpaid customers to:&lt;br&gt;&lt;br&gt;- Consult your account in real time: minutes, sms, internet&lt;br&gt;- Top up your account or a friend account &lt;br&gt;- Buy Internet Bundles&lt;br&gt;- Discover the latest offers and promotions &lt;br&gt;- Access to </t>
+        </is>
+      </c>
+      <c r="T838" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U838" t="inlineStr"/>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E839" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F839" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G839" t="n">
+        <v>6443607903</v>
+      </c>
+      <c r="H839" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I839" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J839" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K839" t="n">
+        <v>0</v>
+      </c>
+      <c r="L839" t="b">
+        <v>1</v>
+      </c>
+      <c r="M839" t="n">
+        <v>3.69948</v>
+      </c>
+      <c r="N839" t="n">
+        <v>193</v>
+      </c>
+      <c r="O839" t="n">
+        <v>4</v>
+      </c>
+      <c r="P839" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R839" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S839" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The merger of My Orange &amp; Orange Money has given birth to Max it the all-in-one super app, a free application which allows all Orange Sierra Leone customers to 
+Track calls, SMS, and Data usage and monitor balance. 
+Make a secure mobile/Orange Money payment.
+Easily transfer credit to other users </t>
+        </is>
+      </c>
+      <c r="T839" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U839" t="inlineStr"/>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E840" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F840" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G840" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osn</t>
+        </is>
+      </c>
+      <c r="H840" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I840" t="inlineStr">
+        <is>
+          <t>Orange Sénégal</t>
+        </is>
+      </c>
+      <c r="J840" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K840" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L840" t="b">
+        <v>0</v>
+      </c>
+      <c r="M840" t="n">
+        <v>4.2952437</v>
+      </c>
+      <c r="N840" t="n">
+        <v>51365</v>
+      </c>
+      <c r="O840" t="n">
+        <v>8</v>
+      </c>
+      <c r="P840" t="inlineStr"/>
+      <c r="Q840" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R840" t="inlineStr">
+        <is>
+          <t>22.0.1</t>
+        </is>
+      </c>
+      <c r="S840" t="inlineStr">
+        <is>
+          <t>Lu bees ak Max it ! &lt;br&gt;Une application repensée pour être plus simple, plus rapide et adaptée à vos besoins. Une expérience optimisée pour faciliter vos usages au quotidien, avec des parcours simplifiés et un accès plus fluide à vos services. Que vous soyez client Orange ou non, Max it vous accompa</t>
+        </is>
+      </c>
+      <c r="T840" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U840" t="inlineStr"/>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D841" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E841" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F841" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G841" t="n">
+        <v>1039327980</v>
+      </c>
+      <c r="H841" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I841" t="inlineStr">
+        <is>
+          <t>Orange Senegal</t>
+        </is>
+      </c>
+      <c r="J841" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K841" t="n">
+        <v>0</v>
+      </c>
+      <c r="L841" t="b">
+        <v>1</v>
+      </c>
+      <c r="M841" t="n">
+        <v>4.16917</v>
+      </c>
+      <c r="N841" t="n">
+        <v>30236</v>
+      </c>
+      <c r="O841" t="n">
+        <v>7</v>
+      </c>
+      <c r="P841" t="inlineStr"/>
+      <c r="R841" t="inlineStr">
+        <is>
+          <t>22.0.0</t>
+        </is>
+      </c>
+      <c r="S841" t="inlineStr">
+        <is>
+          <t>Here is the English translation:
+Welcome to Max it!
+A redesigned app to be simpler, faster, and tailored to your needs. An optimized experience to make your daily life easier, with streamlined journeys and smoother access to your services. Whether you are an Orange customer or not, Max it is your e</t>
+        </is>
+      </c>
+      <c r="T841" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U841" t="inlineStr"/>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D842" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E842" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F842" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G842" t="inlineStr">
+        <is>
+          <t>com.orange.meditel.mediteletmoi</t>
+        </is>
+      </c>
+      <c r="H842" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I842" t="inlineStr">
+        <is>
+          <t>Orange Maroc</t>
+        </is>
+      </c>
+      <c r="J842" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K842" t="inlineStr">
+        <is>
+          <t>MAD 0.00</t>
+        </is>
+      </c>
+      <c r="L842" t="b">
+        <v>0</v>
+      </c>
+      <c r="M842" t="n">
+        <v>3.718974</v>
+      </c>
+      <c r="N842" t="n">
+        <v>110949</v>
+      </c>
+      <c r="O842" t="n">
+        <v>52</v>
+      </c>
+      <c r="P842" t="inlineStr"/>
+      <c r="Q842" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R842" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S842" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l&amp;#39;expérience mobile réinventé&lt;br&gt;&lt;br&gt;Max it, c&amp;#39;est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d&amp;#39;une multitude de services exclusifs. &lt;br&gt;&lt;br&gt;Créez votre espace sur</t>
+        </is>
+      </c>
+      <c r="T842" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U842" t="inlineStr"/>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F843" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G843" t="n">
+        <v>596028698</v>
+      </c>
+      <c r="H843" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I843" t="inlineStr">
+        <is>
+          <t>Méditel</t>
+        </is>
+      </c>
+      <c r="J843" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K843" t="n">
+        <v>0</v>
+      </c>
+      <c r="L843" t="b">
+        <v>1</v>
+      </c>
+      <c r="M843" t="n">
+        <v>3.94388</v>
+      </c>
+      <c r="N843" t="n">
+        <v>2762</v>
+      </c>
+      <c r="P843" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "MA" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R843" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S843" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l'expérience mobile réinventé
+Max it, c'est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d'une multitude de services exclusifs. 
+Créez votre espace sur mesure et bénéficiez d'</t>
+        </is>
+      </c>
+      <c r="T843" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U843" t="inlineStr"/>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E844" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F844" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G844" t="inlineStr">
+        <is>
+          <t>com.oml.dsi.orangemobile</t>
+        </is>
+      </c>
+      <c r="H844" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I844" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J844" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K844" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L844" t="b">
+        <v>0</v>
+      </c>
+      <c r="M844" t="n">
+        <v>2.7076283</v>
+      </c>
+      <c r="N844" t="n">
+        <v>38240</v>
+      </c>
+      <c r="P844" t="inlineStr"/>
+      <c r="Q844" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R844" t="inlineStr">
+        <is>
+          <t>6.5.0</t>
+        </is>
+      </c>
+      <c r="S844" t="inlineStr">
+        <is>
+          <t>Easily manage your Orange Mali line&lt;br&gt;● Manage your account and view all essential information, your offers, and your phone lines.&lt;br&gt;● Subscribe to call, SMS, Internet, and international call packages.&lt;br&gt;● Track your usage by checking your credit and Internet balance.&lt;br&gt;● Recharge your line by p</t>
+        </is>
+      </c>
+      <c r="T844" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U844" t="inlineStr"/>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F845" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G845" t="n">
+        <v>1494321079</v>
+      </c>
+      <c r="H845" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I845" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J845" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K845" t="n">
+        <v>0</v>
+      </c>
+      <c r="L845" t="b">
+        <v>1</v>
+      </c>
+      <c r="M845" t="n">
+        <v>2.52269</v>
+      </c>
+      <c r="N845" t="n">
+        <v>4760</v>
+      </c>
+      <c r="O845" t="n">
+        <v>10</v>
+      </c>
+      <c r="P845" t="inlineStr"/>
+      <c r="R845" t="inlineStr">
+        <is>
+          <t>6.5.2</t>
+        </is>
+      </c>
+      <c r="S845" t="inlineStr">
+        <is>
+          <t>Gérez facilement votre ligne Orange Mali 
+●        Gérez votre compte et consultez toutes les informations essentielles sur celui-ci, vos offres, ainsi que vos lignes téléphoniques.
+●        Souscrivez aux forfaits appels, SMS, Internet, et appels internationaux.
+●        Suivez votre consommation e</t>
+        </is>
+      </c>
+      <c r="T845" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U845" t="inlineStr"/>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F846" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G846" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.omg</t>
+        </is>
+      </c>
+      <c r="H846" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I846" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J846" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K846" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L846" t="b">
+        <v>0</v>
+      </c>
+      <c r="M846" t="n">
+        <v>4.148148</v>
+      </c>
+      <c r="N846" t="n">
+        <v>1391</v>
+      </c>
+      <c r="O846" t="n">
+        <v>58</v>
+      </c>
+      <c r="P846" t="inlineStr"/>
+      <c r="Q846" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R846" t="inlineStr">
+        <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="S846" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.&lt;br&gt;&lt;br&gt;Simplify Your Life with Max it&lt;br&gt;With Max It, ac</t>
+        </is>
+      </c>
+      <c r="T846" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U846" t="inlineStr"/>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E847" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F847" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G847" t="n">
+        <v>1295171817</v>
+      </c>
+      <c r="H847" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I847" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J847" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K847" t="n">
+        <v>0</v>
+      </c>
+      <c r="L847" t="b">
+        <v>1</v>
+      </c>
+      <c r="M847" t="n">
+        <v>3.05714</v>
+      </c>
+      <c r="N847" t="n">
+        <v>70</v>
+      </c>
+      <c r="O847" t="n">
+        <v>34</v>
+      </c>
+      <c r="P847" t="inlineStr"/>
+      <c r="R847" t="inlineStr">
+        <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="S847" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.
+Simplify Your Life with Max it
+With Max it, access a se</t>
+        </is>
+      </c>
+      <c r="T847" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U847" t="inlineStr"/>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E848" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F848" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G848" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.olr</t>
+        </is>
+      </c>
+      <c r="H848" t="inlineStr">
+        <is>
+          <t>Orange Max it - Liberia</t>
+        </is>
+      </c>
+      <c r="I848" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J848" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K848" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L848" t="b">
+        <v>0</v>
+      </c>
+      <c r="M848" t="n">
+        <v>4.5207667</v>
+      </c>
+      <c r="N848" t="n">
+        <v>3108</v>
+      </c>
+      <c r="O848" t="n">
+        <v>80</v>
+      </c>
+      <c r="P848" t="inlineStr"/>
+      <c r="Q848" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R848" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="S848" t="inlineStr">
+        <is>
+          <t>Max it: your personalized experience by Orange Liberia!&lt;br&gt;&lt;br&gt;Step into Max it, your all-in-one solution for telecom, marketplace, and financial services! Manage your mobile line, customize offers, pay your bills, keep&lt;br&gt;track of your usage with ease, and recharge your credit. Access exclusive eve</t>
+        </is>
+      </c>
+      <c r="T848" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U848" t="inlineStr"/>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E849" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F849" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G849" t="n">
+        <v>6746187327</v>
+      </c>
+      <c r="H849" t="inlineStr">
+        <is>
+          <t>Orange Max it – Liberia</t>
+        </is>
+      </c>
+      <c r="I849" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J849" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K849" t="n">
+        <v>0</v>
+      </c>
+      <c r="L849" t="b">
+        <v>1</v>
+      </c>
+      <c r="M849" t="n">
+        <v>4.0625</v>
+      </c>
+      <c r="N849" t="n">
+        <v>48</v>
+      </c>
+      <c r="P849" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "LR" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R849" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="S849" t="inlineStr">
+        <is>
+          <t>Max it is a free application, which allows Orange Liberia customers to:
+- Consult your account in real time: minutes, sms, internet
+- Top up your account or a friend account 
+- Buy  Bundles (voice, data, SMS, roaming, international)
+- Discover the latest offers and promotions 
+- Access to Orange se</t>
+        </is>
+      </c>
+      <c r="T849" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U849" t="inlineStr"/>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E850" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F850" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G850" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ojo</t>
+        </is>
+      </c>
+      <c r="H850" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I850" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J850" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K850" t="inlineStr">
+        <is>
+          <t>JOD 0.000</t>
+        </is>
+      </c>
+      <c r="L850" t="b">
+        <v>0</v>
+      </c>
+      <c r="M850" t="n">
+        <v>4.4289455</v>
+      </c>
+      <c r="N850" t="n">
+        <v>97886</v>
+      </c>
+      <c r="O850" t="n">
+        <v>42</v>
+      </c>
+      <c r="P850" t="inlineStr"/>
+      <c r="Q850" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R850" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S850" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience&lt;br&gt;Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.&lt;br&gt;Important Update:&lt;br&gt;The jood app (jood Orange) w</t>
+        </is>
+      </c>
+      <c r="T850" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U850" t="inlineStr"/>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E851" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F851" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G851" t="n">
+        <v>808824590</v>
+      </c>
+      <c r="H851" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I851" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J851" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K851" t="n">
+        <v>0</v>
+      </c>
+      <c r="L851" t="b">
+        <v>1</v>
+      </c>
+      <c r="M851" t="n">
+        <v>4.20429</v>
+      </c>
+      <c r="N851" t="n">
+        <v>3074</v>
+      </c>
+      <c r="O851" t="n">
+        <v>50</v>
+      </c>
+      <c r="P851" t="inlineStr"/>
+      <c r="R851" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S851" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience
+Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.
+Important Update:
+The jood app (jood Orange) will be di</t>
+        </is>
+      </c>
+      <c r="T851" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U851" t="inlineStr"/>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F852" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G852" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.oci</t>
+        </is>
+      </c>
+      <c r="H852" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I852" t="inlineStr">
+        <is>
+          <t>Orange Côte d'Ivoire S.A</t>
+        </is>
+      </c>
+      <c r="J852" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K852" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L852" t="b">
+        <v>0</v>
+      </c>
+      <c r="M852" t="n">
+        <v>4.1500297</v>
+      </c>
+      <c r="N852" t="n">
+        <v>67357</v>
+      </c>
+      <c r="O852" t="n">
+        <v>15</v>
+      </c>
+      <c r="P852" t="inlineStr"/>
+      <c r="Q852" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R852" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S852" t="inlineStr">
+        <is>
+          <t>Aaaahhh, ta super app Max it, n&amp;#39;a pas fini de te surprendre... &lt;br&gt;Est-ce que tu as remarqué ? Maintenant, tu as ton QR code personnalisé en haut de ton écran d&amp;#39;accueil ! Ainsi, tu peux :&lt;br&gt;     scanner le QR code de ton ami(e) pour lui faire un transfert d&amp;#39;&amp;#39;argent&lt;br&gt;     scanner l</t>
+        </is>
+      </c>
+      <c r="T852" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U852" t="inlineStr"/>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F853" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G853" t="n">
+        <v>1061120855</v>
+      </c>
+      <c r="H853" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I853" t="inlineStr">
+        <is>
+          <t>Orange CI</t>
+        </is>
+      </c>
+      <c r="J853" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K853" t="n">
+        <v>0</v>
+      </c>
+      <c r="L853" t="b">
+        <v>1</v>
+      </c>
+      <c r="M853" t="n">
+        <v>3.78645</v>
+      </c>
+      <c r="N853" t="n">
+        <v>5980</v>
+      </c>
+      <c r="O853" t="n">
+        <v>10</v>
+      </c>
+      <c r="P853" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R853" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S853" t="inlineStr">
+        <is>
+          <t>Max it, la super app all-in-one te fais gagner du temps, et diminue tes soucis... Gagne plus d'espace de stockage sur ton téléphone ; plus besoin de cumuler plusieurs appli d'Orange pour avoir accès à un maximum de services. Max it est là ! Gère ta ligne (SIM) au niveau des pass, des soldes, réalise</t>
+        </is>
+      </c>
+      <c r="T853" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U853" t="inlineStr"/>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F854" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G854" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogw</t>
+        </is>
+      </c>
+      <c r="H854" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I854" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J854" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K854" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L854" t="b">
+        <v>0</v>
+      </c>
+      <c r="M854" t="n">
+        <v>4.4248366</v>
+      </c>
+      <c r="N854" t="n">
+        <v>1551</v>
+      </c>
+      <c r="O854" t="n">
+        <v>4</v>
+      </c>
+      <c r="P854" t="inlineStr"/>
+      <c r="Q854" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R854" t="inlineStr">
+        <is>
+          <t>4.0.18</t>
+        </is>
+      </c>
+      <c r="S854" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T854" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U854" t="inlineStr"/>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F855" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G855" t="n">
+        <v>1574668652</v>
+      </c>
+      <c r="H855" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I855" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J855" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K855" t="n">
+        <v>0</v>
+      </c>
+      <c r="L855" t="b">
+        <v>1</v>
+      </c>
+      <c r="M855" t="n">
+        <v>4.05333</v>
+      </c>
+      <c r="N855" t="n">
+        <v>75</v>
+      </c>
+      <c r="O855" t="n">
+        <v>1</v>
+      </c>
+      <c r="P855" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R855" t="inlineStr">
+        <is>
+          <t>6.0.35</t>
+        </is>
+      </c>
+      <c r="S855" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T855" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U855" t="inlineStr"/>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E856" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F856" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G856" t="inlineStr">
+        <is>
+          <t>com.orange.sugu.ocd</t>
+        </is>
+      </c>
+      <c r="H856" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I856" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J856" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K856" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L856" t="b">
+        <v>0</v>
+      </c>
+      <c r="M856" t="n">
+        <v>4.1345797</v>
+      </c>
+      <c r="N856" t="n">
+        <v>5323</v>
+      </c>
+      <c r="O856" t="n">
+        <v>87</v>
+      </c>
+      <c r="P856" t="inlineStr"/>
+      <c r="Q856" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R856" t="inlineStr">
+        <is>
+          <t>9.0.12</t>
+        </is>
+      </c>
+      <c r="S856" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DRC that brings together the features of MyOrange, and Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Plans, Mobile Payments, money transfers, bill payments, subscriptions, and entertai</t>
+        </is>
+      </c>
+      <c r="T856" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U856" t="inlineStr"/>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F857" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G857" t="n">
+        <v>6447896435</v>
+      </c>
+      <c r="H857" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I857" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J857" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K857" t="n">
+        <v>0</v>
+      </c>
+      <c r="L857" t="b">
+        <v>1</v>
+      </c>
+      <c r="M857" t="n">
+        <v>3.55351</v>
+      </c>
+      <c r="N857" t="n">
+        <v>271</v>
+      </c>
+      <c r="P857" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "CD" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R857" t="inlineStr">
+        <is>
+          <t>9.0.6</t>
+        </is>
+      </c>
+      <c r="S857" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DR Congo. It brings together the features of Orange et Moi, as well as Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Packages, Mobile payment, money transfers, bill payment and subscri</t>
+        </is>
+      </c>
+      <c r="T857" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U857" t="inlineStr"/>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F858" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G858" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ocm</t>
+        </is>
+      </c>
+      <c r="H858" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroon</t>
+        </is>
+      </c>
+      <c r="I858" t="inlineStr">
+        <is>
+          <t>Orange MEA</t>
+        </is>
+      </c>
+      <c r="J858" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K858" t="inlineStr">
+        <is>
+          <t>FCFA 0</t>
+        </is>
+      </c>
+      <c r="L858" t="b">
+        <v>0</v>
+      </c>
+      <c r="M858" t="n">
+        <v>3.9178343</v>
+      </c>
+      <c r="N858" t="n">
+        <v>47065</v>
+      </c>
+      <c r="O858" t="n">
+        <v>11</v>
+      </c>
+      <c r="P858" t="inlineStr"/>
+      <c r="Q858" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R858" t="inlineStr">
+        <is>
+          <t>7.0.23</t>
+        </is>
+      </c>
+      <c r="S858" t="inlineStr">
+        <is>
+          <t>Max it brings together everything that matters to you in one app: managing your lines, money transfer, bill payment, exclusive offers, and a universe of lifestyle and entertainment. Simple, fast, and 100% secure..&lt;br&gt;&lt;br&gt;📞 My line&lt;br&gt;Manage your Orange mobile and landline bundles in a single click:</t>
+        </is>
+      </c>
+      <c r="T858" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U858" t="inlineStr"/>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F859" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G859" t="n">
+        <v>1116920093</v>
+      </c>
+      <c r="H859" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroun</t>
+        </is>
+      </c>
+      <c r="I859" t="inlineStr">
+        <is>
+          <t>Orange Middle East &amp; Africa</t>
+        </is>
+      </c>
+      <c r="J859" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K859" t="n">
+        <v>0</v>
+      </c>
+      <c r="L859" t="b">
+        <v>1</v>
+      </c>
+      <c r="M859" t="n">
+        <v>3.7683</v>
+      </c>
+      <c r="N859" t="n">
+        <v>16172</v>
+      </c>
+      <c r="O859" t="n">
+        <v>4</v>
+      </c>
+      <c r="P859" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R859" t="inlineStr">
+        <is>
+          <t>7.0.24</t>
+        </is>
+      </c>
+      <c r="S859" t="inlineStr">
+        <is>
+          <t>Avec Max it, Orange rassemble tout ce qui compte pour vous dans une même application : la gestion de vos lignes, les transferts d’argent, payement de vos factures, des offres exclusives et un univers lifestyle et divertissement.
+Simple, rapide et 100 % sécurisée.
+Ma ligne
+Gérez vos forfaits mobiles</t>
+        </is>
+      </c>
+      <c r="T859" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U859" t="inlineStr"/>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F860" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G860" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obf</t>
+        </is>
+      </c>
+      <c r="H860" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I860" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso</t>
+        </is>
+      </c>
+      <c r="J860" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K860" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L860" t="b">
+        <v>0</v>
+      </c>
+      <c r="M860" t="n">
+        <v>4.133255</v>
+      </c>
+      <c r="N860" t="n">
+        <v>25556</v>
+      </c>
+      <c r="O860" t="n">
+        <v>11</v>
+      </c>
+      <c r="P860" t="inlineStr"/>
+      <c r="Q860" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R860" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S860" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.&lt;br&gt;Gérez vos lignes mobiles, effectuez des transferts d&amp;#39;argent sécurisés, réglez vos factures, profitez d&amp;#39;offres exclusives, effectuez des paiements marchands fiables, et bien plus enco</t>
+        </is>
+      </c>
+      <c r="T860" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U860" t="inlineStr"/>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F861" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G861" t="n">
+        <v>1553774707</v>
+      </c>
+      <c r="H861" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I861" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso SA</t>
+        </is>
+      </c>
+      <c r="J861" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K861" t="n">
+        <v>0</v>
+      </c>
+      <c r="L861" t="b">
+        <v>1</v>
+      </c>
+      <c r="M861" t="n">
+        <v>3.45555</v>
+      </c>
+      <c r="N861" t="n">
+        <v>1181</v>
+      </c>
+      <c r="O861" t="n">
+        <v>8</v>
+      </c>
+      <c r="P861" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R861" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S861" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.
+Gérez vos lignes mobiles, effectuez des transferts d'argent sécurisés, réglez vos factures, profitez d'offres exclusives, effectuez des paiements marchands fiables, et bien plus encore, le tout</t>
+        </is>
+      </c>
+      <c r="T861" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U861" t="inlineStr"/>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F862" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G862" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obw</t>
+        </is>
+      </c>
+      <c r="H862" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I862" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J862" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K862" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L862" t="b">
+        <v>0</v>
+      </c>
+      <c r="M862" t="n">
+        <v>3.9714286</v>
+      </c>
+      <c r="N862" t="n">
+        <v>2967</v>
+      </c>
+      <c r="O862" t="n">
+        <v>34</v>
+      </c>
+      <c r="P862" t="inlineStr"/>
+      <c r="Q862" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R862" t="inlineStr">
+        <is>
+          <t>7.3.8</t>
+        </is>
+      </c>
+      <c r="S862" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it, the brand-new Orange Botswana Super App that follows Yame and gives you access to four distinct universes for a one-of-a-kind experience!&lt;br&gt;&lt;br&gt;Manage your accounts, make quick payments using QR codes, investigate a range of online goods and services, and discover the many options provided </t>
+        </is>
+      </c>
+      <c r="T862" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U862" t="inlineStr"/>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E863" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F863" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G863" t="n">
+        <v>1195839458</v>
+      </c>
+      <c r="H863" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I863" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J863" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K863" t="n">
+        <v>0</v>
+      </c>
+      <c r="L863" t="b">
+        <v>1</v>
+      </c>
+      <c r="M863" t="n">
+        <v>3.00806</v>
+      </c>
+      <c r="N863" t="n">
+        <v>124</v>
+      </c>
+      <c r="O863" t="n">
+        <v>46</v>
+      </c>
+      <c r="P863" t="inlineStr"/>
+      <c r="R863" t="inlineStr">
+        <is>
+          <t>7.3.1</t>
+        </is>
+      </c>
+      <c r="S863" t="inlineStr">
+        <is>
+          <t>A free mobile self-care application for Orange Botswana’s mobile customers.
+Full Description :
+Max it is a free application, which allows Orange Botswana customers to:
+- Consult your account in real time: minutes, sms, internet ...
+- Top up your account or a friend account  with Orange Money
+-</t>
+        </is>
+      </c>
+      <c r="T863" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U863" t="inlineStr"/>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F864" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G864" t="inlineStr">
+        <is>
+          <t>com.orange.mobinilandme</t>
+        </is>
+      </c>
+      <c r="H864" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I864" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J864" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K864" t="inlineStr">
+        <is>
+          <t>EGP 0.00</t>
+        </is>
+      </c>
+      <c r="L864" t="b">
+        <v>0</v>
+      </c>
+      <c r="M864" t="n">
+        <v>4.5568175</v>
+      </c>
+      <c r="N864" t="n">
+        <v>935873</v>
+      </c>
+      <c r="O864" t="n">
+        <v>19</v>
+      </c>
+      <c r="P864" t="inlineStr"/>
+      <c r="Q864" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R864" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S864" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion&lt;br&gt;Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.&lt;br&gt;Key services include:&lt;br&gt;• Account Management: Easily manage</t>
+        </is>
+      </c>
+      <c r="T864" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U864" t="inlineStr"/>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>d7ae874f-50c6-4b7a-8d80-29efda9ca6f7</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>2026-08-03 07:28:28</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E865" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F865" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G865" t="n">
+        <v>942568333</v>
+      </c>
+      <c r="H865" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I865" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J865" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K865" t="n">
+        <v>0</v>
+      </c>
+      <c r="L865" t="b">
+        <v>1</v>
+      </c>
+      <c r="M865" t="n">
+        <v>4.25279</v>
+      </c>
+      <c r="N865" t="n">
+        <v>118619</v>
+      </c>
+      <c r="O865" t="n">
+        <v>65</v>
+      </c>
+      <c r="P865" t="inlineStr"/>
+      <c r="R865" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S865" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion
+Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.
+Key services include:
+• Account Management: Easily manage your Ora</t>
+        </is>
+      </c>
+      <c r="T865" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U865" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-08-04
</commit_message>
<xml_diff>
--- a/maxit_store_history.xlsx
+++ b/maxit_store_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U865"/>
+  <dimension ref="A1:U897"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -71755,7 +71755,6 @@
       <c r="O834" t="n">
         <v>40</v>
       </c>
-      <c r="P834" t="inlineStr"/>
       <c r="Q834" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -71776,7 +71775,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U834" t="inlineStr"/>
     </row>
     <row r="835">
       <c r="A835" t="inlineStr">
@@ -71839,7 +71837,6 @@
       <c r="N835" t="n">
         <v>327</v>
       </c>
-      <c r="P835" t="inlineStr"/>
       <c r="R835" t="inlineStr">
         <is>
           <t>6.4.12</t>
@@ -71855,7 +71852,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U835" t="inlineStr"/>
     </row>
     <row r="836">
       <c r="A836" t="inlineStr">
@@ -71925,7 +71921,6 @@
       <c r="O836" t="n">
         <v>26</v>
       </c>
-      <c r="P836" t="inlineStr"/>
       <c r="Q836" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -71946,7 +71941,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U836" t="inlineStr"/>
     </row>
     <row r="837">
       <c r="A837" t="inlineStr">
@@ -72012,7 +72006,6 @@
       <c r="O837" t="n">
         <v>43</v>
       </c>
-      <c r="P837" t="inlineStr"/>
       <c r="R837" t="inlineStr">
         <is>
           <t>10.0.7</t>
@@ -72030,7 +72023,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U837" t="inlineStr"/>
     </row>
     <row r="838">
       <c r="A838" t="inlineStr">
@@ -72100,7 +72092,6 @@
       <c r="O838" t="n">
         <v>10</v>
       </c>
-      <c r="P838" t="inlineStr"/>
       <c r="Q838" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -72121,7 +72112,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U838" t="inlineStr"/>
     </row>
     <row r="839">
       <c r="A839" t="inlineStr">
@@ -72210,7 +72200,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U839" t="inlineStr"/>
     </row>
     <row r="840">
       <c r="A840" t="inlineStr">
@@ -72280,7 +72269,6 @@
       <c r="O840" t="n">
         <v>8</v>
       </c>
-      <c r="P840" t="inlineStr"/>
       <c r="Q840" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -72301,7 +72289,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U840" t="inlineStr"/>
     </row>
     <row r="841">
       <c r="A841" t="inlineStr">
@@ -72367,7 +72354,6 @@
       <c r="O841" t="n">
         <v>7</v>
       </c>
-      <c r="P841" t="inlineStr"/>
       <c r="R841" t="inlineStr">
         <is>
           <t>22.0.0</t>
@@ -72385,7 +72371,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U841" t="inlineStr"/>
     </row>
     <row r="842">
       <c r="A842" t="inlineStr">
@@ -72455,7 +72440,6 @@
       <c r="O842" t="n">
         <v>52</v>
       </c>
-      <c r="P842" t="inlineStr"/>
       <c r="Q842" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -72476,7 +72460,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U842" t="inlineStr"/>
     </row>
     <row r="843">
       <c r="A843" t="inlineStr">
@@ -72561,7 +72544,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U843" t="inlineStr"/>
     </row>
     <row r="844">
       <c r="A844" t="inlineStr">
@@ -72628,7 +72610,6 @@
       <c r="N844" t="n">
         <v>38240</v>
       </c>
-      <c r="P844" t="inlineStr"/>
       <c r="Q844" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -72649,7 +72630,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U844" t="inlineStr"/>
     </row>
     <row r="845">
       <c r="A845" t="inlineStr">
@@ -72715,7 +72695,6 @@
       <c r="O845" t="n">
         <v>10</v>
       </c>
-      <c r="P845" t="inlineStr"/>
       <c r="R845" t="inlineStr">
         <is>
           <t>6.5.2</t>
@@ -72734,7 +72713,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U845" t="inlineStr"/>
     </row>
     <row r="846">
       <c r="A846" t="inlineStr">
@@ -72804,7 +72782,6 @@
       <c r="O846" t="n">
         <v>58</v>
       </c>
-      <c r="P846" t="inlineStr"/>
       <c r="Q846" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -72825,7 +72802,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U846" t="inlineStr"/>
     </row>
     <row r="847">
       <c r="A847" t="inlineStr">
@@ -72891,7 +72867,6 @@
       <c r="O847" t="n">
         <v>34</v>
       </c>
-      <c r="P847" t="inlineStr"/>
       <c r="R847" t="inlineStr">
         <is>
           <t>5.0.2</t>
@@ -72909,7 +72884,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U847" t="inlineStr"/>
     </row>
     <row r="848">
       <c r="A848" t="inlineStr">
@@ -72979,7 +72953,6 @@
       <c r="O848" t="n">
         <v>80</v>
       </c>
-      <c r="P848" t="inlineStr"/>
       <c r="Q848" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -73000,7 +72973,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U848" t="inlineStr"/>
     </row>
     <row r="849">
       <c r="A849" t="inlineStr">
@@ -73088,7 +73060,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U849" t="inlineStr"/>
     </row>
     <row r="850">
       <c r="A850" t="inlineStr">
@@ -73158,7 +73129,6 @@
       <c r="O850" t="n">
         <v>42</v>
       </c>
-      <c r="P850" t="inlineStr"/>
       <c r="Q850" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -73179,7 +73149,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U850" t="inlineStr"/>
     </row>
     <row r="851">
       <c r="A851" t="inlineStr">
@@ -73245,7 +73214,6 @@
       <c r="O851" t="n">
         <v>50</v>
       </c>
-      <c r="P851" t="inlineStr"/>
       <c r="R851" t="inlineStr">
         <is>
           <t>10.0.21</t>
@@ -73264,7 +73232,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U851" t="inlineStr"/>
     </row>
     <row r="852">
       <c r="A852" t="inlineStr">
@@ -73334,7 +73301,6 @@
       <c r="O852" t="n">
         <v>15</v>
       </c>
-      <c r="P852" t="inlineStr"/>
       <c r="Q852" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -73355,7 +73321,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U852" t="inlineStr"/>
     </row>
     <row r="853">
       <c r="A853" t="inlineStr">
@@ -73441,7 +73406,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U853" t="inlineStr"/>
     </row>
     <row r="854">
       <c r="A854" t="inlineStr">
@@ -73511,7 +73475,6 @@
       <c r="O854" t="n">
         <v>4</v>
       </c>
-      <c r="P854" t="inlineStr"/>
       <c r="Q854" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -73532,7 +73495,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U854" t="inlineStr"/>
     </row>
     <row r="855">
       <c r="A855" t="inlineStr">
@@ -73618,7 +73580,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U855" t="inlineStr"/>
     </row>
     <row r="856">
       <c r="A856" t="inlineStr">
@@ -73688,7 +73649,6 @@
       <c r="O856" t="n">
         <v>87</v>
       </c>
-      <c r="P856" t="inlineStr"/>
       <c r="Q856" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -73709,7 +73669,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U856" t="inlineStr"/>
     </row>
     <row r="857">
       <c r="A857" t="inlineStr">
@@ -73792,7 +73751,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U857" t="inlineStr"/>
     </row>
     <row r="858">
       <c r="A858" t="inlineStr">
@@ -73862,7 +73820,6 @@
       <c r="O858" t="n">
         <v>11</v>
       </c>
-      <c r="P858" t="inlineStr"/>
       <c r="Q858" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -73883,7 +73840,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U858" t="inlineStr"/>
     </row>
     <row r="859">
       <c r="A859" t="inlineStr">
@@ -73972,7 +73928,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U859" t="inlineStr"/>
     </row>
     <row r="860">
       <c r="A860" t="inlineStr">
@@ -74042,7 +73997,6 @@
       <c r="O860" t="n">
         <v>11</v>
       </c>
-      <c r="P860" t="inlineStr"/>
       <c r="Q860" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -74063,7 +74017,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U860" t="inlineStr"/>
     </row>
     <row r="861">
       <c r="A861" t="inlineStr">
@@ -74150,7 +74103,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U861" t="inlineStr"/>
     </row>
     <row r="862">
       <c r="A862" t="inlineStr">
@@ -74220,7 +74172,6 @@
       <c r="O862" t="n">
         <v>34</v>
       </c>
-      <c r="P862" t="inlineStr"/>
       <c r="Q862" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -74241,7 +74192,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U862" t="inlineStr"/>
     </row>
     <row r="863">
       <c r="A863" t="inlineStr">
@@ -74307,7 +74257,6 @@
       <c r="O863" t="n">
         <v>46</v>
       </c>
-      <c r="P863" t="inlineStr"/>
       <c r="R863" t="inlineStr">
         <is>
           <t>7.3.1</t>
@@ -74328,7 +74277,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U863" t="inlineStr"/>
     </row>
     <row r="864">
       <c r="A864" t="inlineStr">
@@ -74398,7 +74346,6 @@
       <c r="O864" t="n">
         <v>19</v>
       </c>
-      <c r="P864" t="inlineStr"/>
       <c r="Q864" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -74419,7 +74366,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U864" t="inlineStr"/>
     </row>
     <row r="865">
       <c r="A865" t="inlineStr">
@@ -74485,7 +74431,6 @@
       <c r="O865" t="n">
         <v>65</v>
       </c>
-      <c r="P865" t="inlineStr"/>
       <c r="R865" t="inlineStr">
         <is>
           <t>10.1.0</t>
@@ -74504,7 +74449,2825 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U865" t="inlineStr"/>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E866" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F866" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G866" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogn</t>
+        </is>
+      </c>
+      <c r="H866" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I866" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J866" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K866" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L866" t="b">
+        <v>0</v>
+      </c>
+      <c r="M866" t="n">
+        <v>4.451193</v>
+      </c>
+      <c r="N866" t="n">
+        <v>9381</v>
+      </c>
+      <c r="O866" t="n">
+        <v>39</v>
+      </c>
+      <c r="P866" t="inlineStr"/>
+      <c r="Q866" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R866" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S866" t="inlineStr">
+        <is>
+          <t>Bien plus qu&amp;#39;une application, un véritable assistant personnel pour une vie connectée et simplifiée.&lt;br&gt;Suivi de consommation: Votre tableau de bord tout-en-un pour une gestion simplifiée !&lt;br&gt;- Gestion de votre offre: Accédez à une vue détaillée de votre offre actuelle et de vos forfaits Orange</t>
+        </is>
+      </c>
+      <c r="T866" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U866" t="inlineStr"/>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E867" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F867" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G867" t="n">
+        <v>1177999485</v>
+      </c>
+      <c r="H867" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I867" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J867" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K867" t="n">
+        <v>0</v>
+      </c>
+      <c r="L867" t="b">
+        <v>1</v>
+      </c>
+      <c r="M867" t="n">
+        <v>3.89759</v>
+      </c>
+      <c r="N867" t="n">
+        <v>332</v>
+      </c>
+      <c r="P867" t="inlineStr"/>
+      <c r="R867" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S867" t="inlineStr">
+        <is>
+          <t>La fusion d’Orange et Moi et Orange Money donne naissance à Max it, la nouvelle Super Application Tout-en-Un. Profitez du suivi de consommation, de paiements mobiles, de toutes les fonctionnalités Orange et Moi et Money avec un large éventail de divertissements, le tout regroupé en un seul endroit !</t>
+        </is>
+      </c>
+      <c r="T867" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U867" t="inlineStr"/>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E868" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F868" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G868" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.otn</t>
+        </is>
+      </c>
+      <c r="H868" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I868" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J868" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K868" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L868" t="b">
+        <v>0</v>
+      </c>
+      <c r="M868" t="n">
+        <v>3.965507</v>
+      </c>
+      <c r="N868" t="n">
+        <v>35390</v>
+      </c>
+      <c r="O868" t="n">
+        <v>31</v>
+      </c>
+      <c r="P868" t="inlineStr"/>
+      <c r="Q868" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R868" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S868" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Max it par Orange Tunisie facilite votre vie au quotidien !&lt;/h2&gt;&lt;br&gt;&lt;br&gt;Welcome sur Max it !&lt;br&gt;Accédez rapidement à vos fonctionnalités Max it préférées et profitez également de contenus exclusifs, d’activités divertissantes, et de jeux interactifs pour une expérience enrichissante avec la roue</t>
+        </is>
+      </c>
+      <c r="T868" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U868" t="inlineStr"/>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E869" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F869" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G869" t="n">
+        <v>1146892088</v>
+      </c>
+      <c r="H869" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I869" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J869" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K869" t="n">
+        <v>0</v>
+      </c>
+      <c r="L869" t="b">
+        <v>1</v>
+      </c>
+      <c r="M869" t="n">
+        <v>3.02862</v>
+      </c>
+      <c r="N869" t="n">
+        <v>1642</v>
+      </c>
+      <c r="O869" t="n">
+        <v>41</v>
+      </c>
+      <c r="P869" t="inlineStr"/>
+      <c r="R869" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S869" t="inlineStr">
+        <is>
+          <t>Max it by Orange Tunisie : Votre appli incontournable pour une vie connectée
+Welcome sur Max it : Découvrez fonctionnalités, jeux &amp; contenus de divertissement by Orange Tunisie !
+Trouvez vite vos fonctionnalités Max it favorites et explorez des contenus exclusifs et des jeux pour une expérience im</t>
+        </is>
+      </c>
+      <c r="T869" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U869" t="inlineStr"/>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F870" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G870" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osl</t>
+        </is>
+      </c>
+      <c r="H870" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I870" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J870" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K870" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L870" t="b">
+        <v>0</v>
+      </c>
+      <c r="M870" t="n">
+        <v>4.447005</v>
+      </c>
+      <c r="N870" t="n">
+        <v>2160</v>
+      </c>
+      <c r="O870" t="n">
+        <v>10</v>
+      </c>
+      <c r="P870" t="inlineStr"/>
+      <c r="Q870" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R870" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S870" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it is a free application, which allows Orange Sierra Leone prepaid and postpaid customers to:&lt;br&gt;&lt;br&gt;- Consult your account in real time: minutes, sms, internet&lt;br&gt;- Top up your account or a friend account &lt;br&gt;- Buy Internet Bundles&lt;br&gt;- Discover the latest offers and promotions &lt;br&gt;- Access to </t>
+        </is>
+      </c>
+      <c r="T870" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U870" t="inlineStr"/>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E871" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F871" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G871" t="n">
+        <v>6443607903</v>
+      </c>
+      <c r="H871" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I871" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J871" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K871" t="n">
+        <v>0</v>
+      </c>
+      <c r="L871" t="b">
+        <v>1</v>
+      </c>
+      <c r="M871" t="n">
+        <v>3.69948</v>
+      </c>
+      <c r="N871" t="n">
+        <v>193</v>
+      </c>
+      <c r="O871" t="n">
+        <v>5</v>
+      </c>
+      <c r="P871" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R871" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S871" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The merger of My Orange &amp; Orange Money has given birth to Max it the all-in-one super app, a free application which allows all Orange Sierra Leone customers to 
+Track calls, SMS, and Data usage and monitor balance. 
+Make a secure mobile/Orange Money payment.
+Easily transfer credit to other users </t>
+        </is>
+      </c>
+      <c r="T871" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U871" t="inlineStr"/>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D872" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E872" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F872" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G872" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osn</t>
+        </is>
+      </c>
+      <c r="H872" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I872" t="inlineStr">
+        <is>
+          <t>Orange Sénégal</t>
+        </is>
+      </c>
+      <c r="J872" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K872" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L872" t="b">
+        <v>0</v>
+      </c>
+      <c r="M872" t="n">
+        <v>4.294166</v>
+      </c>
+      <c r="N872" t="n">
+        <v>51379</v>
+      </c>
+      <c r="O872" t="n">
+        <v>8</v>
+      </c>
+      <c r="P872" t="inlineStr"/>
+      <c r="Q872" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R872" t="inlineStr">
+        <is>
+          <t>22.0.1</t>
+        </is>
+      </c>
+      <c r="S872" t="inlineStr">
+        <is>
+          <t>Lu bees ak Max it ! &lt;br&gt;Une application repensée pour être plus simple, plus rapide et adaptée à vos besoins. Une expérience optimisée pour faciliter vos usages au quotidien, avec des parcours simplifiés et un accès plus fluide à vos services. Que vous soyez client Orange ou non, Max it vous accompa</t>
+        </is>
+      </c>
+      <c r="T872" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U872" t="inlineStr"/>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D873" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E873" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F873" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G873" t="n">
+        <v>1039327980</v>
+      </c>
+      <c r="H873" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I873" t="inlineStr">
+        <is>
+          <t>Orange Senegal</t>
+        </is>
+      </c>
+      <c r="J873" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K873" t="n">
+        <v>0</v>
+      </c>
+      <c r="L873" t="b">
+        <v>1</v>
+      </c>
+      <c r="M873" t="n">
+        <v>4.16922</v>
+      </c>
+      <c r="N873" t="n">
+        <v>30239</v>
+      </c>
+      <c r="O873" t="n">
+        <v>12</v>
+      </c>
+      <c r="P873" t="inlineStr"/>
+      <c r="R873" t="inlineStr">
+        <is>
+          <t>22.0.1</t>
+        </is>
+      </c>
+      <c r="S873" t="inlineStr">
+        <is>
+          <t>Here is the English translation:
+Welcome to Max it!
+A redesigned app to be simpler, faster, and tailored to your needs. An optimized experience to make your daily life easier, with streamlined journeys and smoother access to your services. Whether you are an Orange customer or not, Max it is your e</t>
+        </is>
+      </c>
+      <c r="T873" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U873" t="inlineStr"/>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D874" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E874" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F874" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G874" t="inlineStr">
+        <is>
+          <t>com.orange.meditel.mediteletmoi</t>
+        </is>
+      </c>
+      <c r="H874" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I874" t="inlineStr">
+        <is>
+          <t>Orange Maroc</t>
+        </is>
+      </c>
+      <c r="J874" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K874" t="inlineStr">
+        <is>
+          <t>MAD 0.00</t>
+        </is>
+      </c>
+      <c r="L874" t="b">
+        <v>0</v>
+      </c>
+      <c r="M874" t="n">
+        <v>3.7150326</v>
+      </c>
+      <c r="N874" t="n">
+        <v>110950</v>
+      </c>
+      <c r="O874" t="n">
+        <v>49</v>
+      </c>
+      <c r="P874" t="inlineStr"/>
+      <c r="Q874" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R874" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S874" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l&amp;#39;expérience mobile réinventé&lt;br&gt;&lt;br&gt;Max it, c&amp;#39;est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d&amp;#39;une multitude de services exclusifs. &lt;br&gt;&lt;br&gt;Créez votre espace sur</t>
+        </is>
+      </c>
+      <c r="T874" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U874" t="inlineStr"/>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D875" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E875" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F875" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G875" t="n">
+        <v>596028698</v>
+      </c>
+      <c r="H875" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I875" t="inlineStr">
+        <is>
+          <t>Méditel</t>
+        </is>
+      </c>
+      <c r="J875" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K875" t="n">
+        <v>0</v>
+      </c>
+      <c r="L875" t="b">
+        <v>1</v>
+      </c>
+      <c r="M875" t="n">
+        <v>3.94388</v>
+      </c>
+      <c r="N875" t="n">
+        <v>2762</v>
+      </c>
+      <c r="P875" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "MA" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R875" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S875" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l'expérience mobile réinventé
+Max it, c'est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d'une multitude de services exclusifs. 
+Créez votre espace sur mesure et bénéficiez d'</t>
+        </is>
+      </c>
+      <c r="T875" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U875" t="inlineStr"/>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D876" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E876" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F876" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G876" t="inlineStr">
+        <is>
+          <t>com.oml.dsi.orangemobile</t>
+        </is>
+      </c>
+      <c r="H876" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I876" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J876" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K876" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L876" t="b">
+        <v>0</v>
+      </c>
+      <c r="M876" t="n">
+        <v>2.7085178</v>
+      </c>
+      <c r="N876" t="n">
+        <v>38237</v>
+      </c>
+      <c r="P876" t="inlineStr"/>
+      <c r="Q876" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R876" t="inlineStr">
+        <is>
+          <t>6.5.0</t>
+        </is>
+      </c>
+      <c r="S876" t="inlineStr">
+        <is>
+          <t>Easily manage your Orange Mali line&lt;br&gt;● Manage your account and view all essential information, your offers, and your phone lines.&lt;br&gt;● Subscribe to call, SMS, Internet, and international call packages.&lt;br&gt;● Track your usage by checking your credit and Internet balance.&lt;br&gt;● Recharge your line by p</t>
+        </is>
+      </c>
+      <c r="T876" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U876" t="inlineStr"/>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D877" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E877" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F877" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G877" t="n">
+        <v>1494321079</v>
+      </c>
+      <c r="H877" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I877" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J877" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K877" t="n">
+        <v>0</v>
+      </c>
+      <c r="L877" t="b">
+        <v>1</v>
+      </c>
+      <c r="M877" t="n">
+        <v>2.52394</v>
+      </c>
+      <c r="N877" t="n">
+        <v>4762</v>
+      </c>
+      <c r="O877" t="n">
+        <v>13</v>
+      </c>
+      <c r="P877" t="inlineStr"/>
+      <c r="R877" t="inlineStr">
+        <is>
+          <t>6.5.2</t>
+        </is>
+      </c>
+      <c r="S877" t="inlineStr">
+        <is>
+          <t>Gérez facilement votre ligne Orange Mali 
+●        Gérez votre compte et consultez toutes les informations essentielles sur celui-ci, vos offres, ainsi que vos lignes téléphoniques.
+●        Souscrivez aux forfaits appels, SMS, Internet, et appels internationaux.
+●        Suivez votre consommation e</t>
+        </is>
+      </c>
+      <c r="T877" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U877" t="inlineStr"/>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D878" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E878" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F878" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G878" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.omg</t>
+        </is>
+      </c>
+      <c r="H878" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I878" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J878" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K878" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L878" t="b">
+        <v>0</v>
+      </c>
+      <c r="M878" t="n">
+        <v>4.1654677</v>
+      </c>
+      <c r="N878" t="n">
+        <v>1394</v>
+      </c>
+      <c r="O878" t="n">
+        <v>62</v>
+      </c>
+      <c r="P878" t="inlineStr"/>
+      <c r="Q878" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R878" t="inlineStr">
+        <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="S878" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.&lt;br&gt;&lt;br&gt;Simplify Your Life with Max it&lt;br&gt;With Max It, ac</t>
+        </is>
+      </c>
+      <c r="T878" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U878" t="inlineStr"/>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D879" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E879" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F879" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G879" t="n">
+        <v>1295171817</v>
+      </c>
+      <c r="H879" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I879" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J879" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K879" t="n">
+        <v>0</v>
+      </c>
+      <c r="L879" t="b">
+        <v>1</v>
+      </c>
+      <c r="M879" t="n">
+        <v>3.05714</v>
+      </c>
+      <c r="N879" t="n">
+        <v>70</v>
+      </c>
+      <c r="O879" t="n">
+        <v>33</v>
+      </c>
+      <c r="P879" t="inlineStr"/>
+      <c r="R879" t="inlineStr">
+        <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="S879" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.
+Simplify Your Life with Max it
+With Max it, access a se</t>
+        </is>
+      </c>
+      <c r="T879" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U879" t="inlineStr"/>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D880" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E880" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F880" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G880" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.olr</t>
+        </is>
+      </c>
+      <c r="H880" t="inlineStr">
+        <is>
+          <t>Orange Max it - Liberia</t>
+        </is>
+      </c>
+      <c r="I880" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J880" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K880" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L880" t="b">
+        <v>0</v>
+      </c>
+      <c r="M880" t="n">
+        <v>4.5207667</v>
+      </c>
+      <c r="N880" t="n">
+        <v>3107</v>
+      </c>
+      <c r="O880" t="n">
+        <v>77</v>
+      </c>
+      <c r="P880" t="inlineStr"/>
+      <c r="Q880" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R880" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="S880" t="inlineStr">
+        <is>
+          <t>Max it: your personalized experience by Orange Liberia!&lt;br&gt;&lt;br&gt;Step into Max it, your all-in-one solution for telecom, marketplace, and financial services! Manage your mobile line, customize offers, pay your bills, keep&lt;br&gt;track of your usage with ease, and recharge your credit. Access exclusive eve</t>
+        </is>
+      </c>
+      <c r="T880" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U880" t="inlineStr"/>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D881" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E881" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F881" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G881" t="n">
+        <v>6746187327</v>
+      </c>
+      <c r="H881" t="inlineStr">
+        <is>
+          <t>Orange Max it – Liberia</t>
+        </is>
+      </c>
+      <c r="I881" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J881" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K881" t="n">
+        <v>0</v>
+      </c>
+      <c r="L881" t="b">
+        <v>1</v>
+      </c>
+      <c r="M881" t="n">
+        <v>4.0625</v>
+      </c>
+      <c r="N881" t="n">
+        <v>48</v>
+      </c>
+      <c r="P881" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "LR" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R881" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="S881" t="inlineStr">
+        <is>
+          <t>Max it is a free application, which allows Orange Liberia customers to:
+- Consult your account in real time: minutes, sms, internet
+- Top up your account or a friend account 
+- Buy  Bundles (voice, data, SMS, roaming, international)
+- Discover the latest offers and promotions 
+- Access to Orange se</t>
+        </is>
+      </c>
+      <c r="T881" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U881" t="inlineStr"/>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E882" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F882" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G882" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ojo</t>
+        </is>
+      </c>
+      <c r="H882" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I882" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J882" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K882" t="inlineStr">
+        <is>
+          <t>JOD 0.000</t>
+        </is>
+      </c>
+      <c r="L882" t="b">
+        <v>0</v>
+      </c>
+      <c r="M882" t="n">
+        <v>4.42854</v>
+      </c>
+      <c r="N882" t="n">
+        <v>97891</v>
+      </c>
+      <c r="O882" t="n">
+        <v>41</v>
+      </c>
+      <c r="P882" t="inlineStr"/>
+      <c r="Q882" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R882" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S882" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience&lt;br&gt;Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.&lt;br&gt;Important Update:&lt;br&gt;The jood app (jood Orange) w</t>
+        </is>
+      </c>
+      <c r="T882" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U882" t="inlineStr"/>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D883" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E883" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F883" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G883" t="n">
+        <v>808824590</v>
+      </c>
+      <c r="H883" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I883" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J883" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K883" t="n">
+        <v>0</v>
+      </c>
+      <c r="L883" t="b">
+        <v>1</v>
+      </c>
+      <c r="M883" t="n">
+        <v>4.20486</v>
+      </c>
+      <c r="N883" t="n">
+        <v>3085</v>
+      </c>
+      <c r="O883" t="n">
+        <v>54</v>
+      </c>
+      <c r="P883" t="inlineStr"/>
+      <c r="R883" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S883" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience
+Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.
+Important Update:
+The jood app (jood Orange) will be di</t>
+        </is>
+      </c>
+      <c r="T883" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U883" t="inlineStr"/>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E884" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F884" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G884" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.oci</t>
+        </is>
+      </c>
+      <c r="H884" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I884" t="inlineStr">
+        <is>
+          <t>Orange Côte d'Ivoire S.A</t>
+        </is>
+      </c>
+      <c r="J884" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K884" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L884" t="b">
+        <v>0</v>
+      </c>
+      <c r="M884" t="n">
+        <v>4.1427503</v>
+      </c>
+      <c r="N884" t="n">
+        <v>67384</v>
+      </c>
+      <c r="O884" t="n">
+        <v>14</v>
+      </c>
+      <c r="P884" t="inlineStr"/>
+      <c r="Q884" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R884" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S884" t="inlineStr">
+        <is>
+          <t>Aaaahhh, ta super app Max it, n&amp;#39;a pas fini de te surprendre... &lt;br&gt;Est-ce que tu as remarqué ? Maintenant, tu as ton QR code personnalisé en haut de ton écran d&amp;#39;accueil ! Ainsi, tu peux :&lt;br&gt;     scanner le QR code de ton ami(e) pour lui faire un transfert d&amp;#39;&amp;#39;argent&lt;br&gt;     scanner l</t>
+        </is>
+      </c>
+      <c r="T884" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U884" t="inlineStr"/>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D885" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E885" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F885" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G885" t="n">
+        <v>1061120855</v>
+      </c>
+      <c r="H885" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I885" t="inlineStr">
+        <is>
+          <t>Orange CI</t>
+        </is>
+      </c>
+      <c r="J885" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K885" t="n">
+        <v>0</v>
+      </c>
+      <c r="L885" t="b">
+        <v>1</v>
+      </c>
+      <c r="M885" t="n">
+        <v>3.78666</v>
+      </c>
+      <c r="N885" t="n">
+        <v>5981</v>
+      </c>
+      <c r="O885" t="n">
+        <v>14</v>
+      </c>
+      <c r="P885" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R885" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S885" t="inlineStr">
+        <is>
+          <t>Max it, la super app all-in-one te fais gagner du temps, et diminue tes soucis... Gagne plus d'espace de stockage sur ton téléphone ; plus besoin de cumuler plusieurs appli d'Orange pour avoir accès à un maximum de services. Max it est là ! Gère ta ligne (SIM) au niveau des pass, des soldes, réalise</t>
+        </is>
+      </c>
+      <c r="T885" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U885" t="inlineStr"/>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D886" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E886" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F886" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G886" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogw</t>
+        </is>
+      </c>
+      <c r="H886" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I886" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J886" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K886" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L886" t="b">
+        <v>0</v>
+      </c>
+      <c r="M886" t="n">
+        <v>4.428571</v>
+      </c>
+      <c r="N886" t="n">
+        <v>1553</v>
+      </c>
+      <c r="O886" t="n">
+        <v>4</v>
+      </c>
+      <c r="P886" t="inlineStr"/>
+      <c r="Q886" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R886" t="inlineStr">
+        <is>
+          <t>4.0.18</t>
+        </is>
+      </c>
+      <c r="S886" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T886" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U886" t="inlineStr"/>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D887" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E887" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F887" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G887" t="n">
+        <v>1574668652</v>
+      </c>
+      <c r="H887" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I887" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J887" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K887" t="n">
+        <v>0</v>
+      </c>
+      <c r="L887" t="b">
+        <v>1</v>
+      </c>
+      <c r="M887" t="n">
+        <v>4.01316</v>
+      </c>
+      <c r="N887" t="n">
+        <v>76</v>
+      </c>
+      <c r="O887" t="n">
+        <v>1</v>
+      </c>
+      <c r="P887" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R887" t="inlineStr">
+        <is>
+          <t>6.0.35</t>
+        </is>
+      </c>
+      <c r="S887" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T887" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U887" t="inlineStr"/>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D888" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E888" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F888" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G888" t="inlineStr">
+        <is>
+          <t>com.orange.sugu.ocd</t>
+        </is>
+      </c>
+      <c r="H888" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I888" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J888" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K888" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L888" t="b">
+        <v>0</v>
+      </c>
+      <c r="M888" t="n">
+        <v>4.1571164</v>
+      </c>
+      <c r="N888" t="n">
+        <v>5334</v>
+      </c>
+      <c r="O888" t="n">
+        <v>95</v>
+      </c>
+      <c r="P888" t="inlineStr"/>
+      <c r="Q888" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R888" t="inlineStr">
+        <is>
+          <t>9.0.12</t>
+        </is>
+      </c>
+      <c r="S888" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DRC that brings together the features of MyOrange, and Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Plans, Mobile Payments, money transfers, bill payments, subscriptions, and entertai</t>
+        </is>
+      </c>
+      <c r="T888" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U888" t="inlineStr"/>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D889" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E889" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F889" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G889" t="n">
+        <v>6447896435</v>
+      </c>
+      <c r="H889" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I889" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J889" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K889" t="n">
+        <v>0</v>
+      </c>
+      <c r="L889" t="b">
+        <v>1</v>
+      </c>
+      <c r="M889" t="n">
+        <v>3.55351</v>
+      </c>
+      <c r="N889" t="n">
+        <v>271</v>
+      </c>
+      <c r="P889" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "CD" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R889" t="inlineStr">
+        <is>
+          <t>9.0.6</t>
+        </is>
+      </c>
+      <c r="S889" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DR Congo. It brings together the features of Orange et Moi, as well as Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Packages, Mobile payment, money transfers, bill payment and subscri</t>
+        </is>
+      </c>
+      <c r="T889" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U889" t="inlineStr"/>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D890" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E890" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F890" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G890" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ocm</t>
+        </is>
+      </c>
+      <c r="H890" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroon</t>
+        </is>
+      </c>
+      <c r="I890" t="inlineStr">
+        <is>
+          <t>Orange MEA</t>
+        </is>
+      </c>
+      <c r="J890" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K890" t="inlineStr">
+        <is>
+          <t>FCFA 0</t>
+        </is>
+      </c>
+      <c r="L890" t="b">
+        <v>0</v>
+      </c>
+      <c r="M890" t="n">
+        <v>3.917552</v>
+      </c>
+      <c r="N890" t="n">
+        <v>47100</v>
+      </c>
+      <c r="O890" t="n">
+        <v>11</v>
+      </c>
+      <c r="P890" t="inlineStr"/>
+      <c r="Q890" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R890" t="inlineStr">
+        <is>
+          <t>7.0.23</t>
+        </is>
+      </c>
+      <c r="S890" t="inlineStr">
+        <is>
+          <t>Max it brings together everything that matters to you in one app: managing your lines, money transfer, bill payment, exclusive offers, and a universe of lifestyle and entertainment. Simple, fast, and 100% secure..&lt;br&gt;&lt;br&gt;📞 My line&lt;br&gt;Manage your Orange mobile and landline bundles in a single click:</t>
+        </is>
+      </c>
+      <c r="T890" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U890" t="inlineStr"/>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D891" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E891" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F891" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G891" t="n">
+        <v>1116920093</v>
+      </c>
+      <c r="H891" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroun</t>
+        </is>
+      </c>
+      <c r="I891" t="inlineStr">
+        <is>
+          <t>Orange Middle East &amp; Africa</t>
+        </is>
+      </c>
+      <c r="J891" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K891" t="n">
+        <v>0</v>
+      </c>
+      <c r="L891" t="b">
+        <v>1</v>
+      </c>
+      <c r="M891" t="n">
+        <v>3.76774</v>
+      </c>
+      <c r="N891" t="n">
+        <v>16176</v>
+      </c>
+      <c r="O891" t="n">
+        <v>3</v>
+      </c>
+      <c r="P891" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R891" t="inlineStr">
+        <is>
+          <t>7.0.24</t>
+        </is>
+      </c>
+      <c r="S891" t="inlineStr">
+        <is>
+          <t>Avec Max it, Orange rassemble tout ce qui compte pour vous dans une même application : la gestion de vos lignes, les transferts d’argent, payement de vos factures, des offres exclusives et un univers lifestyle et divertissement.
+Simple, rapide et 100 % sécurisée.
+Ma ligne
+Gérez vos forfaits mobiles</t>
+        </is>
+      </c>
+      <c r="T891" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U891" t="inlineStr"/>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D892" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E892" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F892" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G892" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obf</t>
+        </is>
+      </c>
+      <c r="H892" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I892" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso</t>
+        </is>
+      </c>
+      <c r="J892" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K892" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L892" t="b">
+        <v>0</v>
+      </c>
+      <c r="M892" t="n">
+        <v>4.137783</v>
+      </c>
+      <c r="N892" t="n">
+        <v>25572</v>
+      </c>
+      <c r="O892" t="n">
+        <v>11</v>
+      </c>
+      <c r="P892" t="inlineStr"/>
+      <c r="Q892" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R892" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S892" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.&lt;br&gt;Gérez vos lignes mobiles, effectuez des transferts d&amp;#39;argent sécurisés, réglez vos factures, profitez d&amp;#39;offres exclusives, effectuez des paiements marchands fiables, et bien plus enco</t>
+        </is>
+      </c>
+      <c r="T892" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U892" t="inlineStr"/>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E893" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F893" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G893" t="n">
+        <v>1553774707</v>
+      </c>
+      <c r="H893" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I893" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso SA</t>
+        </is>
+      </c>
+      <c r="J893" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K893" t="n">
+        <v>0</v>
+      </c>
+      <c r="L893" t="b">
+        <v>1</v>
+      </c>
+      <c r="M893" t="n">
+        <v>3.45555</v>
+      </c>
+      <c r="N893" t="n">
+        <v>1181</v>
+      </c>
+      <c r="O893" t="n">
+        <v>7</v>
+      </c>
+      <c r="P893" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R893" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S893" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.
+Gérez vos lignes mobiles, effectuez des transferts d'argent sécurisés, réglez vos factures, profitez d'offres exclusives, effectuez des paiements marchands fiables, et bien plus encore, le tout</t>
+        </is>
+      </c>
+      <c r="T893" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U893" t="inlineStr"/>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E894" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F894" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G894" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obw</t>
+        </is>
+      </c>
+      <c r="H894" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I894" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J894" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K894" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L894" t="b">
+        <v>0</v>
+      </c>
+      <c r="M894" t="n">
+        <v>3.9602888</v>
+      </c>
+      <c r="N894" t="n">
+        <v>2968</v>
+      </c>
+      <c r="O894" t="n">
+        <v>34</v>
+      </c>
+      <c r="P894" t="inlineStr"/>
+      <c r="Q894" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R894" t="inlineStr">
+        <is>
+          <t>7.3.8</t>
+        </is>
+      </c>
+      <c r="S894" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it, the brand-new Orange Botswana Super App that follows Yame and gives you access to four distinct universes for a one-of-a-kind experience!&lt;br&gt;&lt;br&gt;Manage your accounts, make quick payments using QR codes, investigate a range of online goods and services, and discover the many options provided </t>
+        </is>
+      </c>
+      <c r="T894" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U894" t="inlineStr"/>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E895" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F895" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G895" t="n">
+        <v>1195839458</v>
+      </c>
+      <c r="H895" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I895" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J895" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K895" t="n">
+        <v>0</v>
+      </c>
+      <c r="L895" t="b">
+        <v>1</v>
+      </c>
+      <c r="M895" t="n">
+        <v>3.00806</v>
+      </c>
+      <c r="N895" t="n">
+        <v>124</v>
+      </c>
+      <c r="O895" t="n">
+        <v>24</v>
+      </c>
+      <c r="P895" t="inlineStr"/>
+      <c r="R895" t="inlineStr">
+        <is>
+          <t>7.3.1</t>
+        </is>
+      </c>
+      <c r="S895" t="inlineStr">
+        <is>
+          <t>A free mobile self-care application for Orange Botswana’s mobile customers.
+Full Description :
+Max it is a free application, which allows Orange Botswana customers to:
+- Consult your account in real time: minutes, sms, internet ...
+- Top up your account or a friend account  with Orange Money
+-</t>
+        </is>
+      </c>
+      <c r="T895" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U895" t="inlineStr"/>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E896" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F896" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G896" t="inlineStr">
+        <is>
+          <t>com.orange.mobinilandme</t>
+        </is>
+      </c>
+      <c r="H896" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I896" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J896" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K896" t="inlineStr">
+        <is>
+          <t>EGP 0.00</t>
+        </is>
+      </c>
+      <c r="L896" t="b">
+        <v>0</v>
+      </c>
+      <c r="M896" t="n">
+        <v>4.557035</v>
+      </c>
+      <c r="N896" t="n">
+        <v>937117</v>
+      </c>
+      <c r="O896" t="n">
+        <v>19</v>
+      </c>
+      <c r="P896" t="inlineStr"/>
+      <c r="Q896" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R896" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S896" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion&lt;br&gt;Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.&lt;br&gt;Key services include:&lt;br&gt;• Account Management: Easily manage</t>
+        </is>
+      </c>
+      <c r="T896" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U896" t="inlineStr"/>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>e2bb7be7-3cb8-45f4-84c8-974b983e034c</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:29:10</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E897" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F897" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G897" t="n">
+        <v>942568333</v>
+      </c>
+      <c r="H897" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I897" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J897" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K897" t="n">
+        <v>0</v>
+      </c>
+      <c r="L897" t="b">
+        <v>1</v>
+      </c>
+      <c r="M897" t="n">
+        <v>4.25281</v>
+      </c>
+      <c r="N897" t="n">
+        <v>118838</v>
+      </c>
+      <c r="O897" t="n">
+        <v>58</v>
+      </c>
+      <c r="P897" t="inlineStr"/>
+      <c r="R897" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S897" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion
+Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.
+Key services include:
+• Account Management: Easily manage your Ora</t>
+        </is>
+      </c>
+      <c r="T897" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U897" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-08-05
</commit_message>
<xml_diff>
--- a/maxit_store_history.xlsx
+++ b/maxit_store_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U897"/>
+  <dimension ref="A1:U929"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74518,7 +74518,6 @@
       <c r="O866" t="n">
         <v>39</v>
       </c>
-      <c r="P866" t="inlineStr"/>
       <c r="Q866" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -74539,7 +74538,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U866" t="inlineStr"/>
     </row>
     <row r="867">
       <c r="A867" t="inlineStr">
@@ -74602,7 +74600,6 @@
       <c r="N867" t="n">
         <v>332</v>
       </c>
-      <c r="P867" t="inlineStr"/>
       <c r="R867" t="inlineStr">
         <is>
           <t>6.4.12</t>
@@ -74618,7 +74615,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U867" t="inlineStr"/>
     </row>
     <row r="868">
       <c r="A868" t="inlineStr">
@@ -74688,7 +74684,6 @@
       <c r="O868" t="n">
         <v>31</v>
       </c>
-      <c r="P868" t="inlineStr"/>
       <c r="Q868" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -74709,7 +74704,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U868" t="inlineStr"/>
     </row>
     <row r="869">
       <c r="A869" t="inlineStr">
@@ -74775,7 +74769,6 @@
       <c r="O869" t="n">
         <v>41</v>
       </c>
-      <c r="P869" t="inlineStr"/>
       <c r="R869" t="inlineStr">
         <is>
           <t>10.0.7</t>
@@ -74793,7 +74786,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U869" t="inlineStr"/>
     </row>
     <row r="870">
       <c r="A870" t="inlineStr">
@@ -74863,7 +74855,6 @@
       <c r="O870" t="n">
         <v>10</v>
       </c>
-      <c r="P870" t="inlineStr"/>
       <c r="Q870" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -74884,7 +74875,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U870" t="inlineStr"/>
     </row>
     <row r="871">
       <c r="A871" t="inlineStr">
@@ -74973,7 +74963,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U871" t="inlineStr"/>
     </row>
     <row r="872">
       <c r="A872" t="inlineStr">
@@ -75043,7 +75032,6 @@
       <c r="O872" t="n">
         <v>8</v>
       </c>
-      <c r="P872" t="inlineStr"/>
       <c r="Q872" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -75064,7 +75052,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U872" t="inlineStr"/>
     </row>
     <row r="873">
       <c r="A873" t="inlineStr">
@@ -75130,7 +75117,6 @@
       <c r="O873" t="n">
         <v>12</v>
       </c>
-      <c r="P873" t="inlineStr"/>
       <c r="R873" t="inlineStr">
         <is>
           <t>22.0.1</t>
@@ -75148,7 +75134,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U873" t="inlineStr"/>
     </row>
     <row r="874">
       <c r="A874" t="inlineStr">
@@ -75218,7 +75203,6 @@
       <c r="O874" t="n">
         <v>49</v>
       </c>
-      <c r="P874" t="inlineStr"/>
       <c r="Q874" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -75239,7 +75223,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U874" t="inlineStr"/>
     </row>
     <row r="875">
       <c r="A875" t="inlineStr">
@@ -75324,7 +75307,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U875" t="inlineStr"/>
     </row>
     <row r="876">
       <c r="A876" t="inlineStr">
@@ -75391,7 +75373,6 @@
       <c r="N876" t="n">
         <v>38237</v>
       </c>
-      <c r="P876" t="inlineStr"/>
       <c r="Q876" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -75412,7 +75393,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U876" t="inlineStr"/>
     </row>
     <row r="877">
       <c r="A877" t="inlineStr">
@@ -75478,7 +75458,6 @@
       <c r="O877" t="n">
         <v>13</v>
       </c>
-      <c r="P877" t="inlineStr"/>
       <c r="R877" t="inlineStr">
         <is>
           <t>6.5.2</t>
@@ -75497,7 +75476,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U877" t="inlineStr"/>
     </row>
     <row r="878">
       <c r="A878" t="inlineStr">
@@ -75567,7 +75545,6 @@
       <c r="O878" t="n">
         <v>62</v>
       </c>
-      <c r="P878" t="inlineStr"/>
       <c r="Q878" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -75588,7 +75565,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U878" t="inlineStr"/>
     </row>
     <row r="879">
       <c r="A879" t="inlineStr">
@@ -75654,7 +75630,6 @@
       <c r="O879" t="n">
         <v>33</v>
       </c>
-      <c r="P879" t="inlineStr"/>
       <c r="R879" t="inlineStr">
         <is>
           <t>5.0.2</t>
@@ -75672,7 +75647,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U879" t="inlineStr"/>
     </row>
     <row r="880">
       <c r="A880" t="inlineStr">
@@ -75742,7 +75716,6 @@
       <c r="O880" t="n">
         <v>77</v>
       </c>
-      <c r="P880" t="inlineStr"/>
       <c r="Q880" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -75763,7 +75736,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U880" t="inlineStr"/>
     </row>
     <row r="881">
       <c r="A881" t="inlineStr">
@@ -75851,7 +75823,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U881" t="inlineStr"/>
     </row>
     <row r="882">
       <c r="A882" t="inlineStr">
@@ -75921,7 +75892,6 @@
       <c r="O882" t="n">
         <v>41</v>
       </c>
-      <c r="P882" t="inlineStr"/>
       <c r="Q882" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -75942,7 +75912,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U882" t="inlineStr"/>
     </row>
     <row r="883">
       <c r="A883" t="inlineStr">
@@ -76008,7 +75977,6 @@
       <c r="O883" t="n">
         <v>54</v>
       </c>
-      <c r="P883" t="inlineStr"/>
       <c r="R883" t="inlineStr">
         <is>
           <t>10.0.21</t>
@@ -76027,7 +75995,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U883" t="inlineStr"/>
     </row>
     <row r="884">
       <c r="A884" t="inlineStr">
@@ -76097,7 +76064,6 @@
       <c r="O884" t="n">
         <v>14</v>
       </c>
-      <c r="P884" t="inlineStr"/>
       <c r="Q884" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -76118,7 +76084,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U884" t="inlineStr"/>
     </row>
     <row r="885">
       <c r="A885" t="inlineStr">
@@ -76204,7 +76169,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U885" t="inlineStr"/>
     </row>
     <row r="886">
       <c r="A886" t="inlineStr">
@@ -76274,7 +76238,6 @@
       <c r="O886" t="n">
         <v>4</v>
       </c>
-      <c r="P886" t="inlineStr"/>
       <c r="Q886" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -76295,7 +76258,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U886" t="inlineStr"/>
     </row>
     <row r="887">
       <c r="A887" t="inlineStr">
@@ -76381,7 +76343,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U887" t="inlineStr"/>
     </row>
     <row r="888">
       <c r="A888" t="inlineStr">
@@ -76451,7 +76412,6 @@
       <c r="O888" t="n">
         <v>95</v>
       </c>
-      <c r="P888" t="inlineStr"/>
       <c r="Q888" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -76472,7 +76432,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U888" t="inlineStr"/>
     </row>
     <row r="889">
       <c r="A889" t="inlineStr">
@@ -76555,7 +76514,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U889" t="inlineStr"/>
     </row>
     <row r="890">
       <c r="A890" t="inlineStr">
@@ -76625,7 +76583,6 @@
       <c r="O890" t="n">
         <v>11</v>
       </c>
-      <c r="P890" t="inlineStr"/>
       <c r="Q890" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -76646,7 +76603,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U890" t="inlineStr"/>
     </row>
     <row r="891">
       <c r="A891" t="inlineStr">
@@ -76735,7 +76691,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U891" t="inlineStr"/>
     </row>
     <row r="892">
       <c r="A892" t="inlineStr">
@@ -76805,7 +76760,6 @@
       <c r="O892" t="n">
         <v>11</v>
       </c>
-      <c r="P892" t="inlineStr"/>
       <c r="Q892" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -76826,7 +76780,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U892" t="inlineStr"/>
     </row>
     <row r="893">
       <c r="A893" t="inlineStr">
@@ -76913,7 +76866,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U893" t="inlineStr"/>
     </row>
     <row r="894">
       <c r="A894" t="inlineStr">
@@ -76983,7 +76935,6 @@
       <c r="O894" t="n">
         <v>34</v>
       </c>
-      <c r="P894" t="inlineStr"/>
       <c r="Q894" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -77004,7 +76955,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U894" t="inlineStr"/>
     </row>
     <row r="895">
       <c r="A895" t="inlineStr">
@@ -77070,7 +77020,6 @@
       <c r="O895" t="n">
         <v>24</v>
       </c>
-      <c r="P895" t="inlineStr"/>
       <c r="R895" t="inlineStr">
         <is>
           <t>7.3.1</t>
@@ -77091,7 +77040,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U895" t="inlineStr"/>
     </row>
     <row r="896">
       <c r="A896" t="inlineStr">
@@ -77161,7 +77109,6 @@
       <c r="O896" t="n">
         <v>19</v>
       </c>
-      <c r="P896" t="inlineStr"/>
       <c r="Q896" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -77182,7 +77129,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U896" t="inlineStr"/>
     </row>
     <row r="897">
       <c r="A897" t="inlineStr">
@@ -77248,7 +77194,6 @@
       <c r="O897" t="n">
         <v>58</v>
       </c>
-      <c r="P897" t="inlineStr"/>
       <c r="R897" t="inlineStr">
         <is>
           <t>10.1.0</t>
@@ -77267,7 +77212,2825 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U897" t="inlineStr"/>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F898" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G898" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogn</t>
+        </is>
+      </c>
+      <c r="H898" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I898" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J898" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K898" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L898" t="b">
+        <v>0</v>
+      </c>
+      <c r="M898" t="n">
+        <v>4.4555197</v>
+      </c>
+      <c r="N898" t="n">
+        <v>9392</v>
+      </c>
+      <c r="O898" t="n">
+        <v>43</v>
+      </c>
+      <c r="P898" t="inlineStr"/>
+      <c r="Q898" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R898" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S898" t="inlineStr">
+        <is>
+          <t>Bien plus qu&amp;#39;une application, un véritable assistant personnel pour une vie connectée et simplifiée.&lt;br&gt;Suivi de consommation: Votre tableau de bord tout-en-un pour une gestion simplifiée !&lt;br&gt;- Gestion de votre offre: Accédez à une vue détaillée de votre offre actuelle et de vos forfaits Orange</t>
+        </is>
+      </c>
+      <c r="T898" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U898" t="inlineStr"/>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F899" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G899" t="n">
+        <v>1177999485</v>
+      </c>
+      <c r="H899" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I899" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J899" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K899" t="n">
+        <v>0</v>
+      </c>
+      <c r="L899" t="b">
+        <v>1</v>
+      </c>
+      <c r="M899" t="n">
+        <v>3.89941</v>
+      </c>
+      <c r="N899" t="n">
+        <v>338</v>
+      </c>
+      <c r="P899" t="inlineStr"/>
+      <c r="R899" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S899" t="inlineStr">
+        <is>
+          <t>La fusion d’Orange et Moi et Orange Money donne naissance à Max it, la nouvelle Super Application Tout-en-Un. Profitez du suivi de consommation, de paiements mobiles, de toutes les fonctionnalités Orange et Moi et Money avec un large éventail de divertissements, le tout regroupé en un seul endroit !</t>
+        </is>
+      </c>
+      <c r="T899" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U899" t="inlineStr"/>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E900" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F900" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G900" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.otn</t>
+        </is>
+      </c>
+      <c r="H900" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I900" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J900" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K900" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L900" t="b">
+        <v>0</v>
+      </c>
+      <c r="M900" t="n">
+        <v>3.9660816</v>
+      </c>
+      <c r="N900" t="n">
+        <v>35389</v>
+      </c>
+      <c r="O900" t="n">
+        <v>28</v>
+      </c>
+      <c r="P900" t="inlineStr"/>
+      <c r="Q900" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R900" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S900" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Max it par Orange Tunisie facilite votre vie au quotidien !&lt;/h2&gt;&lt;br&gt;&lt;br&gt;Welcome sur Max it !&lt;br&gt;Accédez rapidement à vos fonctionnalités Max it préférées et profitez également de contenus exclusifs, d’activités divertissantes, et de jeux interactifs pour une expérience enrichissante avec la roue</t>
+        </is>
+      </c>
+      <c r="T900" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U900" t="inlineStr"/>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E901" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F901" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G901" t="n">
+        <v>1146892088</v>
+      </c>
+      <c r="H901" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I901" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J901" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K901" t="n">
+        <v>0</v>
+      </c>
+      <c r="L901" t="b">
+        <v>1</v>
+      </c>
+      <c r="M901" t="n">
+        <v>3.02862</v>
+      </c>
+      <c r="N901" t="n">
+        <v>1642</v>
+      </c>
+      <c r="O901" t="n">
+        <v>40</v>
+      </c>
+      <c r="P901" t="inlineStr"/>
+      <c r="R901" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S901" t="inlineStr">
+        <is>
+          <t>Max it by Orange Tunisie : Votre appli incontournable pour une vie connectée
+Welcome sur Max it : Découvrez fonctionnalités, jeux &amp; contenus de divertissement by Orange Tunisie !
+Trouvez vite vos fonctionnalités Max it favorites et explorez des contenus exclusifs et des jeux pour une expérience im</t>
+        </is>
+      </c>
+      <c r="T901" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U901" t="inlineStr"/>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E902" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F902" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G902" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osl</t>
+        </is>
+      </c>
+      <c r="H902" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I902" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J902" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K902" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L902" t="b">
+        <v>0</v>
+      </c>
+      <c r="M902" t="n">
+        <v>4.46789</v>
+      </c>
+      <c r="N902" t="n">
+        <v>2171</v>
+      </c>
+      <c r="O902" t="n">
+        <v>11</v>
+      </c>
+      <c r="P902" t="inlineStr"/>
+      <c r="Q902" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R902" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S902" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it is a free application, which allows Orange Sierra Leone prepaid and postpaid customers to:&lt;br&gt;&lt;br&gt;- Consult your account in real time: minutes, sms, internet&lt;br&gt;- Top up your account or a friend account &lt;br&gt;- Buy Internet Bundles&lt;br&gt;- Discover the latest offers and promotions &lt;br&gt;- Access to </t>
+        </is>
+      </c>
+      <c r="T902" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U902" t="inlineStr"/>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D903" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E903" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F903" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G903" t="n">
+        <v>6443607903</v>
+      </c>
+      <c r="H903" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I903" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J903" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K903" t="n">
+        <v>0</v>
+      </c>
+      <c r="L903" t="b">
+        <v>1</v>
+      </c>
+      <c r="M903" t="n">
+        <v>3.69072</v>
+      </c>
+      <c r="N903" t="n">
+        <v>194</v>
+      </c>
+      <c r="O903" t="n">
+        <v>5</v>
+      </c>
+      <c r="P903" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R903" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S903" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The merger of My Orange &amp; Orange Money has given birth to Max it the all-in-one super app, a free application which allows all Orange Sierra Leone customers to 
+Track calls, SMS, and Data usage and monitor balance. 
+Make a secure mobile/Orange Money payment.
+Easily transfer credit to other users </t>
+        </is>
+      </c>
+      <c r="T903" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U903" t="inlineStr"/>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D904" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E904" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F904" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G904" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osn</t>
+        </is>
+      </c>
+      <c r="H904" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I904" t="inlineStr">
+        <is>
+          <t>Orange Sénégal</t>
+        </is>
+      </c>
+      <c r="J904" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K904" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L904" t="b">
+        <v>0</v>
+      </c>
+      <c r="M904" t="n">
+        <v>4.29368</v>
+      </c>
+      <c r="N904" t="n">
+        <v>51389</v>
+      </c>
+      <c r="O904" t="n">
+        <v>8</v>
+      </c>
+      <c r="P904" t="inlineStr"/>
+      <c r="Q904" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R904" t="inlineStr">
+        <is>
+          <t>22.0.1</t>
+        </is>
+      </c>
+      <c r="S904" t="inlineStr">
+        <is>
+          <t>Lu bees ak Max it ! &lt;br&gt;Une application repensée pour être plus simple, plus rapide et adaptée à vos besoins. Une expérience optimisée pour faciliter vos usages au quotidien, avec des parcours simplifiés et un accès plus fluide à vos services. Que vous soyez client Orange ou non, Max it vous accompa</t>
+        </is>
+      </c>
+      <c r="T904" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U904" t="inlineStr"/>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D905" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E905" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F905" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G905" t="n">
+        <v>1039327980</v>
+      </c>
+      <c r="H905" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I905" t="inlineStr">
+        <is>
+          <t>Orange Senegal</t>
+        </is>
+      </c>
+      <c r="J905" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K905" t="n">
+        <v>0</v>
+      </c>
+      <c r="L905" t="b">
+        <v>1</v>
+      </c>
+      <c r="M905" t="n">
+        <v>4.16904</v>
+      </c>
+      <c r="N905" t="n">
+        <v>30242</v>
+      </c>
+      <c r="O905" t="n">
+        <v>12</v>
+      </c>
+      <c r="P905" t="inlineStr"/>
+      <c r="R905" t="inlineStr">
+        <is>
+          <t>22.0.1</t>
+        </is>
+      </c>
+      <c r="S905" t="inlineStr">
+        <is>
+          <t>Here is the English translation:
+Welcome to Max it!
+A redesigned app to be simpler, faster, and tailored to your needs. An optimized experience to make your daily life easier, with streamlined journeys and smoother access to your services. Whether you are an Orange customer or not, Max it is your e</t>
+        </is>
+      </c>
+      <c r="T905" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U905" t="inlineStr"/>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D906" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E906" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F906" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G906" t="inlineStr">
+        <is>
+          <t>com.orange.meditel.mediteletmoi</t>
+        </is>
+      </c>
+      <c r="H906" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I906" t="inlineStr">
+        <is>
+          <t>Orange Maroc</t>
+        </is>
+      </c>
+      <c r="J906" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K906" t="inlineStr">
+        <is>
+          <t>MAD 0.00</t>
+        </is>
+      </c>
+      <c r="L906" t="b">
+        <v>0</v>
+      </c>
+      <c r="M906" t="n">
+        <v>3.7159326</v>
+      </c>
+      <c r="N906" t="n">
+        <v>110961</v>
+      </c>
+      <c r="O906" t="n">
+        <v>58</v>
+      </c>
+      <c r="P906" t="inlineStr"/>
+      <c r="Q906" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R906" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S906" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l&amp;#39;expérience mobile réinventé&lt;br&gt;&lt;br&gt;Max it, c&amp;#39;est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d&amp;#39;une multitude de services exclusifs. &lt;br&gt;&lt;br&gt;Créez votre espace sur</t>
+        </is>
+      </c>
+      <c r="T906" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U906" t="inlineStr"/>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D907" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E907" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F907" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G907" t="n">
+        <v>596028698</v>
+      </c>
+      <c r="H907" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I907" t="inlineStr">
+        <is>
+          <t>Méditel</t>
+        </is>
+      </c>
+      <c r="J907" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K907" t="n">
+        <v>0</v>
+      </c>
+      <c r="L907" t="b">
+        <v>1</v>
+      </c>
+      <c r="M907" t="n">
+        <v>3.94282</v>
+      </c>
+      <c r="N907" t="n">
+        <v>2763</v>
+      </c>
+      <c r="P907" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "MA" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R907" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S907" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l'expérience mobile réinventé
+Max it, c'est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d'une multitude de services exclusifs. 
+Créez votre espace sur mesure et bénéficiez d'</t>
+        </is>
+      </c>
+      <c r="T907" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U907" t="inlineStr"/>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E908" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F908" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G908" t="inlineStr">
+        <is>
+          <t>com.oml.dsi.orangemobile</t>
+        </is>
+      </c>
+      <c r="H908" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I908" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J908" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K908" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L908" t="b">
+        <v>0</v>
+      </c>
+      <c r="M908" t="n">
+        <v>2.7094083</v>
+      </c>
+      <c r="N908" t="n">
+        <v>38235</v>
+      </c>
+      <c r="P908" t="inlineStr"/>
+      <c r="Q908" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R908" t="inlineStr">
+        <is>
+          <t>6.5.0</t>
+        </is>
+      </c>
+      <c r="S908" t="inlineStr">
+        <is>
+          <t>Easily manage your Orange Mali line&lt;br&gt;● Manage your account and view all essential information, your offers, and your phone lines.&lt;br&gt;● Subscribe to call, SMS, Internet, and international call packages.&lt;br&gt;● Track your usage by checking your credit and Internet balance.&lt;br&gt;● Recharge your line by p</t>
+        </is>
+      </c>
+      <c r="T908" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U908" t="inlineStr"/>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D909" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E909" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F909" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G909" t="n">
+        <v>1494321079</v>
+      </c>
+      <c r="H909" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I909" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J909" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K909" t="n">
+        <v>0</v>
+      </c>
+      <c r="L909" t="b">
+        <v>1</v>
+      </c>
+      <c r="M909" t="n">
+        <v>2.5255</v>
+      </c>
+      <c r="N909" t="n">
+        <v>4765</v>
+      </c>
+      <c r="O909" t="n">
+        <v>13</v>
+      </c>
+      <c r="P909" t="inlineStr"/>
+      <c r="R909" t="inlineStr">
+        <is>
+          <t>6.5.2</t>
+        </is>
+      </c>
+      <c r="S909" t="inlineStr">
+        <is>
+          <t>Gérez facilement votre ligne Orange Mali 
+●        Gérez votre compte et consultez toutes les informations essentielles sur celui-ci, vos offres, ainsi que vos lignes téléphoniques.
+●        Souscrivez aux forfaits appels, SMS, Internet, et appels internationaux.
+●        Suivez votre consommation e</t>
+        </is>
+      </c>
+      <c r="T909" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U909" t="inlineStr"/>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D910" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E910" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F910" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G910" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.omg</t>
+        </is>
+      </c>
+      <c r="H910" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I910" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J910" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K910" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L910" t="b">
+        <v>0</v>
+      </c>
+      <c r="M910" t="n">
+        <v>4.1532845</v>
+      </c>
+      <c r="N910" t="n">
+        <v>1392</v>
+      </c>
+      <c r="O910" t="n">
+        <v>71</v>
+      </c>
+      <c r="P910" t="inlineStr"/>
+      <c r="Q910" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R910" t="inlineStr">
+        <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="S910" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.&lt;br&gt;&lt;br&gt;Simplify Your Life with Max it&lt;br&gt;With Max It, ac</t>
+        </is>
+      </c>
+      <c r="T910" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U910" t="inlineStr"/>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D911" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E911" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F911" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G911" t="n">
+        <v>1295171817</v>
+      </c>
+      <c r="H911" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I911" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J911" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K911" t="n">
+        <v>0</v>
+      </c>
+      <c r="L911" t="b">
+        <v>1</v>
+      </c>
+      <c r="M911" t="n">
+        <v>3.05714</v>
+      </c>
+      <c r="N911" t="n">
+        <v>70</v>
+      </c>
+      <c r="O911" t="n">
+        <v>20</v>
+      </c>
+      <c r="P911" t="inlineStr"/>
+      <c r="R911" t="inlineStr">
+        <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="S911" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.
+Simplify Your Life with Max it
+With Max it, access a se</t>
+        </is>
+      </c>
+      <c r="T911" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U911" t="inlineStr"/>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D912" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E912" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F912" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G912" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.olr</t>
+        </is>
+      </c>
+      <c r="H912" t="inlineStr">
+        <is>
+          <t>Orange Max it - Liberia</t>
+        </is>
+      </c>
+      <c r="I912" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J912" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K912" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L912" t="b">
+        <v>0</v>
+      </c>
+      <c r="M912" t="n">
+        <v>4.535032</v>
+      </c>
+      <c r="N912" t="n">
+        <v>3112</v>
+      </c>
+      <c r="O912" t="n">
+        <v>73</v>
+      </c>
+      <c r="P912" t="inlineStr"/>
+      <c r="Q912" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R912" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="S912" t="inlineStr">
+        <is>
+          <t>Max it: your personalized experience by Orange Liberia!&lt;br&gt;&lt;br&gt;Step into Max it, your all-in-one solution for telecom, marketplace, and financial services! Manage your mobile line, customize offers, pay your bills, keep&lt;br&gt;track of your usage with ease, and recharge your credit. Access exclusive eve</t>
+        </is>
+      </c>
+      <c r="T912" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U912" t="inlineStr"/>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D913" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E913" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F913" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G913" t="n">
+        <v>6746187327</v>
+      </c>
+      <c r="H913" t="inlineStr">
+        <is>
+          <t>Orange Max it – Liberia</t>
+        </is>
+      </c>
+      <c r="I913" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J913" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K913" t="n">
+        <v>0</v>
+      </c>
+      <c r="L913" t="b">
+        <v>1</v>
+      </c>
+      <c r="M913" t="n">
+        <v>4.0625</v>
+      </c>
+      <c r="N913" t="n">
+        <v>48</v>
+      </c>
+      <c r="P913" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "LR" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R913" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="S913" t="inlineStr">
+        <is>
+          <t>Max it is a free application, which allows Orange Liberia customers to:
+- Consult your account in real time: minutes, sms, internet
+- Top up your account or a friend account 
+- Buy  Bundles (voice, data, SMS, roaming, international)
+- Discover the latest offers and promotions 
+- Access to Orange se</t>
+        </is>
+      </c>
+      <c r="T913" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U913" t="inlineStr"/>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D914" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E914" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F914" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G914" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ojo</t>
+        </is>
+      </c>
+      <c r="H914" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I914" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J914" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K914" t="inlineStr">
+        <is>
+          <t>JOD 0.000</t>
+        </is>
+      </c>
+      <c r="L914" t="b">
+        <v>0</v>
+      </c>
+      <c r="M914" t="n">
+        <v>4.4292107</v>
+      </c>
+      <c r="N914" t="n">
+        <v>97911</v>
+      </c>
+      <c r="O914" t="n">
+        <v>45</v>
+      </c>
+      <c r="P914" t="inlineStr"/>
+      <c r="Q914" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R914" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S914" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience&lt;br&gt;Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.&lt;br&gt;Important Update:&lt;br&gt;The jood app (jood Orange) w</t>
+        </is>
+      </c>
+      <c r="T914" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U914" t="inlineStr"/>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D915" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E915" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F915" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G915" t="n">
+        <v>808824590</v>
+      </c>
+      <c r="H915" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I915" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J915" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K915" t="n">
+        <v>0</v>
+      </c>
+      <c r="L915" t="b">
+        <v>1</v>
+      </c>
+      <c r="M915" t="n">
+        <v>4.20563</v>
+      </c>
+      <c r="N915" t="n">
+        <v>3088</v>
+      </c>
+      <c r="O915" t="n">
+        <v>46</v>
+      </c>
+      <c r="P915" t="inlineStr"/>
+      <c r="R915" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S915" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience
+Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.
+Important Update:
+The jood app (jood Orange) will be di</t>
+        </is>
+      </c>
+      <c r="T915" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U915" t="inlineStr"/>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D916" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E916" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F916" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G916" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.oci</t>
+        </is>
+      </c>
+      <c r="H916" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I916" t="inlineStr">
+        <is>
+          <t>Orange Côte d'Ivoire S.A</t>
+        </is>
+      </c>
+      <c r="J916" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K916" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L916" t="b">
+        <v>0</v>
+      </c>
+      <c r="M916" t="n">
+        <v>4.14226</v>
+      </c>
+      <c r="N916" t="n">
+        <v>67398</v>
+      </c>
+      <c r="O916" t="n">
+        <v>13</v>
+      </c>
+      <c r="P916" t="inlineStr"/>
+      <c r="Q916" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R916" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S916" t="inlineStr">
+        <is>
+          <t>Aaaahhh, ta super app Max it, n&amp;#39;a pas fini de te surprendre... &lt;br&gt;Est-ce que tu as remarqué ? Maintenant, tu as ton QR code personnalisé en haut de ton écran d&amp;#39;accueil ! Ainsi, tu peux :&lt;br&gt;     scanner le QR code de ton ami(e) pour lui faire un transfert d&amp;#39;&amp;#39;argent&lt;br&gt;     scanner l</t>
+        </is>
+      </c>
+      <c r="T916" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U916" t="inlineStr"/>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D917" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E917" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F917" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G917" t="n">
+        <v>1061120855</v>
+      </c>
+      <c r="H917" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I917" t="inlineStr">
+        <is>
+          <t>Orange CI</t>
+        </is>
+      </c>
+      <c r="J917" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K917" t="n">
+        <v>0</v>
+      </c>
+      <c r="L917" t="b">
+        <v>1</v>
+      </c>
+      <c r="M917" t="n">
+        <v>3.78613</v>
+      </c>
+      <c r="N917" t="n">
+        <v>5985</v>
+      </c>
+      <c r="O917" t="n">
+        <v>10</v>
+      </c>
+      <c r="P917" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R917" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S917" t="inlineStr">
+        <is>
+          <t>Max it, la super app all-in-one te fais gagner du temps, et diminue tes soucis... Gagne plus d'espace de stockage sur ton téléphone ; plus besoin de cumuler plusieurs appli d'Orange pour avoir accès à un maximum de services. Max it est là ! Gère ta ligne (SIM) au niveau des pass, des soldes, réalise</t>
+        </is>
+      </c>
+      <c r="T917" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U917" t="inlineStr"/>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D918" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E918" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F918" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G918" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogw</t>
+        </is>
+      </c>
+      <c r="H918" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I918" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J918" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K918" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L918" t="b">
+        <v>0</v>
+      </c>
+      <c r="M918" t="n">
+        <v>4.422078</v>
+      </c>
+      <c r="N918" t="n">
+        <v>1555</v>
+      </c>
+      <c r="O918" t="n">
+        <v>4</v>
+      </c>
+      <c r="P918" t="inlineStr"/>
+      <c r="Q918" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R918" t="inlineStr">
+        <is>
+          <t>4.0.18</t>
+        </is>
+      </c>
+      <c r="S918" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T918" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U918" t="inlineStr"/>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D919" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E919" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F919" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G919" t="n">
+        <v>1574668652</v>
+      </c>
+      <c r="H919" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I919" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J919" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K919" t="n">
+        <v>0</v>
+      </c>
+      <c r="L919" t="b">
+        <v>1</v>
+      </c>
+      <c r="M919" t="n">
+        <v>4.01316</v>
+      </c>
+      <c r="N919" t="n">
+        <v>76</v>
+      </c>
+      <c r="O919" t="n">
+        <v>1</v>
+      </c>
+      <c r="P919" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R919" t="inlineStr">
+        <is>
+          <t>6.0.35</t>
+        </is>
+      </c>
+      <c r="S919" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T919" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U919" t="inlineStr"/>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D920" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E920" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F920" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G920" t="inlineStr">
+        <is>
+          <t>com.orange.sugu.ocd</t>
+        </is>
+      </c>
+      <c r="H920" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I920" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J920" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K920" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L920" t="b">
+        <v>0</v>
+      </c>
+      <c r="M920" t="n">
+        <v>4.1657557</v>
+      </c>
+      <c r="N920" t="n">
+        <v>5342</v>
+      </c>
+      <c r="O920" t="n">
+        <v>114</v>
+      </c>
+      <c r="P920" t="inlineStr"/>
+      <c r="Q920" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R920" t="inlineStr">
+        <is>
+          <t>9.0.12</t>
+        </is>
+      </c>
+      <c r="S920" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DRC that brings together the features of MyOrange, and Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Plans, Mobile Payments, money transfers, bill payments, subscriptions, and entertai</t>
+        </is>
+      </c>
+      <c r="T920" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U920" t="inlineStr"/>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D921" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E921" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F921" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G921" t="n">
+        <v>6447896435</v>
+      </c>
+      <c r="H921" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I921" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J921" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K921" t="n">
+        <v>0</v>
+      </c>
+      <c r="L921" t="b">
+        <v>1</v>
+      </c>
+      <c r="M921" t="n">
+        <v>3.55351</v>
+      </c>
+      <c r="N921" t="n">
+        <v>271</v>
+      </c>
+      <c r="P921" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "CD" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R921" t="inlineStr">
+        <is>
+          <t>9.0.6</t>
+        </is>
+      </c>
+      <c r="S921" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DR Congo. It brings together the features of Orange et Moi, as well as Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Packages, Mobile payment, money transfers, bill payment and subscri</t>
+        </is>
+      </c>
+      <c r="T921" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U921" t="inlineStr"/>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D922" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E922" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F922" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G922" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ocm</t>
+        </is>
+      </c>
+      <c r="H922" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroon</t>
+        </is>
+      </c>
+      <c r="I922" t="inlineStr">
+        <is>
+          <t>Orange MEA</t>
+        </is>
+      </c>
+      <c r="J922" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K922" t="inlineStr">
+        <is>
+          <t>FCFA 0</t>
+        </is>
+      </c>
+      <c r="L922" t="b">
+        <v>0</v>
+      </c>
+      <c r="M922" t="n">
+        <v>3.9162238</v>
+      </c>
+      <c r="N922" t="n">
+        <v>47147</v>
+      </c>
+      <c r="O922" t="n">
+        <v>13</v>
+      </c>
+      <c r="P922" t="inlineStr"/>
+      <c r="Q922" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R922" t="inlineStr">
+        <is>
+          <t>7.0.23</t>
+        </is>
+      </c>
+      <c r="S922" t="inlineStr">
+        <is>
+          <t>Max it brings together everything that matters to you in one app: managing your lines, money transfer, bill payment, exclusive offers, and a universe of lifestyle and entertainment. Simple, fast, and 100% secure..&lt;br&gt;&lt;br&gt;📞 My line&lt;br&gt;Manage your Orange mobile and landline bundles in a single click:</t>
+        </is>
+      </c>
+      <c r="T922" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U922" t="inlineStr"/>
+    </row>
+    <row r="923">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D923" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E923" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F923" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G923" t="n">
+        <v>1116920093</v>
+      </c>
+      <c r="H923" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroun</t>
+        </is>
+      </c>
+      <c r="I923" t="inlineStr">
+        <is>
+          <t>Orange Middle East &amp; Africa</t>
+        </is>
+      </c>
+      <c r="J923" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K923" t="n">
+        <v>0</v>
+      </c>
+      <c r="L923" t="b">
+        <v>1</v>
+      </c>
+      <c r="M923" t="n">
+        <v>3.76808</v>
+      </c>
+      <c r="N923" t="n">
+        <v>16178</v>
+      </c>
+      <c r="O923" t="n">
+        <v>5</v>
+      </c>
+      <c r="P923" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R923" t="inlineStr">
+        <is>
+          <t>7.0.24</t>
+        </is>
+      </c>
+      <c r="S923" t="inlineStr">
+        <is>
+          <t>Avec Max it, Orange rassemble tout ce qui compte pour vous dans une même application : la gestion de vos lignes, les transferts d’argent, payement de vos factures, des offres exclusives et un univers lifestyle et divertissement.
+Simple, rapide et 100 % sécurisée.
+Ma ligne
+Gérez vos forfaits mobiles</t>
+        </is>
+      </c>
+      <c r="T923" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U923" t="inlineStr"/>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D924" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E924" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F924" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G924" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obf</t>
+        </is>
+      </c>
+      <c r="H924" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I924" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso</t>
+        </is>
+      </c>
+      <c r="J924" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K924" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L924" t="b">
+        <v>0</v>
+      </c>
+      <c r="M924" t="n">
+        <v>4.1396885</v>
+      </c>
+      <c r="N924" t="n">
+        <v>25580</v>
+      </c>
+      <c r="O924" t="n">
+        <v>12</v>
+      </c>
+      <c r="P924" t="inlineStr"/>
+      <c r="Q924" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R924" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S924" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.&lt;br&gt;Gérez vos lignes mobiles, effectuez des transferts d&amp;#39;argent sécurisés, réglez vos factures, profitez d&amp;#39;offres exclusives, effectuez des paiements marchands fiables, et bien plus enco</t>
+        </is>
+      </c>
+      <c r="T924" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U924" t="inlineStr"/>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D925" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E925" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F925" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G925" t="n">
+        <v>1553774707</v>
+      </c>
+      <c r="H925" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I925" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso SA</t>
+        </is>
+      </c>
+      <c r="J925" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K925" t="n">
+        <v>0</v>
+      </c>
+      <c r="L925" t="b">
+        <v>1</v>
+      </c>
+      <c r="M925" t="n">
+        <v>3.45816</v>
+      </c>
+      <c r="N925" t="n">
+        <v>1183</v>
+      </c>
+      <c r="O925" t="n">
+        <v>4</v>
+      </c>
+      <c r="P925" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R925" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S925" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.
+Gérez vos lignes mobiles, effectuez des transferts d'argent sécurisés, réglez vos factures, profitez d'offres exclusives, effectuez des paiements marchands fiables, et bien plus encore, le tout</t>
+        </is>
+      </c>
+      <c r="T925" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U925" t="inlineStr"/>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D926" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E926" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F926" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G926" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obw</t>
+        </is>
+      </c>
+      <c r="H926" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I926" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J926" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K926" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L926" t="b">
+        <v>0</v>
+      </c>
+      <c r="M926" t="n">
+        <v>3.9640288</v>
+      </c>
+      <c r="N926" t="n">
+        <v>2968</v>
+      </c>
+      <c r="O926" t="n">
+        <v>37</v>
+      </c>
+      <c r="P926" t="inlineStr"/>
+      <c r="Q926" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R926" t="inlineStr">
+        <is>
+          <t>7.3.8</t>
+        </is>
+      </c>
+      <c r="S926" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it, the brand-new Orange Botswana Super App that follows Yame and gives you access to four distinct universes for a one-of-a-kind experience!&lt;br&gt;&lt;br&gt;Manage your accounts, make quick payments using QR codes, investigate a range of online goods and services, and discover the many options provided </t>
+        </is>
+      </c>
+      <c r="T926" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U926" t="inlineStr"/>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D927" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E927" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F927" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G927" t="n">
+        <v>1195839458</v>
+      </c>
+      <c r="H927" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I927" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J927" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K927" t="n">
+        <v>0</v>
+      </c>
+      <c r="L927" t="b">
+        <v>1</v>
+      </c>
+      <c r="M927" t="n">
+        <v>3.00806</v>
+      </c>
+      <c r="N927" t="n">
+        <v>124</v>
+      </c>
+      <c r="O927" t="n">
+        <v>25</v>
+      </c>
+      <c r="P927" t="inlineStr"/>
+      <c r="R927" t="inlineStr">
+        <is>
+          <t>7.3.1</t>
+        </is>
+      </c>
+      <c r="S927" t="inlineStr">
+        <is>
+          <t>A free mobile self-care application for Orange Botswana’s mobile customers.
+Full Description :
+Max it is a free application, which allows Orange Botswana customers to:
+- Consult your account in real time: minutes, sms, internet ...
+- Top up your account or a friend account  with Orange Money
+-</t>
+        </is>
+      </c>
+      <c r="T927" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U927" t="inlineStr"/>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D928" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E928" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F928" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G928" t="inlineStr">
+        <is>
+          <t>com.orange.mobinilandme</t>
+        </is>
+      </c>
+      <c r="H928" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I928" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J928" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K928" t="inlineStr">
+        <is>
+          <t>EGP 0.00</t>
+        </is>
+      </c>
+      <c r="L928" t="b">
+        <v>0</v>
+      </c>
+      <c r="M928" t="n">
+        <v>4.555653</v>
+      </c>
+      <c r="N928" t="n">
+        <v>938289</v>
+      </c>
+      <c r="O928" t="n">
+        <v>19</v>
+      </c>
+      <c r="P928" t="inlineStr"/>
+      <c r="Q928" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R928" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S928" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion&lt;br&gt;Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.&lt;br&gt;Key services include:&lt;br&gt;• Account Management: Easily manage</t>
+        </is>
+      </c>
+      <c r="T928" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U928" t="inlineStr"/>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>a1ef9bdb-77d1-4802-afc2-e05a04259a39</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>2026-08-05 06:29:48</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D929" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E929" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F929" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G929" t="n">
+        <v>942568333</v>
+      </c>
+      <c r="H929" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I929" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J929" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K929" t="n">
+        <v>0</v>
+      </c>
+      <c r="L929" t="b">
+        <v>1</v>
+      </c>
+      <c r="M929" t="n">
+        <v>4.25301</v>
+      </c>
+      <c r="N929" t="n">
+        <v>119017</v>
+      </c>
+      <c r="O929" t="n">
+        <v>56</v>
+      </c>
+      <c r="P929" t="inlineStr"/>
+      <c r="R929" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S929" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion
+Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.
+Key services include:
+• Account Management: Easily manage your Ora</t>
+        </is>
+      </c>
+      <c r="T929" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U929" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-08-06
</commit_message>
<xml_diff>
--- a/maxit_store_history.xlsx
+++ b/maxit_store_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U929"/>
+  <dimension ref="A1:U961"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77281,7 +77281,6 @@
       <c r="O898" t="n">
         <v>43</v>
       </c>
-      <c r="P898" t="inlineStr"/>
       <c r="Q898" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -77302,7 +77301,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U898" t="inlineStr"/>
     </row>
     <row r="899">
       <c r="A899" t="inlineStr">
@@ -77365,7 +77363,6 @@
       <c r="N899" t="n">
         <v>338</v>
       </c>
-      <c r="P899" t="inlineStr"/>
       <c r="R899" t="inlineStr">
         <is>
           <t>6.4.12</t>
@@ -77381,7 +77378,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U899" t="inlineStr"/>
     </row>
     <row r="900">
       <c r="A900" t="inlineStr">
@@ -77451,7 +77447,6 @@
       <c r="O900" t="n">
         <v>28</v>
       </c>
-      <c r="P900" t="inlineStr"/>
       <c r="Q900" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -77472,7 +77467,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U900" t="inlineStr"/>
     </row>
     <row r="901">
       <c r="A901" t="inlineStr">
@@ -77538,7 +77532,6 @@
       <c r="O901" t="n">
         <v>40</v>
       </c>
-      <c r="P901" t="inlineStr"/>
       <c r="R901" t="inlineStr">
         <is>
           <t>10.0.7</t>
@@ -77556,7 +77549,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U901" t="inlineStr"/>
     </row>
     <row r="902">
       <c r="A902" t="inlineStr">
@@ -77626,7 +77618,6 @@
       <c r="O902" t="n">
         <v>11</v>
       </c>
-      <c r="P902" t="inlineStr"/>
       <c r="Q902" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -77647,7 +77638,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U902" t="inlineStr"/>
     </row>
     <row r="903">
       <c r="A903" t="inlineStr">
@@ -77736,7 +77726,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U903" t="inlineStr"/>
     </row>
     <row r="904">
       <c r="A904" t="inlineStr">
@@ -77806,7 +77795,6 @@
       <c r="O904" t="n">
         <v>8</v>
       </c>
-      <c r="P904" t="inlineStr"/>
       <c r="Q904" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -77827,7 +77815,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U904" t="inlineStr"/>
     </row>
     <row r="905">
       <c r="A905" t="inlineStr">
@@ -77893,7 +77880,6 @@
       <c r="O905" t="n">
         <v>12</v>
       </c>
-      <c r="P905" t="inlineStr"/>
       <c r="R905" t="inlineStr">
         <is>
           <t>22.0.1</t>
@@ -77911,7 +77897,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U905" t="inlineStr"/>
     </row>
     <row r="906">
       <c r="A906" t="inlineStr">
@@ -77981,7 +77966,6 @@
       <c r="O906" t="n">
         <v>58</v>
       </c>
-      <c r="P906" t="inlineStr"/>
       <c r="Q906" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -78002,7 +77986,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U906" t="inlineStr"/>
     </row>
     <row r="907">
       <c r="A907" t="inlineStr">
@@ -78087,7 +78070,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U907" t="inlineStr"/>
     </row>
     <row r="908">
       <c r="A908" t="inlineStr">
@@ -78154,7 +78136,6 @@
       <c r="N908" t="n">
         <v>38235</v>
       </c>
-      <c r="P908" t="inlineStr"/>
       <c r="Q908" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -78175,7 +78156,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U908" t="inlineStr"/>
     </row>
     <row r="909">
       <c r="A909" t="inlineStr">
@@ -78241,7 +78221,6 @@
       <c r="O909" t="n">
         <v>13</v>
       </c>
-      <c r="P909" t="inlineStr"/>
       <c r="R909" t="inlineStr">
         <is>
           <t>6.5.2</t>
@@ -78260,7 +78239,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U909" t="inlineStr"/>
     </row>
     <row r="910">
       <c r="A910" t="inlineStr">
@@ -78330,7 +78308,6 @@
       <c r="O910" t="n">
         <v>71</v>
       </c>
-      <c r="P910" t="inlineStr"/>
       <c r="Q910" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -78351,7 +78328,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U910" t="inlineStr"/>
     </row>
     <row r="911">
       <c r="A911" t="inlineStr">
@@ -78417,7 +78393,6 @@
       <c r="O911" t="n">
         <v>20</v>
       </c>
-      <c r="P911" t="inlineStr"/>
       <c r="R911" t="inlineStr">
         <is>
           <t>5.0.2</t>
@@ -78435,7 +78410,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U911" t="inlineStr"/>
     </row>
     <row r="912">
       <c r="A912" t="inlineStr">
@@ -78505,7 +78479,6 @@
       <c r="O912" t="n">
         <v>73</v>
       </c>
-      <c r="P912" t="inlineStr"/>
       <c r="Q912" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -78526,7 +78499,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U912" t="inlineStr"/>
     </row>
     <row r="913">
       <c r="A913" t="inlineStr">
@@ -78614,7 +78586,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U913" t="inlineStr"/>
     </row>
     <row r="914">
       <c r="A914" t="inlineStr">
@@ -78684,7 +78655,6 @@
       <c r="O914" t="n">
         <v>45</v>
       </c>
-      <c r="P914" t="inlineStr"/>
       <c r="Q914" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -78705,7 +78675,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U914" t="inlineStr"/>
     </row>
     <row r="915">
       <c r="A915" t="inlineStr">
@@ -78771,7 +78740,6 @@
       <c r="O915" t="n">
         <v>46</v>
       </c>
-      <c r="P915" t="inlineStr"/>
       <c r="R915" t="inlineStr">
         <is>
           <t>10.0.21</t>
@@ -78790,7 +78758,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U915" t="inlineStr"/>
     </row>
     <row r="916">
       <c r="A916" t="inlineStr">
@@ -78860,7 +78827,6 @@
       <c r="O916" t="n">
         <v>13</v>
       </c>
-      <c r="P916" t="inlineStr"/>
       <c r="Q916" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -78881,7 +78847,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U916" t="inlineStr"/>
     </row>
     <row r="917">
       <c r="A917" t="inlineStr">
@@ -78967,7 +78932,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U917" t="inlineStr"/>
     </row>
     <row r="918">
       <c r="A918" t="inlineStr">
@@ -79037,7 +79001,6 @@
       <c r="O918" t="n">
         <v>4</v>
       </c>
-      <c r="P918" t="inlineStr"/>
       <c r="Q918" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -79058,7 +79021,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U918" t="inlineStr"/>
     </row>
     <row r="919">
       <c r="A919" t="inlineStr">
@@ -79144,7 +79106,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U919" t="inlineStr"/>
     </row>
     <row r="920">
       <c r="A920" t="inlineStr">
@@ -79214,7 +79175,6 @@
       <c r="O920" t="n">
         <v>114</v>
       </c>
-      <c r="P920" t="inlineStr"/>
       <c r="Q920" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -79235,7 +79195,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U920" t="inlineStr"/>
     </row>
     <row r="921">
       <c r="A921" t="inlineStr">
@@ -79318,7 +79277,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U921" t="inlineStr"/>
     </row>
     <row r="922">
       <c r="A922" t="inlineStr">
@@ -79388,7 +79346,6 @@
       <c r="O922" t="n">
         <v>13</v>
       </c>
-      <c r="P922" t="inlineStr"/>
       <c r="Q922" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -79409,7 +79366,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U922" t="inlineStr"/>
     </row>
     <row r="923">
       <c r="A923" t="inlineStr">
@@ -79498,7 +79454,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U923" t="inlineStr"/>
     </row>
     <row r="924">
       <c r="A924" t="inlineStr">
@@ -79568,7 +79523,6 @@
       <c r="O924" t="n">
         <v>12</v>
       </c>
-      <c r="P924" t="inlineStr"/>
       <c r="Q924" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -79589,7 +79543,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U924" t="inlineStr"/>
     </row>
     <row r="925">
       <c r="A925" t="inlineStr">
@@ -79676,7 +79629,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U925" t="inlineStr"/>
     </row>
     <row r="926">
       <c r="A926" t="inlineStr">
@@ -79746,7 +79698,6 @@
       <c r="O926" t="n">
         <v>37</v>
       </c>
-      <c r="P926" t="inlineStr"/>
       <c r="Q926" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -79767,7 +79718,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U926" t="inlineStr"/>
     </row>
     <row r="927">
       <c r="A927" t="inlineStr">
@@ -79833,7 +79783,6 @@
       <c r="O927" t="n">
         <v>25</v>
       </c>
-      <c r="P927" t="inlineStr"/>
       <c r="R927" t="inlineStr">
         <is>
           <t>7.3.1</t>
@@ -79854,7 +79803,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U927" t="inlineStr"/>
     </row>
     <row r="928">
       <c r="A928" t="inlineStr">
@@ -79924,7 +79872,6 @@
       <c r="O928" t="n">
         <v>19</v>
       </c>
-      <c r="P928" t="inlineStr"/>
       <c r="Q928" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -79945,7 +79892,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U928" t="inlineStr"/>
     </row>
     <row r="929">
       <c r="A929" t="inlineStr">
@@ -80011,7 +79957,6 @@
       <c r="O929" t="n">
         <v>56</v>
       </c>
-      <c r="P929" t="inlineStr"/>
       <c r="R929" t="inlineStr">
         <is>
           <t>10.1.0</t>
@@ -80030,7 +79975,2825 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U929" t="inlineStr"/>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D930" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E930" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F930" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G930" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogn</t>
+        </is>
+      </c>
+      <c r="H930" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I930" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J930" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K930" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L930" t="b">
+        <v>0</v>
+      </c>
+      <c r="M930" t="n">
+        <v>4.4439607</v>
+      </c>
+      <c r="N930" t="n">
+        <v>9406</v>
+      </c>
+      <c r="O930" t="n">
+        <v>43</v>
+      </c>
+      <c r="P930" t="inlineStr"/>
+      <c r="Q930" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R930" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S930" t="inlineStr">
+        <is>
+          <t>Bien plus qu&amp;#39;une application, un véritable assistant personnel pour une vie connectée et simplifiée.&lt;br&gt;Suivi de consommation: Votre tableau de bord tout-en-un pour une gestion simplifiée !&lt;br&gt;- Gestion de votre offre: Accédez à une vue détaillée de votre offre actuelle et de vos forfaits Orange</t>
+        </is>
+      </c>
+      <c r="T930" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U930" t="inlineStr"/>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D931" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E931" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F931" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G931" t="n">
+        <v>1177999485</v>
+      </c>
+      <c r="H931" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I931" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J931" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K931" t="n">
+        <v>0</v>
+      </c>
+      <c r="L931" t="b">
+        <v>1</v>
+      </c>
+      <c r="M931" t="n">
+        <v>3.90909</v>
+      </c>
+      <c r="N931" t="n">
+        <v>341</v>
+      </c>
+      <c r="P931" t="inlineStr"/>
+      <c r="R931" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S931" t="inlineStr">
+        <is>
+          <t>La fusion d’Orange et Moi et Orange Money donne naissance à Max it, la nouvelle Super Application Tout-en-Un. Profitez du suivi de consommation, de paiements mobiles, de toutes les fonctionnalités Orange et Moi et Money avec un large éventail de divertissements, le tout regroupé en un seul endroit !</t>
+        </is>
+      </c>
+      <c r="T931" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U931" t="inlineStr"/>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D932" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E932" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F932" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G932" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.otn</t>
+        </is>
+      </c>
+      <c r="H932" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I932" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J932" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K932" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L932" t="b">
+        <v>0</v>
+      </c>
+      <c r="M932" t="n">
+        <v>3.9649227</v>
+      </c>
+      <c r="N932" t="n">
+        <v>35392</v>
+      </c>
+      <c r="O932" t="n">
+        <v>34</v>
+      </c>
+      <c r="P932" t="inlineStr"/>
+      <c r="Q932" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R932" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S932" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Max it par Orange Tunisie facilite votre vie au quotidien !&lt;/h2&gt;&lt;br&gt;&lt;br&gt;Welcome sur Max it !&lt;br&gt;Accédez rapidement à vos fonctionnalités Max it préférées et profitez également de contenus exclusifs, d’activités divertissantes, et de jeux interactifs pour une expérience enrichissante avec la roue</t>
+        </is>
+      </c>
+      <c r="T932" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U932" t="inlineStr"/>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D933" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E933" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F933" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G933" t="n">
+        <v>1146892088</v>
+      </c>
+      <c r="H933" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I933" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J933" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K933" t="n">
+        <v>0</v>
+      </c>
+      <c r="L933" t="b">
+        <v>1</v>
+      </c>
+      <c r="M933" t="n">
+        <v>3.028</v>
+      </c>
+      <c r="N933" t="n">
+        <v>1643</v>
+      </c>
+      <c r="O933" t="n">
+        <v>40</v>
+      </c>
+      <c r="P933" t="inlineStr"/>
+      <c r="R933" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S933" t="inlineStr">
+        <is>
+          <t>Max it by Orange Tunisie : Votre appli incontournable pour une vie connectée
+Welcome sur Max it : Découvrez fonctionnalités, jeux &amp; contenus de divertissement by Orange Tunisie !
+Trouvez vite vos fonctionnalités Max it favorites et explorez des contenus exclusifs et des jeux pour une expérience im</t>
+        </is>
+      </c>
+      <c r="T933" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U933" t="inlineStr"/>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D934" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E934" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F934" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G934" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osl</t>
+        </is>
+      </c>
+      <c r="H934" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I934" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J934" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K934" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L934" t="b">
+        <v>0</v>
+      </c>
+      <c r="M934" t="n">
+        <v>4.392694</v>
+      </c>
+      <c r="N934" t="n">
+        <v>2184</v>
+      </c>
+      <c r="O934" t="n">
+        <v>12</v>
+      </c>
+      <c r="P934" t="inlineStr"/>
+      <c r="Q934" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R934" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S934" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it is a free application, which allows Orange Sierra Leone prepaid and postpaid customers to:&lt;br&gt;&lt;br&gt;- Consult your account in real time: minutes, sms, internet&lt;br&gt;- Top up your account or a friend account &lt;br&gt;- Buy Internet Bundles&lt;br&gt;- Discover the latest offers and promotions &lt;br&gt;- Access to </t>
+        </is>
+      </c>
+      <c r="T934" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U934" t="inlineStr"/>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D935" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E935" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F935" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G935" t="n">
+        <v>6443607903</v>
+      </c>
+      <c r="H935" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I935" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J935" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K935" t="n">
+        <v>0</v>
+      </c>
+      <c r="L935" t="b">
+        <v>1</v>
+      </c>
+      <c r="M935" t="n">
+        <v>3.69072</v>
+      </c>
+      <c r="N935" t="n">
+        <v>194</v>
+      </c>
+      <c r="O935" t="n">
+        <v>8</v>
+      </c>
+      <c r="P935" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R935" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S935" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The merger of My Orange &amp; Orange Money has given birth to Max it the all-in-one super app, a free application which allows all Orange Sierra Leone customers to 
+Track calls, SMS, and Data usage and monitor balance. 
+Make a secure mobile/Orange Money payment.
+Easily transfer credit to other users </t>
+        </is>
+      </c>
+      <c r="T935" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U935" t="inlineStr"/>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D936" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E936" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F936" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G936" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osn</t>
+        </is>
+      </c>
+      <c r="H936" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I936" t="inlineStr">
+        <is>
+          <t>Orange Sénégal</t>
+        </is>
+      </c>
+      <c r="J936" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K936" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L936" t="b">
+        <v>0</v>
+      </c>
+      <c r="M936" t="n">
+        <v>4.2948585</v>
+      </c>
+      <c r="N936" t="n">
+        <v>51405</v>
+      </c>
+      <c r="O936" t="n">
+        <v>12</v>
+      </c>
+      <c r="P936" t="inlineStr"/>
+      <c r="Q936" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R936" t="inlineStr">
+        <is>
+          <t>22.0.1</t>
+        </is>
+      </c>
+      <c r="S936" t="inlineStr">
+        <is>
+          <t>Lu bees ak Max it ! &lt;br&gt;Une application repensée pour être plus simple, plus rapide et adaptée à vos besoins. Une expérience optimisée pour faciliter vos usages au quotidien, avec des parcours simplifiés et un accès plus fluide à vos services. Que vous soyez client Orange ou non, Max it vous accompa</t>
+        </is>
+      </c>
+      <c r="T936" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U936" t="inlineStr"/>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D937" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E937" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F937" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G937" t="n">
+        <v>1039327980</v>
+      </c>
+      <c r="H937" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I937" t="inlineStr">
+        <is>
+          <t>Orange Senegal</t>
+        </is>
+      </c>
+      <c r="J937" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K937" t="n">
+        <v>0</v>
+      </c>
+      <c r="L937" t="b">
+        <v>1</v>
+      </c>
+      <c r="M937" t="n">
+        <v>4.16909</v>
+      </c>
+      <c r="N937" t="n">
+        <v>30245</v>
+      </c>
+      <c r="O937" t="n">
+        <v>13</v>
+      </c>
+      <c r="P937" t="inlineStr"/>
+      <c r="R937" t="inlineStr">
+        <is>
+          <t>22.0.1</t>
+        </is>
+      </c>
+      <c r="S937" t="inlineStr">
+        <is>
+          <t>Here is the English translation:
+Welcome to Max it!
+A redesigned app to be simpler, faster, and tailored to your needs. An optimized experience to make your daily life easier, with streamlined journeys and smoother access to your services. Whether you are an Orange customer or not, Max it is your e</t>
+        </is>
+      </c>
+      <c r="T937" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U937" t="inlineStr"/>
+    </row>
+    <row r="938">
+      <c r="A938" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D938" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E938" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F938" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G938" t="inlineStr">
+        <is>
+          <t>com.orange.meditel.mediteletmoi</t>
+        </is>
+      </c>
+      <c r="H938" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I938" t="inlineStr">
+        <is>
+          <t>Orange Maroc</t>
+        </is>
+      </c>
+      <c r="J938" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K938" t="inlineStr">
+        <is>
+          <t>MAD 0.00</t>
+        </is>
+      </c>
+      <c r="L938" t="b">
+        <v>0</v>
+      </c>
+      <c r="M938" t="n">
+        <v>3.7168324</v>
+      </c>
+      <c r="N938" t="n">
+        <v>110966</v>
+      </c>
+      <c r="O938" t="n">
+        <v>72</v>
+      </c>
+      <c r="P938" t="inlineStr"/>
+      <c r="Q938" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R938" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S938" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l&amp;#39;expérience mobile réinventé&lt;br&gt;&lt;br&gt;Max it, c&amp;#39;est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d&amp;#39;une multitude de services exclusifs. &lt;br&gt;&lt;br&gt;Créez votre espace sur</t>
+        </is>
+      </c>
+      <c r="T938" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U938" t="inlineStr"/>
+    </row>
+    <row r="939">
+      <c r="A939" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D939" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E939" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F939" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G939" t="n">
+        <v>596028698</v>
+      </c>
+      <c r="H939" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I939" t="inlineStr">
+        <is>
+          <t>Méditel</t>
+        </is>
+      </c>
+      <c r="J939" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K939" t="n">
+        <v>0</v>
+      </c>
+      <c r="L939" t="b">
+        <v>1</v>
+      </c>
+      <c r="M939" t="n">
+        <v>3.94284</v>
+      </c>
+      <c r="N939" t="n">
+        <v>2764</v>
+      </c>
+      <c r="P939" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "MA" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R939" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S939" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l'expérience mobile réinventé
+Max it, c'est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d'une multitude de services exclusifs. 
+Créez votre espace sur mesure et bénéficiez d'</t>
+        </is>
+      </c>
+      <c r="T939" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U939" t="inlineStr"/>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D940" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E940" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F940" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G940" t="inlineStr">
+        <is>
+          <t>com.oml.dsi.orangemobile</t>
+        </is>
+      </c>
+      <c r="H940" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I940" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J940" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K940" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L940" t="b">
+        <v>0</v>
+      </c>
+      <c r="M940" t="n">
+        <v>2.7094083</v>
+      </c>
+      <c r="N940" t="n">
+        <v>38236</v>
+      </c>
+      <c r="P940" t="inlineStr"/>
+      <c r="Q940" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R940" t="inlineStr">
+        <is>
+          <t>6.5.0</t>
+        </is>
+      </c>
+      <c r="S940" t="inlineStr">
+        <is>
+          <t>Easily manage your Orange Mali line&lt;br&gt;● Manage your account and view all essential information, your offers, and your phone lines.&lt;br&gt;● Subscribe to call, SMS, Internet, and international call packages.&lt;br&gt;● Track your usage by checking your credit and Internet balance.&lt;br&gt;● Recharge your line by p</t>
+        </is>
+      </c>
+      <c r="T940" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U940" t="inlineStr"/>
+    </row>
+    <row r="941">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D941" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E941" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F941" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G941" t="n">
+        <v>1494321079</v>
+      </c>
+      <c r="H941" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I941" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J941" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K941" t="n">
+        <v>0</v>
+      </c>
+      <c r="L941" t="b">
+        <v>1</v>
+      </c>
+      <c r="M941" t="n">
+        <v>2.52518</v>
+      </c>
+      <c r="N941" t="n">
+        <v>4766</v>
+      </c>
+      <c r="O941" t="n">
+        <v>11</v>
+      </c>
+      <c r="P941" t="inlineStr"/>
+      <c r="R941" t="inlineStr">
+        <is>
+          <t>6.5.2</t>
+        </is>
+      </c>
+      <c r="S941" t="inlineStr">
+        <is>
+          <t>Gérez facilement votre ligne Orange Mali 
+●        Gérez votre compte et consultez toutes les informations essentielles sur celui-ci, vos offres, ainsi que vos lignes téléphoniques.
+●        Souscrivez aux forfaits appels, SMS, Internet, et appels internationaux.
+●        Suivez votre consommation e</t>
+        </is>
+      </c>
+      <c r="T941" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U941" t="inlineStr"/>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D942" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E942" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F942" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G942" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.omg</t>
+        </is>
+      </c>
+      <c r="H942" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I942" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J942" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K942" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L942" t="b">
+        <v>0</v>
+      </c>
+      <c r="M942" t="n">
+        <v>4.1594205</v>
+      </c>
+      <c r="N942" t="n">
+        <v>1393</v>
+      </c>
+      <c r="O942" t="n">
+        <v>76</v>
+      </c>
+      <c r="P942" t="inlineStr"/>
+      <c r="Q942" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R942" t="inlineStr">
+        <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="S942" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.&lt;br&gt;&lt;br&gt;Simplify Your Life with Max it&lt;br&gt;With Max It, ac</t>
+        </is>
+      </c>
+      <c r="T942" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U942" t="inlineStr"/>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D943" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E943" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F943" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G943" t="n">
+        <v>1295171817</v>
+      </c>
+      <c r="H943" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I943" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J943" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K943" t="n">
+        <v>0</v>
+      </c>
+      <c r="L943" t="b">
+        <v>1</v>
+      </c>
+      <c r="M943" t="n">
+        <v>3.05714</v>
+      </c>
+      <c r="N943" t="n">
+        <v>70</v>
+      </c>
+      <c r="O943" t="n">
+        <v>22</v>
+      </c>
+      <c r="P943" t="inlineStr"/>
+      <c r="R943" t="inlineStr">
+        <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="S943" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.
+Simplify Your Life with Max it
+With Max it, access a se</t>
+        </is>
+      </c>
+      <c r="T943" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U943" t="inlineStr"/>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D944" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E944" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F944" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G944" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.olr</t>
+        </is>
+      </c>
+      <c r="H944" t="inlineStr">
+        <is>
+          <t>Orange Max it - Liberia</t>
+        </is>
+      </c>
+      <c r="I944" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J944" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K944" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L944" t="b">
+        <v>0</v>
+      </c>
+      <c r="M944" t="n">
+        <v>4.532051</v>
+      </c>
+      <c r="N944" t="n">
+        <v>3116</v>
+      </c>
+      <c r="O944" t="n">
+        <v>76</v>
+      </c>
+      <c r="P944" t="inlineStr"/>
+      <c r="Q944" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R944" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="S944" t="inlineStr">
+        <is>
+          <t>Max it: your personalized experience by Orange Liberia!&lt;br&gt;&lt;br&gt;Step into Max it, your all-in-one solution for telecom, marketplace, and financial services! Manage your mobile line, customize offers, pay your bills, keep&lt;br&gt;track of your usage with ease, and recharge your credit. Access exclusive eve</t>
+        </is>
+      </c>
+      <c r="T944" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U944" t="inlineStr"/>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D945" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E945" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F945" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G945" t="n">
+        <v>6746187327</v>
+      </c>
+      <c r="H945" t="inlineStr">
+        <is>
+          <t>Orange Max it – Liberia</t>
+        </is>
+      </c>
+      <c r="I945" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J945" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K945" t="n">
+        <v>0</v>
+      </c>
+      <c r="L945" t="b">
+        <v>1</v>
+      </c>
+      <c r="M945" t="n">
+        <v>4.0625</v>
+      </c>
+      <c r="N945" t="n">
+        <v>48</v>
+      </c>
+      <c r="P945" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "LR" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R945" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="S945" t="inlineStr">
+        <is>
+          <t>Max it is a free application, which allows Orange Liberia customers to:
+- Consult your account in real time: minutes, sms, internet
+- Top up your account or a friend account 
+- Buy  Bundles (voice, data, SMS, roaming, international)
+- Discover the latest offers and promotions 
+- Access to Orange se</t>
+        </is>
+      </c>
+      <c r="T945" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U945" t="inlineStr"/>
+    </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D946" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E946" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F946" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G946" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ojo</t>
+        </is>
+      </c>
+      <c r="H946" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I946" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J946" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K946" t="inlineStr">
+        <is>
+          <t>JOD 0.000</t>
+        </is>
+      </c>
+      <c r="L946" t="b">
+        <v>0</v>
+      </c>
+      <c r="M946" t="n">
+        <v>4.429194</v>
+      </c>
+      <c r="N946" t="n">
+        <v>97943</v>
+      </c>
+      <c r="O946" t="n">
+        <v>50</v>
+      </c>
+      <c r="P946" t="inlineStr"/>
+      <c r="Q946" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R946" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S946" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience&lt;br&gt;Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.&lt;br&gt;Important Update:&lt;br&gt;The jood app (jood Orange) w</t>
+        </is>
+      </c>
+      <c r="T946" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U946" t="inlineStr"/>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D947" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E947" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F947" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G947" t="n">
+        <v>808824590</v>
+      </c>
+      <c r="H947" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I947" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J947" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K947" t="n">
+        <v>0</v>
+      </c>
+      <c r="L947" t="b">
+        <v>1</v>
+      </c>
+      <c r="M947" t="n">
+        <v>4.20594</v>
+      </c>
+      <c r="N947" t="n">
+        <v>3098</v>
+      </c>
+      <c r="O947" t="n">
+        <v>50</v>
+      </c>
+      <c r="P947" t="inlineStr"/>
+      <c r="R947" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S947" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience
+Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.
+Important Update:
+The jood app (jood Orange) will be di</t>
+        </is>
+      </c>
+      <c r="T947" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U947" t="inlineStr"/>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D948" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E948" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F948" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G948" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.oci</t>
+        </is>
+      </c>
+      <c r="H948" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I948" t="inlineStr">
+        <is>
+          <t>Orange Côte d'Ivoire S.A</t>
+        </is>
+      </c>
+      <c r="J948" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K948" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L948" t="b">
+        <v>0</v>
+      </c>
+      <c r="M948" t="n">
+        <v>4.142073</v>
+      </c>
+      <c r="N948" t="n">
+        <v>67441</v>
+      </c>
+      <c r="O948" t="n">
+        <v>12</v>
+      </c>
+      <c r="P948" t="inlineStr"/>
+      <c r="Q948" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R948" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S948" t="inlineStr">
+        <is>
+          <t>Aaaahhh, ta super app Max it, n&amp;#39;a pas fini de te surprendre... &lt;br&gt;Est-ce que tu as remarqué ? Maintenant, tu as ton QR code personnalisé en haut de ton écran d&amp;#39;accueil ! Ainsi, tu peux :&lt;br&gt;     scanner le QR code de ton ami(e) pour lui faire un transfert d&amp;#39;&amp;#39;argent&lt;br&gt;     scanner l</t>
+        </is>
+      </c>
+      <c r="T948" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U948" t="inlineStr"/>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D949" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E949" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F949" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G949" t="n">
+        <v>1061120855</v>
+      </c>
+      <c r="H949" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I949" t="inlineStr">
+        <is>
+          <t>Orange CI</t>
+        </is>
+      </c>
+      <c r="J949" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K949" t="n">
+        <v>0</v>
+      </c>
+      <c r="L949" t="b">
+        <v>1</v>
+      </c>
+      <c r="M949" t="n">
+        <v>3.78637</v>
+      </c>
+      <c r="N949" t="n">
+        <v>5987</v>
+      </c>
+      <c r="O949" t="n">
+        <v>4</v>
+      </c>
+      <c r="P949" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R949" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S949" t="inlineStr">
+        <is>
+          <t>Max it, la super app all-in-one te fais gagner du temps, et diminue tes soucis... Gagne plus d'espace de stockage sur ton téléphone ; plus besoin de cumuler plusieurs appli d'Orange pour avoir accès à un maximum de services. Max it est là ! Gère ta ligne (SIM) au niveau des pass, des soldes, réalise</t>
+        </is>
+      </c>
+      <c r="T949" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U949" t="inlineStr"/>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D950" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E950" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F950" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G950" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogw</t>
+        </is>
+      </c>
+      <c r="H950" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I950" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J950" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K950" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L950" t="b">
+        <v>0</v>
+      </c>
+      <c r="M950" t="n">
+        <v>4.428571</v>
+      </c>
+      <c r="N950" t="n">
+        <v>1557</v>
+      </c>
+      <c r="O950" t="n">
+        <v>8</v>
+      </c>
+      <c r="P950" t="inlineStr"/>
+      <c r="Q950" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R950" t="inlineStr">
+        <is>
+          <t>4.0.18</t>
+        </is>
+      </c>
+      <c r="S950" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T950" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U950" t="inlineStr"/>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D951" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E951" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F951" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G951" t="n">
+        <v>1574668652</v>
+      </c>
+      <c r="H951" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I951" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J951" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K951" t="n">
+        <v>0</v>
+      </c>
+      <c r="L951" t="b">
+        <v>1</v>
+      </c>
+      <c r="M951" t="n">
+        <v>4.01316</v>
+      </c>
+      <c r="N951" t="n">
+        <v>76</v>
+      </c>
+      <c r="O951" t="n">
+        <v>1</v>
+      </c>
+      <c r="P951" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R951" t="inlineStr">
+        <is>
+          <t>6.0.35</t>
+        </is>
+      </c>
+      <c r="S951" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T951" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U951" t="inlineStr"/>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D952" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E952" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F952" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G952" t="inlineStr">
+        <is>
+          <t>com.orange.sugu.ocd</t>
+        </is>
+      </c>
+      <c r="H952" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I952" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J952" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K952" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L952" t="b">
+        <v>0</v>
+      </c>
+      <c r="M952" t="n">
+        <v>4.1660447</v>
+      </c>
+      <c r="N952" t="n">
+        <v>5345</v>
+      </c>
+      <c r="O952" t="n">
+        <v>120</v>
+      </c>
+      <c r="P952" t="inlineStr"/>
+      <c r="Q952" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R952" t="inlineStr">
+        <is>
+          <t>9.0.12</t>
+        </is>
+      </c>
+      <c r="S952" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DRC that brings together the features of MyOrange, and Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Plans, Mobile Payments, money transfers, bill payments, subscriptions, and entertai</t>
+        </is>
+      </c>
+      <c r="T952" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U952" t="inlineStr"/>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D953" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E953" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F953" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G953" t="n">
+        <v>6447896435</v>
+      </c>
+      <c r="H953" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I953" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J953" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K953" t="n">
+        <v>0</v>
+      </c>
+      <c r="L953" t="b">
+        <v>1</v>
+      </c>
+      <c r="M953" t="n">
+        <v>3.55351</v>
+      </c>
+      <c r="N953" t="n">
+        <v>271</v>
+      </c>
+      <c r="P953" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "CD" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R953" t="inlineStr">
+        <is>
+          <t>9.0.6</t>
+        </is>
+      </c>
+      <c r="S953" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DR Congo. It brings together the features of Orange et Moi, as well as Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Packages, Mobile payment, money transfers, bill payment and subscri</t>
+        </is>
+      </c>
+      <c r="T953" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U953" t="inlineStr"/>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D954" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E954" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F954" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G954" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ocm</t>
+        </is>
+      </c>
+      <c r="H954" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroon</t>
+        </is>
+      </c>
+      <c r="I954" t="inlineStr">
+        <is>
+          <t>Orange MEA</t>
+        </is>
+      </c>
+      <c r="J954" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K954" t="inlineStr">
+        <is>
+          <t>FCFA 0</t>
+        </is>
+      </c>
+      <c r="L954" t="b">
+        <v>0</v>
+      </c>
+      <c r="M954" t="n">
+        <v>3.9150743</v>
+      </c>
+      <c r="N954" t="n">
+        <v>47204</v>
+      </c>
+      <c r="O954" t="n">
+        <v>13</v>
+      </c>
+      <c r="P954" t="inlineStr"/>
+      <c r="Q954" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R954" t="inlineStr">
+        <is>
+          <t>7.0.23</t>
+        </is>
+      </c>
+      <c r="S954" t="inlineStr">
+        <is>
+          <t>Max it brings together everything that matters to you in one app: managing your lines, money transfer, bill payment, exclusive offers, and a universe of lifestyle and entertainment. Simple, fast, and 100% secure..&lt;br&gt;&lt;br&gt;📞 My line&lt;br&gt;Manage your Orange mobile and landline bundles in a single click:</t>
+        </is>
+      </c>
+      <c r="T954" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U954" t="inlineStr"/>
+    </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D955" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E955" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F955" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G955" t="n">
+        <v>1116920093</v>
+      </c>
+      <c r="H955" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroun</t>
+        </is>
+      </c>
+      <c r="I955" t="inlineStr">
+        <is>
+          <t>Orange Middle East &amp; Africa</t>
+        </is>
+      </c>
+      <c r="J955" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K955" t="n">
+        <v>0</v>
+      </c>
+      <c r="L955" t="b">
+        <v>1</v>
+      </c>
+      <c r="M955" t="n">
+        <v>3.76781</v>
+      </c>
+      <c r="N955" t="n">
+        <v>16181</v>
+      </c>
+      <c r="O955" t="n">
+        <v>6</v>
+      </c>
+      <c r="P955" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R955" t="inlineStr">
+        <is>
+          <t>7.0.24</t>
+        </is>
+      </c>
+      <c r="S955" t="inlineStr">
+        <is>
+          <t>Avec Max it, Orange rassemble tout ce qui compte pour vous dans une même application : la gestion de vos lignes, les transferts d’argent, payement de vos factures, des offres exclusives et un univers lifestyle et divertissement.
+Simple, rapide et 100 % sécurisée.
+Ma ligne
+Gérez vos forfaits mobiles</t>
+        </is>
+      </c>
+      <c r="T955" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U955" t="inlineStr"/>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D956" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E956" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F956" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G956" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obf</t>
+        </is>
+      </c>
+      <c r="H956" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I956" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso</t>
+        </is>
+      </c>
+      <c r="J956" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K956" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L956" t="b">
+        <v>0</v>
+      </c>
+      <c r="M956" t="n">
+        <v>4.139852</v>
+      </c>
+      <c r="N956" t="n">
+        <v>25593</v>
+      </c>
+      <c r="O956" t="n">
+        <v>13</v>
+      </c>
+      <c r="P956" t="inlineStr"/>
+      <c r="Q956" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R956" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S956" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.&lt;br&gt;Gérez vos lignes mobiles, effectuez des transferts d&amp;#39;argent sécurisés, réglez vos factures, profitez d&amp;#39;offres exclusives, effectuez des paiements marchands fiables, et bien plus enco</t>
+        </is>
+      </c>
+      <c r="T956" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U956" t="inlineStr"/>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D957" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E957" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F957" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G957" t="n">
+        <v>1553774707</v>
+      </c>
+      <c r="H957" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I957" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso SA</t>
+        </is>
+      </c>
+      <c r="J957" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K957" t="n">
+        <v>0</v>
+      </c>
+      <c r="L957" t="b">
+        <v>1</v>
+      </c>
+      <c r="M957" t="n">
+        <v>3.46076</v>
+      </c>
+      <c r="N957" t="n">
+        <v>1185</v>
+      </c>
+      <c r="O957" t="n">
+        <v>11</v>
+      </c>
+      <c r="P957" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R957" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S957" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.
+Gérez vos lignes mobiles, effectuez des transferts d'argent sécurisés, réglez vos factures, profitez d'offres exclusives, effectuez des paiements marchands fiables, et bien plus encore, le tout</t>
+        </is>
+      </c>
+      <c r="T957" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U957" t="inlineStr"/>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D958" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E958" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F958" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G958" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obw</t>
+        </is>
+      </c>
+      <c r="H958" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I958" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J958" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K958" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L958" t="b">
+        <v>0</v>
+      </c>
+      <c r="M958" t="n">
+        <v>3.9714286</v>
+      </c>
+      <c r="N958" t="n">
+        <v>2971</v>
+      </c>
+      <c r="O958" t="n">
+        <v>47</v>
+      </c>
+      <c r="P958" t="inlineStr"/>
+      <c r="Q958" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R958" t="inlineStr">
+        <is>
+          <t>7.3.8</t>
+        </is>
+      </c>
+      <c r="S958" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it, the brand-new Orange Botswana Super App that follows Yame and gives you access to four distinct universes for a one-of-a-kind experience!&lt;br&gt;&lt;br&gt;Manage your accounts, make quick payments using QR codes, investigate a range of online goods and services, and discover the many options provided </t>
+        </is>
+      </c>
+      <c r="T958" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U958" t="inlineStr"/>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D959" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E959" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F959" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G959" t="n">
+        <v>1195839458</v>
+      </c>
+      <c r="H959" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I959" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J959" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K959" t="n">
+        <v>0</v>
+      </c>
+      <c r="L959" t="b">
+        <v>1</v>
+      </c>
+      <c r="M959" t="n">
+        <v>3.00806</v>
+      </c>
+      <c r="N959" t="n">
+        <v>124</v>
+      </c>
+      <c r="O959" t="n">
+        <v>37</v>
+      </c>
+      <c r="P959" t="inlineStr"/>
+      <c r="R959" t="inlineStr">
+        <is>
+          <t>7.3.1</t>
+        </is>
+      </c>
+      <c r="S959" t="inlineStr">
+        <is>
+          <t>A free mobile self-care application for Orange Botswana’s mobile customers.
+Full Description :
+Max it is a free application, which allows Orange Botswana customers to:
+- Consult your account in real time: minutes, sms, internet ...
+- Top up your account or a friend account  with Orange Money
+-</t>
+        </is>
+      </c>
+      <c r="T959" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U959" t="inlineStr"/>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D960" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E960" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F960" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G960" t="inlineStr">
+        <is>
+          <t>com.orange.mobinilandme</t>
+        </is>
+      </c>
+      <c r="H960" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I960" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J960" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K960" t="inlineStr">
+        <is>
+          <t>EGP 0.00</t>
+        </is>
+      </c>
+      <c r="L960" t="b">
+        <v>0</v>
+      </c>
+      <c r="M960" t="n">
+        <v>4.556035</v>
+      </c>
+      <c r="N960" t="n">
+        <v>939639</v>
+      </c>
+      <c r="O960" t="n">
+        <v>27</v>
+      </c>
+      <c r="P960" t="inlineStr"/>
+      <c r="Q960" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R960" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S960" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion&lt;br&gt;Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.&lt;br&gt;Key services include:&lt;br&gt;• Account Management: Easily manage</t>
+        </is>
+      </c>
+      <c r="T960" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U960" t="inlineStr"/>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>42947182-69b2-451a-89a2-b3ff1898532c</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>2026-08-06 06:32:40</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D961" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E961" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F961" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G961" t="n">
+        <v>942568333</v>
+      </c>
+      <c r="H961" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I961" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J961" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K961" t="n">
+        <v>0</v>
+      </c>
+      <c r="L961" t="b">
+        <v>1</v>
+      </c>
+      <c r="M961" t="n">
+        <v>4.25302</v>
+      </c>
+      <c r="N961" t="n">
+        <v>119188</v>
+      </c>
+      <c r="O961" t="n">
+        <v>51</v>
+      </c>
+      <c r="P961" t="inlineStr"/>
+      <c r="R961" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S961" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion
+Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.
+Key services include:
+• Account Management: Easily manage your Ora</t>
+        </is>
+      </c>
+      <c r="T961" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U961" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-08-07
</commit_message>
<xml_diff>
--- a/maxit_store_history.xlsx
+++ b/maxit_store_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U961"/>
+  <dimension ref="A1:U993"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -80044,7 +80044,6 @@
       <c r="O930" t="n">
         <v>43</v>
       </c>
-      <c r="P930" t="inlineStr"/>
       <c r="Q930" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -80065,7 +80064,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U930" t="inlineStr"/>
     </row>
     <row r="931">
       <c r="A931" t="inlineStr">
@@ -80128,7 +80126,6 @@
       <c r="N931" t="n">
         <v>341</v>
       </c>
-      <c r="P931" t="inlineStr"/>
       <c r="R931" t="inlineStr">
         <is>
           <t>6.4.12</t>
@@ -80144,7 +80141,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U931" t="inlineStr"/>
     </row>
     <row r="932">
       <c r="A932" t="inlineStr">
@@ -80214,7 +80210,6 @@
       <c r="O932" t="n">
         <v>34</v>
       </c>
-      <c r="P932" t="inlineStr"/>
       <c r="Q932" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -80235,7 +80230,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U932" t="inlineStr"/>
     </row>
     <row r="933">
       <c r="A933" t="inlineStr">
@@ -80301,7 +80295,6 @@
       <c r="O933" t="n">
         <v>40</v>
       </c>
-      <c r="P933" t="inlineStr"/>
       <c r="R933" t="inlineStr">
         <is>
           <t>10.0.7</t>
@@ -80319,7 +80312,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U933" t="inlineStr"/>
     </row>
     <row r="934">
       <c r="A934" t="inlineStr">
@@ -80389,7 +80381,6 @@
       <c r="O934" t="n">
         <v>12</v>
       </c>
-      <c r="P934" t="inlineStr"/>
       <c r="Q934" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -80410,7 +80401,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U934" t="inlineStr"/>
     </row>
     <row r="935">
       <c r="A935" t="inlineStr">
@@ -80499,7 +80489,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U935" t="inlineStr"/>
     </row>
     <row r="936">
       <c r="A936" t="inlineStr">
@@ -80569,7 +80558,6 @@
       <c r="O936" t="n">
         <v>12</v>
       </c>
-      <c r="P936" t="inlineStr"/>
       <c r="Q936" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -80590,7 +80578,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U936" t="inlineStr"/>
     </row>
     <row r="937">
       <c r="A937" t="inlineStr">
@@ -80656,7 +80643,6 @@
       <c r="O937" t="n">
         <v>13</v>
       </c>
-      <c r="P937" t="inlineStr"/>
       <c r="R937" t="inlineStr">
         <is>
           <t>22.0.1</t>
@@ -80674,7 +80660,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U937" t="inlineStr"/>
     </row>
     <row r="938">
       <c r="A938" t="inlineStr">
@@ -80744,7 +80729,6 @@
       <c r="O938" t="n">
         <v>72</v>
       </c>
-      <c r="P938" t="inlineStr"/>
       <c r="Q938" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -80765,7 +80749,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U938" t="inlineStr"/>
     </row>
     <row r="939">
       <c r="A939" t="inlineStr">
@@ -80850,7 +80833,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U939" t="inlineStr"/>
     </row>
     <row r="940">
       <c r="A940" t="inlineStr">
@@ -80917,7 +80899,6 @@
       <c r="N940" t="n">
         <v>38236</v>
       </c>
-      <c r="P940" t="inlineStr"/>
       <c r="Q940" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -80938,7 +80919,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U940" t="inlineStr"/>
     </row>
     <row r="941">
       <c r="A941" t="inlineStr">
@@ -81004,7 +80984,6 @@
       <c r="O941" t="n">
         <v>11</v>
       </c>
-      <c r="P941" t="inlineStr"/>
       <c r="R941" t="inlineStr">
         <is>
           <t>6.5.2</t>
@@ -81023,7 +81002,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U941" t="inlineStr"/>
     </row>
     <row r="942">
       <c r="A942" t="inlineStr">
@@ -81093,7 +81071,6 @@
       <c r="O942" t="n">
         <v>76</v>
       </c>
-      <c r="P942" t="inlineStr"/>
       <c r="Q942" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -81114,7 +81091,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U942" t="inlineStr"/>
     </row>
     <row r="943">
       <c r="A943" t="inlineStr">
@@ -81180,7 +81156,6 @@
       <c r="O943" t="n">
         <v>22</v>
       </c>
-      <c r="P943" t="inlineStr"/>
       <c r="R943" t="inlineStr">
         <is>
           <t>5.0.2</t>
@@ -81198,7 +81173,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U943" t="inlineStr"/>
     </row>
     <row r="944">
       <c r="A944" t="inlineStr">
@@ -81268,7 +81242,6 @@
       <c r="O944" t="n">
         <v>76</v>
       </c>
-      <c r="P944" t="inlineStr"/>
       <c r="Q944" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -81289,7 +81262,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U944" t="inlineStr"/>
     </row>
     <row r="945">
       <c r="A945" t="inlineStr">
@@ -81377,7 +81349,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U945" t="inlineStr"/>
     </row>
     <row r="946">
       <c r="A946" t="inlineStr">
@@ -81447,7 +81418,6 @@
       <c r="O946" t="n">
         <v>50</v>
       </c>
-      <c r="P946" t="inlineStr"/>
       <c r="Q946" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -81468,7 +81438,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U946" t="inlineStr"/>
     </row>
     <row r="947">
       <c r="A947" t="inlineStr">
@@ -81534,7 +81503,6 @@
       <c r="O947" t="n">
         <v>50</v>
       </c>
-      <c r="P947" t="inlineStr"/>
       <c r="R947" t="inlineStr">
         <is>
           <t>10.0.21</t>
@@ -81553,7 +81521,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U947" t="inlineStr"/>
     </row>
     <row r="948">
       <c r="A948" t="inlineStr">
@@ -81623,7 +81590,6 @@
       <c r="O948" t="n">
         <v>12</v>
       </c>
-      <c r="P948" t="inlineStr"/>
       <c r="Q948" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -81644,7 +81610,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U948" t="inlineStr"/>
     </row>
     <row r="949">
       <c r="A949" t="inlineStr">
@@ -81730,7 +81695,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U949" t="inlineStr"/>
     </row>
     <row r="950">
       <c r="A950" t="inlineStr">
@@ -81800,7 +81764,6 @@
       <c r="O950" t="n">
         <v>8</v>
       </c>
-      <c r="P950" t="inlineStr"/>
       <c r="Q950" t="inlineStr">
         <is>
           <t>100,000+</t>
@@ -81821,7 +81784,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U950" t="inlineStr"/>
     </row>
     <row r="951">
       <c r="A951" t="inlineStr">
@@ -81907,7 +81869,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U951" t="inlineStr"/>
     </row>
     <row r="952">
       <c r="A952" t="inlineStr">
@@ -81977,7 +81938,6 @@
       <c r="O952" t="n">
         <v>120</v>
       </c>
-      <c r="P952" t="inlineStr"/>
       <c r="Q952" t="inlineStr">
         <is>
           <t>1,000,000+</t>
@@ -81998,7 +81958,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U952" t="inlineStr"/>
     </row>
     <row r="953">
       <c r="A953" t="inlineStr">
@@ -82081,7 +82040,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U953" t="inlineStr"/>
     </row>
     <row r="954">
       <c r="A954" t="inlineStr">
@@ -82151,7 +82109,6 @@
       <c r="O954" t="n">
         <v>13</v>
       </c>
-      <c r="P954" t="inlineStr"/>
       <c r="Q954" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -82172,7 +82129,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U954" t="inlineStr"/>
     </row>
     <row r="955">
       <c r="A955" t="inlineStr">
@@ -82261,7 +82217,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U955" t="inlineStr"/>
     </row>
     <row r="956">
       <c r="A956" t="inlineStr">
@@ -82331,7 +82286,6 @@
       <c r="O956" t="n">
         <v>13</v>
       </c>
-      <c r="P956" t="inlineStr"/>
       <c r="Q956" t="inlineStr">
         <is>
           <t>5,000,000+</t>
@@ -82352,7 +82306,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U956" t="inlineStr"/>
     </row>
     <row r="957">
       <c r="A957" t="inlineStr">
@@ -82439,7 +82392,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U957" t="inlineStr"/>
     </row>
     <row r="958">
       <c r="A958" t="inlineStr">
@@ -82509,7 +82461,6 @@
       <c r="O958" t="n">
         <v>47</v>
       </c>
-      <c r="P958" t="inlineStr"/>
       <c r="Q958" t="inlineStr">
         <is>
           <t>500,000+</t>
@@ -82530,7 +82481,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U958" t="inlineStr"/>
     </row>
     <row r="959">
       <c r="A959" t="inlineStr">
@@ -82596,7 +82546,6 @@
       <c r="O959" t="n">
         <v>37</v>
       </c>
-      <c r="P959" t="inlineStr"/>
       <c r="R959" t="inlineStr">
         <is>
           <t>7.3.1</t>
@@ -82617,7 +82566,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U959" t="inlineStr"/>
     </row>
     <row r="960">
       <c r="A960" t="inlineStr">
@@ -82687,7 +82635,6 @@
       <c r="O960" t="n">
         <v>27</v>
       </c>
-      <c r="P960" t="inlineStr"/>
       <c r="Q960" t="inlineStr">
         <is>
           <t>10,000,000+</t>
@@ -82708,7 +82655,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U960" t="inlineStr"/>
     </row>
     <row r="961">
       <c r="A961" t="inlineStr">
@@ -82774,7 +82720,6 @@
       <c r="O961" t="n">
         <v>51</v>
       </c>
-      <c r="P961" t="inlineStr"/>
       <c r="R961" t="inlineStr">
         <is>
           <t>10.1.0</t>
@@ -82793,7 +82738,2825 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="U961" t="inlineStr"/>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D962" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E962" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F962" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G962" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogn</t>
+        </is>
+      </c>
+      <c r="H962" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I962" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J962" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K962" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L962" t="b">
+        <v>0</v>
+      </c>
+      <c r="M962" t="n">
+        <v>4.443478</v>
+      </c>
+      <c r="N962" t="n">
+        <v>9414</v>
+      </c>
+      <c r="O962" t="n">
+        <v>43</v>
+      </c>
+      <c r="P962" t="inlineStr"/>
+      <c r="Q962" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R962" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S962" t="inlineStr">
+        <is>
+          <t>Bien plus qu&amp;#39;une application, un véritable assistant personnel pour une vie connectée et simplifiée.&lt;br&gt;Suivi de consommation: Votre tableau de bord tout-en-un pour une gestion simplifiée !&lt;br&gt;- Gestion de votre offre: Accédez à une vue détaillée de votre offre actuelle et de vos forfaits Orange</t>
+        </is>
+      </c>
+      <c r="T962" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U962" t="inlineStr"/>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D963" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="E963" t="inlineStr">
+        <is>
+          <t>Guinée</t>
+        </is>
+      </c>
+      <c r="F963" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G963" t="n">
+        <v>1177999485</v>
+      </c>
+      <c r="H963" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinée</t>
+        </is>
+      </c>
+      <c r="I963" t="inlineStr">
+        <is>
+          <t>Orange Guinée</t>
+        </is>
+      </c>
+      <c r="J963" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K963" t="n">
+        <v>0</v>
+      </c>
+      <c r="L963" t="b">
+        <v>1</v>
+      </c>
+      <c r="M963" t="n">
+        <v>3.9186</v>
+      </c>
+      <c r="N963" t="n">
+        <v>344</v>
+      </c>
+      <c r="P963" t="inlineStr"/>
+      <c r="R963" t="inlineStr">
+        <is>
+          <t>6.4.12</t>
+        </is>
+      </c>
+      <c r="S963" t="inlineStr">
+        <is>
+          <t>La fusion d’Orange et Moi et Orange Money donne naissance à Max it, la nouvelle Super Application Tout-en-Un. Profitez du suivi de consommation, de paiements mobiles, de toutes les fonctionnalités Orange et Moi et Money avec un large éventail de divertissements, le tout regroupé en un seul endroit !</t>
+        </is>
+      </c>
+      <c r="T963" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U963" t="inlineStr"/>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D964" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E964" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F964" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G964" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.otn</t>
+        </is>
+      </c>
+      <c r="H964" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I964" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J964" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K964" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L964" t="b">
+        <v>0</v>
+      </c>
+      <c r="M964" t="n">
+        <v>3.9650266</v>
+      </c>
+      <c r="N964" t="n">
+        <v>35401</v>
+      </c>
+      <c r="O964" t="n">
+        <v>34</v>
+      </c>
+      <c r="P964" t="inlineStr"/>
+      <c r="Q964" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R964" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S964" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Max it par Orange Tunisie facilite votre vie au quotidien !&lt;/h2&gt;&lt;br&gt;&lt;br&gt;Welcome sur Max it !&lt;br&gt;Accédez rapidement à vos fonctionnalités Max it préférées et profitez également de contenus exclusifs, d’activités divertissantes, et de jeux interactifs pour une expérience enrichissante avec la roue</t>
+        </is>
+      </c>
+      <c r="T964" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U964" t="inlineStr"/>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D965" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E965" t="inlineStr">
+        <is>
+          <t>Tunisie</t>
+        </is>
+      </c>
+      <c r="F965" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G965" t="n">
+        <v>1146892088</v>
+      </c>
+      <c r="H965" t="inlineStr">
+        <is>
+          <t>Orange Max it - Tunisie</t>
+        </is>
+      </c>
+      <c r="I965" t="inlineStr">
+        <is>
+          <t>Orange Tunisie</t>
+        </is>
+      </c>
+      <c r="J965" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K965" t="n">
+        <v>0</v>
+      </c>
+      <c r="L965" t="b">
+        <v>1</v>
+      </c>
+      <c r="M965" t="n">
+        <v>3.028</v>
+      </c>
+      <c r="N965" t="n">
+        <v>1643</v>
+      </c>
+      <c r="O965" t="n">
+        <v>39</v>
+      </c>
+      <c r="P965" t="inlineStr"/>
+      <c r="R965" t="inlineStr">
+        <is>
+          <t>10.0.7</t>
+        </is>
+      </c>
+      <c r="S965" t="inlineStr">
+        <is>
+          <t>Max it by Orange Tunisie : Votre appli incontournable pour une vie connectée
+Welcome sur Max it : Découvrez fonctionnalités, jeux &amp; contenus de divertissement by Orange Tunisie !
+Trouvez vite vos fonctionnalités Max it favorites et explorez des contenus exclusifs et des jeux pour une expérience im</t>
+        </is>
+      </c>
+      <c r="T965" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U965" t="inlineStr"/>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D966" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E966" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F966" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G966" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osl</t>
+        </is>
+      </c>
+      <c r="H966" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I966" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J966" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K966" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L966" t="b">
+        <v>0</v>
+      </c>
+      <c r="M966" t="n">
+        <v>4.39819</v>
+      </c>
+      <c r="N966" t="n">
+        <v>2185</v>
+      </c>
+      <c r="O966" t="n">
+        <v>12</v>
+      </c>
+      <c r="P966" t="inlineStr"/>
+      <c r="Q966" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R966" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S966" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it is a free application, which allows Orange Sierra Leone prepaid and postpaid customers to:&lt;br&gt;&lt;br&gt;- Consult your account in real time: minutes, sms, internet&lt;br&gt;- Top up your account or a friend account &lt;br&gt;- Buy Internet Bundles&lt;br&gt;- Discover the latest offers and promotions &lt;br&gt;- Access to </t>
+        </is>
+      </c>
+      <c r="T966" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U966" t="inlineStr"/>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D967" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E967" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="F967" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G967" t="n">
+        <v>6443607903</v>
+      </c>
+      <c r="H967" t="inlineStr">
+        <is>
+          <t>Orange Max it - Sierra Leone</t>
+        </is>
+      </c>
+      <c r="I967" t="inlineStr">
+        <is>
+          <t>Orange Sierra Leone</t>
+        </is>
+      </c>
+      <c r="J967" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K967" t="n">
+        <v>0</v>
+      </c>
+      <c r="L967" t="b">
+        <v>1</v>
+      </c>
+      <c r="M967" t="n">
+        <v>3.69072</v>
+      </c>
+      <c r="N967" t="n">
+        <v>194</v>
+      </c>
+      <c r="O967" t="n">
+        <v>7</v>
+      </c>
+      <c r="P967" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R967" t="inlineStr">
+        <is>
+          <t>4.0.3</t>
+        </is>
+      </c>
+      <c r="S967" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The merger of My Orange &amp; Orange Money has given birth to Max it the all-in-one super app, a free application which allows all Orange Sierra Leone customers to 
+Track calls, SMS, and Data usage and monitor balance. 
+Make a secure mobile/Orange Money payment.
+Easily transfer credit to other users </t>
+        </is>
+      </c>
+      <c r="T967" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U967" t="inlineStr"/>
+    </row>
+    <row r="968">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D968" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E968" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F968" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G968" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.osn</t>
+        </is>
+      </c>
+      <c r="H968" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I968" t="inlineStr">
+        <is>
+          <t>Orange Sénégal</t>
+        </is>
+      </c>
+      <c r="J968" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K968" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L968" t="b">
+        <v>0</v>
+      </c>
+      <c r="M968" t="n">
+        <v>4.2972302</v>
+      </c>
+      <c r="N968" t="n">
+        <v>51431</v>
+      </c>
+      <c r="O968" t="n">
+        <v>8</v>
+      </c>
+      <c r="P968" t="inlineStr"/>
+      <c r="Q968" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R968" t="inlineStr">
+        <is>
+          <t>22.0.1</t>
+        </is>
+      </c>
+      <c r="S968" t="inlineStr">
+        <is>
+          <t>Lu bees ak Max it ! &lt;br&gt;Une application repensée pour être plus simple, plus rapide et adaptée à vos besoins. Une expérience optimisée pour faciliter vos usages au quotidien, avec des parcours simplifiés et un accès plus fluide à vos services. Que vous soyez client Orange ou non, Max it vous accompa</t>
+        </is>
+      </c>
+      <c r="T968" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U968" t="inlineStr"/>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D969" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="E969" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F969" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G969" t="n">
+        <v>1039327980</v>
+      </c>
+      <c r="H969" t="inlineStr">
+        <is>
+          <t>Orange Max it Sénégal</t>
+        </is>
+      </c>
+      <c r="I969" t="inlineStr">
+        <is>
+          <t>Orange Senegal</t>
+        </is>
+      </c>
+      <c r="J969" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K969" t="n">
+        <v>0</v>
+      </c>
+      <c r="L969" t="b">
+        <v>1</v>
+      </c>
+      <c r="M969" t="n">
+        <v>4.16896</v>
+      </c>
+      <c r="N969" t="n">
+        <v>30250</v>
+      </c>
+      <c r="O969" t="n">
+        <v>3</v>
+      </c>
+      <c r="P969" t="inlineStr"/>
+      <c r="R969" t="inlineStr">
+        <is>
+          <t>22.0.1</t>
+        </is>
+      </c>
+      <c r="S969" t="inlineStr">
+        <is>
+          <t>Here is the English translation:
+Welcome to Max it!
+A redesigned app to be simpler, faster, and tailored to your needs. An optimized experience to make your daily life easier, with streamlined journeys and smoother access to your services. Whether you are an Orange customer or not, Max it is your e</t>
+        </is>
+      </c>
+      <c r="T969" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U969" t="inlineStr"/>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D970" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E970" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F970" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G970" t="inlineStr">
+        <is>
+          <t>com.orange.meditel.mediteletmoi</t>
+        </is>
+      </c>
+      <c r="H970" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I970" t="inlineStr">
+        <is>
+          <t>Orange Maroc</t>
+        </is>
+      </c>
+      <c r="J970" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K970" t="inlineStr">
+        <is>
+          <t>MAD 0.00</t>
+        </is>
+      </c>
+      <c r="L970" t="b">
+        <v>0</v>
+      </c>
+      <c r="M970" t="n">
+        <v>3.71655</v>
+      </c>
+      <c r="N970" t="n">
+        <v>110970</v>
+      </c>
+      <c r="O970" t="n">
+        <v>78</v>
+      </c>
+      <c r="P970" t="inlineStr"/>
+      <c r="Q970" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R970" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S970" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l&amp;#39;expérience mobile réinventé&lt;br&gt;&lt;br&gt;Max it, c&amp;#39;est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d&amp;#39;une multitude de services exclusifs. &lt;br&gt;&lt;br&gt;Créez votre espace sur</t>
+        </is>
+      </c>
+      <c r="T970" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U970" t="inlineStr"/>
+    </row>
+    <row r="971">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D971" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E971" t="inlineStr">
+        <is>
+          <t>Maroc</t>
+        </is>
+      </c>
+      <c r="F971" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G971" t="n">
+        <v>596028698</v>
+      </c>
+      <c r="H971" t="inlineStr">
+        <is>
+          <t>Max it – Maroc</t>
+        </is>
+      </c>
+      <c r="I971" t="inlineStr">
+        <is>
+          <t>Méditel</t>
+        </is>
+      </c>
+      <c r="J971" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K971" t="n">
+        <v>0</v>
+      </c>
+      <c r="L971" t="b">
+        <v>1</v>
+      </c>
+      <c r="M971" t="n">
+        <v>3.94322</v>
+      </c>
+      <c r="N971" t="n">
+        <v>2765</v>
+      </c>
+      <c r="P971" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "MA" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R971" t="inlineStr">
+        <is>
+          <t>10.9.0</t>
+        </is>
+      </c>
+      <c r="S971" t="inlineStr">
+        <is>
+          <t>Max it par Orange Maroc : l'expérience mobile réinventé
+Max it, c'est votre espace Orange entièrement personnalisé. Gérez vos lignes mobiles et fixes, consultez votre consommation,payez vos factures, et profitez d'une multitude de services exclusifs. 
+Créez votre espace sur mesure et bénéficiez d'</t>
+        </is>
+      </c>
+      <c r="T971" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U971" t="inlineStr"/>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D972" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E972" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F972" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G972" t="inlineStr">
+        <is>
+          <t>com.oml.dsi.orangemobile</t>
+        </is>
+      </c>
+      <c r="H972" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I972" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J972" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K972" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L972" t="b">
+        <v>0</v>
+      </c>
+      <c r="M972" t="n">
+        <v>2.7088113</v>
+      </c>
+      <c r="N972" t="n">
+        <v>38232</v>
+      </c>
+      <c r="P972" t="inlineStr"/>
+      <c r="Q972" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R972" t="inlineStr">
+        <is>
+          <t>6.5.0</t>
+        </is>
+      </c>
+      <c r="S972" t="inlineStr">
+        <is>
+          <t>Easily manage your Orange Mali line&lt;br&gt;● Manage your account and view all essential information, your offers, and your phone lines.&lt;br&gt;● Subscribe to call, SMS, Internet, and international call packages.&lt;br&gt;● Track your usage by checking your credit and Internet balance.&lt;br&gt;● Recharge your line by p</t>
+        </is>
+      </c>
+      <c r="T972" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U972" t="inlineStr"/>
+    </row>
+    <row r="973">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D973" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E973" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F973" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G973" t="n">
+        <v>1494321079</v>
+      </c>
+      <c r="H973" t="inlineStr">
+        <is>
+          <t>Orange Max it – Mali</t>
+        </is>
+      </c>
+      <c r="I973" t="inlineStr">
+        <is>
+          <t>Orange Mali</t>
+        </is>
+      </c>
+      <c r="J973" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K973" t="n">
+        <v>0</v>
+      </c>
+      <c r="L973" t="b">
+        <v>1</v>
+      </c>
+      <c r="M973" t="n">
+        <v>2.5257</v>
+      </c>
+      <c r="N973" t="n">
+        <v>4767</v>
+      </c>
+      <c r="O973" t="n">
+        <v>11</v>
+      </c>
+      <c r="P973" t="inlineStr"/>
+      <c r="R973" t="inlineStr">
+        <is>
+          <t>6.5.2</t>
+        </is>
+      </c>
+      <c r="S973" t="inlineStr">
+        <is>
+          <t>Gérez facilement votre ligne Orange Mali 
+●        Gérez votre compte et consultez toutes les informations essentielles sur celui-ci, vos offres, ainsi que vos lignes téléphoniques.
+●        Souscrivez aux forfaits appels, SMS, Internet, et appels internationaux.
+●        Suivez votre consommation e</t>
+        </is>
+      </c>
+      <c r="T973" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U973" t="inlineStr"/>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D974" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E974" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F974" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G974" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.omg</t>
+        </is>
+      </c>
+      <c r="H974" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I974" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J974" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K974" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L974" t="b">
+        <v>0</v>
+      </c>
+      <c r="M974" t="n">
+        <v>4.1642857</v>
+      </c>
+      <c r="N974" t="n">
+        <v>1395</v>
+      </c>
+      <c r="O974" t="n">
+        <v>59</v>
+      </c>
+      <c r="P974" t="inlineStr"/>
+      <c r="Q974" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R974" t="inlineStr">
+        <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="S974" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.&lt;br&gt;&lt;br&gt;Simplify Your Life with Max it&lt;br&gt;With Max It, ac</t>
+        </is>
+      </c>
+      <c r="T974" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U974" t="inlineStr"/>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D975" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E975" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="F975" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G975" t="n">
+        <v>1295171817</v>
+      </c>
+      <c r="H975" t="inlineStr">
+        <is>
+          <t>Orange Max it - Madagascar</t>
+        </is>
+      </c>
+      <c r="I975" t="inlineStr">
+        <is>
+          <t>Orange Madagascar</t>
+        </is>
+      </c>
+      <c r="J975" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K975" t="n">
+        <v>0</v>
+      </c>
+      <c r="L975" t="b">
+        <v>1</v>
+      </c>
+      <c r="M975" t="n">
+        <v>3.05714</v>
+      </c>
+      <c r="N975" t="n">
+        <v>70</v>
+      </c>
+      <c r="O975" t="n">
+        <v>22</v>
+      </c>
+      <c r="P975" t="inlineStr"/>
+      <c r="R975" t="inlineStr">
+        <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="S975" t="inlineStr">
+        <is>
+          <t>Discover Max it, the super app that brings together all mobile and Orange Money features, offering you a unique and complete mobile experience. Save time and simplify your daily life with a multitude of services centralized in one application.
+Simplify Your Life with Max it
+With Max it, access a se</t>
+        </is>
+      </c>
+      <c r="T975" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U975" t="inlineStr"/>
+    </row>
+    <row r="976">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D976" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E976" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F976" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G976" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.olr</t>
+        </is>
+      </c>
+      <c r="H976" t="inlineStr">
+        <is>
+          <t>Orange Max it - Liberia</t>
+        </is>
+      </c>
+      <c r="I976" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J976" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K976" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L976" t="b">
+        <v>0</v>
+      </c>
+      <c r="M976" t="n">
+        <v>4.5335464</v>
+      </c>
+      <c r="N976" t="n">
+        <v>3117</v>
+      </c>
+      <c r="O976" t="n">
+        <v>58</v>
+      </c>
+      <c r="P976" t="inlineStr"/>
+      <c r="Q976" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R976" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="S976" t="inlineStr">
+        <is>
+          <t>Max it: your personalized experience by Orange Liberia!&lt;br&gt;&lt;br&gt;Step into Max it, your all-in-one solution for telecom, marketplace, and financial services! Manage your mobile line, customize offers, pay your bills, keep&lt;br&gt;track of your usage with ease, and recharge your credit. Access exclusive eve</t>
+        </is>
+      </c>
+      <c r="T976" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U976" t="inlineStr"/>
+    </row>
+    <row r="977">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D977" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="E977" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="F977" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G977" t="n">
+        <v>6746187327</v>
+      </c>
+      <c r="H977" t="inlineStr">
+        <is>
+          <t>Orange Max it – Liberia</t>
+        </is>
+      </c>
+      <c r="I977" t="inlineStr">
+        <is>
+          <t>Orange Liberia</t>
+        </is>
+      </c>
+      <c r="J977" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K977" t="n">
+        <v>0</v>
+      </c>
+      <c r="L977" t="b">
+        <v>1</v>
+      </c>
+      <c r="M977" t="n">
+        <v>4.0625</v>
+      </c>
+      <c r="N977" t="n">
+        <v>48</v>
+      </c>
+      <c r="P977" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "LR" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R977" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="S977" t="inlineStr">
+        <is>
+          <t>Max it is a free application, which allows Orange Liberia customers to:
+- Consult your account in real time: minutes, sms, internet
+- Top up your account or a friend account 
+- Buy  Bundles (voice, data, SMS, roaming, international)
+- Discover the latest offers and promotions 
+- Access to Orange se</t>
+        </is>
+      </c>
+      <c r="T977" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U977" t="inlineStr"/>
+    </row>
+    <row r="978">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D978" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E978" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F978" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G978" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ojo</t>
+        </is>
+      </c>
+      <c r="H978" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I978" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J978" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K978" t="inlineStr">
+        <is>
+          <t>JOD 0.000</t>
+        </is>
+      </c>
+      <c r="L978" t="b">
+        <v>0</v>
+      </c>
+      <c r="M978" t="n">
+        <v>4.428432</v>
+      </c>
+      <c r="N978" t="n">
+        <v>97970</v>
+      </c>
+      <c r="O978" t="n">
+        <v>56</v>
+      </c>
+      <c r="P978" t="inlineStr"/>
+      <c r="Q978" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R978" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S978" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience&lt;br&gt;Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.&lt;br&gt;Important Update:&lt;br&gt;The jood app (jood Orange) w</t>
+        </is>
+      </c>
+      <c r="T978" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U978" t="inlineStr"/>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D979" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="E979" t="inlineStr">
+        <is>
+          <t>Jordanie</t>
+        </is>
+      </c>
+      <c r="F979" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G979" t="n">
+        <v>808824590</v>
+      </c>
+      <c r="H979" t="inlineStr">
+        <is>
+          <t>Orange Max it - Jordan</t>
+        </is>
+      </c>
+      <c r="I979" t="inlineStr">
+        <is>
+          <t>Orange Jordan</t>
+        </is>
+      </c>
+      <c r="J979" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K979" t="n">
+        <v>0</v>
+      </c>
+      <c r="L979" t="b">
+        <v>1</v>
+      </c>
+      <c r="M979" t="n">
+        <v>4.20348</v>
+      </c>
+      <c r="N979" t="n">
+        <v>3106</v>
+      </c>
+      <c r="O979" t="n">
+        <v>45</v>
+      </c>
+      <c r="P979" t="inlineStr"/>
+      <c r="R979" t="inlineStr">
+        <is>
+          <t>10.0.21</t>
+        </is>
+      </c>
+      <c r="S979" t="inlineStr">
+        <is>
+          <t>Max it by Orange Jordan – Your All-in-One Digital Experience
+Max it by Orange Jordan is your new all-in-one super app, bringing together telecom services, rewards, entertainment, marketplace, and Orange Money in one simple, powerful experience.
+Important Update:
+The jood app (jood Orange) will be di</t>
+        </is>
+      </c>
+      <c r="T979" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U979" t="inlineStr"/>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D980" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E980" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F980" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G980" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.oci</t>
+        </is>
+      </c>
+      <c r="H980" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I980" t="inlineStr">
+        <is>
+          <t>Orange Côte d'Ivoire S.A</t>
+        </is>
+      </c>
+      <c r="J980" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K980" t="inlineStr">
+        <is>
+          <t>F CFA 0</t>
+        </is>
+      </c>
+      <c r="L980" t="b">
+        <v>0</v>
+      </c>
+      <c r="M980" t="n">
+        <v>4.1410103</v>
+      </c>
+      <c r="N980" t="n">
+        <v>67475</v>
+      </c>
+      <c r="O980" t="n">
+        <v>11</v>
+      </c>
+      <c r="P980" t="inlineStr"/>
+      <c r="Q980" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R980" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S980" t="inlineStr">
+        <is>
+          <t>Aaaahhh, ta super app Max it, n&amp;#39;a pas fini de te surprendre... &lt;br&gt;Est-ce que tu as remarqué ? Maintenant, tu as ton QR code personnalisé en haut de ton écran d&amp;#39;accueil ! Ainsi, tu peux :&lt;br&gt;     scanner le QR code de ton ami(e) pour lui faire un transfert d&amp;#39;&amp;#39;argent&lt;br&gt;     scanner l</t>
+        </is>
+      </c>
+      <c r="T980" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U980" t="inlineStr"/>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D981" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E981" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F981" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G981" t="n">
+        <v>1061120855</v>
+      </c>
+      <c r="H981" t="inlineStr">
+        <is>
+          <t>Orange Max it - Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="I981" t="inlineStr">
+        <is>
+          <t>Orange CI</t>
+        </is>
+      </c>
+      <c r="J981" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K981" t="n">
+        <v>0</v>
+      </c>
+      <c r="L981" t="b">
+        <v>1</v>
+      </c>
+      <c r="M981" t="n">
+        <v>3.78655</v>
+      </c>
+      <c r="N981" t="n">
+        <v>5992</v>
+      </c>
+      <c r="O981" t="n">
+        <v>6</v>
+      </c>
+      <c r="P981" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R981" t="inlineStr">
+        <is>
+          <t>10.0.33</t>
+        </is>
+      </c>
+      <c r="S981" t="inlineStr">
+        <is>
+          <t>Max it, la super app all-in-one te fais gagner du temps, et diminue tes soucis... Gagne plus d'espace de stockage sur ton téléphone ; plus besoin de cumuler plusieurs appli d'Orange pour avoir accès à un maximum de services. Max it est là ! Gère ta ligne (SIM) au niveau des pass, des soldes, réalise</t>
+        </is>
+      </c>
+      <c r="T981" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U981" t="inlineStr"/>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D982" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E982" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F982" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G982" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ogw</t>
+        </is>
+      </c>
+      <c r="H982" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I982" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J982" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K982" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L982" t="b">
+        <v>0</v>
+      </c>
+      <c r="M982" t="n">
+        <v>4.443038</v>
+      </c>
+      <c r="N982" t="n">
+        <v>1561</v>
+      </c>
+      <c r="O982" t="n">
+        <v>5</v>
+      </c>
+      <c r="P982" t="inlineStr"/>
+      <c r="Q982" t="inlineStr">
+        <is>
+          <t>100,000+</t>
+        </is>
+      </c>
+      <c r="R982" t="inlineStr">
+        <is>
+          <t>4.0.18</t>
+        </is>
+      </c>
+      <c r="S982" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T982" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U982" t="inlineStr"/>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D983" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E983" t="inlineStr">
+        <is>
+          <t>Guinée-Bissau</t>
+        </is>
+      </c>
+      <c r="F983" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G983" t="n">
+        <v>1574668652</v>
+      </c>
+      <c r="H983" t="inlineStr">
+        <is>
+          <t>Orange Max it - Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="I983" t="inlineStr">
+        <is>
+          <t>Orange Bissau</t>
+        </is>
+      </c>
+      <c r="J983" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K983" t="n">
+        <v>0</v>
+      </c>
+      <c r="L983" t="b">
+        <v>1</v>
+      </c>
+      <c r="M983" t="n">
+        <v>4.02597</v>
+      </c>
+      <c r="N983" t="n">
+        <v>77</v>
+      </c>
+      <c r="O983" t="n">
+        <v>1</v>
+      </c>
+      <c r="P983" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R983" t="inlineStr">
+        <is>
+          <t>6.0.35</t>
+        </is>
+      </c>
+      <c r="S983" t="inlineStr">
+        <is>
+          <t>Max it is your new all-in-one app from Orange Bissau. Discover the new version of the Orange Max it Guinea Bissau application, an all-in-one application that brings together all your Orange services, Orange Money and your online store with a completely new interface, even more fluid, faster and easi</t>
+        </is>
+      </c>
+      <c r="T983" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U983" t="inlineStr"/>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D984" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E984" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F984" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G984" t="inlineStr">
+        <is>
+          <t>com.orange.sugu.ocd</t>
+        </is>
+      </c>
+      <c r="H984" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I984" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J984" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K984" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="L984" t="b">
+        <v>0</v>
+      </c>
+      <c r="M984" t="n">
+        <v>4.167598</v>
+      </c>
+      <c r="N984" t="n">
+        <v>5346</v>
+      </c>
+      <c r="O984" t="n">
+        <v>107</v>
+      </c>
+      <c r="P984" t="inlineStr"/>
+      <c r="Q984" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="R984" t="inlineStr">
+        <is>
+          <t>9.0.12</t>
+        </is>
+      </c>
+      <c r="S984" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DRC that brings together the features of MyOrange, and Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Plans, Mobile Payments, money transfers, bill payments, subscriptions, and entertai</t>
+        </is>
+      </c>
+      <c r="T984" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U984" t="inlineStr"/>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D985" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="E985" t="inlineStr">
+        <is>
+          <t>RDC</t>
+        </is>
+      </c>
+      <c r="F985" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G985" t="n">
+        <v>6447896435</v>
+      </c>
+      <c r="H985" t="inlineStr">
+        <is>
+          <t>Orange Max it - RDC</t>
+        </is>
+      </c>
+      <c r="I985" t="inlineStr">
+        <is>
+          <t>Orange RD Congo</t>
+        </is>
+      </c>
+      <c r="J985" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K985" t="n">
+        <v>0</v>
+      </c>
+      <c r="L985" t="b">
+        <v>1</v>
+      </c>
+      <c r="M985" t="n">
+        <v>3.55351</v>
+      </c>
+      <c r="N985" t="n">
+        <v>271</v>
+      </c>
+      <c r="P985" t="inlineStr">
+        <is>
+          <t>Non trouvé dans le top 25 web (méthode de repli limitée à 25, pays "CD" non couvert par app-store-scraper).</t>
+        </is>
+      </c>
+      <c r="R985" t="inlineStr">
+        <is>
+          <t>9.0.6</t>
+        </is>
+      </c>
+      <c r="S985" t="inlineStr">
+        <is>
+          <t>Experience Max it: the new Super App from Orange DR Congo. It brings together the features of Orange et Moi, as well as Orange Money, for a unique experience. Max it becomes your ally to manage everything: Telephone Credit, Internet Packages, Mobile payment, money transfers, bill payment and subscri</t>
+        </is>
+      </c>
+      <c r="T985" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U985" t="inlineStr"/>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D986" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E986" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F986" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G986" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.ocm</t>
+        </is>
+      </c>
+      <c r="H986" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroon</t>
+        </is>
+      </c>
+      <c r="I986" t="inlineStr">
+        <is>
+          <t>Orange MEA</t>
+        </is>
+      </c>
+      <c r="J986" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K986" t="inlineStr">
+        <is>
+          <t>FCFA 0</t>
+        </is>
+      </c>
+      <c r="L986" t="b">
+        <v>0</v>
+      </c>
+      <c r="M986" t="n">
+        <v>3.9146729</v>
+      </c>
+      <c r="N986" t="n">
+        <v>47262</v>
+      </c>
+      <c r="O986" t="n">
+        <v>12</v>
+      </c>
+      <c r="P986" t="inlineStr"/>
+      <c r="Q986" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R986" t="inlineStr">
+        <is>
+          <t>7.0.23</t>
+        </is>
+      </c>
+      <c r="S986" t="inlineStr">
+        <is>
+          <t>Max it brings together everything that matters to you in one app: managing your lines, money transfer, bill payment, exclusive offers, and a universe of lifestyle and entertainment. Simple, fast, and 100% secure..&lt;br&gt;&lt;br&gt;📞 My line&lt;br&gt;Manage your Orange mobile and landline bundles in a single click:</t>
+        </is>
+      </c>
+      <c r="T986" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U986" t="inlineStr"/>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D987" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="E987" t="inlineStr">
+        <is>
+          <t>Cameroun</t>
+        </is>
+      </c>
+      <c r="F987" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G987" t="n">
+        <v>1116920093</v>
+      </c>
+      <c r="H987" t="inlineStr">
+        <is>
+          <t>Orange Max it - Cameroun</t>
+        </is>
+      </c>
+      <c r="I987" t="inlineStr">
+        <is>
+          <t>Orange Middle East &amp; Africa</t>
+        </is>
+      </c>
+      <c r="J987" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K987" t="n">
+        <v>0</v>
+      </c>
+      <c r="L987" t="b">
+        <v>1</v>
+      </c>
+      <c r="M987" t="n">
+        <v>3.76783</v>
+      </c>
+      <c r="N987" t="n">
+        <v>16182</v>
+      </c>
+      <c r="O987" t="n">
+        <v>6</v>
+      </c>
+      <c r="P987" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R987" t="inlineStr">
+        <is>
+          <t>7.0.24</t>
+        </is>
+      </c>
+      <c r="S987" t="inlineStr">
+        <is>
+          <t>Avec Max it, Orange rassemble tout ce qui compte pour vous dans une même application : la gestion de vos lignes, les transferts d’argent, payement de vos factures, des offres exclusives et un univers lifestyle et divertissement.
+Simple, rapide et 100 % sécurisée.
+Ma ligne
+Gérez vos forfaits mobiles</t>
+        </is>
+      </c>
+      <c r="T987" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U987" t="inlineStr"/>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D988" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E988" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F988" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G988" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obf</t>
+        </is>
+      </c>
+      <c r="H988" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I988" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso</t>
+        </is>
+      </c>
+      <c r="J988" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K988" t="inlineStr">
+        <is>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="L988" t="b">
+        <v>0</v>
+      </c>
+      <c r="M988" t="n">
+        <v>4.141966</v>
+      </c>
+      <c r="N988" t="n">
+        <v>25605</v>
+      </c>
+      <c r="O988" t="n">
+        <v>13</v>
+      </c>
+      <c r="P988" t="inlineStr"/>
+      <c r="Q988" t="inlineStr">
+        <is>
+          <t>5,000,000+</t>
+        </is>
+      </c>
+      <c r="R988" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S988" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.&lt;br&gt;Gérez vos lignes mobiles, effectuez des transferts d&amp;#39;argent sécurisés, réglez vos factures, profitez d&amp;#39;offres exclusives, effectuez des paiements marchands fiables, et bien plus enco</t>
+        </is>
+      </c>
+      <c r="T988" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U988" t="inlineStr"/>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D989" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="E989" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F989" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G989" t="n">
+        <v>1553774707</v>
+      </c>
+      <c r="H989" t="inlineStr">
+        <is>
+          <t>Orange Max it - Burkina Faso</t>
+        </is>
+      </c>
+      <c r="I989" t="inlineStr">
+        <is>
+          <t>Orange Burkina Faso SA</t>
+        </is>
+      </c>
+      <c r="J989" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K989" t="n">
+        <v>0</v>
+      </c>
+      <c r="L989" t="b">
+        <v>1</v>
+      </c>
+      <c r="M989" t="n">
+        <v>3.46076</v>
+      </c>
+      <c r="N989" t="n">
+        <v>1185</v>
+      </c>
+      <c r="O989" t="n">
+        <v>13</v>
+      </c>
+      <c r="P989" t="inlineStr">
+        <is>
+          <t>Rang obtenu via la page web des classements (méthode de repli, top 25 max), pas via app-store-scraper.</t>
+        </is>
+      </c>
+      <c r="R989" t="inlineStr">
+        <is>
+          <t>5.0.48</t>
+        </is>
+      </c>
+      <c r="S989" t="inlineStr">
+        <is>
+          <t>Max it vous offre une solution unique pour gérer votre ligne mobile, vos finances et votre divertissement.
+Gérez vos lignes mobiles, effectuez des transferts d'argent sécurisés, réglez vos factures, profitez d'offres exclusives, effectuez des paiements marchands fiables, et bien plus encore, le tout</t>
+        </is>
+      </c>
+      <c r="T989" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U989" t="inlineStr"/>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D990" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E990" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F990" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G990" t="inlineStr">
+        <is>
+          <t>com.orange.myorange.obw</t>
+        </is>
+      </c>
+      <c r="H990" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I990" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J990" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K990" t="inlineStr">
+        <is>
+          <t>US$0.00</t>
+        </is>
+      </c>
+      <c r="L990" t="b">
+        <v>0</v>
+      </c>
+      <c r="M990" t="n">
+        <v>3.967742</v>
+      </c>
+      <c r="N990" t="n">
+        <v>2970</v>
+      </c>
+      <c r="O990" t="n">
+        <v>51</v>
+      </c>
+      <c r="P990" t="inlineStr"/>
+      <c r="Q990" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="R990" t="inlineStr">
+        <is>
+          <t>7.3.8</t>
+        </is>
+      </c>
+      <c r="S990" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max it, the brand-new Orange Botswana Super App that follows Yame and gives you access to four distinct universes for a one-of-a-kind experience!&lt;br&gt;&lt;br&gt;Manage your accounts, make quick payments using QR codes, investigate a range of online goods and services, and discover the many options provided </t>
+        </is>
+      </c>
+      <c r="T990" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U990" t="inlineStr"/>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D991" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="E991" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="F991" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G991" t="n">
+        <v>1195839458</v>
+      </c>
+      <c r="H991" t="inlineStr">
+        <is>
+          <t>Orange Max it - Botswana</t>
+        </is>
+      </c>
+      <c r="I991" t="inlineStr">
+        <is>
+          <t>Orange Botswana</t>
+        </is>
+      </c>
+      <c r="J991" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K991" t="n">
+        <v>0</v>
+      </c>
+      <c r="L991" t="b">
+        <v>1</v>
+      </c>
+      <c r="M991" t="n">
+        <v>3.00806</v>
+      </c>
+      <c r="N991" t="n">
+        <v>124</v>
+      </c>
+      <c r="O991" t="n">
+        <v>31</v>
+      </c>
+      <c r="P991" t="inlineStr"/>
+      <c r="R991" t="inlineStr">
+        <is>
+          <t>7.3.1</t>
+        </is>
+      </c>
+      <c r="S991" t="inlineStr">
+        <is>
+          <t>A free mobile self-care application for Orange Botswana’s mobile customers.
+Full Description :
+Max it is a free application, which allows Orange Botswana customers to:
+- Consult your account in real time: minutes, sms, internet ...
+- Top up your account or a friend account  with Orange Money
+-</t>
+        </is>
+      </c>
+      <c r="T991" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U991" t="inlineStr"/>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D992" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E992" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F992" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="G992" t="inlineStr">
+        <is>
+          <t>com.orange.mobinilandme</t>
+        </is>
+      </c>
+      <c r="H992" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I992" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J992" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="K992" t="inlineStr">
+        <is>
+          <t>EGP 0.00</t>
+        </is>
+      </c>
+      <c r="L992" t="b">
+        <v>0</v>
+      </c>
+      <c r="M992" t="n">
+        <v>4.55614</v>
+      </c>
+      <c r="N992" t="n">
+        <v>941015</v>
+      </c>
+      <c r="O992" t="n">
+        <v>23</v>
+      </c>
+      <c r="P992" t="inlineStr"/>
+      <c r="Q992" t="inlineStr">
+        <is>
+          <t>10,000,000+</t>
+        </is>
+      </c>
+      <c r="R992" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S992" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion&lt;br&gt;Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.&lt;br&gt;Key services include:&lt;br&gt;• Account Management: Easily manage</t>
+        </is>
+      </c>
+      <c r="T992" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U992" t="inlineStr"/>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>8ada0338-46c9-4aa5-9d65-79f4a70c5fba</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>2026-08-07 05:41:17</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D993" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="E993" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="F993" t="inlineStr">
+        <is>
+          <t>ios</t>
+        </is>
+      </c>
+      <c r="G993" t="n">
+        <v>942568333</v>
+      </c>
+      <c r="H993" t="inlineStr">
+        <is>
+          <t>My Orange Egypt</t>
+        </is>
+      </c>
+      <c r="I993" t="inlineStr">
+        <is>
+          <t>Orange Egypt</t>
+        </is>
+      </c>
+      <c r="J993" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K993" t="n">
+        <v>0</v>
+      </c>
+      <c r="L993" t="b">
+        <v>1</v>
+      </c>
+      <c r="M993" t="n">
+        <v>4.25338</v>
+      </c>
+      <c r="N993" t="n">
+        <v>119368</v>
+      </c>
+      <c r="O993" t="n">
+        <v>52</v>
+      </c>
+      <c r="P993" t="inlineStr"/>
+      <c r="R993" t="inlineStr">
+        <is>
+          <t>10.1.0</t>
+        </is>
+      </c>
+      <c r="S993" t="inlineStr">
+        <is>
+          <t>My Orange Egypt and Orange Cash: Your Ultimate Orange Companion
+Both My Orange Egypt and Orange Cash offer a range of essential services, making it easier for you to manage your Orange account and enjoy seamless digital interactions.
+Key services include:
+• Account Management: Easily manage your Ora</t>
+        </is>
+      </c>
+      <c r="T993" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="U993" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>